<commit_message>
chore: clean up repo for public Streamlit Cloud deployment
- Replace 80MB monolithic rounds CSV with per-year file concat in load_rounds_all()
- Compute round_position/round_position_text at load time (cached) from per-year files
- Convert sg_production_tab live stats from file read to direct DataGolf API call
- Add git_push() to refresh_data.py; Blocks 1/2/3 auto-push updated data files
- Block 2 now saves round positions into the per-year clean CSV before pushing
- Remove raw per-tour CSVs, notebooks, IDE files, and large intermediate files from git
- Update .gitignore to permanently exclude those categories
- Add new production scripts: refresh_data.py, live_tab.py, refresh_live_odds.py
- Add new data files: field_status.json, data_changelog.json, distacc weight files
- Fix NaT date filter bug in overview_tab, grass_putting_deepdive, elite_finish_tab

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -589,7 +589,7 @@
       </c>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="n">
-        <v>257</v>
+        <v>244</v>
       </c>
     </row>
     <row r="11">
@@ -715,7 +715,7 @@
       </c>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="n">
-        <v>428</v>
+        <v>414</v>
       </c>
     </row>
     <row r="19">
@@ -837,7 +837,7 @@
       </c>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="n">
-        <v>211</v>
+        <v>192</v>
       </c>
     </row>
     <row r="27">
@@ -1087,7 +1087,7 @@
       </c>
       <c r="C42" t="inlineStr"/>
       <c r="D42" t="n">
-        <v>207</v>
+        <v>225</v>
       </c>
     </row>
     <row r="43">
@@ -1133,7 +1133,7 @@
       </c>
       <c r="C45" t="inlineStr"/>
       <c r="D45" t="n">
-        <v>154</v>
+        <v>161</v>
       </c>
     </row>
     <row r="46">
@@ -1195,7 +1195,7 @@
       </c>
       <c r="C49" t="inlineStr"/>
       <c r="D49" t="n">
-        <v>148</v>
+        <v>154</v>
       </c>
     </row>
     <row r="50">
@@ -1263,7 +1263,7 @@
       </c>
       <c r="C53" t="inlineStr"/>
       <c r="D53" t="n">
-        <v>317</v>
+        <v>279</v>
       </c>
     </row>
     <row r="54">
@@ -1311,9 +1311,13 @@
       <c r="B56" t="n">
         <v>11451</v>
       </c>
-      <c r="C56" t="inlineStr"/>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>https://pga-tour-res.cloudinary.com/image/upload/c_fill,g_face:center,q_auto,f_auto,dpr_2.0,h_220,w_200,d_stub:default_avatar_light.webp/headshots_29535</t>
+        </is>
+      </c>
       <c r="D56" t="n">
-        <v>348</v>
+        <v>383</v>
       </c>
     </row>
     <row r="57">
@@ -1349,7 +1353,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>168</v>
+        <v>175</v>
       </c>
     </row>
     <row r="59">
@@ -1507,7 +1511,7 @@
       </c>
       <c r="C68" t="inlineStr"/>
       <c r="D68" t="n">
-        <v>209</v>
+        <v>218</v>
       </c>
     </row>
     <row r="69">
@@ -1733,7 +1737,7 @@
       </c>
       <c r="C82" t="inlineStr"/>
       <c r="D82" t="n">
-        <v>327</v>
+        <v>347</v>
       </c>
     </row>
     <row r="83">
@@ -1823,7 +1827,7 @@
         </is>
       </c>
       <c r="D87" t="n">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
     <row r="88">
@@ -1851,7 +1855,7 @@
       </c>
       <c r="C89" t="inlineStr"/>
       <c r="D89" t="n">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="90">
@@ -2061,7 +2065,7 @@
         </is>
       </c>
       <c r="D102" t="n">
-        <v>116</v>
+        <v>124</v>
       </c>
     </row>
     <row r="103">
@@ -2217,7 +2221,7 @@
       </c>
       <c r="C112" t="inlineStr"/>
       <c r="D112" t="n">
-        <v>143</v>
+        <v>147</v>
       </c>
     </row>
     <row r="113">
@@ -2299,9 +2303,13 @@
       <c r="B118" t="n">
         <v>15980</v>
       </c>
-      <c r="C118" t="inlineStr"/>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>https://pga-tour-res.cloudinary.com/image/upload/c_fill,g_face:center,q_auto,f_auto,dpr_2.0,h_220,w_200,d_stub:default_avatar_light.webp/headshots_36326</t>
+        </is>
+      </c>
       <c r="D118" t="n">
-        <v>146</v>
+        <v>150</v>
       </c>
     </row>
     <row r="119">
@@ -2671,7 +2679,7 @@
       </c>
       <c r="C141" t="inlineStr"/>
       <c r="D141" t="n">
-        <v>58</v>
+        <v>63</v>
       </c>
     </row>
     <row r="142">
@@ -2843,7 +2851,7 @@
       </c>
       <c r="C153" t="inlineStr"/>
       <c r="D153" t="n">
-        <v>303</v>
+        <v>293</v>
       </c>
     </row>
     <row r="154">
@@ -2855,7 +2863,11 @@
       <c r="B154" t="n">
         <v>19960</v>
       </c>
-      <c r="C154" t="inlineStr"/>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>https://pga-tour-res.cloudinary.com/image/upload/c_fill,g_face:center,q_auto,f_auto,dpr_2.0,h_220,w_200,d_stub:default_avatar_light.webp/headshots_48153</t>
+        </is>
+      </c>
       <c r="D154" t="n">
         <v>263</v>
       </c>
@@ -2925,7 +2937,7 @@
       </c>
       <c r="C158" t="inlineStr"/>
       <c r="D158" t="n">
-        <v>246</v>
+        <v>232</v>
       </c>
     </row>
     <row r="159">
@@ -3231,7 +3243,7 @@
       </c>
       <c r="C177" t="inlineStr"/>
       <c r="D177" t="n">
-        <v>229</v>
+        <v>239</v>
       </c>
     </row>
     <row r="178">
@@ -3309,7 +3321,11 @@
       <c r="B182" t="n">
         <v>20722</v>
       </c>
-      <c r="C182" t="inlineStr"/>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>https://pga-tour-res.cloudinary.com/image/upload/c_fill,g_face:center,q_auto,f_auto,dpr_2.0,h_220,w_200,d_stub:default_avatar_light.webp/headshots_48867</t>
+        </is>
+      </c>
       <c r="D182" t="n">
         <v>90</v>
       </c>
@@ -3323,7 +3339,11 @@
       <c r="B183" t="n">
         <v>20722</v>
       </c>
-      <c r="C183" t="inlineStr"/>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>https://pga-tour-res.cloudinary.com/image/upload/c_fill,g_face:center,q_auto,f_auto,dpr_2.0,h_220,w_200,d_stub:default_avatar_light.webp/headshots_48867</t>
+        </is>
+      </c>
       <c r="D183" t="n">
         <v>90</v>
       </c>
@@ -3383,9 +3403,13 @@
       <c r="B187" t="n">
         <v>11049</v>
       </c>
-      <c r="C187" t="inlineStr"/>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>https://pga-tour-res.cloudinary.com/image/upload/c_fill,g_face:center,q_auto,f_auto,dpr_2.0,h_220,w_200,d_stub:default_avatar_light.webp/headshots_29221</t>
+        </is>
+      </c>
       <c r="D187" t="n">
-        <v>474</v>
+        <v>485</v>
       </c>
     </row>
     <row r="188">
@@ -3399,7 +3423,7 @@
       </c>
       <c r="C188" t="inlineStr"/>
       <c r="D188" t="n">
-        <v>270</v>
+        <v>272</v>
       </c>
     </row>
     <row r="189">
@@ -3449,7 +3473,7 @@
       </c>
       <c r="C191" t="inlineStr"/>
       <c r="D191" t="n">
-        <v>289</v>
+        <v>305</v>
       </c>
     </row>
     <row r="192">
@@ -3561,8 +3585,14 @@
       <c r="B198" t="n">
         <v>8480</v>
       </c>
-      <c r="C198" t="inlineStr"/>
-      <c r="D198" t="inlineStr"/>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>https://pga-tour-res.cloudinary.com/image/upload/c_fill,g_face:center,q_auto,f_auto,dpr_2.0,h_220,w_200,d_stub:default_avatar_light.webp/headshots_27214</t>
+        </is>
+      </c>
+      <c r="D198" t="n">
+        <v>409</v>
+      </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -3575,7 +3605,7 @@
       </c>
       <c r="C199" t="inlineStr"/>
       <c r="D199" t="n">
-        <v>186</v>
+        <v>194</v>
       </c>
     </row>
     <row r="200">
@@ -3589,7 +3619,7 @@
       </c>
       <c r="C200" t="inlineStr"/>
       <c r="D200" t="n">
-        <v>341</v>
+        <v>353</v>
       </c>
     </row>
     <row r="201">
@@ -3603,7 +3633,7 @@
       </c>
       <c r="C201" t="inlineStr"/>
       <c r="D201" t="n">
-        <v>165</v>
+        <v>167</v>
       </c>
     </row>
     <row r="202">
@@ -3731,7 +3761,7 @@
       </c>
       <c r="C209" t="inlineStr"/>
       <c r="D209" t="n">
-        <v>285</v>
+        <v>309</v>
       </c>
     </row>
     <row r="210">
@@ -3883,9 +3913,13 @@
       <c r="B219" t="n">
         <v>20706</v>
       </c>
-      <c r="C219" t="inlineStr"/>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>https://pga-tour-res.cloudinary.com/image/upload/c_fill,g_face:center,q_auto,f_auto,dpr_2.0,h_220,w_200,d_stub:default_avatar_light.webp/headshots_48887</t>
+        </is>
+      </c>
       <c r="D219" t="n">
-        <v>91</v>
+        <v>97</v>
       </c>
     </row>
     <row r="220">
@@ -3897,9 +3931,13 @@
       <c r="B220" t="n">
         <v>12426</v>
       </c>
-      <c r="C220" t="inlineStr"/>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>https://pga-tour-res.cloudinary.com/image/upload/c_fill,g_face:center,q_auto,f_auto,dpr_2.0,h_220,w_200,d_stub:default_avatar_light.webp/headshots_31113</t>
+        </is>
+      </c>
       <c r="D220" t="n">
-        <v>268</v>
+        <v>292</v>
       </c>
     </row>
     <row r="221">
@@ -3943,7 +3981,7 @@
       </c>
       <c r="C223" t="inlineStr"/>
       <c r="D223" t="n">
-        <v>375</v>
+        <v>377</v>
       </c>
     </row>
     <row r="224">
@@ -3967,7 +4005,11 @@
       <c r="B225" t="n">
         <v>12577</v>
       </c>
-      <c r="C225" t="inlineStr"/>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>https://pga-tour-res.cloudinary.com/image/upload/c_fill,g_face:center,q_auto,f_auto,dpr_2.0,h_220,w_200,d_stub:default_avatar_light.webp/headshots_31323</t>
+        </is>
+      </c>
       <c r="D225" t="n">
         <v>148</v>
       </c>
@@ -3983,7 +4025,7 @@
       </c>
       <c r="C226" t="inlineStr"/>
       <c r="D226" t="n">
-        <v>349</v>
+        <v>361</v>
       </c>
     </row>
     <row r="227">

</xml_diff>

<commit_message>
data: field/odds refresh 2026-03-16 14:20 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -557,7 +557,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="9">
@@ -575,7 +575,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
     </row>
     <row r="10">
@@ -589,7 +589,7 @@
       </c>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="n">
-        <v>244</v>
+        <v>240</v>
       </c>
     </row>
     <row r="11">
@@ -607,7 +607,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="12">
@@ -639,7 +639,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="14">
@@ -701,7 +701,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>96</v>
+        <v>99</v>
       </c>
     </row>
     <row r="18">
@@ -715,7 +715,7 @@
       </c>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="n">
-        <v>414</v>
+        <v>417</v>
       </c>
     </row>
     <row r="19">
@@ -747,7 +747,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="21">
@@ -779,7 +779,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>95</v>
+        <v>90</v>
       </c>
     </row>
     <row r="23">
@@ -797,7 +797,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="24">
@@ -837,7 +837,7 @@
       </c>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="n">
-        <v>192</v>
+        <v>201</v>
       </c>
     </row>
     <row r="27">
@@ -855,7 +855,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="28">
@@ -873,7 +873,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>121</v>
+        <v>117</v>
       </c>
     </row>
     <row r="29">
@@ -905,7 +905,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="31">
@@ -923,7 +923,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>48</v>
+        <v>52</v>
       </c>
     </row>
     <row r="32">
@@ -985,7 +985,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>179</v>
+        <v>188</v>
       </c>
     </row>
     <row r="36">
@@ -1181,7 +1181,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="49">
@@ -1195,7 +1195,7 @@
       </c>
       <c r="C49" t="inlineStr"/>
       <c r="D49" t="n">
-        <v>154</v>
+        <v>159</v>
       </c>
     </row>
     <row r="50">
@@ -1213,7 +1213,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
     <row r="51">
@@ -1231,7 +1231,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>24</v>
+        <v>15</v>
       </c>
     </row>
     <row r="52">
@@ -1263,7 +1263,7 @@
       </c>
       <c r="C53" t="inlineStr"/>
       <c r="D53" t="n">
-        <v>279</v>
+        <v>275</v>
       </c>
     </row>
     <row r="54">
@@ -1317,7 +1317,7 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>383</v>
+        <v>377</v>
       </c>
     </row>
     <row r="57">
@@ -1353,7 +1353,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>175</v>
+        <v>181</v>
       </c>
     </row>
     <row r="59">
@@ -1371,7 +1371,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>78</v>
+        <v>81</v>
       </c>
     </row>
     <row r="60">
@@ -1435,7 +1435,7 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="64">
@@ -1453,7 +1453,7 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
     </row>
     <row r="65">
@@ -1485,7 +1485,7 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>113</v>
+        <v>115</v>
       </c>
     </row>
     <row r="67">
@@ -1511,7 +1511,7 @@
       </c>
       <c r="C68" t="inlineStr"/>
       <c r="D68" t="n">
-        <v>218</v>
+        <v>219</v>
       </c>
     </row>
     <row r="69">
@@ -1641,7 +1641,7 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="77">
@@ -1673,7 +1673,7 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="79">
@@ -1691,7 +1691,7 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>65</v>
+        <v>61</v>
       </c>
     </row>
     <row r="80">
@@ -1737,7 +1737,7 @@
       </c>
       <c r="C82" t="inlineStr"/>
       <c r="D82" t="n">
-        <v>347</v>
+        <v>353</v>
       </c>
     </row>
     <row r="83">
@@ -1773,7 +1773,7 @@
         </is>
       </c>
       <c r="D84" t="n">
-        <v>52</v>
+        <v>47</v>
       </c>
     </row>
     <row r="85">
@@ -1791,7 +1791,7 @@
         </is>
       </c>
       <c r="D85" t="n">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="86">
@@ -1809,7 +1809,7 @@
         </is>
       </c>
       <c r="D86" t="n">
-        <v>149</v>
+        <v>142</v>
       </c>
     </row>
     <row r="87">
@@ -1827,7 +1827,7 @@
         </is>
       </c>
       <c r="D87" t="n">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="88">
@@ -1855,7 +1855,7 @@
       </c>
       <c r="C89" t="inlineStr"/>
       <c r="D89" t="n">
-        <v>152</v>
+        <v>156</v>
       </c>
     </row>
     <row r="90">
@@ -1887,7 +1887,7 @@
       </c>
       <c r="C91" t="inlineStr"/>
       <c r="D91" t="n">
-        <v>139</v>
+        <v>140</v>
       </c>
     </row>
     <row r="92">
@@ -1905,7 +1905,7 @@
         </is>
       </c>
       <c r="D92" t="n">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
     <row r="93">
@@ -1923,7 +1923,7 @@
         </is>
       </c>
       <c r="D93" t="n">
-        <v>79</v>
+        <v>82</v>
       </c>
     </row>
     <row r="94">
@@ -1941,7 +1941,7 @@
         </is>
       </c>
       <c r="D94" t="n">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="95">
@@ -1985,7 +1985,7 @@
       </c>
       <c r="C97" t="inlineStr"/>
       <c r="D97" t="n">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="98">
@@ -2029,7 +2029,7 @@
         </is>
       </c>
       <c r="D100" t="n">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="101">
@@ -2065,7 +2065,7 @@
         </is>
       </c>
       <c r="D102" t="n">
-        <v>124</v>
+        <v>127</v>
       </c>
     </row>
     <row r="103">
@@ -2127,7 +2127,7 @@
       </c>
       <c r="C106" t="inlineStr"/>
       <c r="D106" t="n">
-        <v>230</v>
+        <v>234</v>
       </c>
     </row>
     <row r="107">
@@ -2175,7 +2175,7 @@
         </is>
       </c>
       <c r="D109" t="n">
-        <v>221</v>
+        <v>173</v>
       </c>
     </row>
     <row r="110">
@@ -2221,7 +2221,7 @@
       </c>
       <c r="C112" t="inlineStr"/>
       <c r="D112" t="n">
-        <v>147</v>
+        <v>153</v>
       </c>
     </row>
     <row r="113">
@@ -2309,7 +2309,7 @@
         </is>
       </c>
       <c r="D118" t="n">
-        <v>150</v>
+        <v>154</v>
       </c>
     </row>
     <row r="119">
@@ -2449,7 +2449,7 @@
         </is>
       </c>
       <c r="D127" t="n">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
     <row r="128">
@@ -2485,7 +2485,7 @@
         </is>
       </c>
       <c r="D129" t="n">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="130">
@@ -2539,7 +2539,7 @@
         </is>
       </c>
       <c r="D132" t="n">
-        <v>106</v>
+        <v>111</v>
       </c>
     </row>
     <row r="133">
@@ -2619,7 +2619,7 @@
         </is>
       </c>
       <c r="D137" t="n">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="138">
@@ -2651,7 +2651,7 @@
       </c>
       <c r="C139" t="inlineStr"/>
       <c r="D139" t="n">
-        <v>126</v>
+        <v>118</v>
       </c>
     </row>
     <row r="140">
@@ -2679,7 +2679,7 @@
       </c>
       <c r="C141" t="inlineStr"/>
       <c r="D141" t="n">
-        <v>63</v>
+        <v>65</v>
       </c>
     </row>
     <row r="142">
@@ -2743,7 +2743,7 @@
       </c>
       <c r="C145" t="inlineStr"/>
       <c r="D145" t="n">
-        <v>292</v>
+        <v>320</v>
       </c>
     </row>
     <row r="146">
@@ -2773,7 +2773,7 @@
         </is>
       </c>
       <c r="D147" t="n">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="148">
@@ -2851,7 +2851,7 @@
       </c>
       <c r="C153" t="inlineStr"/>
       <c r="D153" t="n">
-        <v>293</v>
+        <v>294</v>
       </c>
     </row>
     <row r="154">
@@ -2869,7 +2869,7 @@
         </is>
       </c>
       <c r="D154" t="n">
-        <v>263</v>
+        <v>272</v>
       </c>
     </row>
     <row r="155">
@@ -2905,7 +2905,7 @@
         </is>
       </c>
       <c r="D156" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="157">
@@ -2937,7 +2937,7 @@
       </c>
       <c r="C158" t="inlineStr"/>
       <c r="D158" t="n">
-        <v>232</v>
+        <v>233</v>
       </c>
     </row>
     <row r="159">
@@ -2951,7 +2951,7 @@
       </c>
       <c r="C159" t="inlineStr"/>
       <c r="D159" t="n">
-        <v>168</v>
+        <v>176</v>
       </c>
     </row>
     <row r="160">
@@ -3001,7 +3001,7 @@
       </c>
       <c r="C162" t="inlineStr"/>
       <c r="D162" t="n">
-        <v>157</v>
+        <v>160</v>
       </c>
     </row>
     <row r="163">
@@ -3019,7 +3019,7 @@
         </is>
       </c>
       <c r="D163" t="n">
-        <v>122</v>
+        <v>116</v>
       </c>
     </row>
     <row r="164">
@@ -3055,7 +3055,7 @@
         </is>
       </c>
       <c r="D165" t="n">
-        <v>35</v>
+        <v>38</v>
       </c>
     </row>
     <row r="166">
@@ -3069,7 +3069,7 @@
       </c>
       <c r="C166" t="inlineStr"/>
       <c r="D166" t="n">
-        <v>155</v>
+        <v>146</v>
       </c>
     </row>
     <row r="167">
@@ -3129,7 +3129,7 @@
         </is>
       </c>
       <c r="D170" t="n">
-        <v>107</v>
+        <v>109</v>
       </c>
     </row>
     <row r="171">
@@ -3147,7 +3147,7 @@
         </is>
       </c>
       <c r="D171" t="n">
-        <v>85</v>
+        <v>70</v>
       </c>
     </row>
     <row r="172">
@@ -3193,7 +3193,7 @@
       </c>
       <c r="C174" t="inlineStr"/>
       <c r="D174" t="n">
-        <v>138</v>
+        <v>134</v>
       </c>
     </row>
     <row r="175">
@@ -3243,7 +3243,7 @@
       </c>
       <c r="C177" t="inlineStr"/>
       <c r="D177" t="n">
-        <v>239</v>
+        <v>242</v>
       </c>
     </row>
     <row r="178">
@@ -3273,7 +3273,7 @@
         </is>
       </c>
       <c r="D179" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="180">
@@ -3309,7 +3309,7 @@
         </is>
       </c>
       <c r="D181" t="n">
-        <v>141</v>
+        <v>144</v>
       </c>
     </row>
     <row r="182">
@@ -3327,7 +3327,7 @@
         </is>
       </c>
       <c r="D182" t="n">
-        <v>90</v>
+        <v>86</v>
       </c>
     </row>
     <row r="183">
@@ -3345,7 +3345,7 @@
         </is>
       </c>
       <c r="D183" t="n">
-        <v>90</v>
+        <v>86</v>
       </c>
     </row>
     <row r="184">
@@ -3423,7 +3423,7 @@
       </c>
       <c r="C188" t="inlineStr"/>
       <c r="D188" t="n">
-        <v>272</v>
+        <v>268</v>
       </c>
     </row>
     <row r="189">
@@ -3441,7 +3441,7 @@
         </is>
       </c>
       <c r="D189" t="n">
-        <v>123</v>
+        <v>112</v>
       </c>
     </row>
     <row r="190">
@@ -3473,7 +3473,7 @@
       </c>
       <c r="C191" t="inlineStr"/>
       <c r="D191" t="n">
-        <v>305</v>
+        <v>306</v>
       </c>
     </row>
     <row r="192">
@@ -3491,7 +3491,7 @@
         </is>
       </c>
       <c r="D192" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="193">
@@ -3591,7 +3591,7 @@
         </is>
       </c>
       <c r="D198" t="n">
-        <v>409</v>
+        <v>415</v>
       </c>
     </row>
     <row r="199">
@@ -3605,7 +3605,7 @@
       </c>
       <c r="C199" t="inlineStr"/>
       <c r="D199" t="n">
-        <v>194</v>
+        <v>199</v>
       </c>
     </row>
     <row r="200">
@@ -3619,7 +3619,7 @@
       </c>
       <c r="C200" t="inlineStr"/>
       <c r="D200" t="n">
-        <v>353</v>
+        <v>358</v>
       </c>
     </row>
     <row r="201">
@@ -3633,7 +3633,7 @@
       </c>
       <c r="C201" t="inlineStr"/>
       <c r="D201" t="n">
-        <v>167</v>
+        <v>172</v>
       </c>
     </row>
     <row r="202">
@@ -3669,7 +3669,7 @@
         </is>
       </c>
       <c r="D203" t="n">
-        <v>76</v>
+        <v>73</v>
       </c>
     </row>
     <row r="204">
@@ -3705,7 +3705,7 @@
         </is>
       </c>
       <c r="D205" t="n">
-        <v>111</v>
+        <v>113</v>
       </c>
     </row>
     <row r="206">
@@ -3761,7 +3761,7 @@
       </c>
       <c r="C209" t="inlineStr"/>
       <c r="D209" t="n">
-        <v>309</v>
+        <v>310</v>
       </c>
     </row>
     <row r="210">
@@ -3797,7 +3797,7 @@
         </is>
       </c>
       <c r="D211" t="n">
-        <v>146</v>
+        <v>151</v>
       </c>
     </row>
     <row r="212">
@@ -3841,7 +3841,7 @@
       </c>
       <c r="C214" t="inlineStr"/>
       <c r="D214" t="n">
-        <v>212</v>
+        <v>229</v>
       </c>
     </row>
     <row r="215">
@@ -3855,7 +3855,7 @@
       </c>
       <c r="C215" t="inlineStr"/>
       <c r="D215" t="n">
-        <v>212</v>
+        <v>229</v>
       </c>
     </row>
     <row r="216">
@@ -3873,7 +3873,7 @@
         </is>
       </c>
       <c r="D216" t="n">
-        <v>145</v>
+        <v>149</v>
       </c>
     </row>
     <row r="217">
@@ -3901,7 +3901,7 @@
       </c>
       <c r="C218" t="inlineStr"/>
       <c r="D218" t="n">
-        <v>227</v>
+        <v>224</v>
       </c>
     </row>
     <row r="219">
@@ -3919,7 +3919,7 @@
         </is>
       </c>
       <c r="D219" t="n">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="220">
@@ -3937,7 +3937,7 @@
         </is>
       </c>
       <c r="D220" t="n">
-        <v>292</v>
+        <v>296</v>
       </c>
     </row>
     <row r="221">
@@ -3955,7 +3955,7 @@
         </is>
       </c>
       <c r="D221" t="n">
-        <v>120</v>
+        <v>124</v>
       </c>
     </row>
     <row r="222">
@@ -3981,7 +3981,7 @@
       </c>
       <c r="C223" t="inlineStr"/>
       <c r="D223" t="n">
-        <v>377</v>
+        <v>382</v>
       </c>
     </row>
     <row r="224">
@@ -4011,7 +4011,7 @@
         </is>
       </c>
       <c r="D225" t="n">
-        <v>148</v>
+        <v>152</v>
       </c>
     </row>
     <row r="226">
@@ -4025,7 +4025,7 @@
       </c>
       <c r="C226" t="inlineStr"/>
       <c r="D226" t="n">
-        <v>361</v>
+        <v>359</v>
       </c>
     </row>
     <row r="227">
@@ -4089,7 +4089,7 @@
         </is>
       </c>
       <c r="D230" t="n">
-        <v>115</v>
+        <v>119</v>
       </c>
     </row>
     <row r="231">

</xml_diff>

<commit_message>
data: field/odds refresh 2026-03-23 10:21 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -557,7 +557,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="9">
@@ -666,7 +666,9 @@
         <v>11082</v>
       </c>
       <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr"/>
+      <c r="D15" t="n">
+        <v>480</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -683,7 +685,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="17">
@@ -701,7 +703,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="18">
@@ -715,7 +717,7 @@
       </c>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="n">
-        <v>417</v>
+        <v>424</v>
       </c>
     </row>
     <row r="19">
@@ -779,7 +781,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="23">
@@ -797,7 +799,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="24">
@@ -837,7 +839,7 @@
       </c>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="n">
-        <v>201</v>
+        <v>202</v>
       </c>
     </row>
     <row r="27">
@@ -855,7 +857,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>67</v>
+        <v>72</v>
       </c>
     </row>
     <row r="28">
@@ -873,7 +875,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>117</v>
+        <v>119</v>
       </c>
     </row>
     <row r="29">
@@ -923,7 +925,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="32">
@@ -1003,7 +1005,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="37">
@@ -1087,7 +1089,7 @@
       </c>
       <c r="C42" t="inlineStr"/>
       <c r="D42" t="n">
-        <v>225</v>
+        <v>237</v>
       </c>
     </row>
     <row r="43">
@@ -1105,7 +1107,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="44">
@@ -1119,7 +1121,7 @@
       </c>
       <c r="C44" t="inlineStr"/>
       <c r="D44" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="45">
@@ -1133,7 +1135,7 @@
       </c>
       <c r="C45" t="inlineStr"/>
       <c r="D45" t="n">
-        <v>161</v>
+        <v>172</v>
       </c>
     </row>
     <row r="46">
@@ -1163,7 +1165,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="48">
@@ -1181,7 +1183,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="49">
@@ -1195,7 +1197,7 @@
       </c>
       <c r="C49" t="inlineStr"/>
       <c r="D49" t="n">
-        <v>159</v>
+        <v>161</v>
       </c>
     </row>
     <row r="50">
@@ -1213,7 +1215,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>129</v>
+        <v>134</v>
       </c>
     </row>
     <row r="51">
@@ -1263,7 +1265,7 @@
       </c>
       <c r="C53" t="inlineStr"/>
       <c r="D53" t="n">
-        <v>275</v>
+        <v>262</v>
       </c>
     </row>
     <row r="54">
@@ -1281,7 +1283,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="55">
@@ -1299,7 +1301,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="56">
@@ -1317,7 +1319,7 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>377</v>
+        <v>386</v>
       </c>
     </row>
     <row r="57">
@@ -1371,7 +1373,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>81</v>
+        <v>84</v>
       </c>
     </row>
     <row r="60">
@@ -1417,7 +1419,7 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="63">
@@ -1435,7 +1437,7 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="64">
@@ -1485,7 +1487,7 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>115</v>
+        <v>103</v>
       </c>
     </row>
     <row r="67">
@@ -1529,7 +1531,7 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>56</v>
+        <v>62</v>
       </c>
     </row>
     <row r="70">
@@ -1641,7 +1643,7 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>76</v>
+        <v>83</v>
       </c>
     </row>
     <row r="77">
@@ -1673,7 +1675,7 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="79">
@@ -1705,7 +1707,7 @@
       </c>
       <c r="C80" t="inlineStr"/>
       <c r="D80" t="n">
-        <v>133</v>
+        <v>128</v>
       </c>
     </row>
     <row r="81">
@@ -1723,7 +1725,7 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>80</v>
+        <v>76</v>
       </c>
     </row>
     <row r="82">
@@ -1737,7 +1739,7 @@
       </c>
       <c r="C82" t="inlineStr"/>
       <c r="D82" t="n">
-        <v>353</v>
+        <v>362</v>
       </c>
     </row>
     <row r="83">
@@ -1755,7 +1757,7 @@
         </is>
       </c>
       <c r="D83" t="n">
-        <v>98</v>
+        <v>101</v>
       </c>
     </row>
     <row r="84">
@@ -1827,7 +1829,7 @@
         </is>
       </c>
       <c r="D87" t="n">
-        <v>83</v>
+        <v>87</v>
       </c>
     </row>
     <row r="88">
@@ -1855,7 +1857,7 @@
       </c>
       <c r="C89" t="inlineStr"/>
       <c r="D89" t="n">
-        <v>156</v>
+        <v>164</v>
       </c>
     </row>
     <row r="90">
@@ -1887,7 +1889,7 @@
       </c>
       <c r="C91" t="inlineStr"/>
       <c r="D91" t="n">
-        <v>140</v>
+        <v>143</v>
       </c>
     </row>
     <row r="92">
@@ -1905,7 +1907,7 @@
         </is>
       </c>
       <c r="D92" t="n">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="93">
@@ -1923,7 +1925,7 @@
         </is>
       </c>
       <c r="D93" t="n">
-        <v>82</v>
+        <v>67</v>
       </c>
     </row>
     <row r="94">
@@ -1941,7 +1943,7 @@
         </is>
       </c>
       <c r="D94" t="n">
-        <v>107</v>
+        <v>100</v>
       </c>
     </row>
     <row r="95">
@@ -1985,7 +1987,7 @@
       </c>
       <c r="C97" t="inlineStr"/>
       <c r="D97" t="n">
-        <v>126</v>
+        <v>124</v>
       </c>
     </row>
     <row r="98">
@@ -2065,7 +2067,7 @@
         </is>
       </c>
       <c r="D102" t="n">
-        <v>127</v>
+        <v>123</v>
       </c>
     </row>
     <row r="103">
@@ -2083,7 +2085,7 @@
         </is>
       </c>
       <c r="D103" t="n">
-        <v>99</v>
+        <v>94</v>
       </c>
     </row>
     <row r="104">
@@ -2113,7 +2115,7 @@
         </is>
       </c>
       <c r="D105" t="n">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="106">
@@ -2127,7 +2129,7 @@
       </c>
       <c r="C106" t="inlineStr"/>
       <c r="D106" t="n">
-        <v>234</v>
+        <v>247</v>
       </c>
     </row>
     <row r="107">
@@ -2175,7 +2177,7 @@
         </is>
       </c>
       <c r="D109" t="n">
-        <v>173</v>
+        <v>162</v>
       </c>
     </row>
     <row r="110">
@@ -2272,9 +2274,7 @@
         <v>13497</v>
       </c>
       <c r="C116" t="inlineStr"/>
-      <c r="D116" t="n">
-        <v>496</v>
-      </c>
+      <c r="D116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -2291,7 +2291,7 @@
         </is>
       </c>
       <c r="D117" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="118">
@@ -2309,7 +2309,7 @@
         </is>
       </c>
       <c r="D118" t="n">
-        <v>154</v>
+        <v>88</v>
       </c>
     </row>
     <row r="119">
@@ -2355,7 +2355,7 @@
         </is>
       </c>
       <c r="D121" t="n">
-        <v>29</v>
+        <v>32</v>
       </c>
     </row>
     <row r="122">
@@ -2467,7 +2467,7 @@
         </is>
       </c>
       <c r="D128" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="129">
@@ -2485,7 +2485,7 @@
         </is>
       </c>
       <c r="D129" t="n">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="130">
@@ -2539,7 +2539,7 @@
         </is>
       </c>
       <c r="D132" t="n">
-        <v>111</v>
+        <v>118</v>
       </c>
     </row>
     <row r="133">
@@ -2573,7 +2573,7 @@
         </is>
       </c>
       <c r="D134" t="n">
-        <v>114</v>
+        <v>109</v>
       </c>
     </row>
     <row r="135">
@@ -2651,7 +2651,7 @@
       </c>
       <c r="C139" t="inlineStr"/>
       <c r="D139" t="n">
-        <v>118</v>
+        <v>120</v>
       </c>
     </row>
     <row r="140">
@@ -2665,7 +2665,7 @@
       </c>
       <c r="C140" t="inlineStr"/>
       <c r="D140" t="n">
-        <v>346</v>
+        <v>387</v>
       </c>
     </row>
     <row r="141">
@@ -2679,7 +2679,7 @@
       </c>
       <c r="C141" t="inlineStr"/>
       <c r="D141" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="142">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="C148" t="inlineStr"/>
       <c r="D148" t="n">
-        <v>102</v>
+        <v>108</v>
       </c>
     </row>
     <row r="149">
@@ -2869,7 +2869,7 @@
         </is>
       </c>
       <c r="D154" t="n">
-        <v>272</v>
+        <v>226</v>
       </c>
     </row>
     <row r="155">
@@ -2887,7 +2887,7 @@
         </is>
       </c>
       <c r="D155" t="n">
-        <v>66</v>
+        <v>70</v>
       </c>
     </row>
     <row r="156">
@@ -2905,7 +2905,7 @@
         </is>
       </c>
       <c r="D156" t="n">
-        <v>39</v>
+        <v>36</v>
       </c>
     </row>
     <row r="157">
@@ -2951,7 +2951,7 @@
       </c>
       <c r="C159" t="inlineStr"/>
       <c r="D159" t="n">
-        <v>176</v>
+        <v>177</v>
       </c>
     </row>
     <row r="160">
@@ -2969,7 +2969,7 @@
         </is>
       </c>
       <c r="D160" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="161">
@@ -2987,7 +2987,7 @@
         </is>
       </c>
       <c r="D161" t="n">
-        <v>71</v>
+        <v>77</v>
       </c>
     </row>
     <row r="162">
@@ -3055,7 +3055,7 @@
         </is>
       </c>
       <c r="D165" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="166">
@@ -3069,7 +3069,7 @@
       </c>
       <c r="C166" t="inlineStr"/>
       <c r="D166" t="n">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="167">
@@ -3129,7 +3129,7 @@
         </is>
       </c>
       <c r="D170" t="n">
-        <v>109</v>
+        <v>114</v>
       </c>
     </row>
     <row r="171">
@@ -3147,7 +3147,7 @@
         </is>
       </c>
       <c r="D171" t="n">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="172">
@@ -3193,7 +3193,7 @@
       </c>
       <c r="C174" t="inlineStr"/>
       <c r="D174" t="n">
-        <v>134</v>
+        <v>137</v>
       </c>
     </row>
     <row r="175">
@@ -3243,7 +3243,7 @@
       </c>
       <c r="C177" t="inlineStr"/>
       <c r="D177" t="n">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="178">
@@ -3309,7 +3309,7 @@
         </is>
       </c>
       <c r="D181" t="n">
-        <v>144</v>
+        <v>146</v>
       </c>
     </row>
     <row r="182">
@@ -3327,7 +3327,7 @@
         </is>
       </c>
       <c r="D182" t="n">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="183">
@@ -3345,7 +3345,7 @@
         </is>
       </c>
       <c r="D183" t="n">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="184">
@@ -3363,7 +3363,7 @@
         </is>
       </c>
       <c r="D184" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="185">
@@ -3441,7 +3441,7 @@
         </is>
       </c>
       <c r="D189" t="n">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="190">
@@ -3541,7 +3541,7 @@
         </is>
       </c>
       <c r="D195" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="196">
@@ -3555,7 +3555,7 @@
       </c>
       <c r="C196" t="inlineStr"/>
       <c r="D196" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="197">
@@ -3619,7 +3619,7 @@
       </c>
       <c r="C200" t="inlineStr"/>
       <c r="D200" t="n">
-        <v>358</v>
+        <v>363</v>
       </c>
     </row>
     <row r="201">
@@ -3633,7 +3633,7 @@
       </c>
       <c r="C201" t="inlineStr"/>
       <c r="D201" t="n">
-        <v>172</v>
+        <v>178</v>
       </c>
     </row>
     <row r="202">
@@ -3669,7 +3669,7 @@
         </is>
       </c>
       <c r="D203" t="n">
-        <v>73</v>
+        <v>80</v>
       </c>
     </row>
     <row r="204">
@@ -3705,7 +3705,7 @@
         </is>
       </c>
       <c r="D205" t="n">
-        <v>113</v>
+        <v>115</v>
       </c>
     </row>
     <row r="206">
@@ -3723,7 +3723,7 @@
         </is>
       </c>
       <c r="D206" t="n">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
     <row r="207">
@@ -3761,7 +3761,7 @@
       </c>
       <c r="C209" t="inlineStr"/>
       <c r="D209" t="n">
-        <v>310</v>
+        <v>298</v>
       </c>
     </row>
     <row r="210">
@@ -3797,7 +3797,7 @@
         </is>
       </c>
       <c r="D211" t="n">
-        <v>151</v>
+        <v>156</v>
       </c>
     </row>
     <row r="212">
@@ -3815,7 +3815,7 @@
         </is>
       </c>
       <c r="D212" t="n">
-        <v>101</v>
+        <v>107</v>
       </c>
     </row>
     <row r="213">
@@ -3873,7 +3873,7 @@
         </is>
       </c>
       <c r="D216" t="n">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="217">
@@ -3901,7 +3901,7 @@
       </c>
       <c r="C218" t="inlineStr"/>
       <c r="D218" t="n">
-        <v>224</v>
+        <v>213</v>
       </c>
     </row>
     <row r="219">
@@ -3919,7 +3919,7 @@
         </is>
       </c>
       <c r="D219" t="n">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="220">
@@ -3937,7 +3937,7 @@
         </is>
       </c>
       <c r="D220" t="n">
-        <v>296</v>
+        <v>301</v>
       </c>
     </row>
     <row r="221">
@@ -3955,7 +3955,7 @@
         </is>
       </c>
       <c r="D221" t="n">
-        <v>124</v>
+        <v>127</v>
       </c>
     </row>
     <row r="222">
@@ -3981,7 +3981,7 @@
       </c>
       <c r="C223" t="inlineStr"/>
       <c r="D223" t="n">
-        <v>382</v>
+        <v>399</v>
       </c>
     </row>
     <row r="224">
@@ -4011,7 +4011,7 @@
         </is>
       </c>
       <c r="D225" t="n">
-        <v>152</v>
+        <v>139</v>
       </c>
     </row>
     <row r="226">
@@ -4025,7 +4025,7 @@
       </c>
       <c r="C226" t="inlineStr"/>
       <c r="D226" t="n">
-        <v>359</v>
+        <v>324</v>
       </c>
     </row>
     <row r="227">
@@ -4089,7 +4089,7 @@
         </is>
       </c>
       <c r="D230" t="n">
-        <v>119</v>
+        <v>117</v>
       </c>
     </row>
     <row r="231">
@@ -4107,7 +4107,7 @@
         </is>
       </c>
       <c r="D231" t="n">
-        <v>252</v>
+        <v>291</v>
       </c>
     </row>
     <row r="232">

</xml_diff>

<commit_message>
data: add Yellamaraju, Sudarshan (dg_id=29925) to All_players
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D232"/>
+  <dimension ref="A1:D233"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3465,95 +3465,97 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>Snedeker, Brandt</t>
+          <t>Smotherman, Austin</t>
         </is>
       </c>
       <c r="B191" t="n">
-        <v>8820</v>
-      </c>
-      <c r="C191" t="inlineStr"/>
-      <c r="D191" t="n">
-        <v>306</v>
-      </c>
+        <v>50095</v>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>https://pga-tour-res.cloudinary.com/image/upload/c_fill,g_face:center,q_auto,f_auto,dpr_2.0,h_220,w_200,d_stub:default_avatar_light.webp/headshots_50095</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>Spaun, J.J.</t>
+          <t>Snedeker, Brandt</t>
         </is>
       </c>
       <c r="B192" t="n">
-        <v>17536</v>
-      </c>
-      <c r="C192" t="inlineStr">
-        <is>
-          <t>https://pga-tour-res.cloudinary.com/image/upload/c_fill,g_face:center,q_auto,f_auto,dpr_2.0,h_220,w_200,d_stub:default_avatar_light.webp/headshots_39324</t>
-        </is>
-      </c>
+        <v>8820</v>
+      </c>
+      <c r="C192" t="inlineStr"/>
       <c r="D192" t="n">
-        <v>12</v>
+        <v>306</v>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>Spieth, Jordan</t>
+          <t>Spaun, J.J.</t>
         </is>
       </c>
       <c r="B193" t="n">
-        <v>14636</v>
+        <v>17536</v>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>https://pga-tour-res.cloudinary.com/image/upload/c_fill,g_face:center,q_auto,f_auto,dpr_2.0,h_220,w_200,d_stub:default_avatar_light.webp/headshots_34046</t>
+          <t>https://pga-tour-res.cloudinary.com/image/upload/c_fill,g_face:center,q_auto,f_auto,dpr_2.0,h_220,w_200,d_stub:default_avatar_light.webp/headshots_39324</t>
         </is>
       </c>
       <c r="D193" t="n">
-        <v>64</v>
+        <v>12</v>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>Springer, Hayden</t>
+          <t>Spieth, Jordan</t>
         </is>
       </c>
       <c r="B194" t="n">
-        <v>21995</v>
-      </c>
-      <c r="C194" t="inlineStr"/>
+        <v>14636</v>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>https://pga-tour-res.cloudinary.com/image/upload/c_fill,g_face:center,q_auto,f_auto,dpr_2.0,h_220,w_200,d_stub:default_avatar_light.webp/headshots_34046</t>
+        </is>
+      </c>
       <c r="D194" t="n">
-        <v>219</v>
+        <v>64</v>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>Stevens, Sam</t>
+          <t>Springer, Hayden</t>
         </is>
       </c>
       <c r="B195" t="n">
-        <v>25569</v>
-      </c>
-      <c r="C195" t="inlineStr">
-        <is>
-          <t>https://pga-tour-res.cloudinary.com/image/upload/c_fill,g_face:center,q_auto,f_auto,dpr_2.0,h_220,w_200,d_stub:default_avatar_light.webp/headshots_55893</t>
-        </is>
-      </c>
+        <v>21995</v>
+      </c>
+      <c r="C195" t="inlineStr"/>
       <c r="D195" t="n">
-        <v>50</v>
+        <v>219</v>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>Stevens, Samuel</t>
+          <t>Stevens, Sam</t>
         </is>
       </c>
       <c r="B196" t="n">
         <v>25569</v>
       </c>
-      <c r="C196" t="inlineStr"/>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>https://pga-tour-res.cloudinary.com/image/upload/c_fill,g_face:center,q_auto,f_auto,dpr_2.0,h_220,w_200,d_stub:default_avatar_light.webp/headshots_55893</t>
+        </is>
+      </c>
       <c r="D196" t="n">
         <v>50</v>
       </c>
@@ -3561,191 +3563,193 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>Straka, Sepp</t>
+          <t>Stevens, Samuel</t>
         </is>
       </c>
       <c r="B197" t="n">
-        <v>17511</v>
-      </c>
-      <c r="C197" t="inlineStr">
-        <is>
-          <t>https://pga-tour-res.cloudinary.com/image/upload/c_fill,g_face:center,q_auto,f_auto,dpr_2.0,h_220,w_200,d_stub:default_avatar_light.webp/headshots_49960</t>
-        </is>
-      </c>
+        <v>25569</v>
+      </c>
+      <c r="C197" t="inlineStr"/>
       <c r="D197" t="n">
-        <v>9</v>
+        <v>50</v>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>Streelman, Kevin</t>
+          <t>Straka, Sepp</t>
         </is>
       </c>
       <c r="B198" t="n">
-        <v>8480</v>
+        <v>17511</v>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>https://pga-tour-res.cloudinary.com/image/upload/c_fill,g_face:center,q_auto,f_auto,dpr_2.0,h_220,w_200,d_stub:default_avatar_light.webp/headshots_27214</t>
+          <t>https://pga-tour-res.cloudinary.com/image/upload/c_fill,g_face:center,q_auto,f_auto,dpr_2.0,h_220,w_200,d_stub:default_avatar_light.webp/headshots_49960</t>
         </is>
       </c>
       <c r="D198" t="n">
-        <v>415</v>
+        <v>9</v>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>Suber, Jackson</t>
+          <t>Streelman, Kevin</t>
         </is>
       </c>
       <c r="B199" t="n">
-        <v>29279</v>
-      </c>
-      <c r="C199" t="inlineStr"/>
+        <v>8480</v>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>https://pga-tour-res.cloudinary.com/image/upload/c_fill,g_face:center,q_auto,f_auto,dpr_2.0,h_220,w_200,d_stub:default_avatar_light.webp/headshots_27214</t>
+        </is>
+      </c>
       <c r="D199" t="n">
-        <v>199</v>
+        <v>415</v>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>Svensson, Adam</t>
+          <t>Suber, Jackson</t>
         </is>
       </c>
       <c r="B200" t="n">
-        <v>13997</v>
+        <v>29279</v>
       </c>
       <c r="C200" t="inlineStr"/>
       <c r="D200" t="n">
-        <v>363</v>
+        <v>199</v>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>Svensson, Jesper</t>
+          <t>Svensson, Adam</t>
         </is>
       </c>
       <c r="B201" t="n">
-        <v>26850</v>
+        <v>13997</v>
       </c>
       <c r="C201" t="inlineStr"/>
       <c r="D201" t="n">
-        <v>178</v>
+        <v>363</v>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>Taylor, Nick</t>
+          <t>Svensson, Jesper</t>
         </is>
       </c>
       <c r="B202" t="n">
-        <v>13126</v>
-      </c>
-      <c r="C202" t="inlineStr">
-        <is>
-          <t>https://pga-tour-res.cloudinary.com/image/upload/c_fill,g_face:center,q_auto,f_auto,dpr_2.0,h_220,w_200,d_stub:default_avatar_light.webp/headshots_25493</t>
-        </is>
-      </c>
+        <v>26850</v>
+      </c>
+      <c r="C202" t="inlineStr"/>
       <c r="D202" t="n">
-        <v>62</v>
+        <v>178</v>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>Theegala, Sahith</t>
+          <t>Taylor, Nick</t>
         </is>
       </c>
       <c r="B203" t="n">
-        <v>23014</v>
+        <v>13126</v>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>https://pga-tour-res.cloudinary.com/image/upload/c_fill,g_face:center,q_auto,f_auto,dpr_2.0,h_220,w_200,d_stub:default_avatar_light.webp/headshots_51634</t>
+          <t>https://pga-tour-res.cloudinary.com/image/upload/c_fill,g_face:center,q_auto,f_auto,dpr_2.0,h_220,w_200,d_stub:default_avatar_light.webp/headshots_25493</t>
         </is>
       </c>
       <c r="D203" t="n">
-        <v>80</v>
+        <v>62</v>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>Thomas, Justin</t>
+          <t>Theegala, Sahith</t>
         </is>
       </c>
       <c r="B204" t="n">
-        <v>14139</v>
+        <v>23014</v>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>https://pga-tour-res.cloudinary.com/image/upload/c_fill,g_face:center,q_auto,f_auto,dpr_2.0,h_220,w_200,d_stub:default_avatar_light.webp/headshots_33448</t>
+          <t>https://pga-tour-res.cloudinary.com/image/upload/c_fill,g_face:center,q_auto,f_auto,dpr_2.0,h_220,w_200,d_stub:default_avatar_light.webp/headshots_51634</t>
         </is>
       </c>
       <c r="D204" t="n">
-        <v>14</v>
+        <v>80</v>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>Thompson, Davis</t>
+          <t>Thomas, Justin</t>
         </is>
       </c>
       <c r="B205" t="n">
-        <v>27364</v>
+        <v>14139</v>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>https://pga-tour-res.cloudinary.com/image/upload/c_fill,g_face:center,q_auto,f_auto,dpr_2.0,h_220,w_200,d_stub:default_avatar_light.webp/headshots_58168</t>
+          <t>https://pga-tour-res.cloudinary.com/image/upload/c_fill,g_face:center,q_auto,f_auto,dpr_2.0,h_220,w_200,d_stub:default_avatar_light.webp/headshots_33448</t>
         </is>
       </c>
       <c r="D205" t="n">
-        <v>115</v>
+        <v>14</v>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>Thorbjornsen, Michael</t>
+          <t>Thompson, Davis</t>
         </is>
       </c>
       <c r="B206" t="n">
-        <v>26649</v>
+        <v>27364</v>
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>https://pga-tour-res.cloudinary.com/image/upload/c_fill,g_face:center,q_auto,f_auto,dpr_2.0,h_220,w_200,d_stub:default_avatar_light.webp/headshots_57364</t>
+          <t>https://pga-tour-res.cloudinary.com/image/upload/c_fill,g_face:center,q_auto,f_auto,dpr_2.0,h_220,w_200,d_stub:default_avatar_light.webp/headshots_58168</t>
         </is>
       </c>
       <c r="D206" t="n">
-        <v>56</v>
+        <v>115</v>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>Thornberry, Braden</t>
+          <t>Thorbjornsen, Michael</t>
         </is>
       </c>
       <c r="B207" t="n">
-        <v>23502</v>
-      </c>
-      <c r="C207" t="inlineStr"/>
-      <c r="D207" t="inlineStr"/>
+        <v>26649</v>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>https://pga-tour-res.cloudinary.com/image/upload/c_fill,g_face:center,q_auto,f_auto,dpr_2.0,h_220,w_200,d_stub:default_avatar_light.webp/headshots_57364</t>
+        </is>
+      </c>
+      <c r="D207" t="n">
+        <v>56</v>
+      </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>Todd, Brendon</t>
+          <t>Thornberry, Braden</t>
         </is>
       </c>
       <c r="B208" t="n">
-        <v>12425</v>
+        <v>23502</v>
       </c>
       <c r="C208" t="inlineStr"/>
       <c r="D208" t="inlineStr"/>
@@ -3753,101 +3757,99 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>Tosti, Alejandro</t>
+          <t>Todd, Brendon</t>
         </is>
       </c>
       <c r="B209" t="n">
-        <v>17032</v>
+        <v>12425</v>
       </c>
       <c r="C209" t="inlineStr"/>
-      <c r="D209" t="n">
-        <v>298</v>
-      </c>
+      <c r="D209" t="inlineStr"/>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>Valimaki, Sami</t>
+          <t>Tosti, Alejandro</t>
         </is>
       </c>
       <c r="B210" t="n">
-        <v>23816</v>
-      </c>
-      <c r="C210" t="inlineStr">
-        <is>
-          <t>https://pga-tour-res.cloudinary.com/image/upload/c_fill,g_face:center,q_auto,f_auto,dpr_2.0,h_220,w_200,d_stub:default_avatar_light.webp/headshots_52666</t>
-        </is>
-      </c>
+        <v>17032</v>
+      </c>
+      <c r="C210" t="inlineStr"/>
       <c r="D210" t="n">
-        <v>53</v>
+        <v>298</v>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>Van Rooyen, Erik</t>
+          <t>Valimaki, Sami</t>
         </is>
       </c>
       <c r="B211" t="n">
-        <v>17550</v>
+        <v>23816</v>
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>https://pga-tour-res.cloudinary.com/image/upload/c_fill,g_face:center,q_auto,f_auto,dpr_2.0,h_220,w_200,d_stub:default_avatar_light.webp/headshots_40006</t>
+          <t>https://pga-tour-res.cloudinary.com/image/upload/c_fill,g_face:center,q_auto,f_auto,dpr_2.0,h_220,w_200,d_stub:default_avatar_light.webp/headshots_52666</t>
         </is>
       </c>
       <c r="D211" t="n">
-        <v>156</v>
+        <v>53</v>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>Vegas, Jhonattan</t>
+          <t>Van Rooyen, Erik</t>
         </is>
       </c>
       <c r="B212" t="n">
-        <v>13508</v>
+        <v>17550</v>
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>https://pga-tour-res.cloudinary.com/image/upload/c_fill,g_face:center,q_auto,f_auto,dpr_2.0,h_220,w_200,d_stub:default_avatar_light.webp/headshots_27064</t>
+          <t>https://pga-tour-res.cloudinary.com/image/upload/c_fill,g_face:center,q_auto,f_auto,dpr_2.0,h_220,w_200,d_stub:default_avatar_light.webp/headshots_40006</t>
         </is>
       </c>
       <c r="D212" t="n">
-        <v>107</v>
+        <v>156</v>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>Velo, Kevin</t>
+          <t>Vegas, Jhonattan</t>
         </is>
       </c>
       <c r="B213" t="n">
-        <v>27762</v>
-      </c>
-      <c r="C213" t="inlineStr"/>
-      <c r="D213" t="inlineStr"/>
+        <v>13508</v>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>https://pga-tour-res.cloudinary.com/image/upload/c_fill,g_face:center,q_auto,f_auto,dpr_2.0,h_220,w_200,d_stub:default_avatar_light.webp/headshots_27064</t>
+        </is>
+      </c>
+      <c r="D213" t="n">
+        <v>107</v>
+      </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>Ventura, Kris</t>
+          <t>Velo, Kevin</t>
         </is>
       </c>
       <c r="B214" t="n">
-        <v>15651</v>
+        <v>27762</v>
       </c>
       <c r="C214" t="inlineStr"/>
-      <c r="D214" t="n">
-        <v>229</v>
-      </c>
+      <c r="D214" t="inlineStr"/>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>Ventura, Kristoffer</t>
+          <t>Ventura, Kris</t>
         </is>
       </c>
       <c r="B215" t="n">
@@ -3861,270 +3863,284 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>Vilips, Karl</t>
+          <t>Ventura, Kristoffer</t>
         </is>
       </c>
       <c r="B216" t="n">
-        <v>24304</v>
-      </c>
-      <c r="C216" t="inlineStr">
-        <is>
-          <t>https://pga-tour-res.cloudinary.com/image/upload/c_fill,g_face:center,q_auto,f_auto,dpr_2.0,h_220,w_200,d_stub:default_avatar_light.webp/headshots_54304</t>
-        </is>
-      </c>
+        <v>15651</v>
+      </c>
+      <c r="C216" t="inlineStr"/>
       <c r="D216" t="n">
-        <v>151</v>
+        <v>229</v>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>Villegas, Camilo</t>
+          <t>Vilips, Karl</t>
         </is>
       </c>
       <c r="B217" t="n">
-        <v>9171</v>
-      </c>
-      <c r="C217" t="inlineStr"/>
+        <v>24304</v>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>https://pga-tour-res.cloudinary.com/image/upload/c_fill,g_face:center,q_auto,f_auto,dpr_2.0,h_220,w_200,d_stub:default_avatar_light.webp/headshots_54304</t>
+        </is>
+      </c>
       <c r="D217" t="n">
-        <v>445</v>
+        <v>151</v>
       </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>Walker, Danny</t>
+          <t>Villegas, Camilo</t>
         </is>
       </c>
       <c r="B218" t="n">
-        <v>25003</v>
+        <v>9171</v>
       </c>
       <c r="C218" t="inlineStr"/>
       <c r="D218" t="n">
-        <v>213</v>
+        <v>445</v>
       </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>Wallace, Matt</t>
+          <t>Walker, Danny</t>
         </is>
       </c>
       <c r="B219" t="n">
-        <v>20706</v>
-      </c>
-      <c r="C219" t="inlineStr">
-        <is>
-          <t>https://pga-tour-res.cloudinary.com/image/upload/c_fill,g_face:center,q_auto,f_auto,dpr_2.0,h_220,w_200,d_stub:default_avatar_light.webp/headshots_48887</t>
-        </is>
-      </c>
+        <v>25003</v>
+      </c>
+      <c r="C219" t="inlineStr"/>
       <c r="D219" t="n">
-        <v>95</v>
+        <v>213</v>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>Waring, Paul</t>
+          <t>Wallace, Matt</t>
         </is>
       </c>
       <c r="B220" t="n">
-        <v>12426</v>
+        <v>20706</v>
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>https://pga-tour-res.cloudinary.com/image/upload/c_fill,g_face:center,q_auto,f_auto,dpr_2.0,h_220,w_200,d_stub:default_avatar_light.webp/headshots_31113</t>
+          <t>https://pga-tour-res.cloudinary.com/image/upload/c_fill,g_face:center,q_auto,f_auto,dpr_2.0,h_220,w_200,d_stub:default_avatar_light.webp/headshots_48887</t>
         </is>
       </c>
       <c r="D220" t="n">
-        <v>301</v>
+        <v>95</v>
       </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>Whaley, Vince</t>
+          <t>Waring, Paul</t>
         </is>
       </c>
       <c r="B221" t="n">
-        <v>25908</v>
+        <v>12426</v>
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>https://pga-tour-res.cloudinary.com/image/upload/c_fill,g_face:center,q_auto,f_auto,dpr_2.0,h_220,w_200,d_stub:default_avatar_light.webp/headshots_51894</t>
+          <t>https://pga-tour-res.cloudinary.com/image/upload/c_fill,g_face:center,q_auto,f_auto,dpr_2.0,h_220,w_200,d_stub:default_avatar_light.webp/headshots_31113</t>
         </is>
       </c>
       <c r="D221" t="n">
-        <v>127</v>
+        <v>301</v>
       </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>Widing, Tim</t>
+          <t>Whaley, Vince</t>
         </is>
       </c>
       <c r="B222" t="n">
-        <v>21875</v>
-      </c>
-      <c r="C222" t="inlineStr"/>
-      <c r="D222" t="inlineStr"/>
+        <v>25908</v>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>https://pga-tour-res.cloudinary.com/image/upload/c_fill,g_face:center,q_auto,f_auto,dpr_2.0,h_220,w_200,d_stub:default_avatar_light.webp/headshots_51894</t>
+        </is>
+      </c>
+      <c r="D222" t="n">
+        <v>127</v>
+      </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>Willett, Danny</t>
+          <t>Widing, Tim</t>
         </is>
       </c>
       <c r="B223" t="n">
-        <v>12920</v>
+        <v>21875</v>
       </c>
       <c r="C223" t="inlineStr"/>
-      <c r="D223" t="n">
-        <v>399</v>
-      </c>
+      <c r="D223" t="inlineStr"/>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>Wise, Aaron</t>
+          <t>Willett, Danny</t>
         </is>
       </c>
       <c r="B224" t="n">
-        <v>22051</v>
+        <v>12920</v>
       </c>
       <c r="C224" t="inlineStr"/>
-      <c r="D224" t="inlineStr"/>
+      <c r="D224" t="n">
+        <v>399</v>
+      </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>Woodland, Gary</t>
+          <t>Wise, Aaron</t>
         </is>
       </c>
       <c r="B225" t="n">
-        <v>12577</v>
-      </c>
-      <c r="C225" t="inlineStr">
-        <is>
-          <t>https://pga-tour-res.cloudinary.com/image/upload/c_fill,g_face:center,q_auto,f_auto,dpr_2.0,h_220,w_200,d_stub:default_avatar_light.webp/headshots_31323</t>
-        </is>
-      </c>
-      <c r="D225" t="n">
-        <v>139</v>
-      </c>
+        <v>22051</v>
+      </c>
+      <c r="C225" t="inlineStr"/>
+      <c r="D225" t="inlineStr"/>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>Wu, Dylan</t>
+          <t>Woodland, Gary</t>
         </is>
       </c>
       <c r="B226" t="n">
-        <v>25002</v>
-      </c>
-      <c r="C226" t="inlineStr"/>
+        <v>12577</v>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>https://pga-tour-res.cloudinary.com/image/upload/c_fill,g_face:center,q_auto,f_auto,dpr_2.0,h_220,w_200,d_stub:default_avatar_light.webp/headshots_31323</t>
+        </is>
+      </c>
       <c r="D226" t="n">
-        <v>324</v>
+        <v>139</v>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>Xiong, Norman</t>
+          <t>Wu, Dylan</t>
         </is>
       </c>
       <c r="B227" t="n">
-        <v>24354</v>
+        <v>25002</v>
       </c>
       <c r="C227" t="inlineStr"/>
       <c r="D227" t="n">
-        <v>394</v>
+        <v>324</v>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>Young, Cameron</t>
+          <t>Xiong, Norman</t>
         </is>
       </c>
       <c r="B228" t="n">
-        <v>26651</v>
-      </c>
-      <c r="C228" t="inlineStr">
-        <is>
-          <t>https://pga-tour-res.cloudinary.com/image/upload/c_fill,g_face:center,q_auto,f_auto,dpr_2.0,h_220,w_200,d_stub:default_avatar_light.webp/headshots_57366</t>
-        </is>
-      </c>
+        <v>24354</v>
+      </c>
+      <c r="C228" t="inlineStr"/>
       <c r="D228" t="n">
-        <v>15</v>
+        <v>394</v>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>Young, Carson</t>
+          <t>Yellamaraju, Sudarshan</t>
         </is>
       </c>
       <c r="B229" t="n">
-        <v>23656</v>
-      </c>
-      <c r="C229" t="inlineStr"/>
-      <c r="D229" t="n">
-        <v>158</v>
-      </c>
+        <v>29925</v>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>https://pga-tour-res.cloudinary.com/image/upload/c_fill,g_face:center,q_auto,f_auto,dpr_2.0,h_220,w_200,d_stub:default_avatar_light.webp/headshots_60386</t>
+        </is>
+      </c>
+      <c r="D229" t="inlineStr"/>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>Yu, Kevin</t>
+          <t>Young, Cameron</t>
         </is>
       </c>
       <c r="B230" t="n">
-        <v>17881</v>
+        <v>26651</v>
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>https://pga-tour-res.cloudinary.com/image/upload/c_fill,g_face:center,q_auto,f_auto,dpr_2.0,h_220,w_200,d_stub:default_avatar_light.webp/headshots_45242</t>
+          <t>https://pga-tour-res.cloudinary.com/image/upload/c_fill,g_face:center,q_auto,f_auto,dpr_2.0,h_220,w_200,d_stub:default_avatar_light.webp/headshots_57366</t>
         </is>
       </c>
       <c r="D230" t="n">
-        <v>117</v>
+        <v>15</v>
       </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>Zalatoris, Will</t>
+          <t>Young, Carson</t>
         </is>
       </c>
       <c r="B231" t="n">
-        <v>19428</v>
-      </c>
-      <c r="C231" t="inlineStr">
-        <is>
-          <t>https://pga-tour-res.cloudinary.com/image/upload/c_fill,g_face:center,q_auto,f_auto,dpr_2.0,h_220,w_200,d_stub:default_avatar_light.webp/headshots_47483</t>
-        </is>
-      </c>
+        <v>23656</v>
+      </c>
+      <c r="C231" t="inlineStr"/>
       <c r="D231" t="n">
-        <v>291</v>
+        <v>158</v>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>Smotherman, Austin</t>
+          <t>Yu, Kevin</t>
         </is>
       </c>
       <c r="B232" t="n">
-        <v>50095</v>
+        <v>17881</v>
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>https://pga-tour-res.cloudinary.com/image/upload/c_fill,g_face:center,q_auto,f_auto,dpr_2.0,h_220,w_200,d_stub:default_avatar_light.webp/headshots_50095</t>
-        </is>
-      </c>
-      <c r="D232" t="inlineStr"/>
+          <t>https://pga-tour-res.cloudinary.com/image/upload/c_fill,g_face:center,q_auto,f_auto,dpr_2.0,h_220,w_200,d_stub:default_avatar_light.webp/headshots_45242</t>
+        </is>
+      </c>
+      <c r="D232" t="n">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>Zalatoris, Will</t>
+        </is>
+      </c>
+      <c r="B233" t="n">
+        <v>19428</v>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>https://pga-tour-res.cloudinary.com/image/upload/c_fill,g_face:center,q_auto,f_auto,dpr_2.0,h_220,w_200,d_stub:default_avatar_light.webp/headshots_47483</t>
+        </is>
+      </c>
+      <c r="D233" t="n">
+        <v>291</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
data: field/odds refresh 2026-03-23 12:00 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -4072,7 +4072,9 @@
           <t>https://pga-tour-res.cloudinary.com/image/upload/c_fill,g_face:center,q_auto,f_auto,dpr_2.0,h_220,w_200,d_stub:default_avatar_light.webp/headshots_60386</t>
         </is>
       </c>
-      <c r="D229" t="inlineStr"/>
+      <c r="D229" t="n">
+        <v>145</v>
+      </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">

</xml_diff>

<commit_message>
data: field/odds refresh 2026-03-23 15:04 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -1355,7 +1355,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>181</v>
+        <v>179</v>
       </c>
     </row>
     <row r="59">
@@ -3019,7 +3019,7 @@
         </is>
       </c>
       <c r="D163" t="n">
-        <v>116</v>
+        <v>112</v>
       </c>
     </row>
     <row r="164">
@@ -3857,7 +3857,7 @@
       </c>
       <c r="C215" t="inlineStr"/>
       <c r="D215" t="n">
-        <v>229</v>
+        <v>233</v>
       </c>
     </row>
     <row r="216">
@@ -3871,7 +3871,7 @@
       </c>
       <c r="C216" t="inlineStr"/>
       <c r="D216" t="n">
-        <v>229</v>
+        <v>233</v>
       </c>
     </row>
     <row r="217">

</xml_diff>

<commit_message>
data: field/odds refresh 2026-03-23 18:00 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -1355,7 +1355,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>181</v>
+        <v>179</v>
       </c>
     </row>
     <row r="59">
@@ -3019,7 +3019,7 @@
         </is>
       </c>
       <c r="D163" t="n">
-        <v>116</v>
+        <v>112</v>
       </c>
     </row>
     <row r="164">
@@ -3857,7 +3857,7 @@
       </c>
       <c r="C215" t="inlineStr"/>
       <c r="D215" t="n">
-        <v>229</v>
+        <v>233</v>
       </c>
     </row>
     <row r="216">
@@ -3871,7 +3871,7 @@
       </c>
       <c r="C216" t="inlineStr"/>
       <c r="D216" t="n">
-        <v>229</v>
+        <v>233</v>
       </c>
     </row>
     <row r="217">

</xml_diff>

<commit_message>
data: field/odds refresh 2026-03-24 12:04 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -2223,7 +2223,7 @@
       </c>
       <c r="C112" t="inlineStr"/>
       <c r="D112" t="n">
-        <v>153</v>
+        <v>157</v>
       </c>
     </row>
     <row r="113">
@@ -3001,7 +3001,7 @@
       </c>
       <c r="C162" t="inlineStr"/>
       <c r="D162" t="n">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="163">

</xml_diff>

<commit_message>
data: field/odds refresh 2026-03-24 15:14 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -2223,7 +2223,7 @@
       </c>
       <c r="C112" t="inlineStr"/>
       <c r="D112" t="n">
-        <v>153</v>
+        <v>157</v>
       </c>
     </row>
     <row r="113">
@@ -3001,7 +3001,7 @@
       </c>
       <c r="C162" t="inlineStr"/>
       <c r="D162" t="n">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="163">

</xml_diff>

<commit_message>
data: field/odds refresh 2026-03-30 03:53 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -465,7 +465,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
     </row>
     <row r="3">
@@ -539,7 +539,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>34</v>
+        <v>37</v>
       </c>
     </row>
     <row r="8">
@@ -1251,7 +1251,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="53">
@@ -1563,7 +1563,7 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>58</v>
+        <v>46</v>
       </c>
     </row>
     <row r="72">
@@ -1625,7 +1625,7 @@
         </is>
       </c>
       <c r="D75" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="76">
@@ -1693,7 +1693,7 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="80">
@@ -1811,7 +1811,7 @@
         </is>
       </c>
       <c r="D86" t="n">
-        <v>142</v>
+        <v>148</v>
       </c>
     </row>
     <row r="87">
@@ -2031,7 +2031,7 @@
         </is>
       </c>
       <c r="D100" t="n">
-        <v>57</v>
+        <v>54</v>
       </c>
     </row>
     <row r="101">
@@ -2049,7 +2049,7 @@
         </is>
       </c>
       <c r="D101" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="102">
@@ -2373,7 +2373,7 @@
         </is>
       </c>
       <c r="D122" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
     <row r="123">
@@ -2431,7 +2431,7 @@
         </is>
       </c>
       <c r="D126" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="127">
@@ -2521,7 +2521,7 @@
         </is>
       </c>
       <c r="D131" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="132">
@@ -2637,7 +2637,7 @@
         </is>
       </c>
       <c r="D138" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="139">
@@ -2715,7 +2715,7 @@
         </is>
       </c>
       <c r="D143" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="144">
@@ -3409,7 +3409,7 @@
         </is>
       </c>
       <c r="D187" t="n">
-        <v>485</v>
+        <v>411</v>
       </c>
     </row>
     <row r="188">
@@ -3489,7 +3489,7 @@
       </c>
       <c r="C192" t="inlineStr"/>
       <c r="D192" t="n">
-        <v>306</v>
+        <v>276</v>
       </c>
     </row>
     <row r="193">
@@ -3507,7 +3507,7 @@
         </is>
       </c>
       <c r="D193" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="194">
@@ -3525,7 +3525,7 @@
         </is>
       </c>
       <c r="D194" t="n">
-        <v>64</v>
+        <v>59</v>
       </c>
     </row>
     <row r="195">
@@ -3589,7 +3589,7 @@
         </is>
       </c>
       <c r="D198" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="199">
@@ -3607,7 +3607,7 @@
         </is>
       </c>
       <c r="D199" t="n">
-        <v>415</v>
+        <v>406</v>
       </c>
     </row>
     <row r="200">
@@ -3667,7 +3667,7 @@
         </is>
       </c>
       <c r="D203" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="204">
@@ -3795,7 +3795,7 @@
         </is>
       </c>
       <c r="D211" t="n">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="212">
@@ -3903,7 +3903,7 @@
       </c>
       <c r="C218" t="inlineStr"/>
       <c r="D218" t="n">
-        <v>445</v>
+        <v>453</v>
       </c>
     </row>
     <row r="219">

</xml_diff>

<commit_message>
data: field/odds refresh 2026-03-30 08:52 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -539,7 +539,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="8">
@@ -557,7 +557,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="9">
@@ -667,7 +667,7 @@
       </c>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="n">
-        <v>480</v>
+        <v>320</v>
       </c>
     </row>
     <row r="16">
@@ -717,7 +717,7 @@
       </c>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="n">
-        <v>424</v>
+        <v>423</v>
       </c>
     </row>
     <row r="19">
@@ -781,7 +781,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>91</v>
+        <v>86</v>
       </c>
     </row>
     <row r="23">
@@ -799,7 +799,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="24">
@@ -839,7 +839,7 @@
       </c>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="n">
-        <v>202</v>
+        <v>204</v>
       </c>
     </row>
     <row r="27">
@@ -925,7 +925,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="32">
@@ -1089,7 +1089,7 @@
       </c>
       <c r="C42" t="inlineStr"/>
       <c r="D42" t="n">
-        <v>237</v>
+        <v>244</v>
       </c>
     </row>
     <row r="43">
@@ -1135,7 +1135,7 @@
       </c>
       <c r="C45" t="inlineStr"/>
       <c r="D45" t="n">
-        <v>172</v>
+        <v>174</v>
       </c>
     </row>
     <row r="46">
@@ -1183,7 +1183,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>104</v>
+        <v>107</v>
       </c>
     </row>
     <row r="49">
@@ -1197,7 +1197,7 @@
       </c>
       <c r="C49" t="inlineStr"/>
       <c r="D49" t="n">
-        <v>161</v>
+        <v>168</v>
       </c>
     </row>
     <row r="50">
@@ -1215,7 +1215,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>134</v>
+        <v>137</v>
       </c>
     </row>
     <row r="51">
@@ -1265,7 +1265,7 @@
       </c>
       <c r="C53" t="inlineStr"/>
       <c r="D53" t="n">
-        <v>262</v>
+        <v>267</v>
       </c>
     </row>
     <row r="54">
@@ -1283,7 +1283,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>61</v>
+        <v>65</v>
       </c>
     </row>
     <row r="55">
@@ -1319,7 +1319,7 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>386</v>
+        <v>391</v>
       </c>
     </row>
     <row r="57">
@@ -1355,7 +1355,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>179</v>
+        <v>184</v>
       </c>
     </row>
     <row r="59">
@@ -1373,7 +1373,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>84</v>
+        <v>93</v>
       </c>
     </row>
     <row r="60">
@@ -1487,7 +1487,7 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>103</v>
+        <v>109</v>
       </c>
     </row>
     <row r="67">
@@ -1563,7 +1563,7 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>46</v>
+        <v>50</v>
       </c>
     </row>
     <row r="72">
@@ -1625,7 +1625,7 @@
         </is>
       </c>
       <c r="D75" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="76">
@@ -1675,7 +1675,7 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>132</v>
+        <v>139</v>
       </c>
     </row>
     <row r="79">
@@ -1693,7 +1693,7 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="80">
@@ -1707,7 +1707,7 @@
       </c>
       <c r="C80" t="inlineStr"/>
       <c r="D80" t="n">
-        <v>128</v>
+        <v>132</v>
       </c>
     </row>
     <row r="81">
@@ -1725,7 +1725,7 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="82">
@@ -1739,7 +1739,7 @@
       </c>
       <c r="C82" t="inlineStr"/>
       <c r="D82" t="n">
-        <v>362</v>
+        <v>370</v>
       </c>
     </row>
     <row r="83">
@@ -1757,7 +1757,7 @@
         </is>
       </c>
       <c r="D83" t="n">
-        <v>101</v>
+        <v>106</v>
       </c>
     </row>
     <row r="84">
@@ -1775,7 +1775,7 @@
         </is>
       </c>
       <c r="D84" t="n">
-        <v>47</v>
+        <v>36</v>
       </c>
     </row>
     <row r="85">
@@ -1811,7 +1811,7 @@
         </is>
       </c>
       <c r="D86" t="n">
-        <v>148</v>
+        <v>156</v>
       </c>
     </row>
     <row r="87">
@@ -1829,7 +1829,7 @@
         </is>
       </c>
       <c r="D87" t="n">
-        <v>87</v>
+        <v>94</v>
       </c>
     </row>
     <row r="88">
@@ -1857,7 +1857,7 @@
       </c>
       <c r="C89" t="inlineStr"/>
       <c r="D89" t="n">
-        <v>164</v>
+        <v>159</v>
       </c>
     </row>
     <row r="90">
@@ -1889,7 +1889,7 @@
       </c>
       <c r="C91" t="inlineStr"/>
       <c r="D91" t="n">
-        <v>143</v>
+        <v>149</v>
       </c>
     </row>
     <row r="92">
@@ -1907,7 +1907,7 @@
         </is>
       </c>
       <c r="D92" t="n">
-        <v>116</v>
+        <v>118</v>
       </c>
     </row>
     <row r="93">
@@ -1943,7 +1943,7 @@
         </is>
       </c>
       <c r="D94" t="n">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="95">
@@ -1987,7 +1987,7 @@
       </c>
       <c r="C97" t="inlineStr"/>
       <c r="D97" t="n">
-        <v>124</v>
+        <v>126</v>
       </c>
     </row>
     <row r="98">
@@ -2031,7 +2031,7 @@
         </is>
       </c>
       <c r="D100" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="101">
@@ -2049,7 +2049,7 @@
         </is>
       </c>
       <c r="D101" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="102">
@@ -2067,7 +2067,7 @@
         </is>
       </c>
       <c r="D102" t="n">
-        <v>123</v>
+        <v>129</v>
       </c>
     </row>
     <row r="103">
@@ -2085,7 +2085,7 @@
         </is>
       </c>
       <c r="D103" t="n">
-        <v>94</v>
+        <v>97</v>
       </c>
     </row>
     <row r="104">
@@ -2129,7 +2129,7 @@
       </c>
       <c r="C106" t="inlineStr"/>
       <c r="D106" t="n">
-        <v>247</v>
+        <v>258</v>
       </c>
     </row>
     <row r="107">
@@ -2223,7 +2223,7 @@
       </c>
       <c r="C112" t="inlineStr"/>
       <c r="D112" t="n">
-        <v>157</v>
+        <v>160</v>
       </c>
     </row>
     <row r="113">
@@ -2337,7 +2337,7 @@
       </c>
       <c r="C120" t="inlineStr"/>
       <c r="D120" t="n">
-        <v>195</v>
+        <v>199</v>
       </c>
     </row>
     <row r="121">
@@ -2449,7 +2449,7 @@
         </is>
       </c>
       <c r="D127" t="n">
-        <v>96</v>
+        <v>92</v>
       </c>
     </row>
     <row r="128">
@@ -2467,7 +2467,7 @@
         </is>
       </c>
       <c r="D128" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="129">
@@ -2521,7 +2521,7 @@
         </is>
       </c>
       <c r="D131" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="132">
@@ -2539,7 +2539,7 @@
         </is>
       </c>
       <c r="D132" t="n">
-        <v>118</v>
+        <v>115</v>
       </c>
     </row>
     <row r="133">
@@ -2573,7 +2573,7 @@
         </is>
       </c>
       <c r="D134" t="n">
-        <v>109</v>
+        <v>105</v>
       </c>
     </row>
     <row r="135">
@@ -2651,7 +2651,7 @@
       </c>
       <c r="C139" t="inlineStr"/>
       <c r="D139" t="n">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="140">
@@ -2773,7 +2773,7 @@
         </is>
       </c>
       <c r="D147" t="n">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="148">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="C148" t="inlineStr"/>
       <c r="D148" t="n">
-        <v>108</v>
+        <v>104</v>
       </c>
     </row>
     <row r="149">
@@ -2869,7 +2869,7 @@
         </is>
       </c>
       <c r="D154" t="n">
-        <v>226</v>
+        <v>224</v>
       </c>
     </row>
     <row r="155">
@@ -2905,7 +2905,7 @@
         </is>
       </c>
       <c r="D156" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="157">
@@ -2951,7 +2951,7 @@
       </c>
       <c r="C159" t="inlineStr"/>
       <c r="D159" t="n">
-        <v>177</v>
+        <v>182</v>
       </c>
     </row>
     <row r="160">
@@ -2969,7 +2969,7 @@
         </is>
       </c>
       <c r="D160" t="n">
-        <v>71</v>
+        <v>76</v>
       </c>
     </row>
     <row r="161">
@@ -3001,7 +3001,7 @@
       </c>
       <c r="C162" t="inlineStr"/>
       <c r="D162" t="n">
-        <v>159</v>
+        <v>164</v>
       </c>
     </row>
     <row r="163">
@@ -3019,7 +3019,7 @@
         </is>
       </c>
       <c r="D163" t="n">
-        <v>112</v>
+        <v>114</v>
       </c>
     </row>
     <row r="164">
@@ -3069,7 +3069,7 @@
       </c>
       <c r="C166" t="inlineStr"/>
       <c r="D166" t="n">
-        <v>147</v>
+        <v>144</v>
       </c>
     </row>
     <row r="167">
@@ -3147,7 +3147,7 @@
         </is>
       </c>
       <c r="D171" t="n">
-        <v>68</v>
+        <v>72</v>
       </c>
     </row>
     <row r="172">
@@ -3193,7 +3193,7 @@
       </c>
       <c r="C174" t="inlineStr"/>
       <c r="D174" t="n">
-        <v>137</v>
+        <v>140</v>
       </c>
     </row>
     <row r="175">
@@ -3309,7 +3309,7 @@
         </is>
       </c>
       <c r="D181" t="n">
-        <v>146</v>
+        <v>150</v>
       </c>
     </row>
     <row r="182">
@@ -3327,7 +3327,7 @@
         </is>
       </c>
       <c r="D182" t="n">
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
     <row r="183">
@@ -3345,7 +3345,7 @@
         </is>
       </c>
       <c r="D183" t="n">
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
     <row r="184">
@@ -3409,7 +3409,7 @@
         </is>
       </c>
       <c r="D187" t="n">
-        <v>411</v>
+        <v>416</v>
       </c>
     </row>
     <row r="188">
@@ -3525,7 +3525,7 @@
         </is>
       </c>
       <c r="D194" t="n">
-        <v>59</v>
+        <v>63</v>
       </c>
     </row>
     <row r="195">
@@ -3607,7 +3607,7 @@
         </is>
       </c>
       <c r="D199" t="n">
-        <v>406</v>
+        <v>413</v>
       </c>
     </row>
     <row r="200">
@@ -3635,7 +3635,7 @@
       </c>
       <c r="C201" t="inlineStr"/>
       <c r="D201" t="n">
-        <v>363</v>
+        <v>377</v>
       </c>
     </row>
     <row r="202">
@@ -3649,7 +3649,7 @@
       </c>
       <c r="C202" t="inlineStr"/>
       <c r="D202" t="n">
-        <v>178</v>
+        <v>181</v>
       </c>
     </row>
     <row r="203">
@@ -3667,7 +3667,7 @@
         </is>
       </c>
       <c r="D203" t="n">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="204">
@@ -3721,7 +3721,7 @@
         </is>
       </c>
       <c r="D206" t="n">
-        <v>115</v>
+        <v>120</v>
       </c>
     </row>
     <row r="207">
@@ -3739,7 +3739,7 @@
         </is>
       </c>
       <c r="D207" t="n">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="208">
@@ -3777,7 +3777,7 @@
       </c>
       <c r="C210" t="inlineStr"/>
       <c r="D210" t="n">
-        <v>298</v>
+        <v>308</v>
       </c>
     </row>
     <row r="211">
@@ -3795,7 +3795,7 @@
         </is>
       </c>
       <c r="D211" t="n">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="212">
@@ -3813,7 +3813,7 @@
         </is>
       </c>
       <c r="D212" t="n">
-        <v>156</v>
+        <v>158</v>
       </c>
     </row>
     <row r="213">
@@ -3831,7 +3831,7 @@
         </is>
       </c>
       <c r="D213" t="n">
-        <v>107</v>
+        <v>101</v>
       </c>
     </row>
     <row r="214">
@@ -3857,7 +3857,7 @@
       </c>
       <c r="C215" t="inlineStr"/>
       <c r="D215" t="n">
-        <v>233</v>
+        <v>239</v>
       </c>
     </row>
     <row r="216">
@@ -3871,7 +3871,7 @@
       </c>
       <c r="C216" t="inlineStr"/>
       <c r="D216" t="n">
-        <v>233</v>
+        <v>239</v>
       </c>
     </row>
     <row r="217">
@@ -3889,7 +3889,7 @@
         </is>
       </c>
       <c r="D217" t="n">
-        <v>151</v>
+        <v>146</v>
       </c>
     </row>
     <row r="218">
@@ -3903,7 +3903,7 @@
       </c>
       <c r="C218" t="inlineStr"/>
       <c r="D218" t="n">
-        <v>453</v>
+        <v>460</v>
       </c>
     </row>
     <row r="219">
@@ -3917,7 +3917,7 @@
       </c>
       <c r="C219" t="inlineStr"/>
       <c r="D219" t="n">
-        <v>213</v>
+        <v>215</v>
       </c>
     </row>
     <row r="220">
@@ -3935,7 +3935,7 @@
         </is>
       </c>
       <c r="D220" t="n">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
     <row r="221">
@@ -3953,7 +3953,7 @@
         </is>
       </c>
       <c r="D221" t="n">
-        <v>301</v>
+        <v>298</v>
       </c>
     </row>
     <row r="222">
@@ -3971,7 +3971,7 @@
         </is>
       </c>
       <c r="D222" t="n">
-        <v>127</v>
+        <v>124</v>
       </c>
     </row>
     <row r="223">
@@ -4027,7 +4027,7 @@
         </is>
       </c>
       <c r="D226" t="n">
-        <v>139</v>
+        <v>51</v>
       </c>
     </row>
     <row r="227">
@@ -4041,7 +4041,7 @@
       </c>
       <c r="C227" t="inlineStr"/>
       <c r="D227" t="n">
-        <v>324</v>
+        <v>331</v>
       </c>
     </row>
     <row r="228">
@@ -4073,7 +4073,7 @@
         </is>
       </c>
       <c r="D229" t="n">
-        <v>145</v>
+        <v>131</v>
       </c>
     </row>
     <row r="230">
@@ -4141,7 +4141,7 @@
         </is>
       </c>
       <c r="D233" t="n">
-        <v>291</v>
+        <v>299</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: field/odds refresh 2026-03-30 12:00 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -465,7 +465,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
     </row>
     <row r="3">
@@ -539,7 +539,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>34</v>
+        <v>38</v>
       </c>
     </row>
     <row r="8">
@@ -557,7 +557,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="9">
@@ -667,7 +667,7 @@
       </c>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="n">
-        <v>480</v>
+        <v>320</v>
       </c>
     </row>
     <row r="16">
@@ -717,7 +717,7 @@
       </c>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="n">
-        <v>424</v>
+        <v>423</v>
       </c>
     </row>
     <row r="19">
@@ -781,7 +781,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>91</v>
+        <v>86</v>
       </c>
     </row>
     <row r="23">
@@ -799,7 +799,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="24">
@@ -839,7 +839,7 @@
       </c>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="n">
-        <v>202</v>
+        <v>204</v>
       </c>
     </row>
     <row r="27">
@@ -969,7 +969,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>167</v>
+        <v>175</v>
       </c>
     </row>
     <row r="35">
@@ -1089,7 +1089,7 @@
       </c>
       <c r="C42" t="inlineStr"/>
       <c r="D42" t="n">
-        <v>237</v>
+        <v>244</v>
       </c>
     </row>
     <row r="43">
@@ -1135,7 +1135,7 @@
       </c>
       <c r="C45" t="inlineStr"/>
       <c r="D45" t="n">
-        <v>172</v>
+        <v>174</v>
       </c>
     </row>
     <row r="46">
@@ -1183,7 +1183,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>104</v>
+        <v>107</v>
       </c>
     </row>
     <row r="49">
@@ -1197,7 +1197,7 @@
       </c>
       <c r="C49" t="inlineStr"/>
       <c r="D49" t="n">
-        <v>161</v>
+        <v>168</v>
       </c>
     </row>
     <row r="50">
@@ -1215,7 +1215,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>134</v>
+        <v>137</v>
       </c>
     </row>
     <row r="51">
@@ -1251,7 +1251,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="53">
@@ -1265,7 +1265,7 @@
       </c>
       <c r="C53" t="inlineStr"/>
       <c r="D53" t="n">
-        <v>262</v>
+        <v>267</v>
       </c>
     </row>
     <row r="54">
@@ -1283,7 +1283,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>61</v>
+        <v>65</v>
       </c>
     </row>
     <row r="55">
@@ -1319,7 +1319,7 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>386</v>
+        <v>391</v>
       </c>
     </row>
     <row r="57">
@@ -1355,7 +1355,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>179</v>
+        <v>184</v>
       </c>
     </row>
     <row r="59">
@@ -1373,7 +1373,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>84</v>
+        <v>93</v>
       </c>
     </row>
     <row r="60">
@@ -1487,7 +1487,7 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>103</v>
+        <v>109</v>
       </c>
     </row>
     <row r="67">
@@ -1563,7 +1563,7 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>58</v>
+        <v>50</v>
       </c>
     </row>
     <row r="72">
@@ -1625,7 +1625,7 @@
         </is>
       </c>
       <c r="D75" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="76">
@@ -1675,7 +1675,7 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>132</v>
+        <v>139</v>
       </c>
     </row>
     <row r="79">
@@ -1693,7 +1693,7 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>61</v>
+        <v>64</v>
       </c>
     </row>
     <row r="80">
@@ -1707,7 +1707,7 @@
       </c>
       <c r="C80" t="inlineStr"/>
       <c r="D80" t="n">
-        <v>128</v>
+        <v>132</v>
       </c>
     </row>
     <row r="81">
@@ -1725,7 +1725,7 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="82">
@@ -1739,7 +1739,7 @@
       </c>
       <c r="C82" t="inlineStr"/>
       <c r="D82" t="n">
-        <v>362</v>
+        <v>370</v>
       </c>
     </row>
     <row r="83">
@@ -1757,7 +1757,7 @@
         </is>
       </c>
       <c r="D83" t="n">
-        <v>101</v>
+        <v>106</v>
       </c>
     </row>
     <row r="84">
@@ -1811,7 +1811,7 @@
         </is>
       </c>
       <c r="D86" t="n">
-        <v>142</v>
+        <v>156</v>
       </c>
     </row>
     <row r="87">
@@ -1829,7 +1829,7 @@
         </is>
       </c>
       <c r="D87" t="n">
-        <v>87</v>
+        <v>94</v>
       </c>
     </row>
     <row r="88">
@@ -1857,7 +1857,7 @@
       </c>
       <c r="C89" t="inlineStr"/>
       <c r="D89" t="n">
-        <v>164</v>
+        <v>159</v>
       </c>
     </row>
     <row r="90">
@@ -1889,7 +1889,7 @@
       </c>
       <c r="C91" t="inlineStr"/>
       <c r="D91" t="n">
-        <v>143</v>
+        <v>149</v>
       </c>
     </row>
     <row r="92">
@@ -1907,7 +1907,7 @@
         </is>
       </c>
       <c r="D92" t="n">
-        <v>116</v>
+        <v>118</v>
       </c>
     </row>
     <row r="93">
@@ -1943,7 +1943,7 @@
         </is>
       </c>
       <c r="D94" t="n">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="95">
@@ -1987,7 +1987,7 @@
       </c>
       <c r="C97" t="inlineStr"/>
       <c r="D97" t="n">
-        <v>124</v>
+        <v>126</v>
       </c>
     </row>
     <row r="98">
@@ -2031,7 +2031,7 @@
         </is>
       </c>
       <c r="D100" t="n">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="101">
@@ -2049,7 +2049,7 @@
         </is>
       </c>
       <c r="D101" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="102">
@@ -2067,7 +2067,7 @@
         </is>
       </c>
       <c r="D102" t="n">
-        <v>123</v>
+        <v>129</v>
       </c>
     </row>
     <row r="103">
@@ -2085,7 +2085,7 @@
         </is>
       </c>
       <c r="D103" t="n">
-        <v>94</v>
+        <v>97</v>
       </c>
     </row>
     <row r="104">
@@ -2129,7 +2129,7 @@
       </c>
       <c r="C106" t="inlineStr"/>
       <c r="D106" t="n">
-        <v>247</v>
+        <v>258</v>
       </c>
     </row>
     <row r="107">
@@ -2223,7 +2223,7 @@
       </c>
       <c r="C112" t="inlineStr"/>
       <c r="D112" t="n">
-        <v>157</v>
+        <v>160</v>
       </c>
     </row>
     <row r="113">
@@ -2337,7 +2337,7 @@
       </c>
       <c r="C120" t="inlineStr"/>
       <c r="D120" t="n">
-        <v>195</v>
+        <v>199</v>
       </c>
     </row>
     <row r="121">
@@ -2373,7 +2373,7 @@
         </is>
       </c>
       <c r="D122" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
     <row r="123">
@@ -2431,7 +2431,7 @@
         </is>
       </c>
       <c r="D126" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="127">
@@ -2449,7 +2449,7 @@
         </is>
       </c>
       <c r="D127" t="n">
-        <v>96</v>
+        <v>92</v>
       </c>
     </row>
     <row r="128">
@@ -2467,7 +2467,7 @@
         </is>
       </c>
       <c r="D128" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="129">
@@ -2521,7 +2521,7 @@
         </is>
       </c>
       <c r="D131" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="132">
@@ -2539,7 +2539,7 @@
         </is>
       </c>
       <c r="D132" t="n">
-        <v>118</v>
+        <v>115</v>
       </c>
     </row>
     <row r="133">
@@ -2573,7 +2573,7 @@
         </is>
       </c>
       <c r="D134" t="n">
-        <v>109</v>
+        <v>105</v>
       </c>
     </row>
     <row r="135">
@@ -2619,7 +2619,7 @@
         </is>
       </c>
       <c r="D137" t="n">
-        <v>141</v>
+        <v>147</v>
       </c>
     </row>
     <row r="138">
@@ -2637,7 +2637,7 @@
         </is>
       </c>
       <c r="D138" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="139">
@@ -2651,7 +2651,7 @@
       </c>
       <c r="C139" t="inlineStr"/>
       <c r="D139" t="n">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="140">
@@ -2715,7 +2715,7 @@
         </is>
       </c>
       <c r="D143" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="144">
@@ -2773,7 +2773,7 @@
         </is>
       </c>
       <c r="D147" t="n">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="148">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="C148" t="inlineStr"/>
       <c r="D148" t="n">
-        <v>108</v>
+        <v>104</v>
       </c>
     </row>
     <row r="149">
@@ -2869,7 +2869,7 @@
         </is>
       </c>
       <c r="D154" t="n">
-        <v>226</v>
+        <v>224</v>
       </c>
     </row>
     <row r="155">
@@ -2905,7 +2905,7 @@
         </is>
       </c>
       <c r="D156" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="157">
@@ -2951,7 +2951,7 @@
       </c>
       <c r="C159" t="inlineStr"/>
       <c r="D159" t="n">
-        <v>177</v>
+        <v>182</v>
       </c>
     </row>
     <row r="160">
@@ -2969,7 +2969,7 @@
         </is>
       </c>
       <c r="D160" t="n">
-        <v>71</v>
+        <v>76</v>
       </c>
     </row>
     <row r="161">
@@ -3001,7 +3001,7 @@
       </c>
       <c r="C162" t="inlineStr"/>
       <c r="D162" t="n">
-        <v>159</v>
+        <v>164</v>
       </c>
     </row>
     <row r="163">
@@ -3019,7 +3019,7 @@
         </is>
       </c>
       <c r="D163" t="n">
-        <v>112</v>
+        <v>114</v>
       </c>
     </row>
     <row r="164">
@@ -3069,7 +3069,7 @@
       </c>
       <c r="C166" t="inlineStr"/>
       <c r="D166" t="n">
-        <v>147</v>
+        <v>144</v>
       </c>
     </row>
     <row r="167">
@@ -3147,7 +3147,7 @@
         </is>
       </c>
       <c r="D171" t="n">
-        <v>68</v>
+        <v>72</v>
       </c>
     </row>
     <row r="172">
@@ -3193,7 +3193,7 @@
       </c>
       <c r="C174" t="inlineStr"/>
       <c r="D174" t="n">
-        <v>137</v>
+        <v>140</v>
       </c>
     </row>
     <row r="175">
@@ -3309,7 +3309,7 @@
         </is>
       </c>
       <c r="D181" t="n">
-        <v>146</v>
+        <v>150</v>
       </c>
     </row>
     <row r="182">
@@ -3409,7 +3409,7 @@
         </is>
       </c>
       <c r="D187" t="n">
-        <v>485</v>
+        <v>416</v>
       </c>
     </row>
     <row r="188">
@@ -3489,7 +3489,7 @@
       </c>
       <c r="C192" t="inlineStr"/>
       <c r="D192" t="n">
-        <v>306</v>
+        <v>276</v>
       </c>
     </row>
     <row r="193">
@@ -3507,7 +3507,7 @@
         </is>
       </c>
       <c r="D193" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="194">
@@ -3525,7 +3525,7 @@
         </is>
       </c>
       <c r="D194" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="195">
@@ -3589,7 +3589,7 @@
         </is>
       </c>
       <c r="D198" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="199">
@@ -3607,7 +3607,7 @@
         </is>
       </c>
       <c r="D199" t="n">
-        <v>415</v>
+        <v>413</v>
       </c>
     </row>
     <row r="200">
@@ -3635,7 +3635,7 @@
       </c>
       <c r="C201" t="inlineStr"/>
       <c r="D201" t="n">
-        <v>363</v>
+        <v>377</v>
       </c>
     </row>
     <row r="202">
@@ -3649,7 +3649,7 @@
       </c>
       <c r="C202" t="inlineStr"/>
       <c r="D202" t="n">
-        <v>178</v>
+        <v>181</v>
       </c>
     </row>
     <row r="203">
@@ -3667,7 +3667,7 @@
         </is>
       </c>
       <c r="D203" t="n">
-        <v>62</v>
+        <v>66</v>
       </c>
     </row>
     <row r="204">
@@ -3721,7 +3721,7 @@
         </is>
       </c>
       <c r="D206" t="n">
-        <v>115</v>
+        <v>120</v>
       </c>
     </row>
     <row r="207">
@@ -3739,7 +3739,7 @@
         </is>
       </c>
       <c r="D207" t="n">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="208">
@@ -3777,7 +3777,7 @@
       </c>
       <c r="C210" t="inlineStr"/>
       <c r="D210" t="n">
-        <v>298</v>
+        <v>308</v>
       </c>
     </row>
     <row r="211">
@@ -3795,7 +3795,7 @@
         </is>
       </c>
       <c r="D211" t="n">
-        <v>53</v>
+        <v>57</v>
       </c>
     </row>
     <row r="212">
@@ -3813,7 +3813,7 @@
         </is>
       </c>
       <c r="D212" t="n">
-        <v>156</v>
+        <v>158</v>
       </c>
     </row>
     <row r="213">
@@ -3831,7 +3831,7 @@
         </is>
       </c>
       <c r="D213" t="n">
-        <v>107</v>
+        <v>101</v>
       </c>
     </row>
     <row r="214">
@@ -3857,7 +3857,7 @@
       </c>
       <c r="C215" t="inlineStr"/>
       <c r="D215" t="n">
-        <v>233</v>
+        <v>239</v>
       </c>
     </row>
     <row r="216">
@@ -3871,7 +3871,7 @@
       </c>
       <c r="C216" t="inlineStr"/>
       <c r="D216" t="n">
-        <v>233</v>
+        <v>239</v>
       </c>
     </row>
     <row r="217">
@@ -3889,7 +3889,7 @@
         </is>
       </c>
       <c r="D217" t="n">
-        <v>151</v>
+        <v>146</v>
       </c>
     </row>
     <row r="218">
@@ -3903,7 +3903,7 @@
       </c>
       <c r="C218" t="inlineStr"/>
       <c r="D218" t="n">
-        <v>445</v>
+        <v>460</v>
       </c>
     </row>
     <row r="219">
@@ -3917,7 +3917,7 @@
       </c>
       <c r="C219" t="inlineStr"/>
       <c r="D219" t="n">
-        <v>213</v>
+        <v>215</v>
       </c>
     </row>
     <row r="220">
@@ -3935,7 +3935,7 @@
         </is>
       </c>
       <c r="D220" t="n">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
     <row r="221">
@@ -3953,7 +3953,7 @@
         </is>
       </c>
       <c r="D221" t="n">
-        <v>301</v>
+        <v>298</v>
       </c>
     </row>
     <row r="222">
@@ -3971,7 +3971,7 @@
         </is>
       </c>
       <c r="D222" t="n">
-        <v>127</v>
+        <v>124</v>
       </c>
     </row>
     <row r="223">
@@ -4027,7 +4027,7 @@
         </is>
       </c>
       <c r="D226" t="n">
-        <v>139</v>
+        <v>51</v>
       </c>
     </row>
     <row r="227">
@@ -4041,7 +4041,7 @@
       </c>
       <c r="C227" t="inlineStr"/>
       <c r="D227" t="n">
-        <v>324</v>
+        <v>331</v>
       </c>
     </row>
     <row r="228">
@@ -4073,7 +4073,7 @@
         </is>
       </c>
       <c r="D229" t="n">
-        <v>145</v>
+        <v>131</v>
       </c>
     </row>
     <row r="230">
@@ -4141,7 +4141,7 @@
         </is>
       </c>
       <c r="D233" t="n">
-        <v>291</v>
+        <v>299</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: field/odds refresh 2026-03-30 12:45 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -969,7 +969,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>167</v>
+        <v>175</v>
       </c>
     </row>
     <row r="35">
@@ -2619,7 +2619,7 @@
         </is>
       </c>
       <c r="D137" t="n">
-        <v>141</v>
+        <v>147</v>
       </c>
     </row>
     <row r="138">

</xml_diff>

<commit_message>
data: field/odds refresh 2026-03-31 15:12 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -763,7 +763,7 @@
       </c>
       <c r="C21" t="inlineStr"/>
       <c r="D21" t="n">
-        <v>262</v>
+        <v>299</v>
       </c>
     </row>
     <row r="22">
@@ -4105,7 +4105,7 @@
       </c>
       <c r="C231" t="inlineStr"/>
       <c r="D231" t="n">
-        <v>158</v>
+        <v>163</v>
       </c>
     </row>
     <row r="232">

</xml_diff>

<commit_message>
data: field/odds refresh 2026-03-31 18:00 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -763,7 +763,7 @@
       </c>
       <c r="C21" t="inlineStr"/>
       <c r="D21" t="n">
-        <v>262</v>
+        <v>299</v>
       </c>
     </row>
     <row r="22">
@@ -4105,7 +4105,7 @@
       </c>
       <c r="C231" t="inlineStr"/>
       <c r="D231" t="n">
-        <v>158</v>
+        <v>163</v>
       </c>
     </row>
     <row r="232">

</xml_diff>

<commit_message>
data: field/odds refresh 2026-04-05 12:00 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D233"/>
+  <dimension ref="A1:D234"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4144,6 +4144,22 @@
         <v>299</v>
       </c>
     </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>Jarvis, Casey</t>
+        </is>
+      </c>
+      <c r="B234" t="n">
+        <v>26947</v>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>https://pga-tour-res.cloudinary.com/image/upload/c_fill,g_face:center,q_auto,f_auto,dpr_2.0,h_220,w_200,d_stub:default_avatar_light.webp/headshots_57688</t>
+        </is>
+      </c>
+      <c r="D234" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
data: field/odds refresh 2026-04-06 03:55 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -465,7 +465,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="3">
@@ -575,7 +575,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="10">
@@ -607,7 +607,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="12">
@@ -639,7 +639,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="14">
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>102</v>
+        <v>112</v>
       </c>
     </row>
     <row r="18">
@@ -857,7 +857,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>72</v>
+        <v>78</v>
       </c>
     </row>
     <row r="28">
@@ -907,7 +907,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>40</v>
+        <v>44</v>
       </c>
     </row>
     <row r="31">
@@ -1023,7 +1023,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>33</v>
+        <v>24</v>
       </c>
     </row>
     <row r="38">
@@ -1107,7 +1107,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="44">
@@ -1121,7 +1121,7 @@
       </c>
       <c r="C44" t="inlineStr"/>
       <c r="D44" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="45">
@@ -1233,7 +1233,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
     </row>
     <row r="52">
@@ -1301,7 +1301,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>45</v>
+        <v>51</v>
       </c>
     </row>
     <row r="56">
@@ -1337,7 +1337,7 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="58">
@@ -1419,7 +1419,7 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="63">
@@ -1437,7 +1437,7 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="64">
@@ -1607,7 +1607,7 @@
         </is>
       </c>
       <c r="D74" t="n">
-        <v>25</v>
+        <v>31</v>
       </c>
     </row>
     <row r="75">
@@ -1625,7 +1625,7 @@
         </is>
       </c>
       <c r="D75" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="76">
@@ -1793,7 +1793,7 @@
         </is>
       </c>
       <c r="D85" t="n">
-        <v>53</v>
+        <v>57</v>
       </c>
     </row>
     <row r="86">
@@ -1811,7 +1811,7 @@
         </is>
       </c>
       <c r="D86" t="n">
-        <v>156</v>
+        <v>163</v>
       </c>
     </row>
     <row r="87">
@@ -1875,7 +1875,7 @@
         </is>
       </c>
       <c r="D90" t="n">
-        <v>18</v>
+        <v>22</v>
       </c>
     </row>
     <row r="91">
@@ -1925,7 +1925,7 @@
         </is>
       </c>
       <c r="D93" t="n">
-        <v>67</v>
+        <v>71</v>
       </c>
     </row>
     <row r="94">
@@ -1973,7 +1973,7 @@
       </c>
       <c r="C96" t="inlineStr"/>
       <c r="D96" t="n">
-        <v>278</v>
+        <v>321</v>
       </c>
     </row>
     <row r="97">
@@ -2031,7 +2031,7 @@
         </is>
       </c>
       <c r="D100" t="n">
-        <v>56</v>
+        <v>43</v>
       </c>
     </row>
     <row r="101">
@@ -2049,7 +2049,7 @@
         </is>
       </c>
       <c r="D101" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="102">
@@ -2115,7 +2115,7 @@
         </is>
       </c>
       <c r="D105" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="106">
@@ -2177,7 +2177,7 @@
         </is>
       </c>
       <c r="D109" t="n">
-        <v>162</v>
+        <v>169</v>
       </c>
     </row>
     <row r="110">
@@ -2291,7 +2291,7 @@
         </is>
       </c>
       <c r="D117" t="n">
-        <v>31</v>
+        <v>25</v>
       </c>
     </row>
     <row r="118">
@@ -2373,7 +2373,7 @@
         </is>
       </c>
       <c r="D122" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
     </row>
     <row r="123">
@@ -2467,7 +2467,7 @@
         </is>
       </c>
       <c r="D128" t="n">
-        <v>46</v>
+        <v>49</v>
       </c>
     </row>
     <row r="129">
@@ -2637,7 +2637,7 @@
         </is>
       </c>
       <c r="D138" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="139">
@@ -2679,7 +2679,7 @@
       </c>
       <c r="C141" t="inlineStr"/>
       <c r="D141" t="n">
-        <v>66</v>
+        <v>69</v>
       </c>
     </row>
     <row r="142">
@@ -2773,7 +2773,7 @@
         </is>
       </c>
       <c r="D147" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="148">
@@ -3037,7 +3037,7 @@
         </is>
       </c>
       <c r="D164" t="n">
-        <v>67</v>
+        <v>30</v>
       </c>
     </row>
     <row r="165">
@@ -3099,7 +3099,7 @@
         </is>
       </c>
       <c r="D168" t="n">
-        <v>17</v>
+        <v>23</v>
       </c>
     </row>
     <row r="169">
@@ -3129,7 +3129,7 @@
         </is>
       </c>
       <c r="D170" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
     </row>
     <row r="171">
@@ -3165,7 +3165,7 @@
         </is>
       </c>
       <c r="D172" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="173">
@@ -3273,7 +3273,7 @@
         </is>
       </c>
       <c r="D179" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="180">
@@ -3363,7 +3363,7 @@
         </is>
       </c>
       <c r="D184" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="185">
@@ -3459,7 +3459,7 @@
         </is>
       </c>
       <c r="D190" t="n">
-        <v>227</v>
+        <v>222</v>
       </c>
     </row>
     <row r="191">
@@ -3507,7 +3507,7 @@
         </is>
       </c>
       <c r="D193" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
     </row>
     <row r="194">
@@ -3525,7 +3525,7 @@
         </is>
       </c>
       <c r="D194" t="n">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="195">
@@ -3557,7 +3557,7 @@
         </is>
       </c>
       <c r="D196" t="n">
-        <v>50</v>
+        <v>45</v>
       </c>
     </row>
     <row r="197">
@@ -3571,7 +3571,7 @@
       </c>
       <c r="C197" t="inlineStr"/>
       <c r="D197" t="n">
-        <v>50</v>
+        <v>45</v>
       </c>
     </row>
     <row r="198">
@@ -3589,7 +3589,7 @@
         </is>
       </c>
       <c r="D198" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="199">
@@ -3667,7 +3667,7 @@
         </is>
       </c>
       <c r="D203" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="204">
@@ -3703,7 +3703,7 @@
         </is>
       </c>
       <c r="D205" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="206">
@@ -3795,7 +3795,7 @@
         </is>
       </c>
       <c r="D211" t="n">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="212">
@@ -3997,7 +3997,7 @@
       </c>
       <c r="C224" t="inlineStr"/>
       <c r="D224" t="n">
-        <v>399</v>
+        <v>400</v>
       </c>
     </row>
     <row r="225">
@@ -4027,7 +4027,7 @@
         </is>
       </c>
       <c r="D226" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="227">
@@ -4091,7 +4091,7 @@
         </is>
       </c>
       <c r="D230" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
     </row>
     <row r="231">

</xml_diff>

<commit_message>
data: field/odds refresh 2026-04-07 20:57 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -465,7 +465,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="3">
@@ -575,7 +575,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="10">
@@ -607,7 +607,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="12">
@@ -639,7 +639,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="14">
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>102</v>
+        <v>112</v>
       </c>
     </row>
     <row r="18">
@@ -857,7 +857,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>72</v>
+        <v>78</v>
       </c>
     </row>
     <row r="28">
@@ -907,7 +907,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>40</v>
+        <v>44</v>
       </c>
     </row>
     <row r="31">
@@ -1023,7 +1023,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>33</v>
+        <v>24</v>
       </c>
     </row>
     <row r="38">
@@ -1107,7 +1107,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="44">
@@ -1121,7 +1121,7 @@
       </c>
       <c r="C44" t="inlineStr"/>
       <c r="D44" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="45">
@@ -1233,7 +1233,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
     </row>
     <row r="52">
@@ -1301,7 +1301,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>45</v>
+        <v>51</v>
       </c>
     </row>
     <row r="56">
@@ -1337,7 +1337,7 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="58">
@@ -1419,7 +1419,7 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="63">
@@ -1437,7 +1437,7 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="64">
@@ -1607,7 +1607,7 @@
         </is>
       </c>
       <c r="D74" t="n">
-        <v>25</v>
+        <v>31</v>
       </c>
     </row>
     <row r="75">
@@ -1625,7 +1625,7 @@
         </is>
       </c>
       <c r="D75" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="76">
@@ -1775,7 +1775,7 @@
         </is>
       </c>
       <c r="D84" t="n">
-        <v>47</v>
+        <v>36</v>
       </c>
     </row>
     <row r="85">
@@ -1793,7 +1793,7 @@
         </is>
       </c>
       <c r="D85" t="n">
-        <v>53</v>
+        <v>57</v>
       </c>
     </row>
     <row r="86">
@@ -1811,7 +1811,7 @@
         </is>
       </c>
       <c r="D86" t="n">
-        <v>156</v>
+        <v>163</v>
       </c>
     </row>
     <row r="87">
@@ -1875,7 +1875,7 @@
         </is>
       </c>
       <c r="D90" t="n">
-        <v>18</v>
+        <v>22</v>
       </c>
     </row>
     <row r="91">
@@ -1925,7 +1925,7 @@
         </is>
       </c>
       <c r="D93" t="n">
-        <v>67</v>
+        <v>71</v>
       </c>
     </row>
     <row r="94">
@@ -1973,7 +1973,7 @@
       </c>
       <c r="C96" t="inlineStr"/>
       <c r="D96" t="n">
-        <v>278</v>
+        <v>321</v>
       </c>
     </row>
     <row r="97">
@@ -2031,7 +2031,7 @@
         </is>
       </c>
       <c r="D100" t="n">
-        <v>56</v>
+        <v>43</v>
       </c>
     </row>
     <row r="101">
@@ -2049,7 +2049,7 @@
         </is>
       </c>
       <c r="D101" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="102">
@@ -2115,7 +2115,7 @@
         </is>
       </c>
       <c r="D105" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="106">
@@ -2177,7 +2177,7 @@
         </is>
       </c>
       <c r="D109" t="n">
-        <v>162</v>
+        <v>169</v>
       </c>
     </row>
     <row r="110">
@@ -2291,7 +2291,7 @@
         </is>
       </c>
       <c r="D117" t="n">
-        <v>31</v>
+        <v>25</v>
       </c>
     </row>
     <row r="118">
@@ -2373,7 +2373,7 @@
         </is>
       </c>
       <c r="D122" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
     </row>
     <row r="123">
@@ -2467,7 +2467,7 @@
         </is>
       </c>
       <c r="D128" t="n">
-        <v>46</v>
+        <v>49</v>
       </c>
     </row>
     <row r="129">
@@ -2637,7 +2637,7 @@
         </is>
       </c>
       <c r="D138" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="139">
@@ -2679,7 +2679,7 @@
       </c>
       <c r="C141" t="inlineStr"/>
       <c r="D141" t="n">
-        <v>66</v>
+        <v>69</v>
       </c>
     </row>
     <row r="142">
@@ -2773,7 +2773,7 @@
         </is>
       </c>
       <c r="D147" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="148">
@@ -3037,7 +3037,7 @@
         </is>
       </c>
       <c r="D164" t="n">
-        <v>67</v>
+        <v>30</v>
       </c>
     </row>
     <row r="165">
@@ -3099,7 +3099,7 @@
         </is>
       </c>
       <c r="D168" t="n">
-        <v>17</v>
+        <v>23</v>
       </c>
     </row>
     <row r="169">
@@ -3129,7 +3129,7 @@
         </is>
       </c>
       <c r="D170" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
     </row>
     <row r="171">
@@ -3165,7 +3165,7 @@
         </is>
       </c>
       <c r="D172" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="173">
@@ -3273,7 +3273,7 @@
         </is>
       </c>
       <c r="D179" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="180">
@@ -3363,7 +3363,7 @@
         </is>
       </c>
       <c r="D184" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="185">
@@ -3459,7 +3459,7 @@
         </is>
       </c>
       <c r="D190" t="n">
-        <v>227</v>
+        <v>222</v>
       </c>
     </row>
     <row r="191">
@@ -3507,7 +3507,7 @@
         </is>
       </c>
       <c r="D193" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
     </row>
     <row r="194">
@@ -3525,7 +3525,7 @@
         </is>
       </c>
       <c r="D194" t="n">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="195">
@@ -3557,7 +3557,7 @@
         </is>
       </c>
       <c r="D196" t="n">
-        <v>50</v>
+        <v>45</v>
       </c>
     </row>
     <row r="197">
@@ -3571,7 +3571,7 @@
       </c>
       <c r="C197" t="inlineStr"/>
       <c r="D197" t="n">
-        <v>50</v>
+        <v>45</v>
       </c>
     </row>
     <row r="198">
@@ -3589,7 +3589,7 @@
         </is>
       </c>
       <c r="D198" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="199">
@@ -3667,7 +3667,7 @@
         </is>
       </c>
       <c r="D203" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="204">
@@ -3703,7 +3703,7 @@
         </is>
       </c>
       <c r="D205" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="206">
@@ -3795,7 +3795,7 @@
         </is>
       </c>
       <c r="D211" t="n">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="212">
@@ -3997,7 +3997,7 @@
       </c>
       <c r="C224" t="inlineStr"/>
       <c r="D224" t="n">
-        <v>399</v>
+        <v>400</v>
       </c>
     </row>
     <row r="225">
@@ -4027,7 +4027,7 @@
         </is>
       </c>
       <c r="D226" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="227">
@@ -4091,7 +4091,7 @@
         </is>
       </c>
       <c r="D230" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
     </row>
     <row r="231">
@@ -4158,7 +4158,9 @@
           <t>https://pga-tour-res.cloudinary.com/image/upload/c_fill,g_face:center,q_auto,f_auto,dpr_2.0,h_220,w_200,d_stub:default_avatar_light.webp/headshots_57688</t>
         </is>
       </c>
-      <c r="D234" t="inlineStr"/>
+      <c r="D234" t="n">
+        <v>70</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
data: field/odds refresh 2026-04-13 04:14 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -781,7 +781,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="23">
@@ -799,7 +799,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>80</v>
+        <v>76</v>
       </c>
     </row>
     <row r="24">
@@ -925,7 +925,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="32">
@@ -1183,7 +1183,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>107</v>
+        <v>111</v>
       </c>
     </row>
     <row r="49">
@@ -1215,7 +1215,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="51">
@@ -1373,7 +1373,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>93</v>
+        <v>96</v>
       </c>
     </row>
     <row r="60">
@@ -1643,7 +1643,7 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="77">
@@ -1675,7 +1675,7 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>139</v>
+        <v>141</v>
       </c>
     </row>
     <row r="79">
@@ -1693,7 +1693,7 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>64</v>
+        <v>55</v>
       </c>
     </row>
     <row r="80">
@@ -1757,7 +1757,7 @@
         </is>
       </c>
       <c r="D83" t="n">
-        <v>106</v>
+        <v>110</v>
       </c>
     </row>
     <row r="84">
@@ -2449,7 +2449,7 @@
         </is>
       </c>
       <c r="D127" t="n">
-        <v>92</v>
+        <v>95</v>
       </c>
     </row>
     <row r="128">
@@ -2651,7 +2651,7 @@
       </c>
       <c r="C139" t="inlineStr"/>
       <c r="D139" t="n">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="140">
@@ -2887,7 +2887,7 @@
         </is>
       </c>
       <c r="D155" t="n">
-        <v>70</v>
+        <v>74</v>
       </c>
     </row>
     <row r="156">
@@ -2969,7 +2969,7 @@
         </is>
       </c>
       <c r="D160" t="n">
-        <v>76</v>
+        <v>79</v>
       </c>
     </row>
     <row r="161">
@@ -3019,7 +3019,7 @@
         </is>
       </c>
       <c r="D163" t="n">
-        <v>114</v>
+        <v>93</v>
       </c>
     </row>
     <row r="164">
@@ -3309,7 +3309,7 @@
         </is>
       </c>
       <c r="D181" t="n">
-        <v>150</v>
+        <v>148</v>
       </c>
     </row>
     <row r="182">
@@ -3685,7 +3685,7 @@
         </is>
       </c>
       <c r="D204" t="n">
-        <v>80</v>
+        <v>73</v>
       </c>
     </row>
     <row r="205">
@@ -3831,7 +3831,7 @@
         </is>
       </c>
       <c r="D213" t="n">
-        <v>101</v>
+        <v>107</v>
       </c>
     </row>
     <row r="214">
@@ -3889,7 +3889,7 @@
         </is>
       </c>
       <c r="D217" t="n">
-        <v>146</v>
+        <v>152</v>
       </c>
     </row>
     <row r="218">
@@ -3935,7 +3935,7 @@
         </is>
       </c>
       <c r="D220" t="n">
-        <v>96</v>
+        <v>66</v>
       </c>
     </row>
     <row r="221">
@@ -4073,7 +4073,7 @@
         </is>
       </c>
       <c r="D229" t="n">
-        <v>131</v>
+        <v>119</v>
       </c>
     </row>
     <row r="230">

</xml_diff>

<commit_message>
data: field/odds refresh 2026-04-13 08:59 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -539,7 +539,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="8">
@@ -575,7 +575,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
     </row>
     <row r="10">
@@ -685,7 +685,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>33</v>
+        <v>28</v>
       </c>
     </row>
     <row r="17">
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>112</v>
+        <v>100</v>
       </c>
     </row>
     <row r="18">
@@ -749,7 +749,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="21">
@@ -857,7 +857,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>78</v>
+        <v>71</v>
       </c>
     </row>
     <row r="28">
@@ -907,7 +907,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="31">
@@ -925,7 +925,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="32">
@@ -1005,7 +1005,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="37">
@@ -1107,7 +1107,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="44">
@@ -1121,7 +1121,7 @@
       </c>
       <c r="C44" t="inlineStr"/>
       <c r="D44" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="45">
@@ -1165,7 +1165,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="48">
@@ -1183,7 +1183,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="49">
@@ -1215,7 +1215,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>138</v>
+        <v>142</v>
       </c>
     </row>
     <row r="51">
@@ -1233,7 +1233,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="52">
@@ -1251,7 +1251,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="53">
@@ -1283,7 +1283,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="55">
@@ -1301,7 +1301,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>51</v>
+        <v>54</v>
       </c>
     </row>
     <row r="56">
@@ -1337,7 +1337,7 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>29</v>
+        <v>32</v>
       </c>
     </row>
     <row r="58">
@@ -1373,7 +1373,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="60">
@@ -1531,7 +1531,7 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="70">
@@ -1625,7 +1625,7 @@
         </is>
       </c>
       <c r="D75" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
     </row>
     <row r="76">
@@ -1675,7 +1675,7 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>141</v>
+        <v>144</v>
       </c>
     </row>
     <row r="79">
@@ -1693,7 +1693,7 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="80">
@@ -1757,7 +1757,7 @@
         </is>
       </c>
       <c r="D83" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="84">
@@ -1775,7 +1775,7 @@
         </is>
       </c>
       <c r="D84" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="85">
@@ -1811,7 +1811,7 @@
         </is>
       </c>
       <c r="D86" t="n">
-        <v>163</v>
+        <v>117</v>
       </c>
     </row>
     <row r="87">
@@ -1829,7 +1829,7 @@
         </is>
       </c>
       <c r="D87" t="n">
-        <v>94</v>
+        <v>97</v>
       </c>
     </row>
     <row r="88">
@@ -1925,7 +1925,7 @@
         </is>
       </c>
       <c r="D93" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="94">
@@ -2031,7 +2031,7 @@
         </is>
       </c>
       <c r="D100" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="101">
@@ -2049,7 +2049,7 @@
         </is>
       </c>
       <c r="D101" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="102">
@@ -2115,7 +2115,7 @@
         </is>
       </c>
       <c r="D105" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="106">
@@ -2147,7 +2147,7 @@
         </is>
       </c>
       <c r="D107" t="n">
-        <v>42</v>
+        <v>36</v>
       </c>
     </row>
     <row r="108">
@@ -2291,7 +2291,7 @@
         </is>
       </c>
       <c r="D117" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="118">
@@ -2355,7 +2355,7 @@
         </is>
       </c>
       <c r="D121" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="122">
@@ -2373,7 +2373,7 @@
         </is>
       </c>
       <c r="D122" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="123">
@@ -2449,7 +2449,7 @@
         </is>
       </c>
       <c r="D127" t="n">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
     <row r="128">
@@ -2467,7 +2467,7 @@
         </is>
       </c>
       <c r="D128" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="129">
@@ -2521,7 +2521,7 @@
         </is>
       </c>
       <c r="D131" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="132">
@@ -2637,7 +2637,7 @@
         </is>
       </c>
       <c r="D138" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="139">
@@ -2773,7 +2773,7 @@
         </is>
       </c>
       <c r="D147" t="n">
-        <v>48</v>
+        <v>53</v>
       </c>
     </row>
     <row r="148">
@@ -2887,7 +2887,7 @@
         </is>
       </c>
       <c r="D155" t="n">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="156">
@@ -2987,7 +2987,7 @@
         </is>
       </c>
       <c r="D161" t="n">
-        <v>77</v>
+        <v>81</v>
       </c>
     </row>
     <row r="162">
@@ -3019,7 +3019,7 @@
         </is>
       </c>
       <c r="D163" t="n">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="164">
@@ -3147,7 +3147,7 @@
         </is>
       </c>
       <c r="D171" t="n">
-        <v>72</v>
+        <v>74</v>
       </c>
     </row>
     <row r="172">
@@ -3165,7 +3165,7 @@
         </is>
       </c>
       <c r="D172" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
     </row>
     <row r="173">
@@ -3273,7 +3273,7 @@
         </is>
       </c>
       <c r="D179" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="180">
@@ -3309,7 +3309,7 @@
         </is>
       </c>
       <c r="D181" t="n">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="182">
@@ -3507,7 +3507,7 @@
         </is>
       </c>
       <c r="D193" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="194">
@@ -3525,7 +3525,7 @@
         </is>
       </c>
       <c r="D194" t="n">
-        <v>61</v>
+        <v>52</v>
       </c>
     </row>
     <row r="195">
@@ -3667,7 +3667,7 @@
         </is>
       </c>
       <c r="D203" t="n">
-        <v>67</v>
+        <v>64</v>
       </c>
     </row>
     <row r="204">
@@ -3795,7 +3795,7 @@
         </is>
       </c>
       <c r="D211" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="212">
@@ -3831,7 +3831,7 @@
         </is>
       </c>
       <c r="D213" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="214">
@@ -3889,7 +3889,7 @@
         </is>
       </c>
       <c r="D217" t="n">
-        <v>152</v>
+        <v>154</v>
       </c>
     </row>
     <row r="218">
@@ -3935,7 +3935,7 @@
         </is>
       </c>
       <c r="D220" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="221">
@@ -4027,7 +4027,7 @@
         </is>
       </c>
       <c r="D226" t="n">
-        <v>52</v>
+        <v>49</v>
       </c>
     </row>
     <row r="227">
@@ -4073,7 +4073,7 @@
         </is>
       </c>
       <c r="D229" t="n">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="230">

</xml_diff>

<commit_message>
data: field/odds refresh 2026-04-13 12:00 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -539,7 +539,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="8">
@@ -575,7 +575,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
     </row>
     <row r="10">
@@ -685,7 +685,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>33</v>
+        <v>28</v>
       </c>
     </row>
     <row r="17">
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>112</v>
+        <v>100</v>
       </c>
     </row>
     <row r="18">
@@ -749,7 +749,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="21">
@@ -781,7 +781,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="23">
@@ -799,7 +799,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>80</v>
+        <v>76</v>
       </c>
     </row>
     <row r="24">
@@ -857,7 +857,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>78</v>
+        <v>71</v>
       </c>
     </row>
     <row r="28">
@@ -907,7 +907,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="31">
@@ -925,7 +925,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>51</v>
+        <v>55</v>
       </c>
     </row>
     <row r="32">
@@ -1005,7 +1005,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="37">
@@ -1107,7 +1107,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="44">
@@ -1121,7 +1121,7 @@
       </c>
       <c r="C44" t="inlineStr"/>
       <c r="D44" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="45">
@@ -1165,7 +1165,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="48">
@@ -1183,7 +1183,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>107</v>
+        <v>110</v>
       </c>
     </row>
     <row r="49">
@@ -1215,7 +1215,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>137</v>
+        <v>142</v>
       </c>
     </row>
     <row r="51">
@@ -1233,7 +1233,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="52">
@@ -1251,7 +1251,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="53">
@@ -1283,7 +1283,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="55">
@@ -1301,7 +1301,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>51</v>
+        <v>54</v>
       </c>
     </row>
     <row r="56">
@@ -1337,7 +1337,7 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>29</v>
+        <v>32</v>
       </c>
     </row>
     <row r="58">
@@ -1373,7 +1373,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>93</v>
+        <v>95</v>
       </c>
     </row>
     <row r="60">
@@ -1531,7 +1531,7 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="70">
@@ -1625,7 +1625,7 @@
         </is>
       </c>
       <c r="D75" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
     </row>
     <row r="76">
@@ -1643,7 +1643,7 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="77">
@@ -1675,7 +1675,7 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>139</v>
+        <v>144</v>
       </c>
     </row>
     <row r="79">
@@ -1693,7 +1693,7 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>64</v>
+        <v>56</v>
       </c>
     </row>
     <row r="80">
@@ -1757,7 +1757,7 @@
         </is>
       </c>
       <c r="D83" t="n">
-        <v>106</v>
+        <v>111</v>
       </c>
     </row>
     <row r="84">
@@ -1775,7 +1775,7 @@
         </is>
       </c>
       <c r="D84" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="85">
@@ -1811,7 +1811,7 @@
         </is>
       </c>
       <c r="D86" t="n">
-        <v>163</v>
+        <v>117</v>
       </c>
     </row>
     <row r="87">
@@ -1829,7 +1829,7 @@
         </is>
       </c>
       <c r="D87" t="n">
-        <v>94</v>
+        <v>97</v>
       </c>
     </row>
     <row r="88">
@@ -1925,7 +1925,7 @@
         </is>
       </c>
       <c r="D93" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="94">
@@ -2031,7 +2031,7 @@
         </is>
       </c>
       <c r="D100" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="101">
@@ -2049,7 +2049,7 @@
         </is>
       </c>
       <c r="D101" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="102">
@@ -2115,7 +2115,7 @@
         </is>
       </c>
       <c r="D105" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="106">
@@ -2147,7 +2147,7 @@
         </is>
       </c>
       <c r="D107" t="n">
-        <v>42</v>
+        <v>36</v>
       </c>
     </row>
     <row r="108">
@@ -2291,7 +2291,7 @@
         </is>
       </c>
       <c r="D117" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="118">
@@ -2355,7 +2355,7 @@
         </is>
       </c>
       <c r="D121" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="122">
@@ -2373,7 +2373,7 @@
         </is>
       </c>
       <c r="D122" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="123">
@@ -2449,7 +2449,7 @@
         </is>
       </c>
       <c r="D127" t="n">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="128">
@@ -2467,7 +2467,7 @@
         </is>
       </c>
       <c r="D128" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="129">
@@ -2521,7 +2521,7 @@
         </is>
       </c>
       <c r="D131" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="132">
@@ -2637,7 +2637,7 @@
         </is>
       </c>
       <c r="D138" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="139">
@@ -2651,7 +2651,7 @@
       </c>
       <c r="C139" t="inlineStr"/>
       <c r="D139" t="n">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="140">
@@ -2773,7 +2773,7 @@
         </is>
       </c>
       <c r="D147" t="n">
-        <v>48</v>
+        <v>53</v>
       </c>
     </row>
     <row r="148">
@@ -2887,7 +2887,7 @@
         </is>
       </c>
       <c r="D155" t="n">
-        <v>70</v>
+        <v>77</v>
       </c>
     </row>
     <row r="156">
@@ -2969,7 +2969,7 @@
         </is>
       </c>
       <c r="D160" t="n">
-        <v>76</v>
+        <v>79</v>
       </c>
     </row>
     <row r="161">
@@ -2987,7 +2987,7 @@
         </is>
       </c>
       <c r="D161" t="n">
-        <v>77</v>
+        <v>81</v>
       </c>
     </row>
     <row r="162">
@@ -3019,7 +3019,7 @@
         </is>
       </c>
       <c r="D163" t="n">
-        <v>114</v>
+        <v>92</v>
       </c>
     </row>
     <row r="164">
@@ -3147,7 +3147,7 @@
         </is>
       </c>
       <c r="D171" t="n">
-        <v>72</v>
+        <v>74</v>
       </c>
     </row>
     <row r="172">
@@ -3165,7 +3165,7 @@
         </is>
       </c>
       <c r="D172" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
     </row>
     <row r="173">
@@ -3273,7 +3273,7 @@
         </is>
       </c>
       <c r="D179" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="180">
@@ -3507,7 +3507,7 @@
         </is>
       </c>
       <c r="D193" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="194">
@@ -3525,7 +3525,7 @@
         </is>
       </c>
       <c r="D194" t="n">
-        <v>61</v>
+        <v>52</v>
       </c>
     </row>
     <row r="195">
@@ -3667,7 +3667,7 @@
         </is>
       </c>
       <c r="D203" t="n">
-        <v>67</v>
+        <v>64</v>
       </c>
     </row>
     <row r="204">
@@ -3685,7 +3685,7 @@
         </is>
       </c>
       <c r="D204" t="n">
-        <v>80</v>
+        <v>73</v>
       </c>
     </row>
     <row r="205">
@@ -3795,7 +3795,7 @@
         </is>
       </c>
       <c r="D211" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="212">
@@ -3831,7 +3831,7 @@
         </is>
       </c>
       <c r="D213" t="n">
-        <v>101</v>
+        <v>108</v>
       </c>
     </row>
     <row r="214">
@@ -3889,7 +3889,7 @@
         </is>
       </c>
       <c r="D217" t="n">
-        <v>146</v>
+        <v>154</v>
       </c>
     </row>
     <row r="218">
@@ -3935,7 +3935,7 @@
         </is>
       </c>
       <c r="D220" t="n">
-        <v>96</v>
+        <v>67</v>
       </c>
     </row>
     <row r="221">
@@ -4027,7 +4027,7 @@
         </is>
       </c>
       <c r="D226" t="n">
-        <v>52</v>
+        <v>49</v>
       </c>
     </row>
     <row r="227">
@@ -4073,7 +4073,7 @@
         </is>
       </c>
       <c r="D229" t="n">
-        <v>131</v>
+        <v>120</v>
       </c>
     </row>
     <row r="230">

</xml_diff>

<commit_message>
data: field/odds refresh 2026-04-20 04:21 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -589,7 +589,7 @@
       </c>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="n">
-        <v>240</v>
+        <v>243</v>
       </c>
     </row>
     <row r="11">
@@ -717,7 +717,7 @@
       </c>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="n">
-        <v>423</v>
+        <v>437</v>
       </c>
     </row>
     <row r="19">
@@ -763,7 +763,7 @@
       </c>
       <c r="C21" t="inlineStr"/>
       <c r="D21" t="n">
-        <v>299</v>
+        <v>314</v>
       </c>
     </row>
     <row r="22">
@@ -813,7 +813,7 @@
       </c>
       <c r="C24" t="inlineStr"/>
       <c r="D24" t="n">
-        <v>300</v>
+        <v>294</v>
       </c>
     </row>
     <row r="25">
@@ -839,7 +839,7 @@
       </c>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="n">
-        <v>204</v>
+        <v>210</v>
       </c>
     </row>
     <row r="27">
@@ -875,7 +875,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="29">
@@ -969,7 +969,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>175</v>
+        <v>180</v>
       </c>
     </row>
     <row r="35">
@@ -987,7 +987,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>188</v>
+        <v>211</v>
       </c>
     </row>
     <row r="36">
@@ -1089,7 +1089,7 @@
       </c>
       <c r="C42" t="inlineStr"/>
       <c r="D42" t="n">
-        <v>244</v>
+        <v>265</v>
       </c>
     </row>
     <row r="43">
@@ -1135,7 +1135,7 @@
       </c>
       <c r="C45" t="inlineStr"/>
       <c r="D45" t="n">
-        <v>174</v>
+        <v>158</v>
       </c>
     </row>
     <row r="46">
@@ -1197,7 +1197,7 @@
       </c>
       <c r="C49" t="inlineStr"/>
       <c r="D49" t="n">
-        <v>168</v>
+        <v>175</v>
       </c>
     </row>
     <row r="50">
@@ -1319,7 +1319,7 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>391</v>
+        <v>411</v>
       </c>
     </row>
     <row r="57">
@@ -1355,7 +1355,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>184</v>
+        <v>181</v>
       </c>
     </row>
     <row r="59">
@@ -1387,7 +1387,7 @@
       </c>
       <c r="C60" t="inlineStr"/>
       <c r="D60" t="n">
-        <v>284</v>
+        <v>297</v>
       </c>
     </row>
     <row r="61">
@@ -1401,7 +1401,7 @@
       </c>
       <c r="C61" t="inlineStr"/>
       <c r="D61" t="n">
-        <v>289</v>
+        <v>349</v>
       </c>
     </row>
     <row r="62">
@@ -1437,7 +1437,7 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>59</v>
+        <v>65</v>
       </c>
     </row>
     <row r="64">
@@ -1469,7 +1469,7 @@
       </c>
       <c r="C65" t="inlineStr"/>
       <c r="D65" t="n">
-        <v>216</v>
+        <v>220</v>
       </c>
     </row>
     <row r="66">
@@ -1513,7 +1513,7 @@
       </c>
       <c r="C68" t="inlineStr"/>
       <c r="D68" t="n">
-        <v>219</v>
+        <v>240</v>
       </c>
     </row>
     <row r="69">
@@ -1545,7 +1545,7 @@
       </c>
       <c r="C70" t="inlineStr"/>
       <c r="D70" t="n">
-        <v>484</v>
+        <v>493</v>
       </c>
     </row>
     <row r="71">
@@ -1657,7 +1657,7 @@
       </c>
       <c r="C77" t="inlineStr"/>
       <c r="D77" t="n">
-        <v>227</v>
+        <v>280</v>
       </c>
     </row>
     <row r="78">
@@ -1707,7 +1707,7 @@
       </c>
       <c r="C80" t="inlineStr"/>
       <c r="D80" t="n">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="81">
@@ -1725,7 +1725,7 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>78</v>
+        <v>80</v>
       </c>
     </row>
     <row r="82">
@@ -1739,7 +1739,7 @@
       </c>
       <c r="C82" t="inlineStr"/>
       <c r="D82" t="n">
-        <v>370</v>
+        <v>400</v>
       </c>
     </row>
     <row r="83">
@@ -1857,7 +1857,7 @@
       </c>
       <c r="C89" t="inlineStr"/>
       <c r="D89" t="n">
-        <v>159</v>
+        <v>163</v>
       </c>
     </row>
     <row r="90">
@@ -1889,7 +1889,7 @@
       </c>
       <c r="C91" t="inlineStr"/>
       <c r="D91" t="n">
-        <v>149</v>
+        <v>152</v>
       </c>
     </row>
     <row r="92">
@@ -1907,7 +1907,7 @@
         </is>
       </c>
       <c r="D92" t="n">
-        <v>118</v>
+        <v>123</v>
       </c>
     </row>
     <row r="93">
@@ -1987,7 +1987,7 @@
       </c>
       <c r="C97" t="inlineStr"/>
       <c r="D97" t="n">
-        <v>126</v>
+        <v>128</v>
       </c>
     </row>
     <row r="98">
@@ -2013,7 +2013,7 @@
       </c>
       <c r="C99" t="inlineStr"/>
       <c r="D99" t="n">
-        <v>278</v>
+        <v>287</v>
       </c>
     </row>
     <row r="100">
@@ -2067,7 +2067,7 @@
         </is>
       </c>
       <c r="D102" t="n">
-        <v>129</v>
+        <v>134</v>
       </c>
     </row>
     <row r="103">
@@ -2085,7 +2085,7 @@
         </is>
       </c>
       <c r="D103" t="n">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="104">
@@ -2129,7 +2129,7 @@
       </c>
       <c r="C106" t="inlineStr"/>
       <c r="D106" t="n">
-        <v>258</v>
+        <v>273</v>
       </c>
     </row>
     <row r="107">
@@ -2177,7 +2177,7 @@
         </is>
       </c>
       <c r="D109" t="n">
-        <v>169</v>
+        <v>129</v>
       </c>
     </row>
     <row r="110">
@@ -2191,7 +2191,7 @@
       </c>
       <c r="C110" t="inlineStr"/>
       <c r="D110" t="n">
-        <v>266</v>
+        <v>284</v>
       </c>
     </row>
     <row r="111">
@@ -2223,7 +2223,7 @@
       </c>
       <c r="C112" t="inlineStr"/>
       <c r="D112" t="n">
-        <v>160</v>
+        <v>166</v>
       </c>
     </row>
     <row r="113">
@@ -2322,9 +2322,7 @@
         <v>7960</v>
       </c>
       <c r="C119" t="inlineStr"/>
-      <c r="D119" t="n">
-        <v>484</v>
-      </c>
+      <c r="D119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -2337,7 +2335,7 @@
       </c>
       <c r="C120" t="inlineStr"/>
       <c r="D120" t="n">
-        <v>199</v>
+        <v>208</v>
       </c>
     </row>
     <row r="121">
@@ -2413,7 +2411,7 @@
       </c>
       <c r="C125" t="inlineStr"/>
       <c r="D125" t="n">
-        <v>361</v>
+        <v>422</v>
       </c>
     </row>
     <row r="126">
@@ -2485,7 +2483,7 @@
         </is>
       </c>
       <c r="D129" t="n">
-        <v>73</v>
+        <v>75</v>
       </c>
     </row>
     <row r="130">
@@ -2539,7 +2537,7 @@
         </is>
       </c>
       <c r="D132" t="n">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="133">
@@ -2573,7 +2571,7 @@
         </is>
       </c>
       <c r="D134" t="n">
-        <v>105</v>
+        <v>107</v>
       </c>
     </row>
     <row r="135">
@@ -2601,7 +2599,7 @@
       </c>
       <c r="C136" t="inlineStr"/>
       <c r="D136" t="n">
-        <v>188</v>
+        <v>174</v>
       </c>
     </row>
     <row r="137">
@@ -2665,7 +2663,7 @@
       </c>
       <c r="C140" t="inlineStr"/>
       <c r="D140" t="n">
-        <v>387</v>
+        <v>405</v>
       </c>
     </row>
     <row r="141">
@@ -2679,7 +2677,7 @@
       </c>
       <c r="C141" t="inlineStr"/>
       <c r="D141" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="142">
@@ -2743,7 +2741,7 @@
       </c>
       <c r="C145" t="inlineStr"/>
       <c r="D145" t="n">
-        <v>320</v>
+        <v>339</v>
       </c>
     </row>
     <row r="146">
@@ -2851,7 +2849,7 @@
       </c>
       <c r="C153" t="inlineStr"/>
       <c r="D153" t="n">
-        <v>294</v>
+        <v>312</v>
       </c>
     </row>
     <row r="154">
@@ -2869,7 +2867,7 @@
         </is>
       </c>
       <c r="D154" t="n">
-        <v>224</v>
+        <v>233</v>
       </c>
     </row>
     <row r="155">
@@ -2937,7 +2935,7 @@
       </c>
       <c r="C158" t="inlineStr"/>
       <c r="D158" t="n">
-        <v>233</v>
+        <v>239</v>
       </c>
     </row>
     <row r="159">
@@ -2951,7 +2949,7 @@
       </c>
       <c r="C159" t="inlineStr"/>
       <c r="D159" t="n">
-        <v>182</v>
+        <v>157</v>
       </c>
     </row>
     <row r="160">
@@ -3001,7 +2999,7 @@
       </c>
       <c r="C162" t="inlineStr"/>
       <c r="D162" t="n">
-        <v>164</v>
+        <v>169</v>
       </c>
     </row>
     <row r="163">
@@ -3055,7 +3053,7 @@
         </is>
       </c>
       <c r="D165" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="166">
@@ -3069,7 +3067,7 @@
       </c>
       <c r="C166" t="inlineStr"/>
       <c r="D166" t="n">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="167">
@@ -3129,7 +3127,7 @@
         </is>
       </c>
       <c r="D170" t="n">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="171">
@@ -3193,7 +3191,7 @@
       </c>
       <c r="C174" t="inlineStr"/>
       <c r="D174" t="n">
-        <v>140</v>
+        <v>137</v>
       </c>
     </row>
     <row r="175">
@@ -3229,7 +3227,7 @@
         </is>
       </c>
       <c r="D176" t="n">
-        <v>230</v>
+        <v>216</v>
       </c>
     </row>
     <row r="177">
@@ -3327,7 +3325,7 @@
         </is>
       </c>
       <c r="D182" t="n">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
     <row r="183">
@@ -3345,7 +3343,7 @@
         </is>
       </c>
       <c r="D183" t="n">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
     <row r="184">
@@ -3377,7 +3375,7 @@
       </c>
       <c r="C185" t="inlineStr"/>
       <c r="D185" t="n">
-        <v>274</v>
+        <v>290</v>
       </c>
     </row>
     <row r="186">
@@ -3391,7 +3389,7 @@
       </c>
       <c r="C186" t="inlineStr"/>
       <c r="D186" t="n">
-        <v>260</v>
+        <v>246</v>
       </c>
     </row>
     <row r="187">
@@ -3423,7 +3421,7 @@
       </c>
       <c r="C188" t="inlineStr"/>
       <c r="D188" t="n">
-        <v>268</v>
+        <v>252</v>
       </c>
     </row>
     <row r="189">
@@ -3441,7 +3439,7 @@
         </is>
       </c>
       <c r="D189" t="n">
-        <v>113</v>
+        <v>106</v>
       </c>
     </row>
     <row r="190">
@@ -3489,7 +3487,7 @@
       </c>
       <c r="C192" t="inlineStr"/>
       <c r="D192" t="n">
-        <v>276</v>
+        <v>261</v>
       </c>
     </row>
     <row r="193">
@@ -3539,7 +3537,7 @@
       </c>
       <c r="C195" t="inlineStr"/>
       <c r="D195" t="n">
-        <v>219</v>
+        <v>238</v>
       </c>
     </row>
     <row r="196">
@@ -3607,7 +3605,7 @@
         </is>
       </c>
       <c r="D199" t="n">
-        <v>413</v>
+        <v>377</v>
       </c>
     </row>
     <row r="200">
@@ -3621,7 +3619,7 @@
       </c>
       <c r="C200" t="inlineStr"/>
       <c r="D200" t="n">
-        <v>198</v>
+        <v>206</v>
       </c>
     </row>
     <row r="201">
@@ -3635,7 +3633,7 @@
       </c>
       <c r="C201" t="inlineStr"/>
       <c r="D201" t="n">
-        <v>377</v>
+        <v>368</v>
       </c>
     </row>
     <row r="202">
@@ -3649,7 +3647,7 @@
       </c>
       <c r="C202" t="inlineStr"/>
       <c r="D202" t="n">
-        <v>181</v>
+        <v>186</v>
       </c>
     </row>
     <row r="203">
@@ -3721,7 +3719,7 @@
         </is>
       </c>
       <c r="D206" t="n">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="207">
@@ -3777,7 +3775,7 @@
       </c>
       <c r="C210" t="inlineStr"/>
       <c r="D210" t="n">
-        <v>308</v>
+        <v>317</v>
       </c>
     </row>
     <row r="211">
@@ -3813,7 +3811,7 @@
         </is>
       </c>
       <c r="D212" t="n">
-        <v>158</v>
+        <v>164</v>
       </c>
     </row>
     <row r="213">
@@ -3857,7 +3855,7 @@
       </c>
       <c r="C215" t="inlineStr"/>
       <c r="D215" t="n">
-        <v>239</v>
+        <v>244</v>
       </c>
     </row>
     <row r="216">
@@ -3871,7 +3869,7 @@
       </c>
       <c r="C216" t="inlineStr"/>
       <c r="D216" t="n">
-        <v>239</v>
+        <v>244</v>
       </c>
     </row>
     <row r="217">
@@ -3903,7 +3901,7 @@
       </c>
       <c r="C218" t="inlineStr"/>
       <c r="D218" t="n">
-        <v>460</v>
+        <v>464</v>
       </c>
     </row>
     <row r="219">
@@ -4041,7 +4039,7 @@
       </c>
       <c r="C227" t="inlineStr"/>
       <c r="D227" t="n">
-        <v>331</v>
+        <v>338</v>
       </c>
     </row>
     <row r="228">
@@ -4105,7 +4103,7 @@
       </c>
       <c r="C231" t="inlineStr"/>
       <c r="D231" t="n">
-        <v>163</v>
+        <v>167</v>
       </c>
     </row>
     <row r="232">
@@ -4123,7 +4121,7 @@
         </is>
       </c>
       <c r="D232" t="n">
-        <v>117</v>
+        <v>105</v>
       </c>
     </row>
     <row r="233">

</xml_diff>

<commit_message>
data: field/odds refresh 2026-04-20 12:53 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -557,7 +557,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>91</v>
+        <v>94</v>
       </c>
     </row>
     <row r="9">
@@ -589,7 +589,7 @@
       </c>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="n">
-        <v>243</v>
+        <v>240</v>
       </c>
     </row>
     <row r="11">
@@ -717,7 +717,7 @@
       </c>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="n">
-        <v>437</v>
+        <v>445</v>
       </c>
     </row>
     <row r="19">
@@ -763,7 +763,7 @@
       </c>
       <c r="C21" t="inlineStr"/>
       <c r="D21" t="n">
-        <v>314</v>
+        <v>318</v>
       </c>
     </row>
     <row r="22">
@@ -813,7 +813,7 @@
       </c>
       <c r="C24" t="inlineStr"/>
       <c r="D24" t="n">
-        <v>294</v>
+        <v>304</v>
       </c>
     </row>
     <row r="25">
@@ -839,7 +839,7 @@
       </c>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="n">
-        <v>210</v>
+        <v>219</v>
       </c>
     </row>
     <row r="27">
@@ -857,7 +857,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="28">
@@ -875,7 +875,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="29">
@@ -969,7 +969,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>180</v>
+        <v>182</v>
       </c>
     </row>
     <row r="35">
@@ -987,7 +987,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>211</v>
+        <v>215</v>
       </c>
     </row>
     <row r="36">
@@ -1089,7 +1089,7 @@
       </c>
       <c r="C42" t="inlineStr"/>
       <c r="D42" t="n">
-        <v>265</v>
+        <v>270</v>
       </c>
     </row>
     <row r="43">
@@ -1135,7 +1135,7 @@
       </c>
       <c r="C45" t="inlineStr"/>
       <c r="D45" t="n">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="46">
@@ -1183,7 +1183,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
     <row r="49">
@@ -1197,7 +1197,7 @@
       </c>
       <c r="C49" t="inlineStr"/>
       <c r="D49" t="n">
-        <v>175</v>
+        <v>179</v>
       </c>
     </row>
     <row r="50">
@@ -1233,7 +1233,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="52">
@@ -1319,7 +1319,7 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>411</v>
+        <v>410</v>
       </c>
     </row>
     <row r="57">
@@ -1337,7 +1337,7 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="58">
@@ -1355,7 +1355,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>181</v>
+        <v>183</v>
       </c>
     </row>
     <row r="59">
@@ -1387,7 +1387,7 @@
       </c>
       <c r="C60" t="inlineStr"/>
       <c r="D60" t="n">
-        <v>297</v>
+        <v>306</v>
       </c>
     </row>
     <row r="61">
@@ -1401,7 +1401,7 @@
       </c>
       <c r="C61" t="inlineStr"/>
       <c r="D61" t="n">
-        <v>349</v>
+        <v>358</v>
       </c>
     </row>
     <row r="62">
@@ -1437,7 +1437,7 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="64">
@@ -1513,7 +1513,7 @@
       </c>
       <c r="C68" t="inlineStr"/>
       <c r="D68" t="n">
-        <v>240</v>
+        <v>244</v>
       </c>
     </row>
     <row r="69">
@@ -1545,7 +1545,7 @@
       </c>
       <c r="C70" t="inlineStr"/>
       <c r="D70" t="n">
-        <v>493</v>
+        <v>492</v>
       </c>
     </row>
     <row r="71">
@@ -1643,7 +1643,7 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="77">
@@ -1657,7 +1657,7 @@
       </c>
       <c r="C77" t="inlineStr"/>
       <c r="D77" t="n">
-        <v>280</v>
+        <v>292</v>
       </c>
     </row>
     <row r="78">
@@ -1707,7 +1707,7 @@
       </c>
       <c r="C80" t="inlineStr"/>
       <c r="D80" t="n">
-        <v>133</v>
+        <v>135</v>
       </c>
     </row>
     <row r="81">
@@ -1725,7 +1725,7 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
     </row>
     <row r="82">
@@ -1739,7 +1739,7 @@
       </c>
       <c r="C82" t="inlineStr"/>
       <c r="D82" t="n">
-        <v>400</v>
+        <v>412</v>
       </c>
     </row>
     <row r="83">
@@ -1757,7 +1757,7 @@
         </is>
       </c>
       <c r="D83" t="n">
-        <v>111</v>
+        <v>115</v>
       </c>
     </row>
     <row r="84">
@@ -1829,7 +1829,7 @@
         </is>
       </c>
       <c r="D87" t="n">
-        <v>97</v>
+        <v>99</v>
       </c>
     </row>
     <row r="88">
@@ -1857,7 +1857,7 @@
       </c>
       <c r="C89" t="inlineStr"/>
       <c r="D89" t="n">
-        <v>163</v>
+        <v>166</v>
       </c>
     </row>
     <row r="90">
@@ -1889,7 +1889,7 @@
       </c>
       <c r="C91" t="inlineStr"/>
       <c r="D91" t="n">
-        <v>152</v>
+        <v>156</v>
       </c>
     </row>
     <row r="92">
@@ -1907,7 +1907,7 @@
         </is>
       </c>
       <c r="D92" t="n">
-        <v>123</v>
+        <v>128</v>
       </c>
     </row>
     <row r="93">
@@ -1943,7 +1943,7 @@
         </is>
       </c>
       <c r="D94" t="n">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="95">
@@ -1987,7 +1987,7 @@
       </c>
       <c r="C97" t="inlineStr"/>
       <c r="D97" t="n">
-        <v>128</v>
+        <v>130</v>
       </c>
     </row>
     <row r="98">
@@ -2067,7 +2067,7 @@
         </is>
       </c>
       <c r="D102" t="n">
-        <v>134</v>
+        <v>139</v>
       </c>
     </row>
     <row r="103">
@@ -2085,7 +2085,7 @@
         </is>
       </c>
       <c r="D103" t="n">
-        <v>98</v>
+        <v>96</v>
       </c>
     </row>
     <row r="104">
@@ -2129,7 +2129,7 @@
       </c>
       <c r="C106" t="inlineStr"/>
       <c r="D106" t="n">
-        <v>273</v>
+        <v>275</v>
       </c>
     </row>
     <row r="107">
@@ -2177,7 +2177,7 @@
         </is>
       </c>
       <c r="D109" t="n">
-        <v>129</v>
+        <v>125</v>
       </c>
     </row>
     <row r="110">
@@ -2191,7 +2191,7 @@
       </c>
       <c r="C110" t="inlineStr"/>
       <c r="D110" t="n">
-        <v>284</v>
+        <v>296</v>
       </c>
     </row>
     <row r="111">
@@ -2223,7 +2223,7 @@
       </c>
       <c r="C112" t="inlineStr"/>
       <c r="D112" t="n">
-        <v>166</v>
+        <v>170</v>
       </c>
     </row>
     <row r="113">
@@ -2309,7 +2309,7 @@
         </is>
       </c>
       <c r="D118" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="119">
@@ -2335,7 +2335,7 @@
       </c>
       <c r="C120" t="inlineStr"/>
       <c r="D120" t="n">
-        <v>208</v>
+        <v>213</v>
       </c>
     </row>
     <row r="121">
@@ -2353,7 +2353,7 @@
         </is>
       </c>
       <c r="D121" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="122">
@@ -2411,7 +2411,7 @@
       </c>
       <c r="C125" t="inlineStr"/>
       <c r="D125" t="n">
-        <v>422</v>
+        <v>425</v>
       </c>
     </row>
     <row r="126">
@@ -2465,7 +2465,7 @@
         </is>
       </c>
       <c r="D128" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="129">
@@ -2483,7 +2483,7 @@
         </is>
       </c>
       <c r="D129" t="n">
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="130">
@@ -2599,7 +2599,7 @@
       </c>
       <c r="C136" t="inlineStr"/>
       <c r="D136" t="n">
-        <v>174</v>
+        <v>180</v>
       </c>
     </row>
     <row r="137">
@@ -2617,7 +2617,7 @@
         </is>
       </c>
       <c r="D137" t="n">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="138">
@@ -2663,7 +2663,7 @@
       </c>
       <c r="C140" t="inlineStr"/>
       <c r="D140" t="n">
-        <v>405</v>
+        <v>410</v>
       </c>
     </row>
     <row r="141">
@@ -2677,7 +2677,7 @@
       </c>
       <c r="C141" t="inlineStr"/>
       <c r="D141" t="n">
-        <v>70</v>
+        <v>75</v>
       </c>
     </row>
     <row r="142">
@@ -2741,7 +2741,7 @@
       </c>
       <c r="C145" t="inlineStr"/>
       <c r="D145" t="n">
-        <v>339</v>
+        <v>341</v>
       </c>
     </row>
     <row r="146">
@@ -2771,7 +2771,7 @@
         </is>
       </c>
       <c r="D147" t="n">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="148">
@@ -2849,7 +2849,7 @@
       </c>
       <c r="C153" t="inlineStr"/>
       <c r="D153" t="n">
-        <v>312</v>
+        <v>316</v>
       </c>
     </row>
     <row r="154">
@@ -2867,7 +2867,7 @@
         </is>
       </c>
       <c r="D154" t="n">
-        <v>233</v>
+        <v>236</v>
       </c>
     </row>
     <row r="155">
@@ -2885,7 +2885,7 @@
         </is>
       </c>
       <c r="D155" t="n">
-        <v>77</v>
+        <v>81</v>
       </c>
     </row>
     <row r="156">
@@ -2903,7 +2903,7 @@
         </is>
       </c>
       <c r="D156" t="n">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="157">
@@ -2935,7 +2935,7 @@
       </c>
       <c r="C158" t="inlineStr"/>
       <c r="D158" t="n">
-        <v>239</v>
+        <v>242</v>
       </c>
     </row>
     <row r="159">
@@ -2949,7 +2949,7 @@
       </c>
       <c r="C159" t="inlineStr"/>
       <c r="D159" t="n">
-        <v>157</v>
+        <v>160</v>
       </c>
     </row>
     <row r="160">
@@ -2999,7 +2999,7 @@
       </c>
       <c r="C162" t="inlineStr"/>
       <c r="D162" t="n">
-        <v>169</v>
+        <v>175</v>
       </c>
     </row>
     <row r="163">
@@ -3017,7 +3017,7 @@
         </is>
       </c>
       <c r="D163" t="n">
-        <v>92</v>
+        <v>88</v>
       </c>
     </row>
     <row r="164">
@@ -3067,7 +3067,7 @@
       </c>
       <c r="C166" t="inlineStr"/>
       <c r="D166" t="n">
-        <v>145</v>
+        <v>149</v>
       </c>
     </row>
     <row r="167">
@@ -3127,7 +3127,7 @@
         </is>
       </c>
       <c r="D170" t="n">
-        <v>121</v>
+        <v>124</v>
       </c>
     </row>
     <row r="171">
@@ -3191,7 +3191,7 @@
       </c>
       <c r="C174" t="inlineStr"/>
       <c r="D174" t="n">
-        <v>137</v>
+        <v>140</v>
       </c>
     </row>
     <row r="175">
@@ -3227,7 +3227,7 @@
         </is>
       </c>
       <c r="D176" t="n">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="177">
@@ -3307,7 +3307,7 @@
         </is>
       </c>
       <c r="D181" t="n">
-        <v>150</v>
+        <v>147</v>
       </c>
     </row>
     <row r="182">
@@ -3325,7 +3325,7 @@
         </is>
       </c>
       <c r="D182" t="n">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="183">
@@ -3343,7 +3343,7 @@
         </is>
       </c>
       <c r="D183" t="n">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="184">
@@ -3375,7 +3375,7 @@
       </c>
       <c r="C185" t="inlineStr"/>
       <c r="D185" t="n">
-        <v>290</v>
+        <v>294</v>
       </c>
     </row>
     <row r="186">
@@ -3389,7 +3389,7 @@
       </c>
       <c r="C186" t="inlineStr"/>
       <c r="D186" t="n">
-        <v>246</v>
+        <v>249</v>
       </c>
     </row>
     <row r="187">
@@ -3421,7 +3421,7 @@
       </c>
       <c r="C188" t="inlineStr"/>
       <c r="D188" t="n">
-        <v>252</v>
+        <v>255</v>
       </c>
     </row>
     <row r="189">
@@ -3439,7 +3439,7 @@
         </is>
       </c>
       <c r="D189" t="n">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="190">
@@ -3487,7 +3487,7 @@
       </c>
       <c r="C192" t="inlineStr"/>
       <c r="D192" t="n">
-        <v>261</v>
+        <v>267</v>
       </c>
     </row>
     <row r="193">
@@ -3537,7 +3537,7 @@
       </c>
       <c r="C195" t="inlineStr"/>
       <c r="D195" t="n">
-        <v>238</v>
+        <v>239</v>
       </c>
     </row>
     <row r="196">
@@ -3555,7 +3555,7 @@
         </is>
       </c>
       <c r="D196" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="197">
@@ -3569,7 +3569,7 @@
       </c>
       <c r="C197" t="inlineStr"/>
       <c r="D197" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="198">
@@ -3605,7 +3605,7 @@
         </is>
       </c>
       <c r="D199" t="n">
-        <v>377</v>
+        <v>384</v>
       </c>
     </row>
     <row r="200">
@@ -3619,7 +3619,7 @@
       </c>
       <c r="C200" t="inlineStr"/>
       <c r="D200" t="n">
-        <v>206</v>
+        <v>207</v>
       </c>
     </row>
     <row r="201">
@@ -3633,7 +3633,7 @@
       </c>
       <c r="C201" t="inlineStr"/>
       <c r="D201" t="n">
-        <v>368</v>
+        <v>375</v>
       </c>
     </row>
     <row r="202">
@@ -3647,7 +3647,7 @@
       </c>
       <c r="C202" t="inlineStr"/>
       <c r="D202" t="n">
-        <v>186</v>
+        <v>188</v>
       </c>
     </row>
     <row r="203">
@@ -3683,7 +3683,7 @@
         </is>
       </c>
       <c r="D204" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="205">
@@ -3719,7 +3719,7 @@
         </is>
       </c>
       <c r="D206" t="n">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="207">
@@ -3737,7 +3737,7 @@
         </is>
       </c>
       <c r="D207" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="208">
@@ -3775,7 +3775,7 @@
       </c>
       <c r="C210" t="inlineStr"/>
       <c r="D210" t="n">
-        <v>317</v>
+        <v>319</v>
       </c>
     </row>
     <row r="211">
@@ -3811,7 +3811,7 @@
         </is>
       </c>
       <c r="D212" t="n">
-        <v>164</v>
+        <v>167</v>
       </c>
     </row>
     <row r="213">
@@ -3855,7 +3855,7 @@
       </c>
       <c r="C215" t="inlineStr"/>
       <c r="D215" t="n">
-        <v>244</v>
+        <v>246</v>
       </c>
     </row>
     <row r="216">
@@ -3869,7 +3869,7 @@
       </c>
       <c r="C216" t="inlineStr"/>
       <c r="D216" t="n">
-        <v>244</v>
+        <v>246</v>
       </c>
     </row>
     <row r="217">
@@ -3887,7 +3887,7 @@
         </is>
       </c>
       <c r="D217" t="n">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="218">
@@ -3901,7 +3901,7 @@
       </c>
       <c r="C218" t="inlineStr"/>
       <c r="D218" t="n">
-        <v>464</v>
+        <v>469</v>
       </c>
     </row>
     <row r="219">
@@ -3915,7 +3915,7 @@
       </c>
       <c r="C219" t="inlineStr"/>
       <c r="D219" t="n">
-        <v>215</v>
+        <v>221</v>
       </c>
     </row>
     <row r="220">
@@ -3933,7 +3933,7 @@
         </is>
       </c>
       <c r="D220" t="n">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="221">
@@ -3969,7 +3969,7 @@
         </is>
       </c>
       <c r="D222" t="n">
-        <v>124</v>
+        <v>127</v>
       </c>
     </row>
     <row r="223">
@@ -4039,7 +4039,7 @@
       </c>
       <c r="C227" t="inlineStr"/>
       <c r="D227" t="n">
-        <v>338</v>
+        <v>343</v>
       </c>
     </row>
     <row r="228">
@@ -4071,7 +4071,7 @@
         </is>
       </c>
       <c r="D229" t="n">
-        <v>120</v>
+        <v>118</v>
       </c>
     </row>
     <row r="230">
@@ -4103,7 +4103,7 @@
       </c>
       <c r="C231" t="inlineStr"/>
       <c r="D231" t="n">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="232">
@@ -4121,7 +4121,7 @@
         </is>
       </c>
       <c r="D232" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="233">

</xml_diff>

<commit_message>
data: field/odds refresh 2026-04-20 16:06 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -557,7 +557,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>91</v>
+        <v>94</v>
       </c>
     </row>
     <row r="9">
@@ -717,7 +717,7 @@
       </c>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="n">
-        <v>423</v>
+        <v>445</v>
       </c>
     </row>
     <row r="19">
@@ -763,7 +763,7 @@
       </c>
       <c r="C21" t="inlineStr"/>
       <c r="D21" t="n">
-        <v>299</v>
+        <v>318</v>
       </c>
     </row>
     <row r="22">
@@ -813,7 +813,7 @@
       </c>
       <c r="C24" t="inlineStr"/>
       <c r="D24" t="n">
-        <v>300</v>
+        <v>304</v>
       </c>
     </row>
     <row r="25">
@@ -839,7 +839,7 @@
       </c>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="n">
-        <v>204</v>
+        <v>219</v>
       </c>
     </row>
     <row r="27">
@@ -857,7 +857,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="28">
@@ -969,7 +969,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>175</v>
+        <v>182</v>
       </c>
     </row>
     <row r="35">
@@ -987,7 +987,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>188</v>
+        <v>215</v>
       </c>
     </row>
     <row r="36">
@@ -1089,7 +1089,7 @@
       </c>
       <c r="C42" t="inlineStr"/>
       <c r="D42" t="n">
-        <v>244</v>
+        <v>270</v>
       </c>
     </row>
     <row r="43">
@@ -1135,7 +1135,7 @@
       </c>
       <c r="C45" t="inlineStr"/>
       <c r="D45" t="n">
-        <v>174</v>
+        <v>157</v>
       </c>
     </row>
     <row r="46">
@@ -1183,7 +1183,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
     <row r="49">
@@ -1197,7 +1197,7 @@
       </c>
       <c r="C49" t="inlineStr"/>
       <c r="D49" t="n">
-        <v>168</v>
+        <v>179</v>
       </c>
     </row>
     <row r="50">
@@ -1233,7 +1233,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="52">
@@ -1319,7 +1319,7 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>391</v>
+        <v>410</v>
       </c>
     </row>
     <row r="57">
@@ -1337,7 +1337,7 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="58">
@@ -1355,7 +1355,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="59">
@@ -1387,7 +1387,7 @@
       </c>
       <c r="C60" t="inlineStr"/>
       <c r="D60" t="n">
-        <v>284</v>
+        <v>306</v>
       </c>
     </row>
     <row r="61">
@@ -1401,7 +1401,7 @@
       </c>
       <c r="C61" t="inlineStr"/>
       <c r="D61" t="n">
-        <v>289</v>
+        <v>358</v>
       </c>
     </row>
     <row r="62">
@@ -1437,7 +1437,7 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>59</v>
+        <v>66</v>
       </c>
     </row>
     <row r="64">
@@ -1469,7 +1469,7 @@
       </c>
       <c r="C65" t="inlineStr"/>
       <c r="D65" t="n">
-        <v>216</v>
+        <v>220</v>
       </c>
     </row>
     <row r="66">
@@ -1513,7 +1513,7 @@
       </c>
       <c r="C68" t="inlineStr"/>
       <c r="D68" t="n">
-        <v>219</v>
+        <v>244</v>
       </c>
     </row>
     <row r="69">
@@ -1545,7 +1545,7 @@
       </c>
       <c r="C70" t="inlineStr"/>
       <c r="D70" t="n">
-        <v>484</v>
+        <v>492</v>
       </c>
     </row>
     <row r="71">
@@ -1643,7 +1643,7 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="77">
@@ -1657,7 +1657,7 @@
       </c>
       <c r="C77" t="inlineStr"/>
       <c r="D77" t="n">
-        <v>227</v>
+        <v>292</v>
       </c>
     </row>
     <row r="78">
@@ -1707,7 +1707,7 @@
       </c>
       <c r="C80" t="inlineStr"/>
       <c r="D80" t="n">
-        <v>132</v>
+        <v>135</v>
       </c>
     </row>
     <row r="81">
@@ -1725,7 +1725,7 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>78</v>
+        <v>82</v>
       </c>
     </row>
     <row r="82">
@@ -1739,7 +1739,7 @@
       </c>
       <c r="C82" t="inlineStr"/>
       <c r="D82" t="n">
-        <v>370</v>
+        <v>412</v>
       </c>
     </row>
     <row r="83">
@@ -1757,7 +1757,7 @@
         </is>
       </c>
       <c r="D83" t="n">
-        <v>111</v>
+        <v>115</v>
       </c>
     </row>
     <row r="84">
@@ -1829,7 +1829,7 @@
         </is>
       </c>
       <c r="D87" t="n">
-        <v>97</v>
+        <v>99</v>
       </c>
     </row>
     <row r="88">
@@ -1857,7 +1857,7 @@
       </c>
       <c r="C89" t="inlineStr"/>
       <c r="D89" t="n">
-        <v>159</v>
+        <v>166</v>
       </c>
     </row>
     <row r="90">
@@ -1889,7 +1889,7 @@
       </c>
       <c r="C91" t="inlineStr"/>
       <c r="D91" t="n">
-        <v>149</v>
+        <v>156</v>
       </c>
     </row>
     <row r="92">
@@ -1907,7 +1907,7 @@
         </is>
       </c>
       <c r="D92" t="n">
-        <v>118</v>
+        <v>128</v>
       </c>
     </row>
     <row r="93">
@@ -1943,7 +1943,7 @@
         </is>
       </c>
       <c r="D94" t="n">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="95">
@@ -1987,7 +1987,7 @@
       </c>
       <c r="C97" t="inlineStr"/>
       <c r="D97" t="n">
-        <v>126</v>
+        <v>130</v>
       </c>
     </row>
     <row r="98">
@@ -2013,7 +2013,7 @@
       </c>
       <c r="C99" t="inlineStr"/>
       <c r="D99" t="n">
-        <v>278</v>
+        <v>287</v>
       </c>
     </row>
     <row r="100">
@@ -2067,7 +2067,7 @@
         </is>
       </c>
       <c r="D102" t="n">
-        <v>129</v>
+        <v>139</v>
       </c>
     </row>
     <row r="103">
@@ -2085,7 +2085,7 @@
         </is>
       </c>
       <c r="D103" t="n">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="104">
@@ -2129,7 +2129,7 @@
       </c>
       <c r="C106" t="inlineStr"/>
       <c r="D106" t="n">
-        <v>258</v>
+        <v>275</v>
       </c>
     </row>
     <row r="107">
@@ -2177,7 +2177,7 @@
         </is>
       </c>
       <c r="D109" t="n">
-        <v>169</v>
+        <v>125</v>
       </c>
     </row>
     <row r="110">
@@ -2191,7 +2191,7 @@
       </c>
       <c r="C110" t="inlineStr"/>
       <c r="D110" t="n">
-        <v>266</v>
+        <v>296</v>
       </c>
     </row>
     <row r="111">
@@ -2223,7 +2223,7 @@
       </c>
       <c r="C112" t="inlineStr"/>
       <c r="D112" t="n">
-        <v>160</v>
+        <v>170</v>
       </c>
     </row>
     <row r="113">
@@ -2309,7 +2309,7 @@
         </is>
       </c>
       <c r="D118" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="119">
@@ -2322,9 +2322,7 @@
         <v>7960</v>
       </c>
       <c r="C119" t="inlineStr"/>
-      <c r="D119" t="n">
-        <v>484</v>
-      </c>
+      <c r="D119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -2337,7 +2335,7 @@
       </c>
       <c r="C120" t="inlineStr"/>
       <c r="D120" t="n">
-        <v>199</v>
+        <v>213</v>
       </c>
     </row>
     <row r="121">
@@ -2355,7 +2353,7 @@
         </is>
       </c>
       <c r="D121" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="122">
@@ -2413,7 +2411,7 @@
       </c>
       <c r="C125" t="inlineStr"/>
       <c r="D125" t="n">
-        <v>361</v>
+        <v>425</v>
       </c>
     </row>
     <row r="126">
@@ -2467,7 +2465,7 @@
         </is>
       </c>
       <c r="D128" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="129">
@@ -2485,7 +2483,7 @@
         </is>
       </c>
       <c r="D129" t="n">
-        <v>73</v>
+        <v>78</v>
       </c>
     </row>
     <row r="130">
@@ -2539,7 +2537,7 @@
         </is>
       </c>
       <c r="D132" t="n">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="133">
@@ -2573,7 +2571,7 @@
         </is>
       </c>
       <c r="D134" t="n">
-        <v>105</v>
+        <v>107</v>
       </c>
     </row>
     <row r="135">
@@ -2601,7 +2599,7 @@
       </c>
       <c r="C136" t="inlineStr"/>
       <c r="D136" t="n">
-        <v>188</v>
+        <v>180</v>
       </c>
     </row>
     <row r="137">
@@ -2619,7 +2617,7 @@
         </is>
       </c>
       <c r="D137" t="n">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="138">
@@ -2665,7 +2663,7 @@
       </c>
       <c r="C140" t="inlineStr"/>
       <c r="D140" t="n">
-        <v>387</v>
+        <v>410</v>
       </c>
     </row>
     <row r="141">
@@ -2679,7 +2677,7 @@
       </c>
       <c r="C141" t="inlineStr"/>
       <c r="D141" t="n">
-        <v>69</v>
+        <v>75</v>
       </c>
     </row>
     <row r="142">
@@ -2743,7 +2741,7 @@
       </c>
       <c r="C145" t="inlineStr"/>
       <c r="D145" t="n">
-        <v>320</v>
+        <v>341</v>
       </c>
     </row>
     <row r="146">
@@ -2773,7 +2771,7 @@
         </is>
       </c>
       <c r="D147" t="n">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="148">
@@ -2851,7 +2849,7 @@
       </c>
       <c r="C153" t="inlineStr"/>
       <c r="D153" t="n">
-        <v>294</v>
+        <v>316</v>
       </c>
     </row>
     <row r="154">
@@ -2869,7 +2867,7 @@
         </is>
       </c>
       <c r="D154" t="n">
-        <v>224</v>
+        <v>236</v>
       </c>
     </row>
     <row r="155">
@@ -2887,7 +2885,7 @@
         </is>
       </c>
       <c r="D155" t="n">
-        <v>77</v>
+        <v>81</v>
       </c>
     </row>
     <row r="156">
@@ -2905,7 +2903,7 @@
         </is>
       </c>
       <c r="D156" t="n">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="157">
@@ -2937,7 +2935,7 @@
       </c>
       <c r="C158" t="inlineStr"/>
       <c r="D158" t="n">
-        <v>233</v>
+        <v>242</v>
       </c>
     </row>
     <row r="159">
@@ -2951,7 +2949,7 @@
       </c>
       <c r="C159" t="inlineStr"/>
       <c r="D159" t="n">
-        <v>182</v>
+        <v>160</v>
       </c>
     </row>
     <row r="160">
@@ -3001,7 +2999,7 @@
       </c>
       <c r="C162" t="inlineStr"/>
       <c r="D162" t="n">
-        <v>164</v>
+        <v>175</v>
       </c>
     </row>
     <row r="163">
@@ -3019,7 +3017,7 @@
         </is>
       </c>
       <c r="D163" t="n">
-        <v>92</v>
+        <v>88</v>
       </c>
     </row>
     <row r="164">
@@ -3055,7 +3053,7 @@
         </is>
       </c>
       <c r="D165" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="166">
@@ -3069,7 +3067,7 @@
       </c>
       <c r="C166" t="inlineStr"/>
       <c r="D166" t="n">
-        <v>144</v>
+        <v>149</v>
       </c>
     </row>
     <row r="167">
@@ -3129,7 +3127,7 @@
         </is>
       </c>
       <c r="D170" t="n">
-        <v>120</v>
+        <v>124</v>
       </c>
     </row>
     <row r="171">
@@ -3229,7 +3227,7 @@
         </is>
       </c>
       <c r="D176" t="n">
-        <v>230</v>
+        <v>217</v>
       </c>
     </row>
     <row r="177">
@@ -3309,7 +3307,7 @@
         </is>
       </c>
       <c r="D181" t="n">
-        <v>150</v>
+        <v>147</v>
       </c>
     </row>
     <row r="182">
@@ -3327,7 +3325,7 @@
         </is>
       </c>
       <c r="D182" t="n">
-        <v>85</v>
+        <v>91</v>
       </c>
     </row>
     <row r="183">
@@ -3345,7 +3343,7 @@
         </is>
       </c>
       <c r="D183" t="n">
-        <v>85</v>
+        <v>91</v>
       </c>
     </row>
     <row r="184">
@@ -3377,7 +3375,7 @@
       </c>
       <c r="C185" t="inlineStr"/>
       <c r="D185" t="n">
-        <v>274</v>
+        <v>294</v>
       </c>
     </row>
     <row r="186">
@@ -3391,7 +3389,7 @@
       </c>
       <c r="C186" t="inlineStr"/>
       <c r="D186" t="n">
-        <v>260</v>
+        <v>249</v>
       </c>
     </row>
     <row r="187">
@@ -3423,7 +3421,7 @@
       </c>
       <c r="C188" t="inlineStr"/>
       <c r="D188" t="n">
-        <v>268</v>
+        <v>255</v>
       </c>
     </row>
     <row r="189">
@@ -3441,7 +3439,7 @@
         </is>
       </c>
       <c r="D189" t="n">
-        <v>113</v>
+        <v>104</v>
       </c>
     </row>
     <row r="190">
@@ -3489,7 +3487,7 @@
       </c>
       <c r="C192" t="inlineStr"/>
       <c r="D192" t="n">
-        <v>276</v>
+        <v>267</v>
       </c>
     </row>
     <row r="193">
@@ -3539,7 +3537,7 @@
       </c>
       <c r="C195" t="inlineStr"/>
       <c r="D195" t="n">
-        <v>219</v>
+        <v>239</v>
       </c>
     </row>
     <row r="196">
@@ -3557,7 +3555,7 @@
         </is>
       </c>
       <c r="D196" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="197">
@@ -3571,7 +3569,7 @@
       </c>
       <c r="C197" t="inlineStr"/>
       <c r="D197" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="198">
@@ -3607,7 +3605,7 @@
         </is>
       </c>
       <c r="D199" t="n">
-        <v>413</v>
+        <v>384</v>
       </c>
     </row>
     <row r="200">
@@ -3621,7 +3619,7 @@
       </c>
       <c r="C200" t="inlineStr"/>
       <c r="D200" t="n">
-        <v>198</v>
+        <v>207</v>
       </c>
     </row>
     <row r="201">
@@ -3635,7 +3633,7 @@
       </c>
       <c r="C201" t="inlineStr"/>
       <c r="D201" t="n">
-        <v>377</v>
+        <v>375</v>
       </c>
     </row>
     <row r="202">
@@ -3649,7 +3647,7 @@
       </c>
       <c r="C202" t="inlineStr"/>
       <c r="D202" t="n">
-        <v>181</v>
+        <v>188</v>
       </c>
     </row>
     <row r="203">
@@ -3685,7 +3683,7 @@
         </is>
       </c>
       <c r="D204" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="205">
@@ -3739,7 +3737,7 @@
         </is>
       </c>
       <c r="D207" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="208">
@@ -3777,7 +3775,7 @@
       </c>
       <c r="C210" t="inlineStr"/>
       <c r="D210" t="n">
-        <v>308</v>
+        <v>319</v>
       </c>
     </row>
     <row r="211">
@@ -3813,7 +3811,7 @@
         </is>
       </c>
       <c r="D212" t="n">
-        <v>158</v>
+        <v>167</v>
       </c>
     </row>
     <row r="213">
@@ -3857,7 +3855,7 @@
       </c>
       <c r="C215" t="inlineStr"/>
       <c r="D215" t="n">
-        <v>239</v>
+        <v>246</v>
       </c>
     </row>
     <row r="216">
@@ -3871,7 +3869,7 @@
       </c>
       <c r="C216" t="inlineStr"/>
       <c r="D216" t="n">
-        <v>239</v>
+        <v>246</v>
       </c>
     </row>
     <row r="217">
@@ -3889,7 +3887,7 @@
         </is>
       </c>
       <c r="D217" t="n">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="218">
@@ -3903,7 +3901,7 @@
       </c>
       <c r="C218" t="inlineStr"/>
       <c r="D218" t="n">
-        <v>460</v>
+        <v>469</v>
       </c>
     </row>
     <row r="219">
@@ -3917,7 +3915,7 @@
       </c>
       <c r="C219" t="inlineStr"/>
       <c r="D219" t="n">
-        <v>215</v>
+        <v>221</v>
       </c>
     </row>
     <row r="220">
@@ -3935,7 +3933,7 @@
         </is>
       </c>
       <c r="D220" t="n">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="221">
@@ -3971,7 +3969,7 @@
         </is>
       </c>
       <c r="D222" t="n">
-        <v>124</v>
+        <v>127</v>
       </c>
     </row>
     <row r="223">
@@ -4041,7 +4039,7 @@
       </c>
       <c r="C227" t="inlineStr"/>
       <c r="D227" t="n">
-        <v>331</v>
+        <v>343</v>
       </c>
     </row>
     <row r="228">
@@ -4073,7 +4071,7 @@
         </is>
       </c>
       <c r="D229" t="n">
-        <v>120</v>
+        <v>118</v>
       </c>
     </row>
     <row r="230">
@@ -4105,7 +4103,7 @@
       </c>
       <c r="C231" t="inlineStr"/>
       <c r="D231" t="n">
-        <v>163</v>
+        <v>168</v>
       </c>
     </row>
     <row r="232">
@@ -4123,7 +4121,7 @@
         </is>
       </c>
       <c r="D232" t="n">
-        <v>117</v>
+        <v>106</v>
       </c>
     </row>
     <row r="233">
@@ -4159,7 +4157,7 @@
         </is>
       </c>
       <c r="D234" t="n">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: field/odds refresh 2026-04-27 04:36 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -607,7 +607,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="12">
@@ -639,7 +639,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="14">
@@ -685,7 +685,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="17">
@@ -749,7 +749,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="21">
@@ -781,7 +781,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="23">
@@ -799,7 +799,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>76</v>
+        <v>65</v>
       </c>
     </row>
     <row r="24">
@@ -907,7 +907,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="31">
@@ -1005,7 +1005,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="37">
@@ -1165,7 +1165,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
     </row>
     <row r="48">
@@ -1251,7 +1251,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="53">
@@ -1283,7 +1283,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>63</v>
+        <v>56</v>
       </c>
     </row>
     <row r="55">
@@ -1373,7 +1373,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>95</v>
+        <v>92</v>
       </c>
     </row>
     <row r="60">
@@ -1531,7 +1531,7 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="70">
@@ -1625,7 +1625,7 @@
         </is>
       </c>
       <c r="D75" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="76">
@@ -1693,7 +1693,7 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="80">
@@ -1775,7 +1775,7 @@
         </is>
       </c>
       <c r="D84" t="n">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="85">
@@ -1875,7 +1875,7 @@
         </is>
       </c>
       <c r="D90" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="91">
@@ -1925,7 +1925,7 @@
         </is>
       </c>
       <c r="D93" t="n">
-        <v>72</v>
+        <v>76</v>
       </c>
     </row>
     <row r="94">
@@ -2031,7 +2031,7 @@
         </is>
       </c>
       <c r="D100" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="101">
@@ -2049,7 +2049,7 @@
         </is>
       </c>
       <c r="D101" t="n">
-        <v>30</v>
+        <v>26</v>
       </c>
     </row>
     <row r="102">
@@ -2115,7 +2115,7 @@
         </is>
       </c>
       <c r="D105" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="106">
@@ -2147,7 +2147,7 @@
         </is>
       </c>
       <c r="D107" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="108">
@@ -2291,7 +2291,7 @@
         </is>
       </c>
       <c r="D117" t="n">
-        <v>27</v>
+        <v>32</v>
       </c>
     </row>
     <row r="118">
@@ -2429,7 +2429,7 @@
         </is>
       </c>
       <c r="D126" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="127">
@@ -2519,7 +2519,7 @@
         </is>
       </c>
       <c r="D131" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="132">
@@ -2635,7 +2635,7 @@
         </is>
       </c>
       <c r="D138" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="139">
@@ -2713,7 +2713,7 @@
         </is>
       </c>
       <c r="D143" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="144">
@@ -2985,7 +2985,7 @@
         </is>
       </c>
       <c r="D161" t="n">
-        <v>81</v>
+        <v>77</v>
       </c>
     </row>
     <row r="162">
@@ -3145,7 +3145,7 @@
         </is>
       </c>
       <c r="D171" t="n">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="172">
@@ -3163,7 +3163,7 @@
         </is>
       </c>
       <c r="D172" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="173">
@@ -3523,7 +3523,7 @@
         </is>
       </c>
       <c r="D194" t="n">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="195">
@@ -3665,7 +3665,7 @@
         </is>
       </c>
       <c r="D203" t="n">
-        <v>64</v>
+        <v>67</v>
       </c>
     </row>
     <row r="204">
@@ -3701,7 +3701,7 @@
         </is>
       </c>
       <c r="D205" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="206">
@@ -3829,7 +3829,7 @@
         </is>
       </c>
       <c r="D213" t="n">
-        <v>108</v>
+        <v>111</v>
       </c>
     </row>
     <row r="214">
@@ -4025,7 +4025,7 @@
         </is>
       </c>
       <c r="D226" t="n">
-        <v>49</v>
+        <v>45</v>
       </c>
     </row>
     <row r="227">
@@ -4089,7 +4089,7 @@
         </is>
       </c>
       <c r="D230" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="231">

</xml_diff>

<commit_message>
data: field/odds refresh 2026-04-27 09:15 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -749,7 +749,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="21">
@@ -925,7 +925,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="32">
@@ -969,7 +969,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="35">
@@ -1005,7 +1005,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="37">
@@ -1301,7 +1301,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="56">
@@ -1437,7 +1437,7 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="64">
@@ -1531,7 +1531,7 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="70">
@@ -1563,7 +1563,7 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="72">
@@ -1775,7 +1775,7 @@
         </is>
       </c>
       <c r="D84" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="85">
@@ -1811,7 +1811,7 @@
         </is>
       </c>
       <c r="D86" t="n">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="87">
@@ -1875,7 +1875,7 @@
         </is>
       </c>
       <c r="D90" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="91">
@@ -2049,7 +2049,7 @@
         </is>
       </c>
       <c r="D101" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="102">
@@ -2147,7 +2147,7 @@
         </is>
       </c>
       <c r="D107" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="108">
@@ -2291,7 +2291,7 @@
         </is>
       </c>
       <c r="D117" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="118">
@@ -2571,7 +2571,7 @@
         </is>
       </c>
       <c r="D134" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="135">
@@ -2713,7 +2713,7 @@
         </is>
       </c>
       <c r="D143" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="144">
@@ -2885,7 +2885,7 @@
         </is>
       </c>
       <c r="D155" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="156">
@@ -2967,7 +2967,7 @@
         </is>
       </c>
       <c r="D160" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="161">
@@ -3361,7 +3361,7 @@
         </is>
       </c>
       <c r="D184" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="185">
@@ -3523,7 +3523,7 @@
         </is>
       </c>
       <c r="D194" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="195">
@@ -3665,7 +3665,7 @@
         </is>
       </c>
       <c r="D203" t="n">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="204">
@@ -3829,7 +3829,7 @@
         </is>
       </c>
       <c r="D213" t="n">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="214">
@@ -4071,7 +4071,7 @@
         </is>
       </c>
       <c r="D229" t="n">
-        <v>118</v>
+        <v>113</v>
       </c>
     </row>
     <row r="230">

</xml_diff>

<commit_message>
data: field/odds refresh 2026-04-27 12:06 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -607,7 +607,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="12">
@@ -639,7 +639,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="14">
@@ -685,7 +685,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="17">
@@ -749,7 +749,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="21">
@@ -781,7 +781,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="23">
@@ -799,7 +799,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>76</v>
+        <v>65</v>
       </c>
     </row>
     <row r="24">
@@ -907,7 +907,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="31">
@@ -925,7 +925,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="32">
@@ -969,7 +969,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="35">
@@ -1165,7 +1165,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
     </row>
     <row r="48">
@@ -1251,7 +1251,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="53">
@@ -1283,7 +1283,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>63</v>
+        <v>56</v>
       </c>
     </row>
     <row r="55">
@@ -1301,7 +1301,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="56">
@@ -1373,7 +1373,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>95</v>
+        <v>92</v>
       </c>
     </row>
     <row r="60">
@@ -1437,7 +1437,7 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="64">
@@ -1531,7 +1531,7 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>61</v>
+        <v>64</v>
       </c>
     </row>
     <row r="70">
@@ -1563,7 +1563,7 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="72">
@@ -1625,7 +1625,7 @@
         </is>
       </c>
       <c r="D75" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="76">
@@ -1693,7 +1693,7 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="80">
@@ -1775,7 +1775,7 @@
         </is>
       </c>
       <c r="D84" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="85">
@@ -1811,7 +1811,7 @@
         </is>
       </c>
       <c r="D86" t="n">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="87">
@@ -1875,7 +1875,7 @@
         </is>
       </c>
       <c r="D90" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="91">
@@ -1925,7 +1925,7 @@
         </is>
       </c>
       <c r="D93" t="n">
-        <v>72</v>
+        <v>76</v>
       </c>
     </row>
     <row r="94">
@@ -2031,7 +2031,7 @@
         </is>
       </c>
       <c r="D100" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="101">
@@ -2049,7 +2049,7 @@
         </is>
       </c>
       <c r="D101" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
     </row>
     <row r="102">
@@ -2115,7 +2115,7 @@
         </is>
       </c>
       <c r="D105" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="106">
@@ -2291,7 +2291,7 @@
         </is>
       </c>
       <c r="D117" t="n">
-        <v>27</v>
+        <v>31</v>
       </c>
     </row>
     <row r="118">
@@ -2429,7 +2429,7 @@
         </is>
       </c>
       <c r="D126" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="127">
@@ -2519,7 +2519,7 @@
         </is>
       </c>
       <c r="D131" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="132">
@@ -2571,7 +2571,7 @@
         </is>
       </c>
       <c r="D134" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="135">
@@ -2635,7 +2635,7 @@
         </is>
       </c>
       <c r="D138" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="139">
@@ -2713,7 +2713,7 @@
         </is>
       </c>
       <c r="D143" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
     </row>
     <row r="144">
@@ -2885,7 +2885,7 @@
         </is>
       </c>
       <c r="D155" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="156">
@@ -2967,7 +2967,7 @@
         </is>
       </c>
       <c r="D160" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="161">
@@ -2985,7 +2985,7 @@
         </is>
       </c>
       <c r="D161" t="n">
-        <v>81</v>
+        <v>77</v>
       </c>
     </row>
     <row r="162">
@@ -3145,7 +3145,7 @@
         </is>
       </c>
       <c r="D171" t="n">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="172">
@@ -3163,7 +3163,7 @@
         </is>
       </c>
       <c r="D172" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="173">
@@ -3361,7 +3361,7 @@
         </is>
       </c>
       <c r="D184" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="185">
@@ -3523,7 +3523,7 @@
         </is>
       </c>
       <c r="D194" t="n">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="195">
@@ -3665,7 +3665,7 @@
         </is>
       </c>
       <c r="D203" t="n">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="204">
@@ -3701,7 +3701,7 @@
         </is>
       </c>
       <c r="D205" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="206">
@@ -3829,7 +3829,7 @@
         </is>
       </c>
       <c r="D213" t="n">
-        <v>108</v>
+        <v>112</v>
       </c>
     </row>
     <row r="214">
@@ -4025,7 +4025,7 @@
         </is>
       </c>
       <c r="D226" t="n">
-        <v>49</v>
+        <v>45</v>
       </c>
     </row>
     <row r="227">
@@ -4071,7 +4071,7 @@
         </is>
       </c>
       <c r="D229" t="n">
-        <v>118</v>
+        <v>113</v>
       </c>
     </row>
     <row r="230">
@@ -4089,7 +4089,7 @@
         </is>
       </c>
       <c r="D230" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="231">

</xml_diff>

<commit_message>
data: field/odds refresh 2026-05-04 04:38 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -465,7 +465,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3">
@@ -1183,7 +1183,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="49">
@@ -1907,7 +1907,7 @@
         </is>
       </c>
       <c r="D92" t="n">
-        <v>128</v>
+        <v>134</v>
       </c>
     </row>
     <row r="93">
@@ -3407,7 +3407,7 @@
         </is>
       </c>
       <c r="D187" t="n">
-        <v>416</v>
+        <v>430</v>
       </c>
     </row>
     <row r="188">

</xml_diff>

<commit_message>
data: field/odds refresh 2026-05-04 06:00 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D234"/>
+  <dimension ref="A1:D235"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -465,7 +465,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3">
@@ -1183,7 +1183,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="49">
@@ -1907,7 +1907,7 @@
         </is>
       </c>
       <c r="D92" t="n">
-        <v>128</v>
+        <v>134</v>
       </c>
     </row>
     <row r="93">
@@ -3407,7 +3407,7 @@
         </is>
       </c>
       <c r="D187" t="n">
-        <v>416</v>
+        <v>430</v>
       </c>
     </row>
     <row r="188">
@@ -4158,6 +4158,24 @@
       </c>
       <c r="D234" t="n">
         <v>72</v>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>Fitzpatrick, Alex</t>
+        </is>
+      </c>
+      <c r="B235" t="n">
+        <v>25362</v>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>https://pga-tour-res.cloudinary.com/image/upload/c_fill,g_face:center,q_auto,f_auto,dpr_2.0,h_220,w_200,d_stub:default_avatar_light.webp/headshots_55721</t>
+        </is>
+      </c>
+      <c r="D235" t="n">
+        <v>140</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: field/odds refresh 2026-05-04 09:19 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -465,7 +465,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3">
@@ -607,7 +607,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="12">
@@ -685,7 +685,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="17">
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="18">
@@ -749,7 +749,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="21">
@@ -907,7 +907,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="31">
@@ -925,7 +925,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="32">
@@ -1005,7 +1005,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="37">
@@ -1107,7 +1107,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="44">
@@ -1121,7 +1121,7 @@
       </c>
       <c r="C44" t="inlineStr"/>
       <c r="D44" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="45">
@@ -1165,7 +1165,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>18</v>
+        <v>22</v>
       </c>
     </row>
     <row r="48">
@@ -1183,7 +1183,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="49">
@@ -1233,7 +1233,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="52">
@@ -1283,7 +1283,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>56</v>
+        <v>52</v>
       </c>
     </row>
     <row r="55">
@@ -1337,7 +1337,7 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="58">
@@ -1373,7 +1373,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="60">
@@ -1455,7 +1455,7 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="65">
@@ -1563,7 +1563,7 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="72">
@@ -1693,7 +1693,7 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="80">
@@ -1757,7 +1757,7 @@
         </is>
       </c>
       <c r="D83" t="n">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="84">
@@ -1907,7 +1907,7 @@
         </is>
       </c>
       <c r="D92" t="n">
-        <v>134</v>
+        <v>138</v>
       </c>
     </row>
     <row r="93">
@@ -1925,7 +1925,7 @@
         </is>
       </c>
       <c r="D93" t="n">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="94">
@@ -2031,7 +2031,7 @@
         </is>
       </c>
       <c r="D100" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="101">
@@ -2049,7 +2049,7 @@
         </is>
       </c>
       <c r="D101" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
     </row>
     <row r="102">
@@ -2291,7 +2291,7 @@
         </is>
       </c>
       <c r="D117" t="n">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
     <row r="118">
@@ -2309,7 +2309,7 @@
         </is>
       </c>
       <c r="D118" t="n">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="119">
@@ -2429,7 +2429,7 @@
         </is>
       </c>
       <c r="D126" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="127">
@@ -2447,7 +2447,7 @@
         </is>
       </c>
       <c r="D127" t="n">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="128">
@@ -2465,7 +2465,7 @@
         </is>
       </c>
       <c r="D128" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="129">
@@ -2519,7 +2519,7 @@
         </is>
       </c>
       <c r="D131" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="132">
@@ -2713,7 +2713,7 @@
         </is>
       </c>
       <c r="D143" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
     </row>
     <row r="144">
@@ -2771,7 +2771,7 @@
         </is>
       </c>
       <c r="D147" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="148">
@@ -2885,7 +2885,7 @@
         </is>
       </c>
       <c r="D155" t="n">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="156">
@@ -2985,7 +2985,7 @@
         </is>
       </c>
       <c r="D161" t="n">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="162">
@@ -3017,7 +3017,7 @@
         </is>
       </c>
       <c r="D163" t="n">
-        <v>88</v>
+        <v>84</v>
       </c>
     </row>
     <row r="164">
@@ -3271,7 +3271,7 @@
         </is>
       </c>
       <c r="D179" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="180">
@@ -3361,7 +3361,7 @@
         </is>
       </c>
       <c r="D184" t="n">
-        <v>54</v>
+        <v>43</v>
       </c>
     </row>
     <row r="185">
@@ -3407,7 +3407,7 @@
         </is>
       </c>
       <c r="D187" t="n">
-        <v>430</v>
+        <v>441</v>
       </c>
     </row>
     <row r="188">
@@ -3439,7 +3439,7 @@
         </is>
       </c>
       <c r="D189" t="n">
-        <v>104</v>
+        <v>87</v>
       </c>
     </row>
     <row r="190">
@@ -3505,7 +3505,7 @@
         </is>
       </c>
       <c r="D193" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="194">
@@ -3665,7 +3665,7 @@
         </is>
       </c>
       <c r="D203" t="n">
-        <v>66</v>
+        <v>60</v>
       </c>
     </row>
     <row r="204">
@@ -3683,7 +3683,7 @@
         </is>
       </c>
       <c r="D204" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="205">
@@ -4025,7 +4025,7 @@
         </is>
       </c>
       <c r="D226" t="n">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="227">
@@ -4071,7 +4071,7 @@
         </is>
       </c>
       <c r="D229" t="n">
-        <v>113</v>
+        <v>111</v>
       </c>
     </row>
     <row r="230">
@@ -4089,7 +4089,7 @@
         </is>
       </c>
       <c r="D230" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="231">

</xml_diff>

<commit_message>
data: field/odds refresh 2026-05-04 18:00 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -465,7 +465,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3">
@@ -607,7 +607,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="12">
@@ -685,7 +685,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="17">
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="18">
@@ -749,7 +749,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="21">
@@ -907,7 +907,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="31">
@@ -925,7 +925,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="32">
@@ -1005,7 +1005,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="37">
@@ -1107,7 +1107,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="44">
@@ -1121,7 +1121,7 @@
       </c>
       <c r="C44" t="inlineStr"/>
       <c r="D44" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="45">
@@ -1165,7 +1165,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>18</v>
+        <v>22</v>
       </c>
     </row>
     <row r="48">
@@ -1183,7 +1183,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="49">
@@ -1233,7 +1233,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="52">
@@ -1283,7 +1283,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>56</v>
+        <v>52</v>
       </c>
     </row>
     <row r="55">
@@ -1337,7 +1337,7 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="58">
@@ -1373,7 +1373,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="60">
@@ -1455,7 +1455,7 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="65">
@@ -1563,7 +1563,7 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="72">
@@ -1693,7 +1693,7 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="80">
@@ -1757,7 +1757,7 @@
         </is>
       </c>
       <c r="D83" t="n">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="84">
@@ -1907,7 +1907,7 @@
         </is>
       </c>
       <c r="D92" t="n">
-        <v>134</v>
+        <v>138</v>
       </c>
     </row>
     <row r="93">
@@ -1925,7 +1925,7 @@
         </is>
       </c>
       <c r="D93" t="n">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="94">
@@ -2031,7 +2031,7 @@
         </is>
       </c>
       <c r="D100" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="101">
@@ -2049,7 +2049,7 @@
         </is>
       </c>
       <c r="D101" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
     </row>
     <row r="102">
@@ -2291,7 +2291,7 @@
         </is>
       </c>
       <c r="D117" t="n">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
     <row r="118">
@@ -2309,7 +2309,7 @@
         </is>
       </c>
       <c r="D118" t="n">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="119">
@@ -2429,7 +2429,7 @@
         </is>
       </c>
       <c r="D126" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="127">
@@ -2447,7 +2447,7 @@
         </is>
       </c>
       <c r="D127" t="n">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="128">
@@ -2465,7 +2465,7 @@
         </is>
       </c>
       <c r="D128" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="129">
@@ -2519,7 +2519,7 @@
         </is>
       </c>
       <c r="D131" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="132">
@@ -2713,7 +2713,7 @@
         </is>
       </c>
       <c r="D143" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
     </row>
     <row r="144">
@@ -2771,7 +2771,7 @@
         </is>
       </c>
       <c r="D147" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="148">
@@ -2885,7 +2885,7 @@
         </is>
       </c>
       <c r="D155" t="n">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="156">
@@ -2985,7 +2985,7 @@
         </is>
       </c>
       <c r="D161" t="n">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="162">
@@ -3017,7 +3017,7 @@
         </is>
       </c>
       <c r="D163" t="n">
-        <v>88</v>
+        <v>84</v>
       </c>
     </row>
     <row r="164">
@@ -3271,7 +3271,7 @@
         </is>
       </c>
       <c r="D179" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="180">
@@ -3361,7 +3361,7 @@
         </is>
       </c>
       <c r="D184" t="n">
-        <v>54</v>
+        <v>43</v>
       </c>
     </row>
     <row r="185">
@@ -3407,7 +3407,7 @@
         </is>
       </c>
       <c r="D187" t="n">
-        <v>430</v>
+        <v>441</v>
       </c>
     </row>
     <row r="188">
@@ -3439,7 +3439,7 @@
         </is>
       </c>
       <c r="D189" t="n">
-        <v>104</v>
+        <v>87</v>
       </c>
     </row>
     <row r="190">
@@ -3505,7 +3505,7 @@
         </is>
       </c>
       <c r="D193" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="194">
@@ -3665,7 +3665,7 @@
         </is>
       </c>
       <c r="D203" t="n">
-        <v>66</v>
+        <v>60</v>
       </c>
     </row>
     <row r="204">
@@ -3683,7 +3683,7 @@
         </is>
       </c>
       <c r="D204" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="205">
@@ -4025,7 +4025,7 @@
         </is>
       </c>
       <c r="D226" t="n">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="227">
@@ -4071,7 +4071,7 @@
         </is>
       </c>
       <c r="D229" t="n">
-        <v>113</v>
+        <v>111</v>
       </c>
     </row>
     <row r="230">
@@ -4089,7 +4089,7 @@
         </is>
       </c>
       <c r="D230" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="231">
@@ -4175,7 +4175,7 @@
         </is>
       </c>
       <c r="D235" t="n">
-        <v>140</v>
+        <v>120</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: field/odds refresh 2026-05-10 22:18 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -557,7 +557,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="9">
@@ -1023,7 +1023,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>24</v>
+        <v>29</v>
       </c>
     </row>
     <row r="38">
@@ -1215,7 +1215,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>142</v>
+        <v>126</v>
       </c>
     </row>
     <row r="51">
@@ -1437,7 +1437,7 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="64">
@@ -1607,7 +1607,7 @@
         </is>
       </c>
       <c r="D74" t="n">
-        <v>31</v>
+        <v>25</v>
       </c>
     </row>
     <row r="75">
@@ -1643,7 +1643,7 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
     <row r="77">
@@ -1675,7 +1675,7 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="79">
@@ -1725,7 +1725,7 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="82">
@@ -1793,7 +1793,7 @@
         </is>
       </c>
       <c r="D85" t="n">
-        <v>57</v>
+        <v>61</v>
       </c>
     </row>
     <row r="86">
@@ -1829,7 +1829,7 @@
         </is>
       </c>
       <c r="D87" t="n">
-        <v>99</v>
+        <v>107</v>
       </c>
     </row>
     <row r="88">
@@ -1960,7 +1960,9 @@
           <t>https://pga-tour-res.cloudinary.com/image/upload/c_fill,g_face:center,q_auto,f_auto,dpr_2.0,h_220,w_200,d_stub:default_avatar_light.webp/headshots_30925</t>
         </is>
       </c>
-      <c r="D95" t="inlineStr"/>
+      <c r="D95" t="n">
+        <v>468</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -2085,7 +2087,7 @@
         </is>
       </c>
       <c r="D103" t="n">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="104">
@@ -2177,7 +2179,7 @@
         </is>
       </c>
       <c r="D109" t="n">
-        <v>125</v>
+        <v>127</v>
       </c>
     </row>
     <row r="110">
@@ -2571,7 +2573,7 @@
         </is>
       </c>
       <c r="D134" t="n">
-        <v>108</v>
+        <v>104</v>
       </c>
     </row>
     <row r="135">
@@ -2649,7 +2651,7 @@
       </c>
       <c r="C139" t="inlineStr"/>
       <c r="D139" t="n">
-        <v>122</v>
+        <v>124</v>
       </c>
     </row>
     <row r="140">
@@ -2677,7 +2679,7 @@
       </c>
       <c r="C141" t="inlineStr"/>
       <c r="D141" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="142">
@@ -2695,7 +2697,7 @@
         </is>
       </c>
       <c r="D142" t="n">
-        <v>161</v>
+        <v>178</v>
       </c>
     </row>
     <row r="143">
@@ -3035,7 +3037,7 @@
         </is>
       </c>
       <c r="D164" t="n">
-        <v>30</v>
+        <v>21</v>
       </c>
     </row>
     <row r="165">
@@ -3053,7 +3055,7 @@
         </is>
       </c>
       <c r="D165" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="166">
@@ -3127,7 +3129,7 @@
         </is>
       </c>
       <c r="D170" t="n">
-        <v>124</v>
+        <v>133</v>
       </c>
     </row>
     <row r="171">
@@ -3307,7 +3309,7 @@
         </is>
       </c>
       <c r="D181" t="n">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="182">
@@ -3325,7 +3327,7 @@
         </is>
       </c>
       <c r="D182" t="n">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="183">
@@ -3343,7 +3345,7 @@
         </is>
       </c>
       <c r="D183" t="n">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="184">
@@ -3457,7 +3459,7 @@
         </is>
       </c>
       <c r="D190" t="n">
-        <v>222</v>
+        <v>235</v>
       </c>
     </row>
     <row r="191">
@@ -3487,7 +3489,7 @@
       </c>
       <c r="C192" t="inlineStr"/>
       <c r="D192" t="n">
-        <v>267</v>
+        <v>273</v>
       </c>
     </row>
     <row r="193">
@@ -3737,7 +3739,7 @@
         </is>
       </c>
       <c r="D207" t="n">
-        <v>59</v>
+        <v>62</v>
       </c>
     </row>
     <row r="208">

</xml_diff>

<commit_message>
data: field/odds refresh 2026-05-11 05:53 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -539,7 +539,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="8">
@@ -557,7 +557,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="9">
@@ -575,7 +575,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="10">
@@ -607,7 +607,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="12">
@@ -685,7 +685,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="17">
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>101</v>
+        <v>104</v>
       </c>
     </row>
     <row r="18">
@@ -749,7 +749,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="21">
@@ -781,7 +781,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>86</v>
+        <v>90</v>
       </c>
     </row>
     <row r="23">
@@ -799,7 +799,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="24">
@@ -857,7 +857,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="28">
@@ -907,7 +907,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="31">
@@ -925,7 +925,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="32">
@@ -1005,7 +1005,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>38</v>
+        <v>41</v>
       </c>
     </row>
     <row r="37">
@@ -1023,7 +1023,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>24</v>
+        <v>28</v>
       </c>
     </row>
     <row r="38">
@@ -1049,7 +1049,7 @@
       </c>
       <c r="C39" t="inlineStr"/>
       <c r="D39" t="n">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="40">
@@ -1107,7 +1107,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>44</v>
+        <v>48</v>
       </c>
     </row>
     <row r="44">
@@ -1121,7 +1121,7 @@
       </c>
       <c r="C44" t="inlineStr"/>
       <c r="D44" t="n">
-        <v>44</v>
+        <v>48</v>
       </c>
     </row>
     <row r="45">
@@ -1165,7 +1165,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="48">
@@ -1215,7 +1215,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>142</v>
+        <v>134</v>
       </c>
     </row>
     <row r="51">
@@ -1251,7 +1251,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="53">
@@ -1283,7 +1283,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>52</v>
+        <v>37</v>
       </c>
     </row>
     <row r="55">
@@ -1301,7 +1301,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="56">
@@ -1337,7 +1337,7 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>32</v>
+        <v>36</v>
       </c>
     </row>
     <row r="58">
@@ -1373,7 +1373,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>90</v>
+        <v>93</v>
       </c>
     </row>
     <row r="60">
@@ -1419,7 +1419,7 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="63">
@@ -1437,7 +1437,7 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="64">
@@ -1487,7 +1487,7 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>109</v>
+        <v>115</v>
       </c>
     </row>
     <row r="67">
@@ -1531,7 +1531,7 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>64</v>
+        <v>57</v>
       </c>
     </row>
     <row r="70">
@@ -1607,7 +1607,7 @@
         </is>
       </c>
       <c r="D74" t="n">
-        <v>31</v>
+        <v>26</v>
       </c>
     </row>
     <row r="75">
@@ -1625,7 +1625,7 @@
         </is>
       </c>
       <c r="D75" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="76">
@@ -1643,7 +1643,7 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="77">
@@ -1675,7 +1675,7 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>144</v>
+        <v>151</v>
       </c>
     </row>
     <row r="79">
@@ -1693,7 +1693,7 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="80">
@@ -1725,7 +1725,7 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>82</v>
+        <v>88</v>
       </c>
     </row>
     <row r="82">
@@ -1775,7 +1775,7 @@
         </is>
       </c>
       <c r="D84" t="n">
-        <v>37</v>
+        <v>29</v>
       </c>
     </row>
     <row r="85">
@@ -1793,7 +1793,7 @@
         </is>
       </c>
       <c r="D85" t="n">
-        <v>57</v>
+        <v>64</v>
       </c>
     </row>
     <row r="86">
@@ -1811,7 +1811,7 @@
         </is>
       </c>
       <c r="D86" t="n">
-        <v>118</v>
+        <v>123</v>
       </c>
     </row>
     <row r="87">
@@ -1829,7 +1829,7 @@
         </is>
       </c>
       <c r="D87" t="n">
-        <v>99</v>
+        <v>117</v>
       </c>
     </row>
     <row r="88">
@@ -1875,7 +1875,7 @@
         </is>
       </c>
       <c r="D90" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="91">
@@ -1925,7 +1925,7 @@
         </is>
       </c>
       <c r="D93" t="n">
-        <v>77</v>
+        <v>67</v>
       </c>
     </row>
     <row r="94">
@@ -1943,7 +1943,7 @@
         </is>
       </c>
       <c r="D94" t="n">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="95">
@@ -1960,7 +1960,9 @@
           <t>https://pga-tour-res.cloudinary.com/image/upload/c_fill,g_face:center,q_auto,f_auto,dpr_2.0,h_220,w_200,d_stub:default_avatar_light.webp/headshots_30925</t>
         </is>
       </c>
-      <c r="D95" t="inlineStr"/>
+      <c r="D95" t="n">
+        <v>471</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -2031,7 +2033,7 @@
         </is>
       </c>
       <c r="D100" t="n">
-        <v>41</v>
+        <v>45</v>
       </c>
     </row>
     <row r="101">
@@ -2049,7 +2051,7 @@
         </is>
       </c>
       <c r="D101" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="102">
@@ -2085,7 +2087,7 @@
         </is>
       </c>
       <c r="D103" t="n">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
     <row r="104">
@@ -2147,7 +2149,7 @@
         </is>
       </c>
       <c r="D107" t="n">
-        <v>36</v>
+        <v>39</v>
       </c>
     </row>
     <row r="108">
@@ -2291,7 +2293,7 @@
         </is>
       </c>
       <c r="D117" t="n">
-        <v>27</v>
+        <v>31</v>
       </c>
     </row>
     <row r="118">
@@ -2353,7 +2355,7 @@
         </is>
       </c>
       <c r="D121" t="n">
-        <v>35</v>
+        <v>38</v>
       </c>
     </row>
     <row r="122">
@@ -2429,7 +2431,7 @@
         </is>
       </c>
       <c r="D126" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="127">
@@ -2447,7 +2449,7 @@
         </is>
       </c>
       <c r="D127" t="n">
-        <v>94</v>
+        <v>99</v>
       </c>
     </row>
     <row r="128">
@@ -2465,7 +2467,7 @@
         </is>
       </c>
       <c r="D128" t="n">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="129">
@@ -2483,7 +2485,7 @@
         </is>
       </c>
       <c r="D129" t="n">
-        <v>78</v>
+        <v>80</v>
       </c>
     </row>
     <row r="130">
@@ -2519,7 +2521,7 @@
         </is>
       </c>
       <c r="D131" t="n">
-        <v>28</v>
+        <v>33</v>
       </c>
     </row>
     <row r="132">
@@ -2571,7 +2573,7 @@
         </is>
       </c>
       <c r="D134" t="n">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="135">
@@ -2635,7 +2637,7 @@
         </is>
       </c>
       <c r="D138" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="139">
@@ -2649,7 +2651,7 @@
       </c>
       <c r="C139" t="inlineStr"/>
       <c r="D139" t="n">
-        <v>122</v>
+        <v>132</v>
       </c>
     </row>
     <row r="140">
@@ -2677,7 +2679,7 @@
       </c>
       <c r="C141" t="inlineStr"/>
       <c r="D141" t="n">
-        <v>75</v>
+        <v>77</v>
       </c>
     </row>
     <row r="142">
@@ -2695,7 +2697,7 @@
         </is>
       </c>
       <c r="D142" t="n">
-        <v>161</v>
+        <v>167</v>
       </c>
     </row>
     <row r="143">
@@ -2885,7 +2887,7 @@
         </is>
       </c>
       <c r="D155" t="n">
-        <v>83</v>
+        <v>86</v>
       </c>
     </row>
     <row r="156">
@@ -2903,7 +2905,7 @@
         </is>
       </c>
       <c r="D156" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="157">
@@ -2967,7 +2969,7 @@
         </is>
       </c>
       <c r="D160" t="n">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="161">
@@ -2985,7 +2987,7 @@
         </is>
       </c>
       <c r="D161" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="162">
@@ -3017,7 +3019,7 @@
         </is>
       </c>
       <c r="D163" t="n">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
     <row r="164">
@@ -3035,7 +3037,7 @@
         </is>
       </c>
       <c r="D164" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="165">
@@ -3053,7 +3055,7 @@
         </is>
       </c>
       <c r="D165" t="n">
-        <v>41</v>
+        <v>44</v>
       </c>
     </row>
     <row r="166">
@@ -3097,7 +3099,7 @@
         </is>
       </c>
       <c r="D168" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="169">
@@ -3127,7 +3129,7 @@
         </is>
       </c>
       <c r="D170" t="n">
-        <v>124</v>
+        <v>141</v>
       </c>
     </row>
     <row r="171">
@@ -3163,7 +3165,7 @@
         </is>
       </c>
       <c r="D172" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="173">
@@ -3271,7 +3273,7 @@
         </is>
       </c>
       <c r="D179" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="180">
@@ -3307,7 +3309,7 @@
         </is>
       </c>
       <c r="D181" t="n">
-        <v>147</v>
+        <v>155</v>
       </c>
     </row>
     <row r="182">
@@ -3325,7 +3327,7 @@
         </is>
       </c>
       <c r="D182" t="n">
-        <v>91</v>
+        <v>97</v>
       </c>
     </row>
     <row r="183">
@@ -3343,7 +3345,7 @@
         </is>
       </c>
       <c r="D183" t="n">
-        <v>91</v>
+        <v>97</v>
       </c>
     </row>
     <row r="184">
@@ -3361,7 +3363,7 @@
         </is>
       </c>
       <c r="D184" t="n">
-        <v>43</v>
+        <v>46</v>
       </c>
     </row>
     <row r="185">
@@ -3439,7 +3441,7 @@
         </is>
       </c>
       <c r="D189" t="n">
-        <v>87</v>
+        <v>78</v>
       </c>
     </row>
     <row r="190">
@@ -3457,7 +3459,7 @@
         </is>
       </c>
       <c r="D190" t="n">
-        <v>222</v>
+        <v>239</v>
       </c>
     </row>
     <row r="191">
@@ -3487,7 +3489,7 @@
       </c>
       <c r="C192" t="inlineStr"/>
       <c r="D192" t="n">
-        <v>267</v>
+        <v>131</v>
       </c>
     </row>
     <row r="193">
@@ -3505,7 +3507,7 @@
         </is>
       </c>
       <c r="D193" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="194">
@@ -3523,7 +3525,7 @@
         </is>
       </c>
       <c r="D194" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="195">
@@ -3555,7 +3557,7 @@
         </is>
       </c>
       <c r="D196" t="n">
-        <v>46</v>
+        <v>49</v>
       </c>
     </row>
     <row r="197">
@@ -3569,7 +3571,7 @@
       </c>
       <c r="C197" t="inlineStr"/>
       <c r="D197" t="n">
-        <v>46</v>
+        <v>49</v>
       </c>
     </row>
     <row r="198">
@@ -3665,7 +3667,7 @@
         </is>
       </c>
       <c r="D203" t="n">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="204">
@@ -3683,7 +3685,7 @@
         </is>
       </c>
       <c r="D204" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="205">
@@ -3701,7 +3703,7 @@
         </is>
       </c>
       <c r="D205" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="206">
@@ -3737,7 +3739,7 @@
         </is>
       </c>
       <c r="D207" t="n">
-        <v>59</v>
+        <v>63</v>
       </c>
     </row>
     <row r="208">
@@ -3793,7 +3795,7 @@
         </is>
       </c>
       <c r="D211" t="n">
-        <v>57</v>
+        <v>60</v>
       </c>
     </row>
     <row r="212">
@@ -3829,7 +3831,7 @@
         </is>
       </c>
       <c r="D213" t="n">
-        <v>112</v>
+        <v>126</v>
       </c>
     </row>
     <row r="214">
@@ -4071,7 +4073,7 @@
         </is>
       </c>
       <c r="D229" t="n">
-        <v>111</v>
+        <v>105</v>
       </c>
     </row>
     <row r="230">
@@ -4175,7 +4177,7 @@
         </is>
       </c>
       <c r="D235" t="n">
-        <v>120</v>
+        <v>83</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: field/odds refresh 2026-05-11 12:00 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -539,7 +539,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="8">
@@ -557,7 +557,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>95</v>
+        <v>92</v>
       </c>
     </row>
     <row r="9">
@@ -575,7 +575,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="10">
@@ -607,7 +607,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="12">
@@ -685,7 +685,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="17">
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>101</v>
+        <v>104</v>
       </c>
     </row>
     <row r="18">
@@ -749,7 +749,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="21">
@@ -781,7 +781,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>86</v>
+        <v>90</v>
       </c>
     </row>
     <row r="23">
@@ -799,7 +799,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="24">
@@ -857,7 +857,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="28">
@@ -907,7 +907,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="31">
@@ -925,7 +925,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="32">
@@ -1005,7 +1005,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>38</v>
+        <v>41</v>
       </c>
     </row>
     <row r="37">
@@ -1023,7 +1023,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="38">
@@ -1049,7 +1049,7 @@
       </c>
       <c r="C39" t="inlineStr"/>
       <c r="D39" t="n">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="40">
@@ -1107,7 +1107,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>44</v>
+        <v>48</v>
       </c>
     </row>
     <row r="44">
@@ -1121,7 +1121,7 @@
       </c>
       <c r="C44" t="inlineStr"/>
       <c r="D44" t="n">
-        <v>44</v>
+        <v>48</v>
       </c>
     </row>
     <row r="45">
@@ -1165,7 +1165,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="48">
@@ -1215,7 +1215,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>126</v>
+        <v>134</v>
       </c>
     </row>
     <row r="51">
@@ -1251,7 +1251,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="53">
@@ -1283,7 +1283,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>52</v>
+        <v>37</v>
       </c>
     </row>
     <row r="55">
@@ -1301,7 +1301,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="56">
@@ -1337,7 +1337,7 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>32</v>
+        <v>36</v>
       </c>
     </row>
     <row r="58">
@@ -1373,7 +1373,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>90</v>
+        <v>93</v>
       </c>
     </row>
     <row r="60">
@@ -1419,7 +1419,7 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="63">
@@ -1437,7 +1437,7 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="64">
@@ -1487,7 +1487,7 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>109</v>
+        <v>115</v>
       </c>
     </row>
     <row r="67">
@@ -1531,7 +1531,7 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>64</v>
+        <v>57</v>
       </c>
     </row>
     <row r="70">
@@ -1607,7 +1607,7 @@
         </is>
       </c>
       <c r="D74" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="75">
@@ -1625,7 +1625,7 @@
         </is>
       </c>
       <c r="D75" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="76">
@@ -1643,7 +1643,7 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>82</v>
+        <v>85</v>
       </c>
     </row>
     <row r="77">
@@ -1675,7 +1675,7 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>143</v>
+        <v>151</v>
       </c>
     </row>
     <row r="79">
@@ -1693,7 +1693,7 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="80">
@@ -1725,7 +1725,7 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>81</v>
+        <v>88</v>
       </c>
     </row>
     <row r="82">
@@ -1775,7 +1775,7 @@
         </is>
       </c>
       <c r="D84" t="n">
-        <v>37</v>
+        <v>29</v>
       </c>
     </row>
     <row r="85">
@@ -1793,7 +1793,7 @@
         </is>
       </c>
       <c r="D85" t="n">
-        <v>61</v>
+        <v>64</v>
       </c>
     </row>
     <row r="86">
@@ -1811,7 +1811,7 @@
         </is>
       </c>
       <c r="D86" t="n">
-        <v>118</v>
+        <v>123</v>
       </c>
     </row>
     <row r="87">
@@ -1829,7 +1829,7 @@
         </is>
       </c>
       <c r="D87" t="n">
-        <v>107</v>
+        <v>117</v>
       </c>
     </row>
     <row r="88">
@@ -1875,7 +1875,7 @@
         </is>
       </c>
       <c r="D90" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="91">
@@ -1925,7 +1925,7 @@
         </is>
       </c>
       <c r="D93" t="n">
-        <v>77</v>
+        <v>67</v>
       </c>
     </row>
     <row r="94">
@@ -1943,7 +1943,7 @@
         </is>
       </c>
       <c r="D94" t="n">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="95">
@@ -1961,7 +1961,7 @@
         </is>
       </c>
       <c r="D95" t="n">
-        <v>468</v>
+        <v>471</v>
       </c>
     </row>
     <row r="96">
@@ -2033,7 +2033,7 @@
         </is>
       </c>
       <c r="D100" t="n">
-        <v>41</v>
+        <v>45</v>
       </c>
     </row>
     <row r="101">
@@ -2051,7 +2051,7 @@
         </is>
       </c>
       <c r="D101" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="102">
@@ -2087,7 +2087,7 @@
         </is>
       </c>
       <c r="D103" t="n">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="104">
@@ -2149,7 +2149,7 @@
         </is>
       </c>
       <c r="D107" t="n">
-        <v>36</v>
+        <v>39</v>
       </c>
     </row>
     <row r="108">
@@ -2179,7 +2179,7 @@
         </is>
       </c>
       <c r="D109" t="n">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="110">
@@ -2293,7 +2293,7 @@
         </is>
       </c>
       <c r="D117" t="n">
-        <v>27</v>
+        <v>31</v>
       </c>
     </row>
     <row r="118">
@@ -2355,7 +2355,7 @@
         </is>
       </c>
       <c r="D121" t="n">
-        <v>35</v>
+        <v>38</v>
       </c>
     </row>
     <row r="122">
@@ -2431,7 +2431,7 @@
         </is>
       </c>
       <c r="D126" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="127">
@@ -2449,7 +2449,7 @@
         </is>
       </c>
       <c r="D127" t="n">
-        <v>94</v>
+        <v>99</v>
       </c>
     </row>
     <row r="128">
@@ -2467,7 +2467,7 @@
         </is>
       </c>
       <c r="D128" t="n">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="129">
@@ -2485,7 +2485,7 @@
         </is>
       </c>
       <c r="D129" t="n">
-        <v>78</v>
+        <v>80</v>
       </c>
     </row>
     <row r="130">
@@ -2521,7 +2521,7 @@
         </is>
       </c>
       <c r="D131" t="n">
-        <v>28</v>
+        <v>33</v>
       </c>
     </row>
     <row r="132">
@@ -2573,7 +2573,7 @@
         </is>
       </c>
       <c r="D134" t="n">
-        <v>104</v>
+        <v>109</v>
       </c>
     </row>
     <row r="135">
@@ -2637,7 +2637,7 @@
         </is>
       </c>
       <c r="D138" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="139">
@@ -2651,7 +2651,7 @@
       </c>
       <c r="C139" t="inlineStr"/>
       <c r="D139" t="n">
-        <v>124</v>
+        <v>132</v>
       </c>
     </row>
     <row r="140">
@@ -2679,7 +2679,7 @@
       </c>
       <c r="C141" t="inlineStr"/>
       <c r="D141" t="n">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="142">
@@ -2697,7 +2697,7 @@
         </is>
       </c>
       <c r="D142" t="n">
-        <v>178</v>
+        <v>167</v>
       </c>
     </row>
     <row r="143">
@@ -2887,7 +2887,7 @@
         </is>
       </c>
       <c r="D155" t="n">
-        <v>83</v>
+        <v>86</v>
       </c>
     </row>
     <row r="156">
@@ -2905,7 +2905,7 @@
         </is>
       </c>
       <c r="D156" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="157">
@@ -2969,7 +2969,7 @@
         </is>
       </c>
       <c r="D160" t="n">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="161">
@@ -2987,7 +2987,7 @@
         </is>
       </c>
       <c r="D161" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="162">
@@ -3019,7 +3019,7 @@
         </is>
       </c>
       <c r="D163" t="n">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
     <row r="164">
@@ -3037,7 +3037,7 @@
         </is>
       </c>
       <c r="D164" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="165">
@@ -3055,7 +3055,7 @@
         </is>
       </c>
       <c r="D165" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="166">
@@ -3099,7 +3099,7 @@
         </is>
       </c>
       <c r="D168" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="169">
@@ -3129,7 +3129,7 @@
         </is>
       </c>
       <c r="D170" t="n">
-        <v>133</v>
+        <v>141</v>
       </c>
     </row>
     <row r="171">
@@ -3165,7 +3165,7 @@
         </is>
       </c>
       <c r="D172" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="173">
@@ -3273,7 +3273,7 @@
         </is>
       </c>
       <c r="D179" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="180">
@@ -3309,7 +3309,7 @@
         </is>
       </c>
       <c r="D181" t="n">
-        <v>148</v>
+        <v>155</v>
       </c>
     </row>
     <row r="182">
@@ -3327,7 +3327,7 @@
         </is>
       </c>
       <c r="D182" t="n">
-        <v>93</v>
+        <v>97</v>
       </c>
     </row>
     <row r="183">
@@ -3345,7 +3345,7 @@
         </is>
       </c>
       <c r="D183" t="n">
-        <v>93</v>
+        <v>97</v>
       </c>
     </row>
     <row r="184">
@@ -3363,7 +3363,7 @@
         </is>
       </c>
       <c r="D184" t="n">
-        <v>43</v>
+        <v>46</v>
       </c>
     </row>
     <row r="185">
@@ -3441,7 +3441,7 @@
         </is>
       </c>
       <c r="D189" t="n">
-        <v>87</v>
+        <v>78</v>
       </c>
     </row>
     <row r="190">
@@ -3459,7 +3459,7 @@
         </is>
       </c>
       <c r="D190" t="n">
-        <v>235</v>
+        <v>239</v>
       </c>
     </row>
     <row r="191">
@@ -3489,7 +3489,7 @@
       </c>
       <c r="C192" t="inlineStr"/>
       <c r="D192" t="n">
-        <v>273</v>
+        <v>131</v>
       </c>
     </row>
     <row r="193">
@@ -3507,7 +3507,7 @@
         </is>
       </c>
       <c r="D193" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="194">
@@ -3525,7 +3525,7 @@
         </is>
       </c>
       <c r="D194" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="195">
@@ -3557,7 +3557,7 @@
         </is>
       </c>
       <c r="D196" t="n">
-        <v>46</v>
+        <v>49</v>
       </c>
     </row>
     <row r="197">
@@ -3571,7 +3571,7 @@
       </c>
       <c r="C197" t="inlineStr"/>
       <c r="D197" t="n">
-        <v>46</v>
+        <v>49</v>
       </c>
     </row>
     <row r="198">
@@ -3667,7 +3667,7 @@
         </is>
       </c>
       <c r="D203" t="n">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="204">
@@ -3685,7 +3685,7 @@
         </is>
       </c>
       <c r="D204" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="205">
@@ -3703,7 +3703,7 @@
         </is>
       </c>
       <c r="D205" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="206">
@@ -3739,7 +3739,7 @@
         </is>
       </c>
       <c r="D207" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="208">
@@ -3795,7 +3795,7 @@
         </is>
       </c>
       <c r="D211" t="n">
-        <v>57</v>
+        <v>60</v>
       </c>
     </row>
     <row r="212">
@@ -3831,7 +3831,7 @@
         </is>
       </c>
       <c r="D213" t="n">
-        <v>112</v>
+        <v>126</v>
       </c>
     </row>
     <row r="214">
@@ -4073,7 +4073,7 @@
         </is>
       </c>
       <c r="D229" t="n">
-        <v>111</v>
+        <v>105</v>
       </c>
     </row>
     <row r="230">
@@ -4177,7 +4177,7 @@
         </is>
       </c>
       <c r="D235" t="n">
-        <v>120</v>
+        <v>83</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: field/odds refresh 2026-05-18 06:00 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -589,7 +589,7 @@
       </c>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="n">
-        <v>240</v>
+        <v>256</v>
       </c>
     </row>
     <row r="11">
@@ -717,7 +717,7 @@
       </c>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="n">
-        <v>445</v>
+        <v>466</v>
       </c>
     </row>
     <row r="19">
@@ -813,7 +813,7 @@
       </c>
       <c r="C24" t="inlineStr"/>
       <c r="D24" t="n">
-        <v>304</v>
+        <v>313</v>
       </c>
     </row>
     <row r="25">
@@ -839,7 +839,7 @@
       </c>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="n">
-        <v>219</v>
+        <v>238</v>
       </c>
     </row>
     <row r="27">
@@ -875,7 +875,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>119</v>
+        <v>116</v>
       </c>
     </row>
     <row r="29">
@@ -969,7 +969,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>181</v>
+        <v>193</v>
       </c>
     </row>
     <row r="35">
@@ -987,7 +987,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>215</v>
+        <v>246</v>
       </c>
     </row>
     <row r="36">
@@ -1089,7 +1089,7 @@
       </c>
       <c r="C42" t="inlineStr"/>
       <c r="D42" t="n">
-        <v>270</v>
+        <v>285</v>
       </c>
     </row>
     <row r="43">
@@ -1135,7 +1135,7 @@
       </c>
       <c r="C45" t="inlineStr"/>
       <c r="D45" t="n">
-        <v>157</v>
+        <v>165</v>
       </c>
     </row>
     <row r="46">
@@ -1183,7 +1183,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>117</v>
+        <v>119</v>
       </c>
     </row>
     <row r="49">
@@ -1197,7 +1197,7 @@
       </c>
       <c r="C49" t="inlineStr"/>
       <c r="D49" t="n">
-        <v>179</v>
+        <v>189</v>
       </c>
     </row>
     <row r="50">
@@ -1265,7 +1265,7 @@
       </c>
       <c r="C53" t="inlineStr"/>
       <c r="D53" t="n">
-        <v>267</v>
+        <v>264</v>
       </c>
     </row>
     <row r="54">
@@ -1319,7 +1319,7 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>410</v>
+        <v>389</v>
       </c>
     </row>
     <row r="57">
@@ -1355,7 +1355,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>183</v>
+        <v>187</v>
       </c>
     </row>
     <row r="59">
@@ -1387,7 +1387,7 @@
       </c>
       <c r="C60" t="inlineStr"/>
       <c r="D60" t="n">
-        <v>306</v>
+        <v>323</v>
       </c>
     </row>
     <row r="61">
@@ -1401,7 +1401,7 @@
       </c>
       <c r="C61" t="inlineStr"/>
       <c r="D61" t="n">
-        <v>358</v>
+        <v>386</v>
       </c>
     </row>
     <row r="62">
@@ -1469,7 +1469,7 @@
       </c>
       <c r="C65" t="inlineStr"/>
       <c r="D65" t="n">
-        <v>220</v>
+        <v>206</v>
       </c>
     </row>
     <row r="66">
@@ -1513,7 +1513,7 @@
       </c>
       <c r="C68" t="inlineStr"/>
       <c r="D68" t="n">
-        <v>244</v>
+        <v>262</v>
       </c>
     </row>
     <row r="69">
@@ -1544,9 +1544,7 @@
         <v>19865</v>
       </c>
       <c r="C70" t="inlineStr"/>
-      <c r="D70" t="n">
-        <v>492</v>
-      </c>
+      <c r="D70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -1657,7 +1655,7 @@
       </c>
       <c r="C77" t="inlineStr"/>
       <c r="D77" t="n">
-        <v>292</v>
+        <v>324</v>
       </c>
     </row>
     <row r="78">
@@ -1707,7 +1705,7 @@
       </c>
       <c r="C80" t="inlineStr"/>
       <c r="D80" t="n">
-        <v>135</v>
+        <v>149</v>
       </c>
     </row>
     <row r="81">
@@ -1739,7 +1737,7 @@
       </c>
       <c r="C82" t="inlineStr"/>
       <c r="D82" t="n">
-        <v>412</v>
+        <v>449</v>
       </c>
     </row>
     <row r="83">
@@ -1857,7 +1855,7 @@
       </c>
       <c r="C89" t="inlineStr"/>
       <c r="D89" t="n">
-        <v>166</v>
+        <v>148</v>
       </c>
     </row>
     <row r="90">
@@ -1889,7 +1887,7 @@
       </c>
       <c r="C91" t="inlineStr"/>
       <c r="D91" t="n">
-        <v>156</v>
+        <v>114</v>
       </c>
     </row>
     <row r="92">
@@ -1907,7 +1905,7 @@
         </is>
       </c>
       <c r="D92" t="n">
-        <v>138</v>
+        <v>144</v>
       </c>
     </row>
     <row r="93">
@@ -1989,7 +1987,7 @@
       </c>
       <c r="C97" t="inlineStr"/>
       <c r="D97" t="n">
-        <v>130</v>
+        <v>139</v>
       </c>
     </row>
     <row r="98">
@@ -2015,7 +2013,7 @@
       </c>
       <c r="C99" t="inlineStr"/>
       <c r="D99" t="n">
-        <v>287</v>
+        <v>298</v>
       </c>
     </row>
     <row r="100">
@@ -2069,7 +2067,7 @@
         </is>
       </c>
       <c r="D102" t="n">
-        <v>139</v>
+        <v>142</v>
       </c>
     </row>
     <row r="103">
@@ -2131,7 +2129,7 @@
       </c>
       <c r="C106" t="inlineStr"/>
       <c r="D106" t="n">
-        <v>275</v>
+        <v>294</v>
       </c>
     </row>
     <row r="107">
@@ -2193,7 +2191,7 @@
       </c>
       <c r="C110" t="inlineStr"/>
       <c r="D110" t="n">
-        <v>296</v>
+        <v>303</v>
       </c>
     </row>
     <row r="111">
@@ -2225,7 +2223,7 @@
       </c>
       <c r="C112" t="inlineStr"/>
       <c r="D112" t="n">
-        <v>170</v>
+        <v>178</v>
       </c>
     </row>
     <row r="113">
@@ -2337,7 +2335,7 @@
       </c>
       <c r="C120" t="inlineStr"/>
       <c r="D120" t="n">
-        <v>213</v>
+        <v>227</v>
       </c>
     </row>
     <row r="121">
@@ -2413,7 +2411,7 @@
       </c>
       <c r="C125" t="inlineStr"/>
       <c r="D125" t="n">
-        <v>425</v>
+        <v>446</v>
       </c>
     </row>
     <row r="126">
@@ -2539,7 +2537,7 @@
         </is>
       </c>
       <c r="D132" t="n">
-        <v>116</v>
+        <v>103</v>
       </c>
     </row>
     <row r="133">
@@ -2601,7 +2599,7 @@
       </c>
       <c r="C136" t="inlineStr"/>
       <c r="D136" t="n">
-        <v>180</v>
+        <v>190</v>
       </c>
     </row>
     <row r="137">
@@ -2619,7 +2617,7 @@
         </is>
       </c>
       <c r="D137" t="n">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="138">
@@ -2743,7 +2741,7 @@
       </c>
       <c r="C145" t="inlineStr"/>
       <c r="D145" t="n">
-        <v>341</v>
+        <v>357</v>
       </c>
     </row>
     <row r="146">
@@ -2787,7 +2785,7 @@
       </c>
       <c r="C148" t="inlineStr"/>
       <c r="D148" t="n">
-        <v>104</v>
+        <v>110</v>
       </c>
     </row>
     <row r="149">
@@ -2851,7 +2849,7 @@
       </c>
       <c r="C153" t="inlineStr"/>
       <c r="D153" t="n">
-        <v>316</v>
+        <v>328</v>
       </c>
     </row>
     <row r="154">
@@ -2869,7 +2867,7 @@
         </is>
       </c>
       <c r="D154" t="n">
-        <v>236</v>
+        <v>254</v>
       </c>
     </row>
     <row r="155">
@@ -2937,7 +2935,7 @@
       </c>
       <c r="C158" t="inlineStr"/>
       <c r="D158" t="n">
-        <v>242</v>
+        <v>237</v>
       </c>
     </row>
     <row r="159">
@@ -2951,7 +2949,7 @@
       </c>
       <c r="C159" t="inlineStr"/>
       <c r="D159" t="n">
-        <v>160</v>
+        <v>166</v>
       </c>
     </row>
     <row r="160">
@@ -3001,7 +2999,7 @@
       </c>
       <c r="C162" t="inlineStr"/>
       <c r="D162" t="n">
-        <v>175</v>
+        <v>183</v>
       </c>
     </row>
     <row r="163">
@@ -3069,7 +3067,7 @@
       </c>
       <c r="C166" t="inlineStr"/>
       <c r="D166" t="n">
-        <v>149</v>
+        <v>156</v>
       </c>
     </row>
     <row r="167">
@@ -3193,7 +3191,7 @@
       </c>
       <c r="C174" t="inlineStr"/>
       <c r="D174" t="n">
-        <v>140</v>
+        <v>121</v>
       </c>
     </row>
     <row r="175">
@@ -3229,7 +3227,7 @@
         </is>
       </c>
       <c r="D176" t="n">
-        <v>217</v>
+        <v>210</v>
       </c>
     </row>
     <row r="177">
@@ -3391,7 +3389,7 @@
       </c>
       <c r="C186" t="inlineStr"/>
       <c r="D186" t="n">
-        <v>249</v>
+        <v>268</v>
       </c>
     </row>
     <row r="187">
@@ -3423,7 +3421,7 @@
       </c>
       <c r="C188" t="inlineStr"/>
       <c r="D188" t="n">
-        <v>255</v>
+        <v>258</v>
       </c>
     </row>
     <row r="189">
@@ -3539,7 +3537,7 @@
       </c>
       <c r="C195" t="inlineStr"/>
       <c r="D195" t="n">
-        <v>239</v>
+        <v>247</v>
       </c>
     </row>
     <row r="196">
@@ -3607,7 +3605,7 @@
         </is>
       </c>
       <c r="D199" t="n">
-        <v>384</v>
+        <v>409</v>
       </c>
     </row>
     <row r="200">
@@ -3621,7 +3619,7 @@
       </c>
       <c r="C200" t="inlineStr"/>
       <c r="D200" t="n">
-        <v>207</v>
+        <v>208</v>
       </c>
     </row>
     <row r="201">
@@ -3635,7 +3633,7 @@
       </c>
       <c r="C201" t="inlineStr"/>
       <c r="D201" t="n">
-        <v>375</v>
+        <v>392</v>
       </c>
     </row>
     <row r="202">
@@ -3649,7 +3647,7 @@
       </c>
       <c r="C202" t="inlineStr"/>
       <c r="D202" t="n">
-        <v>188</v>
+        <v>202</v>
       </c>
     </row>
     <row r="203">
@@ -3721,7 +3719,7 @@
         </is>
       </c>
       <c r="D206" t="n">
-        <v>120</v>
+        <v>127</v>
       </c>
     </row>
     <row r="207">
@@ -3777,7 +3775,7 @@
       </c>
       <c r="C210" t="inlineStr"/>
       <c r="D210" t="n">
-        <v>319</v>
+        <v>335</v>
       </c>
     </row>
     <row r="211">
@@ -3813,7 +3811,7 @@
         </is>
       </c>
       <c r="D212" t="n">
-        <v>167</v>
+        <v>174</v>
       </c>
     </row>
     <row r="213">
@@ -3857,7 +3855,7 @@
       </c>
       <c r="C215" t="inlineStr"/>
       <c r="D215" t="n">
-        <v>246</v>
+        <v>265</v>
       </c>
     </row>
     <row r="216">
@@ -3871,7 +3869,7 @@
       </c>
       <c r="C216" t="inlineStr"/>
       <c r="D216" t="n">
-        <v>246</v>
+        <v>265</v>
       </c>
     </row>
     <row r="217">
@@ -3889,7 +3887,7 @@
         </is>
       </c>
       <c r="D217" t="n">
-        <v>153</v>
+        <v>164</v>
       </c>
     </row>
     <row r="218">
@@ -3903,7 +3901,7 @@
       </c>
       <c r="C218" t="inlineStr"/>
       <c r="D218" t="n">
-        <v>469</v>
+        <v>468</v>
       </c>
     </row>
     <row r="219">
@@ -3917,7 +3915,7 @@
       </c>
       <c r="C219" t="inlineStr"/>
       <c r="D219" t="n">
-        <v>221</v>
+        <v>223</v>
       </c>
     </row>
     <row r="220">
@@ -3971,7 +3969,7 @@
         </is>
       </c>
       <c r="D222" t="n">
-        <v>127</v>
+        <v>143</v>
       </c>
     </row>
     <row r="223">
@@ -3997,7 +3995,7 @@
       </c>
       <c r="C224" t="inlineStr"/>
       <c r="D224" t="n">
-        <v>400</v>
+        <v>420</v>
       </c>
     </row>
     <row r="225">
@@ -4041,7 +4039,7 @@
       </c>
       <c r="C227" t="inlineStr"/>
       <c r="D227" t="n">
-        <v>343</v>
+        <v>355</v>
       </c>
     </row>
     <row r="228">
@@ -4105,7 +4103,7 @@
       </c>
       <c r="C231" t="inlineStr"/>
       <c r="D231" t="n">
-        <v>168</v>
+        <v>177</v>
       </c>
     </row>
     <row r="232">
@@ -4123,7 +4121,7 @@
         </is>
       </c>
       <c r="D232" t="n">
-        <v>106</v>
+        <v>111</v>
       </c>
     </row>
     <row r="233">

</xml_diff>

<commit_message>
data: field/odds refresh 2026-05-18 06:17 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -589,7 +589,7 @@
       </c>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="n">
-        <v>240</v>
+        <v>256</v>
       </c>
     </row>
     <row r="11">
@@ -717,7 +717,7 @@
       </c>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="n">
-        <v>445</v>
+        <v>466</v>
       </c>
     </row>
     <row r="19">
@@ -813,7 +813,7 @@
       </c>
       <c r="C24" t="inlineStr"/>
       <c r="D24" t="n">
-        <v>304</v>
+        <v>313</v>
       </c>
     </row>
     <row r="25">
@@ -839,7 +839,7 @@
       </c>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="n">
-        <v>219</v>
+        <v>238</v>
       </c>
     </row>
     <row r="27">
@@ -875,7 +875,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>119</v>
+        <v>116</v>
       </c>
     </row>
     <row r="29">
@@ -969,7 +969,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>181</v>
+        <v>193</v>
       </c>
     </row>
     <row r="35">
@@ -987,7 +987,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>215</v>
+        <v>246</v>
       </c>
     </row>
     <row r="36">
@@ -1089,7 +1089,7 @@
       </c>
       <c r="C42" t="inlineStr"/>
       <c r="D42" t="n">
-        <v>270</v>
+        <v>285</v>
       </c>
     </row>
     <row r="43">
@@ -1135,7 +1135,7 @@
       </c>
       <c r="C45" t="inlineStr"/>
       <c r="D45" t="n">
-        <v>157</v>
+        <v>165</v>
       </c>
     </row>
     <row r="46">
@@ -1183,7 +1183,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>117</v>
+        <v>119</v>
       </c>
     </row>
     <row r="49">
@@ -1197,7 +1197,7 @@
       </c>
       <c r="C49" t="inlineStr"/>
       <c r="D49" t="n">
-        <v>179</v>
+        <v>189</v>
       </c>
     </row>
     <row r="50">
@@ -1265,7 +1265,7 @@
       </c>
       <c r="C53" t="inlineStr"/>
       <c r="D53" t="n">
-        <v>267</v>
+        <v>264</v>
       </c>
     </row>
     <row r="54">
@@ -1319,7 +1319,7 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>410</v>
+        <v>389</v>
       </c>
     </row>
     <row r="57">
@@ -1355,7 +1355,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>183</v>
+        <v>187</v>
       </c>
     </row>
     <row r="59">
@@ -1387,7 +1387,7 @@
       </c>
       <c r="C60" t="inlineStr"/>
       <c r="D60" t="n">
-        <v>306</v>
+        <v>323</v>
       </c>
     </row>
     <row r="61">
@@ -1401,7 +1401,7 @@
       </c>
       <c r="C61" t="inlineStr"/>
       <c r="D61" t="n">
-        <v>358</v>
+        <v>386</v>
       </c>
     </row>
     <row r="62">
@@ -1469,7 +1469,7 @@
       </c>
       <c r="C65" t="inlineStr"/>
       <c r="D65" t="n">
-        <v>220</v>
+        <v>206</v>
       </c>
     </row>
     <row r="66">
@@ -1513,7 +1513,7 @@
       </c>
       <c r="C68" t="inlineStr"/>
       <c r="D68" t="n">
-        <v>244</v>
+        <v>262</v>
       </c>
     </row>
     <row r="69">
@@ -1544,9 +1544,7 @@
         <v>19865</v>
       </c>
       <c r="C70" t="inlineStr"/>
-      <c r="D70" t="n">
-        <v>492</v>
-      </c>
+      <c r="D70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -1657,7 +1655,7 @@
       </c>
       <c r="C77" t="inlineStr"/>
       <c r="D77" t="n">
-        <v>292</v>
+        <v>324</v>
       </c>
     </row>
     <row r="78">
@@ -1707,7 +1705,7 @@
       </c>
       <c r="C80" t="inlineStr"/>
       <c r="D80" t="n">
-        <v>135</v>
+        <v>149</v>
       </c>
     </row>
     <row r="81">
@@ -1739,7 +1737,7 @@
       </c>
       <c r="C82" t="inlineStr"/>
       <c r="D82" t="n">
-        <v>412</v>
+        <v>449</v>
       </c>
     </row>
     <row r="83">
@@ -1857,7 +1855,7 @@
       </c>
       <c r="C89" t="inlineStr"/>
       <c r="D89" t="n">
-        <v>166</v>
+        <v>148</v>
       </c>
     </row>
     <row r="90">
@@ -1889,7 +1887,7 @@
       </c>
       <c r="C91" t="inlineStr"/>
       <c r="D91" t="n">
-        <v>156</v>
+        <v>114</v>
       </c>
     </row>
     <row r="92">
@@ -1907,7 +1905,7 @@
         </is>
       </c>
       <c r="D92" t="n">
-        <v>138</v>
+        <v>144</v>
       </c>
     </row>
     <row r="93">
@@ -1989,7 +1987,7 @@
       </c>
       <c r="C97" t="inlineStr"/>
       <c r="D97" t="n">
-        <v>130</v>
+        <v>139</v>
       </c>
     </row>
     <row r="98">
@@ -2015,7 +2013,7 @@
       </c>
       <c r="C99" t="inlineStr"/>
       <c r="D99" t="n">
-        <v>287</v>
+        <v>298</v>
       </c>
     </row>
     <row r="100">
@@ -2069,7 +2067,7 @@
         </is>
       </c>
       <c r="D102" t="n">
-        <v>139</v>
+        <v>142</v>
       </c>
     </row>
     <row r="103">
@@ -2131,7 +2129,7 @@
       </c>
       <c r="C106" t="inlineStr"/>
       <c r="D106" t="n">
-        <v>275</v>
+        <v>294</v>
       </c>
     </row>
     <row r="107">
@@ -2193,7 +2191,7 @@
       </c>
       <c r="C110" t="inlineStr"/>
       <c r="D110" t="n">
-        <v>296</v>
+        <v>303</v>
       </c>
     </row>
     <row r="111">
@@ -2225,7 +2223,7 @@
       </c>
       <c r="C112" t="inlineStr"/>
       <c r="D112" t="n">
-        <v>170</v>
+        <v>178</v>
       </c>
     </row>
     <row r="113">
@@ -2337,7 +2335,7 @@
       </c>
       <c r="C120" t="inlineStr"/>
       <c r="D120" t="n">
-        <v>213</v>
+        <v>227</v>
       </c>
     </row>
     <row r="121">
@@ -2413,7 +2411,7 @@
       </c>
       <c r="C125" t="inlineStr"/>
       <c r="D125" t="n">
-        <v>425</v>
+        <v>446</v>
       </c>
     </row>
     <row r="126">
@@ -2539,7 +2537,7 @@
         </is>
       </c>
       <c r="D132" t="n">
-        <v>116</v>
+        <v>103</v>
       </c>
     </row>
     <row r="133">
@@ -2601,7 +2599,7 @@
       </c>
       <c r="C136" t="inlineStr"/>
       <c r="D136" t="n">
-        <v>180</v>
+        <v>190</v>
       </c>
     </row>
     <row r="137">
@@ -2619,7 +2617,7 @@
         </is>
       </c>
       <c r="D137" t="n">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="138">
@@ -2743,7 +2741,7 @@
       </c>
       <c r="C145" t="inlineStr"/>
       <c r="D145" t="n">
-        <v>341</v>
+        <v>357</v>
       </c>
     </row>
     <row r="146">
@@ -2787,7 +2785,7 @@
       </c>
       <c r="C148" t="inlineStr"/>
       <c r="D148" t="n">
-        <v>104</v>
+        <v>110</v>
       </c>
     </row>
     <row r="149">
@@ -2851,7 +2849,7 @@
       </c>
       <c r="C153" t="inlineStr"/>
       <c r="D153" t="n">
-        <v>316</v>
+        <v>328</v>
       </c>
     </row>
     <row r="154">
@@ -2869,7 +2867,7 @@
         </is>
       </c>
       <c r="D154" t="n">
-        <v>236</v>
+        <v>254</v>
       </c>
     </row>
     <row r="155">
@@ -2937,7 +2935,7 @@
       </c>
       <c r="C158" t="inlineStr"/>
       <c r="D158" t="n">
-        <v>242</v>
+        <v>237</v>
       </c>
     </row>
     <row r="159">
@@ -2951,7 +2949,7 @@
       </c>
       <c r="C159" t="inlineStr"/>
       <c r="D159" t="n">
-        <v>160</v>
+        <v>166</v>
       </c>
     </row>
     <row r="160">
@@ -3001,7 +2999,7 @@
       </c>
       <c r="C162" t="inlineStr"/>
       <c r="D162" t="n">
-        <v>175</v>
+        <v>183</v>
       </c>
     </row>
     <row r="163">
@@ -3069,7 +3067,7 @@
       </c>
       <c r="C166" t="inlineStr"/>
       <c r="D166" t="n">
-        <v>149</v>
+        <v>156</v>
       </c>
     </row>
     <row r="167">
@@ -3193,7 +3191,7 @@
       </c>
       <c r="C174" t="inlineStr"/>
       <c r="D174" t="n">
-        <v>140</v>
+        <v>121</v>
       </c>
     </row>
     <row r="175">
@@ -3229,7 +3227,7 @@
         </is>
       </c>
       <c r="D176" t="n">
-        <v>217</v>
+        <v>210</v>
       </c>
     </row>
     <row r="177">
@@ -3391,7 +3389,7 @@
       </c>
       <c r="C186" t="inlineStr"/>
       <c r="D186" t="n">
-        <v>249</v>
+        <v>268</v>
       </c>
     </row>
     <row r="187">
@@ -3423,7 +3421,7 @@
       </c>
       <c r="C188" t="inlineStr"/>
       <c r="D188" t="n">
-        <v>255</v>
+        <v>258</v>
       </c>
     </row>
     <row r="189">
@@ -3539,7 +3537,7 @@
       </c>
       <c r="C195" t="inlineStr"/>
       <c r="D195" t="n">
-        <v>239</v>
+        <v>247</v>
       </c>
     </row>
     <row r="196">
@@ -3607,7 +3605,7 @@
         </is>
       </c>
       <c r="D199" t="n">
-        <v>384</v>
+        <v>409</v>
       </c>
     </row>
     <row r="200">
@@ -3621,7 +3619,7 @@
       </c>
       <c r="C200" t="inlineStr"/>
       <c r="D200" t="n">
-        <v>207</v>
+        <v>208</v>
       </c>
     </row>
     <row r="201">
@@ -3635,7 +3633,7 @@
       </c>
       <c r="C201" t="inlineStr"/>
       <c r="D201" t="n">
-        <v>375</v>
+        <v>392</v>
       </c>
     </row>
     <row r="202">
@@ -3649,7 +3647,7 @@
       </c>
       <c r="C202" t="inlineStr"/>
       <c r="D202" t="n">
-        <v>188</v>
+        <v>202</v>
       </c>
     </row>
     <row r="203">
@@ -3721,7 +3719,7 @@
         </is>
       </c>
       <c r="D206" t="n">
-        <v>120</v>
+        <v>127</v>
       </c>
     </row>
     <row r="207">
@@ -3777,7 +3775,7 @@
       </c>
       <c r="C210" t="inlineStr"/>
       <c r="D210" t="n">
-        <v>319</v>
+        <v>335</v>
       </c>
     </row>
     <row r="211">
@@ -3813,7 +3811,7 @@
         </is>
       </c>
       <c r="D212" t="n">
-        <v>167</v>
+        <v>174</v>
       </c>
     </row>
     <row r="213">
@@ -3857,7 +3855,7 @@
       </c>
       <c r="C215" t="inlineStr"/>
       <c r="D215" t="n">
-        <v>246</v>
+        <v>265</v>
       </c>
     </row>
     <row r="216">
@@ -3871,7 +3869,7 @@
       </c>
       <c r="C216" t="inlineStr"/>
       <c r="D216" t="n">
-        <v>246</v>
+        <v>265</v>
       </c>
     </row>
     <row r="217">
@@ -3889,7 +3887,7 @@
         </is>
       </c>
       <c r="D217" t="n">
-        <v>153</v>
+        <v>164</v>
       </c>
     </row>
     <row r="218">
@@ -3903,7 +3901,7 @@
       </c>
       <c r="C218" t="inlineStr"/>
       <c r="D218" t="n">
-        <v>469</v>
+        <v>468</v>
       </c>
     </row>
     <row r="219">
@@ -3917,7 +3915,7 @@
       </c>
       <c r="C219" t="inlineStr"/>
       <c r="D219" t="n">
-        <v>221</v>
+        <v>223</v>
       </c>
     </row>
     <row r="220">
@@ -3971,7 +3969,7 @@
         </is>
       </c>
       <c r="D222" t="n">
-        <v>127</v>
+        <v>143</v>
       </c>
     </row>
     <row r="223">
@@ -3997,7 +3995,7 @@
       </c>
       <c r="C224" t="inlineStr"/>
       <c r="D224" t="n">
-        <v>400</v>
+        <v>420</v>
       </c>
     </row>
     <row r="225">
@@ -4041,7 +4039,7 @@
       </c>
       <c r="C227" t="inlineStr"/>
       <c r="D227" t="n">
-        <v>343</v>
+        <v>355</v>
       </c>
     </row>
     <row r="228">
@@ -4105,7 +4103,7 @@
       </c>
       <c r="C231" t="inlineStr"/>
       <c r="D231" t="n">
-        <v>168</v>
+        <v>177</v>
       </c>
     </row>
     <row r="232">
@@ -4123,7 +4121,7 @@
         </is>
       </c>
       <c r="D232" t="n">
-        <v>106</v>
+        <v>111</v>
       </c>
     </row>
     <row r="233">

</xml_diff>

<commit_message>
data: field/odds refresh 2026-05-18 10:51 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -557,7 +557,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>92</v>
+        <v>88</v>
       </c>
     </row>
     <row r="9">
@@ -589,7 +589,7 @@
       </c>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="n">
-        <v>256</v>
+        <v>196</v>
       </c>
     </row>
     <row r="11">
@@ -717,7 +717,7 @@
       </c>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="n">
-        <v>466</v>
+        <v>476</v>
       </c>
     </row>
     <row r="19">
@@ -813,7 +813,7 @@
       </c>
       <c r="C24" t="inlineStr"/>
       <c r="D24" t="n">
-        <v>313</v>
+        <v>319</v>
       </c>
     </row>
     <row r="25">
@@ -839,7 +839,7 @@
       </c>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="n">
-        <v>238</v>
+        <v>247</v>
       </c>
     </row>
     <row r="27">
@@ -857,7 +857,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>71</v>
+        <v>75</v>
       </c>
     </row>
     <row r="28">
@@ -875,7 +875,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>116</v>
+        <v>118</v>
       </c>
     </row>
     <row r="29">
@@ -925,7 +925,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="32">
@@ -969,7 +969,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>193</v>
+        <v>196</v>
       </c>
     </row>
     <row r="35">
@@ -987,7 +987,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>246</v>
+        <v>249</v>
       </c>
     </row>
     <row r="36">
@@ -1089,7 +1089,7 @@
       </c>
       <c r="C42" t="inlineStr"/>
       <c r="D42" t="n">
-        <v>285</v>
+        <v>288</v>
       </c>
     </row>
     <row r="43">
@@ -1135,7 +1135,7 @@
       </c>
       <c r="C45" t="inlineStr"/>
       <c r="D45" t="n">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="46">
@@ -1183,7 +1183,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="49">
@@ -1197,7 +1197,7 @@
       </c>
       <c r="C49" t="inlineStr"/>
       <c r="D49" t="n">
-        <v>189</v>
+        <v>193</v>
       </c>
     </row>
     <row r="50">
@@ -1215,7 +1215,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="51">
@@ -1265,7 +1265,7 @@
       </c>
       <c r="C53" t="inlineStr"/>
       <c r="D53" t="n">
-        <v>264</v>
+        <v>270</v>
       </c>
     </row>
     <row r="54">
@@ -1319,7 +1319,7 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="57">
@@ -1355,7 +1355,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="59">
@@ -1387,7 +1387,7 @@
       </c>
       <c r="C60" t="inlineStr"/>
       <c r="D60" t="n">
-        <v>323</v>
+        <v>325</v>
       </c>
     </row>
     <row r="61">
@@ -1401,7 +1401,7 @@
       </c>
       <c r="C61" t="inlineStr"/>
       <c r="D61" t="n">
-        <v>386</v>
+        <v>380</v>
       </c>
     </row>
     <row r="62">
@@ -1437,7 +1437,7 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>70</v>
+        <v>63</v>
       </c>
     </row>
     <row r="64">
@@ -1469,7 +1469,7 @@
       </c>
       <c r="C65" t="inlineStr"/>
       <c r="D65" t="n">
-        <v>206</v>
+        <v>212</v>
       </c>
     </row>
     <row r="66">
@@ -1487,7 +1487,7 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>115</v>
+        <v>117</v>
       </c>
     </row>
     <row r="67">
@@ -1513,7 +1513,7 @@
       </c>
       <c r="C68" t="inlineStr"/>
       <c r="D68" t="n">
-        <v>262</v>
+        <v>256</v>
       </c>
     </row>
     <row r="69">
@@ -1641,7 +1641,7 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>85</v>
+        <v>94</v>
       </c>
     </row>
     <row r="77">
@@ -1655,7 +1655,7 @@
       </c>
       <c r="C77" t="inlineStr"/>
       <c r="D77" t="n">
-        <v>324</v>
+        <v>329</v>
       </c>
     </row>
     <row r="78">
@@ -1673,7 +1673,7 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>151</v>
+        <v>155</v>
       </c>
     </row>
     <row r="79">
@@ -1691,7 +1691,7 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="80">
@@ -1705,7 +1705,7 @@
       </c>
       <c r="C80" t="inlineStr"/>
       <c r="D80" t="n">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="81">
@@ -1723,7 +1723,7 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="82">
@@ -1737,7 +1737,7 @@
       </c>
       <c r="C82" t="inlineStr"/>
       <c r="D82" t="n">
-        <v>449</v>
+        <v>460</v>
       </c>
     </row>
     <row r="83">
@@ -1755,7 +1755,7 @@
         </is>
       </c>
       <c r="D83" t="n">
-        <v>124</v>
+        <v>110</v>
       </c>
     </row>
     <row r="84">
@@ -1791,7 +1791,7 @@
         </is>
       </c>
       <c r="D85" t="n">
-        <v>64</v>
+        <v>67</v>
       </c>
     </row>
     <row r="86">
@@ -1827,7 +1827,7 @@
         </is>
       </c>
       <c r="D87" t="n">
-        <v>117</v>
+        <v>123</v>
       </c>
     </row>
     <row r="88">
@@ -1887,7 +1887,7 @@
       </c>
       <c r="C91" t="inlineStr"/>
       <c r="D91" t="n">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="92">
@@ -1905,7 +1905,7 @@
         </is>
       </c>
       <c r="D92" t="n">
-        <v>144</v>
+        <v>142</v>
       </c>
     </row>
     <row r="93">
@@ -1923,7 +1923,7 @@
         </is>
       </c>
       <c r="D93" t="n">
-        <v>67</v>
+        <v>72</v>
       </c>
     </row>
     <row r="94">
@@ -1941,7 +1941,7 @@
         </is>
       </c>
       <c r="D94" t="n">
-        <v>100</v>
+        <v>93</v>
       </c>
     </row>
     <row r="95">
@@ -2013,7 +2013,7 @@
       </c>
       <c r="C99" t="inlineStr"/>
       <c r="D99" t="n">
-        <v>298</v>
+        <v>291</v>
       </c>
     </row>
     <row r="100">
@@ -2049,7 +2049,7 @@
         </is>
       </c>
       <c r="D101" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="102">
@@ -2067,7 +2067,7 @@
         </is>
       </c>
       <c r="D102" t="n">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="103">
@@ -2085,7 +2085,7 @@
         </is>
       </c>
       <c r="D103" t="n">
-        <v>98</v>
+        <v>96</v>
       </c>
     </row>
     <row r="104">
@@ -2129,7 +2129,7 @@
       </c>
       <c r="C106" t="inlineStr"/>
       <c r="D106" t="n">
-        <v>294</v>
+        <v>300</v>
       </c>
     </row>
     <row r="107">
@@ -2177,7 +2177,7 @@
         </is>
       </c>
       <c r="D109" t="n">
-        <v>125</v>
+        <v>111</v>
       </c>
     </row>
     <row r="110">
@@ -2191,7 +2191,7 @@
       </c>
       <c r="C110" t="inlineStr"/>
       <c r="D110" t="n">
-        <v>303</v>
+        <v>286</v>
       </c>
     </row>
     <row r="111">
@@ -2223,7 +2223,7 @@
       </c>
       <c r="C112" t="inlineStr"/>
       <c r="D112" t="n">
-        <v>178</v>
+        <v>181</v>
       </c>
     </row>
     <row r="113">
@@ -2335,7 +2335,7 @@
       </c>
       <c r="C120" t="inlineStr"/>
       <c r="D120" t="n">
-        <v>227</v>
+        <v>235</v>
       </c>
     </row>
     <row r="121">
@@ -2411,7 +2411,7 @@
       </c>
       <c r="C125" t="inlineStr"/>
       <c r="D125" t="n">
-        <v>446</v>
+        <v>447</v>
       </c>
     </row>
     <row r="126">
@@ -2483,7 +2483,7 @@
         </is>
       </c>
       <c r="D129" t="n">
-        <v>80</v>
+        <v>84</v>
       </c>
     </row>
     <row r="130">
@@ -2537,7 +2537,7 @@
         </is>
       </c>
       <c r="D132" t="n">
-        <v>103</v>
+        <v>105</v>
       </c>
     </row>
     <row r="133">
@@ -2571,7 +2571,7 @@
         </is>
       </c>
       <c r="D134" t="n">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="135">
@@ -2599,7 +2599,7 @@
       </c>
       <c r="C136" t="inlineStr"/>
       <c r="D136" t="n">
-        <v>190</v>
+        <v>195</v>
       </c>
     </row>
     <row r="137">
@@ -2617,7 +2617,7 @@
         </is>
       </c>
       <c r="D137" t="n">
-        <v>150</v>
+        <v>152</v>
       </c>
     </row>
     <row r="138">
@@ -2649,7 +2649,7 @@
       </c>
       <c r="C139" t="inlineStr"/>
       <c r="D139" t="n">
-        <v>132</v>
+        <v>129</v>
       </c>
     </row>
     <row r="140">
@@ -2677,7 +2677,7 @@
       </c>
       <c r="C141" t="inlineStr"/>
       <c r="D141" t="n">
-        <v>77</v>
+        <v>79</v>
       </c>
     </row>
     <row r="142">
@@ -2741,7 +2741,7 @@
       </c>
       <c r="C145" t="inlineStr"/>
       <c r="D145" t="n">
-        <v>357</v>
+        <v>367</v>
       </c>
     </row>
     <row r="146">
@@ -2785,7 +2785,7 @@
       </c>
       <c r="C148" t="inlineStr"/>
       <c r="D148" t="n">
-        <v>110</v>
+        <v>113</v>
       </c>
     </row>
     <row r="149">
@@ -2849,7 +2849,7 @@
       </c>
       <c r="C153" t="inlineStr"/>
       <c r="D153" t="n">
-        <v>328</v>
+        <v>332</v>
       </c>
     </row>
     <row r="154">
@@ -2867,7 +2867,7 @@
         </is>
       </c>
       <c r="D154" t="n">
-        <v>254</v>
+        <v>262</v>
       </c>
     </row>
     <row r="155">
@@ -2885,7 +2885,7 @@
         </is>
       </c>
       <c r="D155" t="n">
-        <v>86</v>
+        <v>82</v>
       </c>
     </row>
     <row r="156">
@@ -2935,7 +2935,7 @@
       </c>
       <c r="C158" t="inlineStr"/>
       <c r="D158" t="n">
-        <v>237</v>
+        <v>221</v>
       </c>
     </row>
     <row r="159">
@@ -2949,7 +2949,7 @@
       </c>
       <c r="C159" t="inlineStr"/>
       <c r="D159" t="n">
-        <v>166</v>
+        <v>168</v>
       </c>
     </row>
     <row r="160">
@@ -2999,7 +2999,7 @@
       </c>
       <c r="C162" t="inlineStr"/>
       <c r="D162" t="n">
-        <v>183</v>
+        <v>189</v>
       </c>
     </row>
     <row r="163">
@@ -3017,7 +3017,7 @@
         </is>
       </c>
       <c r="D163" t="n">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="164">
@@ -3053,7 +3053,7 @@
         </is>
       </c>
       <c r="D165" t="n">
-        <v>44</v>
+        <v>15</v>
       </c>
     </row>
     <row r="166">
@@ -3067,7 +3067,7 @@
       </c>
       <c r="C166" t="inlineStr"/>
       <c r="D166" t="n">
-        <v>156</v>
+        <v>160</v>
       </c>
     </row>
     <row r="167">
@@ -3127,7 +3127,7 @@
         </is>
       </c>
       <c r="D170" t="n">
-        <v>141</v>
+        <v>151</v>
       </c>
     </row>
     <row r="171">
@@ -3145,7 +3145,7 @@
         </is>
       </c>
       <c r="D171" t="n">
-        <v>73</v>
+        <v>76</v>
       </c>
     </row>
     <row r="172">
@@ -3191,7 +3191,7 @@
       </c>
       <c r="C174" t="inlineStr"/>
       <c r="D174" t="n">
-        <v>121</v>
+        <v>125</v>
       </c>
     </row>
     <row r="175">
@@ -3227,7 +3227,7 @@
         </is>
       </c>
       <c r="D176" t="n">
-        <v>210</v>
+        <v>214</v>
       </c>
     </row>
     <row r="177">
@@ -3307,7 +3307,7 @@
         </is>
       </c>
       <c r="D181" t="n">
-        <v>155</v>
+        <v>158</v>
       </c>
     </row>
     <row r="182">
@@ -3325,7 +3325,7 @@
         </is>
       </c>
       <c r="D182" t="n">
-        <v>97</v>
+        <v>65</v>
       </c>
     </row>
     <row r="183">
@@ -3343,7 +3343,7 @@
         </is>
       </c>
       <c r="D183" t="n">
-        <v>97</v>
+        <v>65</v>
       </c>
     </row>
     <row r="184">
@@ -3389,7 +3389,7 @@
       </c>
       <c r="C186" t="inlineStr"/>
       <c r="D186" t="n">
-        <v>268</v>
+        <v>278</v>
       </c>
     </row>
     <row r="187">
@@ -3421,7 +3421,7 @@
       </c>
       <c r="C188" t="inlineStr"/>
       <c r="D188" t="n">
-        <v>258</v>
+        <v>264</v>
       </c>
     </row>
     <row r="189">
@@ -3523,7 +3523,7 @@
         </is>
       </c>
       <c r="D194" t="n">
-        <v>51</v>
+        <v>47</v>
       </c>
     </row>
     <row r="195">
@@ -3537,7 +3537,7 @@
       </c>
       <c r="C195" t="inlineStr"/>
       <c r="D195" t="n">
-        <v>247</v>
+        <v>252</v>
       </c>
     </row>
     <row r="196">
@@ -3605,7 +3605,7 @@
         </is>
       </c>
       <c r="D199" t="n">
-        <v>409</v>
+        <v>416</v>
       </c>
     </row>
     <row r="200">
@@ -3619,7 +3619,7 @@
       </c>
       <c r="C200" t="inlineStr"/>
       <c r="D200" t="n">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="201">
@@ -3633,7 +3633,7 @@
       </c>
       <c r="C201" t="inlineStr"/>
       <c r="D201" t="n">
-        <v>392</v>
+        <v>408</v>
       </c>
     </row>
     <row r="202">
@@ -3647,7 +3647,7 @@
       </c>
       <c r="C202" t="inlineStr"/>
       <c r="D202" t="n">
-        <v>202</v>
+        <v>207</v>
       </c>
     </row>
     <row r="203">
@@ -3719,7 +3719,7 @@
         </is>
       </c>
       <c r="D206" t="n">
-        <v>127</v>
+        <v>128</v>
       </c>
     </row>
     <row r="207">
@@ -3737,7 +3737,7 @@
         </is>
       </c>
       <c r="D207" t="n">
-        <v>63</v>
+        <v>70</v>
       </c>
     </row>
     <row r="208">
@@ -3775,7 +3775,7 @@
       </c>
       <c r="C210" t="inlineStr"/>
       <c r="D210" t="n">
-        <v>335</v>
+        <v>331</v>
       </c>
     </row>
     <row r="211">
@@ -3811,7 +3811,7 @@
         </is>
       </c>
       <c r="D212" t="n">
-        <v>174</v>
+        <v>178</v>
       </c>
     </row>
     <row r="213">
@@ -3829,7 +3829,7 @@
         </is>
       </c>
       <c r="D213" t="n">
-        <v>126</v>
+        <v>122</v>
       </c>
     </row>
     <row r="214">
@@ -3855,7 +3855,7 @@
       </c>
       <c r="C215" t="inlineStr"/>
       <c r="D215" t="n">
-        <v>265</v>
+        <v>268</v>
       </c>
     </row>
     <row r="216">
@@ -3869,7 +3869,7 @@
       </c>
       <c r="C216" t="inlineStr"/>
       <c r="D216" t="n">
-        <v>265</v>
+        <v>268</v>
       </c>
     </row>
     <row r="217">
@@ -3887,7 +3887,7 @@
         </is>
       </c>
       <c r="D217" t="n">
-        <v>164</v>
+        <v>167</v>
       </c>
     </row>
     <row r="218">
@@ -3901,7 +3901,7 @@
       </c>
       <c r="C218" t="inlineStr"/>
       <c r="D218" t="n">
-        <v>468</v>
+        <v>471</v>
       </c>
     </row>
     <row r="219">
@@ -3915,7 +3915,7 @@
       </c>
       <c r="C219" t="inlineStr"/>
       <c r="D219" t="n">
-        <v>223</v>
+        <v>226</v>
       </c>
     </row>
     <row r="220">
@@ -3969,7 +3969,7 @@
         </is>
       </c>
       <c r="D222" t="n">
-        <v>143</v>
+        <v>144</v>
       </c>
     </row>
     <row r="223">
@@ -3995,7 +3995,7 @@
       </c>
       <c r="C224" t="inlineStr"/>
       <c r="D224" t="n">
-        <v>420</v>
+        <v>426</v>
       </c>
     </row>
     <row r="225">
@@ -4039,7 +4039,7 @@
       </c>
       <c r="C227" t="inlineStr"/>
       <c r="D227" t="n">
-        <v>355</v>
+        <v>359</v>
       </c>
     </row>
     <row r="228">
@@ -4103,7 +4103,7 @@
       </c>
       <c r="C231" t="inlineStr"/>
       <c r="D231" t="n">
-        <v>177</v>
+        <v>169</v>
       </c>
     </row>
     <row r="232">
@@ -4121,7 +4121,7 @@
         </is>
       </c>
       <c r="D232" t="n">
-        <v>111</v>
+        <v>114</v>
       </c>
     </row>
     <row r="233">

</xml_diff>

<commit_message>
data: field/odds refresh 2026-05-18 12:58 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -557,7 +557,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>92</v>
+        <v>88</v>
       </c>
     </row>
     <row r="9">
@@ -589,7 +589,7 @@
       </c>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="n">
-        <v>256</v>
+        <v>196</v>
       </c>
     </row>
     <row r="11">
@@ -717,7 +717,7 @@
       </c>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="n">
-        <v>466</v>
+        <v>476</v>
       </c>
     </row>
     <row r="19">
@@ -813,7 +813,7 @@
       </c>
       <c r="C24" t="inlineStr"/>
       <c r="D24" t="n">
-        <v>313</v>
+        <v>319</v>
       </c>
     </row>
     <row r="25">
@@ -839,7 +839,7 @@
       </c>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="n">
-        <v>238</v>
+        <v>247</v>
       </c>
     </row>
     <row r="27">
@@ -857,7 +857,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>71</v>
+        <v>75</v>
       </c>
     </row>
     <row r="28">
@@ -875,7 +875,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>116</v>
+        <v>118</v>
       </c>
     </row>
     <row r="29">
@@ -925,7 +925,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="32">
@@ -969,7 +969,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>193</v>
+        <v>196</v>
       </c>
     </row>
     <row r="35">
@@ -987,7 +987,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>246</v>
+        <v>249</v>
       </c>
     </row>
     <row r="36">
@@ -1089,7 +1089,7 @@
       </c>
       <c r="C42" t="inlineStr"/>
       <c r="D42" t="n">
-        <v>285</v>
+        <v>288</v>
       </c>
     </row>
     <row r="43">
@@ -1135,7 +1135,7 @@
       </c>
       <c r="C45" t="inlineStr"/>
       <c r="D45" t="n">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="46">
@@ -1183,7 +1183,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="49">
@@ -1197,7 +1197,7 @@
       </c>
       <c r="C49" t="inlineStr"/>
       <c r="D49" t="n">
-        <v>189</v>
+        <v>193</v>
       </c>
     </row>
     <row r="50">
@@ -1215,7 +1215,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="51">
@@ -1265,7 +1265,7 @@
       </c>
       <c r="C53" t="inlineStr"/>
       <c r="D53" t="n">
-        <v>264</v>
+        <v>270</v>
       </c>
     </row>
     <row r="54">
@@ -1319,7 +1319,7 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="57">
@@ -1355,7 +1355,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="59">
@@ -1387,7 +1387,7 @@
       </c>
       <c r="C60" t="inlineStr"/>
       <c r="D60" t="n">
-        <v>323</v>
+        <v>325</v>
       </c>
     </row>
     <row r="61">
@@ -1401,7 +1401,7 @@
       </c>
       <c r="C61" t="inlineStr"/>
       <c r="D61" t="n">
-        <v>386</v>
+        <v>380</v>
       </c>
     </row>
     <row r="62">
@@ -1437,7 +1437,7 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>70</v>
+        <v>63</v>
       </c>
     </row>
     <row r="64">
@@ -1469,7 +1469,7 @@
       </c>
       <c r="C65" t="inlineStr"/>
       <c r="D65" t="n">
-        <v>206</v>
+        <v>212</v>
       </c>
     </row>
     <row r="66">
@@ -1487,7 +1487,7 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>115</v>
+        <v>117</v>
       </c>
     </row>
     <row r="67">
@@ -1513,7 +1513,7 @@
       </c>
       <c r="C68" t="inlineStr"/>
       <c r="D68" t="n">
-        <v>262</v>
+        <v>256</v>
       </c>
     </row>
     <row r="69">
@@ -1641,7 +1641,7 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>85</v>
+        <v>94</v>
       </c>
     </row>
     <row r="77">
@@ -1655,7 +1655,7 @@
       </c>
       <c r="C77" t="inlineStr"/>
       <c r="D77" t="n">
-        <v>324</v>
+        <v>329</v>
       </c>
     </row>
     <row r="78">
@@ -1673,7 +1673,7 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>151</v>
+        <v>155</v>
       </c>
     </row>
     <row r="79">
@@ -1691,7 +1691,7 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="80">
@@ -1705,7 +1705,7 @@
       </c>
       <c r="C80" t="inlineStr"/>
       <c r="D80" t="n">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="81">
@@ -1723,7 +1723,7 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="82">
@@ -1737,7 +1737,7 @@
       </c>
       <c r="C82" t="inlineStr"/>
       <c r="D82" t="n">
-        <v>449</v>
+        <v>460</v>
       </c>
     </row>
     <row r="83">
@@ -1755,7 +1755,7 @@
         </is>
       </c>
       <c r="D83" t="n">
-        <v>124</v>
+        <v>110</v>
       </c>
     </row>
     <row r="84">
@@ -1791,7 +1791,7 @@
         </is>
       </c>
       <c r="D85" t="n">
-        <v>64</v>
+        <v>67</v>
       </c>
     </row>
     <row r="86">
@@ -1827,7 +1827,7 @@
         </is>
       </c>
       <c r="D87" t="n">
-        <v>117</v>
+        <v>123</v>
       </c>
     </row>
     <row r="88">
@@ -1887,7 +1887,7 @@
       </c>
       <c r="C91" t="inlineStr"/>
       <c r="D91" t="n">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="92">
@@ -1905,7 +1905,7 @@
         </is>
       </c>
       <c r="D92" t="n">
-        <v>144</v>
+        <v>142</v>
       </c>
     </row>
     <row r="93">
@@ -1923,7 +1923,7 @@
         </is>
       </c>
       <c r="D93" t="n">
-        <v>67</v>
+        <v>72</v>
       </c>
     </row>
     <row r="94">
@@ -1941,7 +1941,7 @@
         </is>
       </c>
       <c r="D94" t="n">
-        <v>100</v>
+        <v>93</v>
       </c>
     </row>
     <row r="95">
@@ -2013,7 +2013,7 @@
       </c>
       <c r="C99" t="inlineStr"/>
       <c r="D99" t="n">
-        <v>298</v>
+        <v>291</v>
       </c>
     </row>
     <row r="100">
@@ -2049,7 +2049,7 @@
         </is>
       </c>
       <c r="D101" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="102">
@@ -2067,7 +2067,7 @@
         </is>
       </c>
       <c r="D102" t="n">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="103">
@@ -2085,7 +2085,7 @@
         </is>
       </c>
       <c r="D103" t="n">
-        <v>98</v>
+        <v>96</v>
       </c>
     </row>
     <row r="104">
@@ -2129,7 +2129,7 @@
       </c>
       <c r="C106" t="inlineStr"/>
       <c r="D106" t="n">
-        <v>294</v>
+        <v>300</v>
       </c>
     </row>
     <row r="107">
@@ -2177,7 +2177,7 @@
         </is>
       </c>
       <c r="D109" t="n">
-        <v>125</v>
+        <v>111</v>
       </c>
     </row>
     <row r="110">
@@ -2191,7 +2191,7 @@
       </c>
       <c r="C110" t="inlineStr"/>
       <c r="D110" t="n">
-        <v>303</v>
+        <v>286</v>
       </c>
     </row>
     <row r="111">
@@ -2223,7 +2223,7 @@
       </c>
       <c r="C112" t="inlineStr"/>
       <c r="D112" t="n">
-        <v>178</v>
+        <v>181</v>
       </c>
     </row>
     <row r="113">
@@ -2335,7 +2335,7 @@
       </c>
       <c r="C120" t="inlineStr"/>
       <c r="D120" t="n">
-        <v>227</v>
+        <v>235</v>
       </c>
     </row>
     <row r="121">
@@ -2411,7 +2411,7 @@
       </c>
       <c r="C125" t="inlineStr"/>
       <c r="D125" t="n">
-        <v>446</v>
+        <v>447</v>
       </c>
     </row>
     <row r="126">
@@ -2483,7 +2483,7 @@
         </is>
       </c>
       <c r="D129" t="n">
-        <v>80</v>
+        <v>84</v>
       </c>
     </row>
     <row r="130">
@@ -2537,7 +2537,7 @@
         </is>
       </c>
       <c r="D132" t="n">
-        <v>103</v>
+        <v>105</v>
       </c>
     </row>
     <row r="133">
@@ -2571,7 +2571,7 @@
         </is>
       </c>
       <c r="D134" t="n">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="135">
@@ -2599,7 +2599,7 @@
       </c>
       <c r="C136" t="inlineStr"/>
       <c r="D136" t="n">
-        <v>190</v>
+        <v>195</v>
       </c>
     </row>
     <row r="137">
@@ -2617,7 +2617,7 @@
         </is>
       </c>
       <c r="D137" t="n">
-        <v>150</v>
+        <v>152</v>
       </c>
     </row>
     <row r="138">
@@ -2649,7 +2649,7 @@
       </c>
       <c r="C139" t="inlineStr"/>
       <c r="D139" t="n">
-        <v>132</v>
+        <v>129</v>
       </c>
     </row>
     <row r="140">
@@ -2677,7 +2677,7 @@
       </c>
       <c r="C141" t="inlineStr"/>
       <c r="D141" t="n">
-        <v>77</v>
+        <v>79</v>
       </c>
     </row>
     <row r="142">
@@ -2741,7 +2741,7 @@
       </c>
       <c r="C145" t="inlineStr"/>
       <c r="D145" t="n">
-        <v>357</v>
+        <v>367</v>
       </c>
     </row>
     <row r="146">
@@ -2785,7 +2785,7 @@
       </c>
       <c r="C148" t="inlineStr"/>
       <c r="D148" t="n">
-        <v>110</v>
+        <v>113</v>
       </c>
     </row>
     <row r="149">
@@ -2849,7 +2849,7 @@
       </c>
       <c r="C153" t="inlineStr"/>
       <c r="D153" t="n">
-        <v>328</v>
+        <v>332</v>
       </c>
     </row>
     <row r="154">
@@ -2867,7 +2867,7 @@
         </is>
       </c>
       <c r="D154" t="n">
-        <v>254</v>
+        <v>262</v>
       </c>
     </row>
     <row r="155">
@@ -2885,7 +2885,7 @@
         </is>
       </c>
       <c r="D155" t="n">
-        <v>86</v>
+        <v>82</v>
       </c>
     </row>
     <row r="156">
@@ -2935,7 +2935,7 @@
       </c>
       <c r="C158" t="inlineStr"/>
       <c r="D158" t="n">
-        <v>237</v>
+        <v>221</v>
       </c>
     </row>
     <row r="159">
@@ -2949,7 +2949,7 @@
       </c>
       <c r="C159" t="inlineStr"/>
       <c r="D159" t="n">
-        <v>166</v>
+        <v>168</v>
       </c>
     </row>
     <row r="160">
@@ -2999,7 +2999,7 @@
       </c>
       <c r="C162" t="inlineStr"/>
       <c r="D162" t="n">
-        <v>183</v>
+        <v>189</v>
       </c>
     </row>
     <row r="163">
@@ -3067,7 +3067,7 @@
       </c>
       <c r="C166" t="inlineStr"/>
       <c r="D166" t="n">
-        <v>156</v>
+        <v>160</v>
       </c>
     </row>
     <row r="167">
@@ -3127,7 +3127,7 @@
         </is>
       </c>
       <c r="D170" t="n">
-        <v>141</v>
+        <v>151</v>
       </c>
     </row>
     <row r="171">
@@ -3145,7 +3145,7 @@
         </is>
       </c>
       <c r="D171" t="n">
-        <v>73</v>
+        <v>76</v>
       </c>
     </row>
     <row r="172">
@@ -3191,7 +3191,7 @@
       </c>
       <c r="C174" t="inlineStr"/>
       <c r="D174" t="n">
-        <v>121</v>
+        <v>125</v>
       </c>
     </row>
     <row r="175">
@@ -3227,7 +3227,7 @@
         </is>
       </c>
       <c r="D176" t="n">
-        <v>210</v>
+        <v>214</v>
       </c>
     </row>
     <row r="177">
@@ -3307,7 +3307,7 @@
         </is>
       </c>
       <c r="D181" t="n">
-        <v>155</v>
+        <v>158</v>
       </c>
     </row>
     <row r="182">
@@ -3325,7 +3325,7 @@
         </is>
       </c>
       <c r="D182" t="n">
-        <v>97</v>
+        <v>65</v>
       </c>
     </row>
     <row r="183">
@@ -3343,7 +3343,7 @@
         </is>
       </c>
       <c r="D183" t="n">
-        <v>97</v>
+        <v>65</v>
       </c>
     </row>
     <row r="184">
@@ -3389,7 +3389,7 @@
       </c>
       <c r="C186" t="inlineStr"/>
       <c r="D186" t="n">
-        <v>268</v>
+        <v>278</v>
       </c>
     </row>
     <row r="187">
@@ -3421,7 +3421,7 @@
       </c>
       <c r="C188" t="inlineStr"/>
       <c r="D188" t="n">
-        <v>258</v>
+        <v>264</v>
       </c>
     </row>
     <row r="189">
@@ -3523,7 +3523,7 @@
         </is>
       </c>
       <c r="D194" t="n">
-        <v>51</v>
+        <v>47</v>
       </c>
     </row>
     <row r="195">
@@ -3537,7 +3537,7 @@
       </c>
       <c r="C195" t="inlineStr"/>
       <c r="D195" t="n">
-        <v>247</v>
+        <v>252</v>
       </c>
     </row>
     <row r="196">
@@ -3605,7 +3605,7 @@
         </is>
       </c>
       <c r="D199" t="n">
-        <v>409</v>
+        <v>416</v>
       </c>
     </row>
     <row r="200">
@@ -3619,7 +3619,7 @@
       </c>
       <c r="C200" t="inlineStr"/>
       <c r="D200" t="n">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="201">
@@ -3633,7 +3633,7 @@
       </c>
       <c r="C201" t="inlineStr"/>
       <c r="D201" t="n">
-        <v>392</v>
+        <v>408</v>
       </c>
     </row>
     <row r="202">
@@ -3647,7 +3647,7 @@
       </c>
       <c r="C202" t="inlineStr"/>
       <c r="D202" t="n">
-        <v>202</v>
+        <v>207</v>
       </c>
     </row>
     <row r="203">
@@ -3719,7 +3719,7 @@
         </is>
       </c>
       <c r="D206" t="n">
-        <v>127</v>
+        <v>128</v>
       </c>
     </row>
     <row r="207">
@@ -3737,7 +3737,7 @@
         </is>
       </c>
       <c r="D207" t="n">
-        <v>63</v>
+        <v>70</v>
       </c>
     </row>
     <row r="208">
@@ -3775,7 +3775,7 @@
       </c>
       <c r="C210" t="inlineStr"/>
       <c r="D210" t="n">
-        <v>335</v>
+        <v>331</v>
       </c>
     </row>
     <row r="211">
@@ -3811,7 +3811,7 @@
         </is>
       </c>
       <c r="D212" t="n">
-        <v>174</v>
+        <v>178</v>
       </c>
     </row>
     <row r="213">
@@ -3829,7 +3829,7 @@
         </is>
       </c>
       <c r="D213" t="n">
-        <v>126</v>
+        <v>122</v>
       </c>
     </row>
     <row r="214">
@@ -3855,7 +3855,7 @@
       </c>
       <c r="C215" t="inlineStr"/>
       <c r="D215" t="n">
-        <v>265</v>
+        <v>268</v>
       </c>
     </row>
     <row r="216">
@@ -3869,7 +3869,7 @@
       </c>
       <c r="C216" t="inlineStr"/>
       <c r="D216" t="n">
-        <v>265</v>
+        <v>268</v>
       </c>
     </row>
     <row r="217">
@@ -3887,7 +3887,7 @@
         </is>
       </c>
       <c r="D217" t="n">
-        <v>164</v>
+        <v>167</v>
       </c>
     </row>
     <row r="218">
@@ -3901,7 +3901,7 @@
       </c>
       <c r="C218" t="inlineStr"/>
       <c r="D218" t="n">
-        <v>468</v>
+        <v>471</v>
       </c>
     </row>
     <row r="219">
@@ -3915,7 +3915,7 @@
       </c>
       <c r="C219" t="inlineStr"/>
       <c r="D219" t="n">
-        <v>223</v>
+        <v>226</v>
       </c>
     </row>
     <row r="220">
@@ -3969,7 +3969,7 @@
         </is>
       </c>
       <c r="D222" t="n">
-        <v>143</v>
+        <v>144</v>
       </c>
     </row>
     <row r="223">
@@ -3995,7 +3995,7 @@
       </c>
       <c r="C224" t="inlineStr"/>
       <c r="D224" t="n">
-        <v>420</v>
+        <v>426</v>
       </c>
     </row>
     <row r="225">
@@ -4039,7 +4039,7 @@
       </c>
       <c r="C227" t="inlineStr"/>
       <c r="D227" t="n">
-        <v>355</v>
+        <v>359</v>
       </c>
     </row>
     <row r="228">
@@ -4103,7 +4103,7 @@
       </c>
       <c r="C231" t="inlineStr"/>
       <c r="D231" t="n">
-        <v>177</v>
+        <v>169</v>
       </c>
     </row>
     <row r="232">
@@ -4121,7 +4121,7 @@
         </is>
       </c>
       <c r="D232" t="n">
-        <v>111</v>
+        <v>114</v>
       </c>
     </row>
     <row r="233">

</xml_diff>

<commit_message>
data: field/odds refresh 2026-05-25 06:21 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -465,7 +465,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3">
@@ -575,7 +575,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>23</v>
+        <v>26</v>
       </c>
     </row>
     <row r="10">
@@ -607,7 +607,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>32</v>
+        <v>36</v>
       </c>
     </row>
     <row r="12">
@@ -781,7 +781,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="23">
@@ -1107,7 +1107,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="44">
@@ -1121,7 +1121,7 @@
       </c>
       <c r="C44" t="inlineStr"/>
       <c r="D44" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="45">
@@ -1283,7 +1283,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="55">
@@ -1337,7 +1337,7 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="58">
@@ -1373,7 +1373,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>93</v>
+        <v>97</v>
       </c>
     </row>
     <row r="60">
@@ -1455,7 +1455,7 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="65">
@@ -1531,7 +1531,7 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>57</v>
+        <v>61</v>
       </c>
     </row>
     <row r="70">
@@ -1561,7 +1561,7 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="72">
@@ -1623,7 +1623,7 @@
         </is>
       </c>
       <c r="D75" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="76">
@@ -1809,7 +1809,7 @@
         </is>
       </c>
       <c r="D86" t="n">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="87">
@@ -2309,7 +2309,7 @@
         </is>
       </c>
       <c r="D118" t="n">
-        <v>91</v>
+        <v>95</v>
       </c>
     </row>
     <row r="119">
@@ -2371,7 +2371,7 @@
         </is>
       </c>
       <c r="D122" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="123">
@@ -2429,7 +2429,7 @@
         </is>
       </c>
       <c r="D126" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="127">
@@ -2465,7 +2465,7 @@
         </is>
       </c>
       <c r="D128" t="n">
-        <v>43</v>
+        <v>46</v>
       </c>
     </row>
     <row r="129">
@@ -2771,7 +2771,7 @@
         </is>
       </c>
       <c r="D147" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="148">
@@ -2967,7 +2967,7 @@
         </is>
       </c>
       <c r="D160" t="n">
-        <v>79</v>
+        <v>85</v>
       </c>
     </row>
     <row r="161">
@@ -3439,7 +3439,7 @@
         </is>
       </c>
       <c r="D189" t="n">
-        <v>78</v>
+        <v>42</v>
       </c>
     </row>
     <row r="190">
@@ -3487,7 +3487,7 @@
       </c>
       <c r="C192" t="inlineStr"/>
       <c r="D192" t="n">
-        <v>131</v>
+        <v>134</v>
       </c>
     </row>
     <row r="193">
@@ -3505,7 +3505,7 @@
         </is>
       </c>
       <c r="D193" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="194">
@@ -3555,7 +3555,7 @@
         </is>
       </c>
       <c r="D196" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="197">
@@ -3569,7 +3569,7 @@
       </c>
       <c r="C197" t="inlineStr"/>
       <c r="D197" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="198">
@@ -3683,7 +3683,7 @@
         </is>
       </c>
       <c r="D204" t="n">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="205">
@@ -4025,7 +4025,7 @@
         </is>
       </c>
       <c r="D226" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="227">
@@ -4071,7 +4071,7 @@
         </is>
       </c>
       <c r="D229" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="230">

</xml_diff>

<commit_message>
data: field/odds refresh 2026-05-25 10:31 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -557,7 +557,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>88</v>
+        <v>91</v>
       </c>
     </row>
     <row r="9">
@@ -589,7 +589,7 @@
       </c>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="n">
-        <v>196</v>
+        <v>199</v>
       </c>
     </row>
     <row r="11">
@@ -607,7 +607,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="12">
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>104</v>
+        <v>111</v>
       </c>
     </row>
     <row r="18">
@@ -781,7 +781,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="23">
@@ -799,7 +799,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="24">
@@ -839,7 +839,7 @@
       </c>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="n">
-        <v>247</v>
+        <v>238</v>
       </c>
     </row>
     <row r="27">
@@ -857,7 +857,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>75</v>
+        <v>44</v>
       </c>
     </row>
     <row r="28">
@@ -875,7 +875,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="29">
@@ -925,7 +925,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="32">
@@ -969,7 +969,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>196</v>
+        <v>202</v>
       </c>
     </row>
     <row r="35">
@@ -987,7 +987,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>249</v>
+        <v>262</v>
       </c>
     </row>
     <row r="36">
@@ -1089,7 +1089,7 @@
       </c>
       <c r="C42" t="inlineStr"/>
       <c r="D42" t="n">
-        <v>288</v>
+        <v>308</v>
       </c>
     </row>
     <row r="43">
@@ -1107,7 +1107,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="44">
@@ -1121,7 +1121,7 @@
       </c>
       <c r="C44" t="inlineStr"/>
       <c r="D44" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="45">
@@ -1135,7 +1135,7 @@
       </c>
       <c r="C45" t="inlineStr"/>
       <c r="D45" t="n">
-        <v>166</v>
+        <v>171</v>
       </c>
     </row>
     <row r="46">
@@ -1183,7 +1183,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>120</v>
+        <v>103</v>
       </c>
     </row>
     <row r="49">
@@ -1215,7 +1215,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>135</v>
+        <v>132</v>
       </c>
     </row>
     <row r="51">
@@ -1319,7 +1319,7 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>388</v>
+        <v>407</v>
       </c>
     </row>
     <row r="57">
@@ -1355,7 +1355,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="59">
@@ -1373,7 +1373,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="60">
@@ -1437,7 +1437,7 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="64">
@@ -1487,7 +1487,7 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="67">
@@ -1531,7 +1531,7 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="70">
@@ -1623,7 +1623,7 @@
         </is>
       </c>
       <c r="D75" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="76">
@@ -1641,7 +1641,7 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>94</v>
+        <v>90</v>
       </c>
     </row>
     <row r="77">
@@ -1673,7 +1673,7 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>155</v>
+        <v>160</v>
       </c>
     </row>
     <row r="79">
@@ -1691,7 +1691,7 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="80">
@@ -1705,7 +1705,7 @@
       </c>
       <c r="C80" t="inlineStr"/>
       <c r="D80" t="n">
-        <v>150</v>
+        <v>153</v>
       </c>
     </row>
     <row r="81">
@@ -1723,7 +1723,7 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>89</v>
+        <v>83</v>
       </c>
     </row>
     <row r="82">
@@ -1737,7 +1737,7 @@
       </c>
       <c r="C82" t="inlineStr"/>
       <c r="D82" t="n">
-        <v>460</v>
+        <v>458</v>
       </c>
     </row>
     <row r="83">
@@ -1755,7 +1755,7 @@
         </is>
       </c>
       <c r="D83" t="n">
-        <v>110</v>
+        <v>100</v>
       </c>
     </row>
     <row r="84">
@@ -1791,7 +1791,7 @@
         </is>
       </c>
       <c r="D85" t="n">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="86">
@@ -1809,7 +1809,7 @@
         </is>
       </c>
       <c r="D86" t="n">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="87">
@@ -1827,7 +1827,7 @@
         </is>
       </c>
       <c r="D87" t="n">
-        <v>123</v>
+        <v>130</v>
       </c>
     </row>
     <row r="88">
@@ -1855,7 +1855,7 @@
       </c>
       <c r="C89" t="inlineStr"/>
       <c r="D89" t="n">
-        <v>148</v>
+        <v>151</v>
       </c>
     </row>
     <row r="90">
@@ -1887,7 +1887,7 @@
       </c>
       <c r="C91" t="inlineStr"/>
       <c r="D91" t="n">
-        <v>116</v>
+        <v>114</v>
       </c>
     </row>
     <row r="92">
@@ -1905,7 +1905,7 @@
         </is>
       </c>
       <c r="D92" t="n">
-        <v>142</v>
+        <v>152</v>
       </c>
     </row>
     <row r="93">
@@ -1923,7 +1923,7 @@
         </is>
       </c>
       <c r="D93" t="n">
-        <v>72</v>
+        <v>68</v>
       </c>
     </row>
     <row r="94">
@@ -1941,7 +1941,7 @@
         </is>
       </c>
       <c r="D94" t="n">
-        <v>93</v>
+        <v>84</v>
       </c>
     </row>
     <row r="95">
@@ -1987,7 +1987,7 @@
       </c>
       <c r="C97" t="inlineStr"/>
       <c r="D97" t="n">
-        <v>139</v>
+        <v>145</v>
       </c>
     </row>
     <row r="98">
@@ -2031,7 +2031,7 @@
         </is>
       </c>
       <c r="D100" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
     </row>
     <row r="101">
@@ -2067,7 +2067,7 @@
         </is>
       </c>
       <c r="D102" t="n">
-        <v>141</v>
+        <v>144</v>
       </c>
     </row>
     <row r="103">
@@ -2129,7 +2129,7 @@
       </c>
       <c r="C106" t="inlineStr"/>
       <c r="D106" t="n">
-        <v>300</v>
+        <v>320</v>
       </c>
     </row>
     <row r="107">
@@ -2223,7 +2223,7 @@
       </c>
       <c r="C112" t="inlineStr"/>
       <c r="D112" t="n">
-        <v>181</v>
+        <v>189</v>
       </c>
     </row>
     <row r="113">
@@ -2309,7 +2309,7 @@
         </is>
       </c>
       <c r="D118" t="n">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="119">
@@ -2371,7 +2371,7 @@
         </is>
       </c>
       <c r="D122" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="123">
@@ -2411,7 +2411,7 @@
       </c>
       <c r="C125" t="inlineStr"/>
       <c r="D125" t="n">
-        <v>447</v>
+        <v>454</v>
       </c>
     </row>
     <row r="126">
@@ -2429,7 +2429,7 @@
         </is>
       </c>
       <c r="D126" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="127">
@@ -2465,7 +2465,7 @@
         </is>
       </c>
       <c r="D128" t="n">
-        <v>46</v>
+        <v>49</v>
       </c>
     </row>
     <row r="129">
@@ -2483,7 +2483,7 @@
         </is>
       </c>
       <c r="D129" t="n">
-        <v>84</v>
+        <v>88</v>
       </c>
     </row>
     <row r="130">
@@ -2537,7 +2537,7 @@
         </is>
       </c>
       <c r="D132" t="n">
-        <v>105</v>
+        <v>108</v>
       </c>
     </row>
     <row r="133">
@@ -2571,7 +2571,7 @@
         </is>
       </c>
       <c r="D134" t="n">
-        <v>108</v>
+        <v>95</v>
       </c>
     </row>
     <row r="135">
@@ -2617,7 +2617,7 @@
         </is>
       </c>
       <c r="D137" t="n">
-        <v>152</v>
+        <v>140</v>
       </c>
     </row>
     <row r="138">
@@ -2649,7 +2649,7 @@
       </c>
       <c r="C139" t="inlineStr"/>
       <c r="D139" t="n">
-        <v>129</v>
+        <v>136</v>
       </c>
     </row>
     <row r="140">
@@ -2677,7 +2677,7 @@
       </c>
       <c r="C141" t="inlineStr"/>
       <c r="D141" t="n">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="142">
@@ -2771,7 +2771,7 @@
         </is>
       </c>
       <c r="D147" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="148">
@@ -2785,7 +2785,7 @@
       </c>
       <c r="C148" t="inlineStr"/>
       <c r="D148" t="n">
-        <v>113</v>
+        <v>121</v>
       </c>
     </row>
     <row r="149">
@@ -2867,7 +2867,7 @@
         </is>
       </c>
       <c r="D154" t="n">
-        <v>262</v>
+        <v>260</v>
       </c>
     </row>
     <row r="155">
@@ -2935,7 +2935,7 @@
       </c>
       <c r="C158" t="inlineStr"/>
       <c r="D158" t="n">
-        <v>221</v>
+        <v>226</v>
       </c>
     </row>
     <row r="159">
@@ -2949,7 +2949,7 @@
       </c>
       <c r="C159" t="inlineStr"/>
       <c r="D159" t="n">
-        <v>168</v>
+        <v>174</v>
       </c>
     </row>
     <row r="160">
@@ -2999,7 +2999,7 @@
       </c>
       <c r="C162" t="inlineStr"/>
       <c r="D162" t="n">
-        <v>189</v>
+        <v>184</v>
       </c>
     </row>
     <row r="163">
@@ -3067,7 +3067,7 @@
       </c>
       <c r="C166" t="inlineStr"/>
       <c r="D166" t="n">
-        <v>160</v>
+        <v>163</v>
       </c>
     </row>
     <row r="167">
@@ -3127,7 +3127,7 @@
         </is>
       </c>
       <c r="D170" t="n">
-        <v>151</v>
+        <v>154</v>
       </c>
     </row>
     <row r="171">
@@ -3145,7 +3145,7 @@
         </is>
       </c>
       <c r="D171" t="n">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="172">
@@ -3227,7 +3227,7 @@
         </is>
       </c>
       <c r="D176" t="n">
-        <v>214</v>
+        <v>211</v>
       </c>
     </row>
     <row r="177">
@@ -3307,7 +3307,7 @@
         </is>
       </c>
       <c r="D181" t="n">
-        <v>158</v>
+        <v>164</v>
       </c>
     </row>
     <row r="182">
@@ -3421,7 +3421,7 @@
       </c>
       <c r="C188" t="inlineStr"/>
       <c r="D188" t="n">
-        <v>264</v>
+        <v>268</v>
       </c>
     </row>
     <row r="189">
@@ -3439,7 +3439,7 @@
         </is>
       </c>
       <c r="D189" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="190">
@@ -3487,7 +3487,7 @@
       </c>
       <c r="C192" t="inlineStr"/>
       <c r="D192" t="n">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="193">
@@ -3537,7 +3537,7 @@
       </c>
       <c r="C195" t="inlineStr"/>
       <c r="D195" t="n">
-        <v>252</v>
+        <v>259</v>
       </c>
     </row>
     <row r="196">
@@ -3555,7 +3555,7 @@
         </is>
       </c>
       <c r="D196" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="197">
@@ -3569,7 +3569,7 @@
       </c>
       <c r="C197" t="inlineStr"/>
       <c r="D197" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="198">
@@ -3605,7 +3605,7 @@
         </is>
       </c>
       <c r="D199" t="n">
-        <v>416</v>
+        <v>425</v>
       </c>
     </row>
     <row r="200">
@@ -3619,7 +3619,7 @@
       </c>
       <c r="C200" t="inlineStr"/>
       <c r="D200" t="n">
-        <v>209</v>
+        <v>166</v>
       </c>
     </row>
     <row r="201">
@@ -3633,7 +3633,7 @@
       </c>
       <c r="C201" t="inlineStr"/>
       <c r="D201" t="n">
-        <v>408</v>
+        <v>403</v>
       </c>
     </row>
     <row r="202">
@@ -3683,7 +3683,7 @@
         </is>
       </c>
       <c r="D204" t="n">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="205">
@@ -3719,7 +3719,7 @@
         </is>
       </c>
       <c r="D206" t="n">
-        <v>128</v>
+        <v>137</v>
       </c>
     </row>
     <row r="207">
@@ -3737,7 +3737,7 @@
         </is>
       </c>
       <c r="D207" t="n">
-        <v>70</v>
+        <v>75</v>
       </c>
     </row>
     <row r="208">
@@ -3775,7 +3775,7 @@
       </c>
       <c r="C210" t="inlineStr"/>
       <c r="D210" t="n">
-        <v>331</v>
+        <v>344</v>
       </c>
     </row>
     <row r="211">
@@ -3811,7 +3811,7 @@
         </is>
       </c>
       <c r="D212" t="n">
-        <v>178</v>
+        <v>175</v>
       </c>
     </row>
     <row r="213">
@@ -3855,7 +3855,7 @@
       </c>
       <c r="C215" t="inlineStr"/>
       <c r="D215" t="n">
-        <v>268</v>
+        <v>276</v>
       </c>
     </row>
     <row r="216">
@@ -3869,7 +3869,7 @@
       </c>
       <c r="C216" t="inlineStr"/>
       <c r="D216" t="n">
-        <v>268</v>
+        <v>276</v>
       </c>
     </row>
     <row r="217">
@@ -3887,7 +3887,7 @@
         </is>
       </c>
       <c r="D217" t="n">
-        <v>167</v>
+        <v>176</v>
       </c>
     </row>
     <row r="218">
@@ -3901,7 +3901,7 @@
       </c>
       <c r="C218" t="inlineStr"/>
       <c r="D218" t="n">
-        <v>471</v>
+        <v>453</v>
       </c>
     </row>
     <row r="219">
@@ -3915,7 +3915,7 @@
       </c>
       <c r="C219" t="inlineStr"/>
       <c r="D219" t="n">
-        <v>226</v>
+        <v>230</v>
       </c>
     </row>
     <row r="220">
@@ -3969,7 +3969,7 @@
         </is>
       </c>
       <c r="D222" t="n">
-        <v>144</v>
+        <v>150</v>
       </c>
     </row>
     <row r="223">
@@ -4025,7 +4025,7 @@
         </is>
       </c>
       <c r="D226" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="227">
@@ -4039,7 +4039,7 @@
       </c>
       <c r="C227" t="inlineStr"/>
       <c r="D227" t="n">
-        <v>359</v>
+        <v>370</v>
       </c>
     </row>
     <row r="228">
@@ -4071,7 +4071,7 @@
         </is>
       </c>
       <c r="D229" t="n">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="230">
@@ -4121,7 +4121,7 @@
         </is>
       </c>
       <c r="D232" t="n">
-        <v>114</v>
+        <v>122</v>
       </c>
     </row>
     <row r="233">

</xml_diff>

<commit_message>
data: field/odds refresh 2026-05-25 15:50 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -1469,7 +1469,7 @@
       </c>
       <c r="C65" t="inlineStr"/>
       <c r="D65" t="n">
-        <v>212</v>
+        <v>217</v>
       </c>
     </row>
     <row r="66">
@@ -2191,7 +2191,7 @@
       </c>
       <c r="C110" t="inlineStr"/>
       <c r="D110" t="n">
-        <v>286</v>
+        <v>292</v>
       </c>
     </row>
     <row r="111">

</xml_diff>

<commit_message>
data: field/odds refresh 2026-05-25 16:07 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -465,7 +465,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3">
@@ -557,7 +557,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>88</v>
+        <v>91</v>
       </c>
     </row>
     <row r="9">
@@ -575,7 +575,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>23</v>
+        <v>26</v>
       </c>
     </row>
     <row r="10">
@@ -589,7 +589,7 @@
       </c>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="n">
-        <v>196</v>
+        <v>199</v>
       </c>
     </row>
     <row r="11">
@@ -607,7 +607,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>32</v>
+        <v>35</v>
       </c>
     </row>
     <row r="12">
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>104</v>
+        <v>111</v>
       </c>
     </row>
     <row r="18">
@@ -781,7 +781,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>90</v>
+        <v>93</v>
       </c>
     </row>
     <row r="23">
@@ -799,7 +799,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="24">
@@ -839,7 +839,7 @@
       </c>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="n">
-        <v>247</v>
+        <v>238</v>
       </c>
     </row>
     <row r="27">
@@ -875,7 +875,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="29">
@@ -925,7 +925,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="32">
@@ -969,7 +969,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>196</v>
+        <v>202</v>
       </c>
     </row>
     <row r="35">
@@ -987,7 +987,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>249</v>
+        <v>262</v>
       </c>
     </row>
     <row r="36">
@@ -1089,7 +1089,7 @@
       </c>
       <c r="C42" t="inlineStr"/>
       <c r="D42" t="n">
-        <v>288</v>
+        <v>308</v>
       </c>
     </row>
     <row r="43">
@@ -1107,7 +1107,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>48</v>
+        <v>51</v>
       </c>
     </row>
     <row r="44">
@@ -1121,7 +1121,7 @@
       </c>
       <c r="C44" t="inlineStr"/>
       <c r="D44" t="n">
-        <v>48</v>
+        <v>51</v>
       </c>
     </row>
     <row r="45">
@@ -1135,7 +1135,7 @@
       </c>
       <c r="C45" t="inlineStr"/>
       <c r="D45" t="n">
-        <v>166</v>
+        <v>171</v>
       </c>
     </row>
     <row r="46">
@@ -1183,7 +1183,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>120</v>
+        <v>103</v>
       </c>
     </row>
     <row r="49">
@@ -1215,7 +1215,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>135</v>
+        <v>132</v>
       </c>
     </row>
     <row r="51">
@@ -1283,7 +1283,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="55">
@@ -1319,7 +1319,7 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>388</v>
+        <v>407</v>
       </c>
     </row>
     <row r="57">
@@ -1337,7 +1337,7 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="58">
@@ -1355,7 +1355,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="59">
@@ -1373,7 +1373,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>93</v>
+        <v>98</v>
       </c>
     </row>
     <row r="60">
@@ -1437,7 +1437,7 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="64">
@@ -1455,7 +1455,7 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="65">
@@ -1469,7 +1469,7 @@
       </c>
       <c r="C65" t="inlineStr"/>
       <c r="D65" t="n">
-        <v>212</v>
+        <v>217</v>
       </c>
     </row>
     <row r="66">
@@ -1487,7 +1487,7 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="67">
@@ -1531,7 +1531,7 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>57</v>
+        <v>63</v>
       </c>
     </row>
     <row r="70">
@@ -1561,7 +1561,7 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="72">
@@ -1623,7 +1623,7 @@
         </is>
       </c>
       <c r="D75" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="76">
@@ -1641,7 +1641,7 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>94</v>
+        <v>90</v>
       </c>
     </row>
     <row r="77">
@@ -1673,7 +1673,7 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>155</v>
+        <v>160</v>
       </c>
     </row>
     <row r="79">
@@ -1691,7 +1691,7 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="80">
@@ -1705,7 +1705,7 @@
       </c>
       <c r="C80" t="inlineStr"/>
       <c r="D80" t="n">
-        <v>150</v>
+        <v>153</v>
       </c>
     </row>
     <row r="81">
@@ -1723,7 +1723,7 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>89</v>
+        <v>83</v>
       </c>
     </row>
     <row r="82">
@@ -1737,7 +1737,7 @@
       </c>
       <c r="C82" t="inlineStr"/>
       <c r="D82" t="n">
-        <v>460</v>
+        <v>458</v>
       </c>
     </row>
     <row r="83">
@@ -1755,7 +1755,7 @@
         </is>
       </c>
       <c r="D83" t="n">
-        <v>110</v>
+        <v>100</v>
       </c>
     </row>
     <row r="84">
@@ -1791,7 +1791,7 @@
         </is>
       </c>
       <c r="D85" t="n">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="86">
@@ -1827,7 +1827,7 @@
         </is>
       </c>
       <c r="D87" t="n">
-        <v>123</v>
+        <v>130</v>
       </c>
     </row>
     <row r="88">
@@ -1855,7 +1855,7 @@
       </c>
       <c r="C89" t="inlineStr"/>
       <c r="D89" t="n">
-        <v>148</v>
+        <v>151</v>
       </c>
     </row>
     <row r="90">
@@ -1887,7 +1887,7 @@
       </c>
       <c r="C91" t="inlineStr"/>
       <c r="D91" t="n">
-        <v>116</v>
+        <v>114</v>
       </c>
     </row>
     <row r="92">
@@ -1905,7 +1905,7 @@
         </is>
       </c>
       <c r="D92" t="n">
-        <v>142</v>
+        <v>152</v>
       </c>
     </row>
     <row r="93">
@@ -1923,7 +1923,7 @@
         </is>
       </c>
       <c r="D93" t="n">
-        <v>72</v>
+        <v>68</v>
       </c>
     </row>
     <row r="94">
@@ -1941,7 +1941,7 @@
         </is>
       </c>
       <c r="D94" t="n">
-        <v>93</v>
+        <v>84</v>
       </c>
     </row>
     <row r="95">
@@ -1987,7 +1987,7 @@
       </c>
       <c r="C97" t="inlineStr"/>
       <c r="D97" t="n">
-        <v>139</v>
+        <v>145</v>
       </c>
     </row>
     <row r="98">
@@ -2031,7 +2031,7 @@
         </is>
       </c>
       <c r="D100" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
     </row>
     <row r="101">
@@ -2067,7 +2067,7 @@
         </is>
       </c>
       <c r="D102" t="n">
-        <v>141</v>
+        <v>144</v>
       </c>
     </row>
     <row r="103">
@@ -2129,7 +2129,7 @@
       </c>
       <c r="C106" t="inlineStr"/>
       <c r="D106" t="n">
-        <v>300</v>
+        <v>320</v>
       </c>
     </row>
     <row r="107">
@@ -2191,7 +2191,7 @@
       </c>
       <c r="C110" t="inlineStr"/>
       <c r="D110" t="n">
-        <v>286</v>
+        <v>292</v>
       </c>
     </row>
     <row r="111">
@@ -2223,7 +2223,7 @@
       </c>
       <c r="C112" t="inlineStr"/>
       <c r="D112" t="n">
-        <v>181</v>
+        <v>189</v>
       </c>
     </row>
     <row r="113">
@@ -2309,7 +2309,7 @@
         </is>
       </c>
       <c r="D118" t="n">
-        <v>91</v>
+        <v>97</v>
       </c>
     </row>
     <row r="119">
@@ -2371,7 +2371,7 @@
         </is>
       </c>
       <c r="D122" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
     </row>
     <row r="123">
@@ -2411,7 +2411,7 @@
       </c>
       <c r="C125" t="inlineStr"/>
       <c r="D125" t="n">
-        <v>447</v>
+        <v>454</v>
       </c>
     </row>
     <row r="126">
@@ -2429,7 +2429,7 @@
         </is>
       </c>
       <c r="D126" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
     </row>
     <row r="127">
@@ -2465,7 +2465,7 @@
         </is>
       </c>
       <c r="D128" t="n">
-        <v>43</v>
+        <v>49</v>
       </c>
     </row>
     <row r="129">
@@ -2483,7 +2483,7 @@
         </is>
       </c>
       <c r="D129" t="n">
-        <v>84</v>
+        <v>88</v>
       </c>
     </row>
     <row r="130">
@@ -2537,7 +2537,7 @@
         </is>
       </c>
       <c r="D132" t="n">
-        <v>105</v>
+        <v>108</v>
       </c>
     </row>
     <row r="133">
@@ -2571,7 +2571,7 @@
         </is>
       </c>
       <c r="D134" t="n">
-        <v>108</v>
+        <v>95</v>
       </c>
     </row>
     <row r="135">
@@ -2617,7 +2617,7 @@
         </is>
       </c>
       <c r="D137" t="n">
-        <v>152</v>
+        <v>140</v>
       </c>
     </row>
     <row r="138">
@@ -2649,7 +2649,7 @@
       </c>
       <c r="C139" t="inlineStr"/>
       <c r="D139" t="n">
-        <v>129</v>
+        <v>136</v>
       </c>
     </row>
     <row r="140">
@@ -2677,7 +2677,7 @@
       </c>
       <c r="C141" t="inlineStr"/>
       <c r="D141" t="n">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="142">
@@ -2785,7 +2785,7 @@
       </c>
       <c r="C148" t="inlineStr"/>
       <c r="D148" t="n">
-        <v>113</v>
+        <v>121</v>
       </c>
     </row>
     <row r="149">
@@ -2867,7 +2867,7 @@
         </is>
       </c>
       <c r="D154" t="n">
-        <v>262</v>
+        <v>260</v>
       </c>
     </row>
     <row r="155">
@@ -2935,7 +2935,7 @@
       </c>
       <c r="C158" t="inlineStr"/>
       <c r="D158" t="n">
-        <v>221</v>
+        <v>226</v>
       </c>
     </row>
     <row r="159">
@@ -2949,7 +2949,7 @@
       </c>
       <c r="C159" t="inlineStr"/>
       <c r="D159" t="n">
-        <v>168</v>
+        <v>174</v>
       </c>
     </row>
     <row r="160">
@@ -2967,7 +2967,7 @@
         </is>
       </c>
       <c r="D160" t="n">
-        <v>79</v>
+        <v>85</v>
       </c>
     </row>
     <row r="161">
@@ -2999,7 +2999,7 @@
       </c>
       <c r="C162" t="inlineStr"/>
       <c r="D162" t="n">
-        <v>189</v>
+        <v>184</v>
       </c>
     </row>
     <row r="163">
@@ -3067,7 +3067,7 @@
       </c>
       <c r="C166" t="inlineStr"/>
       <c r="D166" t="n">
-        <v>160</v>
+        <v>163</v>
       </c>
     </row>
     <row r="167">
@@ -3127,7 +3127,7 @@
         </is>
       </c>
       <c r="D170" t="n">
-        <v>151</v>
+        <v>154</v>
       </c>
     </row>
     <row r="171">
@@ -3145,7 +3145,7 @@
         </is>
       </c>
       <c r="D171" t="n">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="172">
@@ -3227,7 +3227,7 @@
         </is>
       </c>
       <c r="D176" t="n">
-        <v>214</v>
+        <v>211</v>
       </c>
     </row>
     <row r="177">
@@ -3307,7 +3307,7 @@
         </is>
       </c>
       <c r="D181" t="n">
-        <v>158</v>
+        <v>164</v>
       </c>
     </row>
     <row r="182">
@@ -3421,7 +3421,7 @@
       </c>
       <c r="C188" t="inlineStr"/>
       <c r="D188" t="n">
-        <v>264</v>
+        <v>268</v>
       </c>
     </row>
     <row r="189">
@@ -3439,7 +3439,7 @@
         </is>
       </c>
       <c r="D189" t="n">
-        <v>78</v>
+        <v>41</v>
       </c>
     </row>
     <row r="190">
@@ -3487,7 +3487,7 @@
       </c>
       <c r="C192" t="inlineStr"/>
       <c r="D192" t="n">
-        <v>131</v>
+        <v>133</v>
       </c>
     </row>
     <row r="193">
@@ -3505,7 +3505,7 @@
         </is>
       </c>
       <c r="D193" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="194">
@@ -3537,7 +3537,7 @@
       </c>
       <c r="C195" t="inlineStr"/>
       <c r="D195" t="n">
-        <v>252</v>
+        <v>259</v>
       </c>
     </row>
     <row r="196">
@@ -3555,7 +3555,7 @@
         </is>
       </c>
       <c r="D196" t="n">
-        <v>49</v>
+        <v>52</v>
       </c>
     </row>
     <row r="197">
@@ -3569,7 +3569,7 @@
       </c>
       <c r="C197" t="inlineStr"/>
       <c r="D197" t="n">
-        <v>49</v>
+        <v>52</v>
       </c>
     </row>
     <row r="198">
@@ -3605,7 +3605,7 @@
         </is>
       </c>
       <c r="D199" t="n">
-        <v>416</v>
+        <v>425</v>
       </c>
     </row>
     <row r="200">
@@ -3619,7 +3619,7 @@
       </c>
       <c r="C200" t="inlineStr"/>
       <c r="D200" t="n">
-        <v>209</v>
+        <v>166</v>
       </c>
     </row>
     <row r="201">
@@ -3633,7 +3633,7 @@
       </c>
       <c r="C201" t="inlineStr"/>
       <c r="D201" t="n">
-        <v>408</v>
+        <v>403</v>
       </c>
     </row>
     <row r="202">
@@ -3683,7 +3683,7 @@
         </is>
       </c>
       <c r="D204" t="n">
-        <v>76</v>
+        <v>79</v>
       </c>
     </row>
     <row r="205">
@@ -3719,7 +3719,7 @@
         </is>
       </c>
       <c r="D206" t="n">
-        <v>128</v>
+        <v>137</v>
       </c>
     </row>
     <row r="207">
@@ -3737,7 +3737,7 @@
         </is>
       </c>
       <c r="D207" t="n">
-        <v>70</v>
+        <v>75</v>
       </c>
     </row>
     <row r="208">
@@ -3775,7 +3775,7 @@
       </c>
       <c r="C210" t="inlineStr"/>
       <c r="D210" t="n">
-        <v>331</v>
+        <v>344</v>
       </c>
     </row>
     <row r="211">
@@ -3811,7 +3811,7 @@
         </is>
       </c>
       <c r="D212" t="n">
-        <v>178</v>
+        <v>175</v>
       </c>
     </row>
     <row r="213">
@@ -3855,7 +3855,7 @@
       </c>
       <c r="C215" t="inlineStr"/>
       <c r="D215" t="n">
-        <v>268</v>
+        <v>276</v>
       </c>
     </row>
     <row r="216">
@@ -3869,7 +3869,7 @@
       </c>
       <c r="C216" t="inlineStr"/>
       <c r="D216" t="n">
-        <v>268</v>
+        <v>276</v>
       </c>
     </row>
     <row r="217">
@@ -3887,7 +3887,7 @@
         </is>
       </c>
       <c r="D217" t="n">
-        <v>167</v>
+        <v>176</v>
       </c>
     </row>
     <row r="218">
@@ -3901,7 +3901,7 @@
       </c>
       <c r="C218" t="inlineStr"/>
       <c r="D218" t="n">
-        <v>471</v>
+        <v>453</v>
       </c>
     </row>
     <row r="219">
@@ -3915,7 +3915,7 @@
       </c>
       <c r="C219" t="inlineStr"/>
       <c r="D219" t="n">
-        <v>226</v>
+        <v>230</v>
       </c>
     </row>
     <row r="220">
@@ -3969,7 +3969,7 @@
         </is>
       </c>
       <c r="D222" t="n">
-        <v>144</v>
+        <v>150</v>
       </c>
     </row>
     <row r="223">
@@ -4039,7 +4039,7 @@
       </c>
       <c r="C227" t="inlineStr"/>
       <c r="D227" t="n">
-        <v>359</v>
+        <v>370</v>
       </c>
     </row>
     <row r="228">
@@ -4071,7 +4071,7 @@
         </is>
       </c>
       <c r="D229" t="n">
-        <v>105</v>
+        <v>107</v>
       </c>
     </row>
     <row r="230">
@@ -4121,7 +4121,7 @@
         </is>
       </c>
       <c r="D232" t="n">
-        <v>114</v>
+        <v>122</v>
       </c>
     </row>
     <row r="233">

</xml_diff>

<commit_message>
data: field/odds refresh 2026-06-01 07:48 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -539,7 +539,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="8">
@@ -639,7 +639,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>19</v>
+        <v>24</v>
       </c>
     </row>
     <row r="14">
@@ -685,7 +685,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="17">
@@ -749,7 +749,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>30</v>
+        <v>33</v>
       </c>
     </row>
     <row r="21">
@@ -907,7 +907,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>50</v>
+        <v>53</v>
       </c>
     </row>
     <row r="31">
@@ -1005,7 +1005,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="37">
@@ -1165,7 +1165,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="48">
@@ -1251,7 +1251,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="53">
@@ -1301,7 +1301,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="56">
@@ -1773,7 +1773,7 @@
         </is>
       </c>
       <c r="D84" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="85">
@@ -2049,7 +2049,7 @@
         </is>
       </c>
       <c r="D101" t="n">
-        <v>24</v>
+        <v>19</v>
       </c>
     </row>
     <row r="102">
@@ -2115,7 +2115,7 @@
         </is>
       </c>
       <c r="D105" t="n">
-        <v>34</v>
+        <v>29</v>
       </c>
     </row>
     <row r="106">
@@ -2291,7 +2291,7 @@
         </is>
       </c>
       <c r="D117" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="118">
@@ -2353,7 +2353,7 @@
         </is>
       </c>
       <c r="D121" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="122">
@@ -2519,7 +2519,7 @@
         </is>
       </c>
       <c r="D131" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="132">
@@ -2713,7 +2713,7 @@
         </is>
       </c>
       <c r="D143" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="144">
@@ -2885,7 +2885,7 @@
         </is>
       </c>
       <c r="D155" t="n">
-        <v>82</v>
+        <v>87</v>
       </c>
     </row>
     <row r="156">
@@ -3053,7 +3053,7 @@
         </is>
       </c>
       <c r="D165" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="166">
@@ -3163,7 +3163,7 @@
         </is>
       </c>
       <c r="D172" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="173">
@@ -3271,7 +3271,7 @@
         </is>
       </c>
       <c r="D179" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
     </row>
     <row r="180">
@@ -3361,7 +3361,7 @@
         </is>
       </c>
       <c r="D184" t="n">
-        <v>46</v>
+        <v>50</v>
       </c>
     </row>
     <row r="185">
@@ -3523,7 +3523,7 @@
         </is>
       </c>
       <c r="D194" t="n">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="195">
@@ -3587,7 +3587,7 @@
         </is>
       </c>
       <c r="D198" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
     </row>
     <row r="199">
@@ -3665,7 +3665,7 @@
         </is>
       </c>
       <c r="D203" t="n">
-        <v>58</v>
+        <v>61</v>
       </c>
     </row>
     <row r="204">
@@ -3829,7 +3829,7 @@
         </is>
       </c>
       <c r="D213" t="n">
-        <v>122</v>
+        <v>131</v>
       </c>
     </row>
     <row r="214">
@@ -4175,7 +4175,7 @@
         </is>
       </c>
       <c r="D235" t="n">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: field/odds refresh 2026-06-01 13:13 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -465,7 +465,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3">
@@ -539,7 +539,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="8">
@@ -607,7 +607,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="12">
@@ -685,7 +685,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="17">
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>111</v>
+        <v>118</v>
       </c>
     </row>
     <row r="18">
@@ -799,7 +799,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="24">
@@ -857,7 +857,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="28">
@@ -875,7 +875,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>117</v>
+        <v>69</v>
       </c>
     </row>
     <row r="29">
@@ -925,7 +925,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="32">
@@ -1005,7 +1005,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="37">
@@ -1107,7 +1107,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>51</v>
+        <v>48</v>
       </c>
     </row>
     <row r="44">
@@ -1121,7 +1121,7 @@
       </c>
       <c r="C44" t="inlineStr"/>
       <c r="D44" t="n">
-        <v>51</v>
+        <v>48</v>
       </c>
     </row>
     <row r="45">
@@ -1165,7 +1165,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="48">
@@ -1183,7 +1183,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>103</v>
+        <v>112</v>
       </c>
     </row>
     <row r="49">
@@ -1251,7 +1251,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="53">
@@ -1283,7 +1283,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="55">
@@ -1301,7 +1301,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="56">
@@ -1337,7 +1337,7 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="58">
@@ -1373,7 +1373,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>98</v>
+        <v>104</v>
       </c>
     </row>
     <row r="60">
@@ -1419,7 +1419,7 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="63">
@@ -1455,7 +1455,7 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="65">
@@ -1531,7 +1531,7 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="70">
@@ -1561,7 +1561,7 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="72">
@@ -1623,7 +1623,7 @@
         </is>
       </c>
       <c r="D75" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
     </row>
     <row r="76">
@@ -1755,7 +1755,7 @@
         </is>
       </c>
       <c r="D83" t="n">
-        <v>100</v>
+        <v>106</v>
       </c>
     </row>
     <row r="84">
@@ -1773,7 +1773,7 @@
         </is>
       </c>
       <c r="D84" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="85">
@@ -1827,7 +1827,7 @@
         </is>
       </c>
       <c r="D87" t="n">
-        <v>130</v>
+        <v>140</v>
       </c>
     </row>
     <row r="88">
@@ -1887,7 +1887,7 @@
       </c>
       <c r="C91" t="inlineStr"/>
       <c r="D91" t="n">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="92">
@@ -1923,7 +1923,7 @@
         </is>
       </c>
       <c r="D93" t="n">
-        <v>68</v>
+        <v>72</v>
       </c>
     </row>
     <row r="94">
@@ -2031,7 +2031,7 @@
         </is>
       </c>
       <c r="D100" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="101">
@@ -2115,7 +2115,7 @@
         </is>
       </c>
       <c r="D105" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="106">
@@ -2147,7 +2147,7 @@
         </is>
       </c>
       <c r="D107" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="108">
@@ -2223,7 +2223,7 @@
       </c>
       <c r="C112" t="inlineStr"/>
       <c r="D112" t="n">
-        <v>189</v>
+        <v>179</v>
       </c>
     </row>
     <row r="113">
@@ -2291,7 +2291,7 @@
         </is>
       </c>
       <c r="D117" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="118">
@@ -2353,7 +2353,7 @@
         </is>
       </c>
       <c r="D121" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="122">
@@ -2371,7 +2371,7 @@
         </is>
       </c>
       <c r="D122" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="123">
@@ -2447,7 +2447,7 @@
         </is>
       </c>
       <c r="D127" t="n">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="128">
@@ -2465,7 +2465,7 @@
         </is>
       </c>
       <c r="D128" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="129">
@@ -2519,7 +2519,7 @@
         </is>
       </c>
       <c r="D131" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="132">
@@ -2537,7 +2537,7 @@
         </is>
       </c>
       <c r="D132" t="n">
-        <v>108</v>
+        <v>81</v>
       </c>
     </row>
     <row r="133">
@@ -2771,7 +2771,7 @@
         </is>
       </c>
       <c r="D147" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="148">
@@ -2885,7 +2885,7 @@
         </is>
       </c>
       <c r="D155" t="n">
-        <v>87</v>
+        <v>92</v>
       </c>
     </row>
     <row r="156">
@@ -2967,7 +2967,7 @@
         </is>
       </c>
       <c r="D160" t="n">
-        <v>85</v>
+        <v>94</v>
       </c>
     </row>
     <row r="161">
@@ -3053,7 +3053,7 @@
         </is>
       </c>
       <c r="D165" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="166">
@@ -3145,7 +3145,7 @@
         </is>
       </c>
       <c r="D171" t="n">
-        <v>77</v>
+        <v>79</v>
       </c>
     </row>
     <row r="172">
@@ -3163,7 +3163,7 @@
         </is>
       </c>
       <c r="D172" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="173">
@@ -3271,7 +3271,7 @@
         </is>
       </c>
       <c r="D179" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="180">
@@ -3439,7 +3439,7 @@
         </is>
       </c>
       <c r="D189" t="n">
-        <v>41</v>
+        <v>38</v>
       </c>
     </row>
     <row r="190">
@@ -3487,7 +3487,7 @@
       </c>
       <c r="C192" t="inlineStr"/>
       <c r="D192" t="n">
-        <v>133</v>
+        <v>127</v>
       </c>
     </row>
     <row r="193">
@@ -3523,7 +3523,7 @@
         </is>
       </c>
       <c r="D194" t="n">
-        <v>46</v>
+        <v>49</v>
       </c>
     </row>
     <row r="195">
@@ -3665,7 +3665,7 @@
         </is>
       </c>
       <c r="D203" t="n">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="204">
@@ -3683,7 +3683,7 @@
         </is>
       </c>
       <c r="D204" t="n">
-        <v>79</v>
+        <v>82</v>
       </c>
     </row>
     <row r="205">
@@ -3829,7 +3829,7 @@
         </is>
       </c>
       <c r="D213" t="n">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="214">
@@ -4025,7 +4025,7 @@
         </is>
       </c>
       <c r="D226" t="n">
-        <v>47</v>
+        <v>43</v>
       </c>
     </row>
     <row r="227">
@@ -4175,7 +4175,7 @@
         </is>
       </c>
       <c r="D235" t="n">
-        <v>82</v>
+        <v>88</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: field/odds refresh 2026-06-01 13:39 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -465,7 +465,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3">
@@ -607,7 +607,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="12">
@@ -639,7 +639,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>19</v>
+        <v>24</v>
       </c>
     </row>
     <row r="14">
@@ -685,7 +685,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="17">
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>111</v>
+        <v>118</v>
       </c>
     </row>
     <row r="18">
@@ -749,7 +749,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>30</v>
+        <v>33</v>
       </c>
     </row>
     <row r="21">
@@ -799,7 +799,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="24">
@@ -857,7 +857,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>75</v>
+        <v>45</v>
       </c>
     </row>
     <row r="28">
@@ -875,7 +875,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>117</v>
+        <v>69</v>
       </c>
     </row>
     <row r="29">
@@ -907,7 +907,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>50</v>
+        <v>53</v>
       </c>
     </row>
     <row r="31">
@@ -925,7 +925,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="32">
@@ -1005,7 +1005,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>41</v>
+        <v>44</v>
       </c>
     </row>
     <row r="37">
@@ -1107,7 +1107,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>51</v>
+        <v>48</v>
       </c>
     </row>
     <row r="44">
@@ -1121,7 +1121,7 @@
       </c>
       <c r="C44" t="inlineStr"/>
       <c r="D44" t="n">
-        <v>51</v>
+        <v>48</v>
       </c>
     </row>
     <row r="45">
@@ -1165,7 +1165,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="48">
@@ -1183,7 +1183,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>103</v>
+        <v>112</v>
       </c>
     </row>
     <row r="49">
@@ -1251,7 +1251,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="53">
@@ -1283,7 +1283,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="55">
@@ -1301,7 +1301,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="56">
@@ -1337,7 +1337,7 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="58">
@@ -1373,7 +1373,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>98</v>
+        <v>104</v>
       </c>
     </row>
     <row r="60">
@@ -1419,7 +1419,7 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="63">
@@ -1455,7 +1455,7 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="65">
@@ -1531,7 +1531,7 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="70">
@@ -1561,7 +1561,7 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="72">
@@ -1623,7 +1623,7 @@
         </is>
       </c>
       <c r="D75" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
     </row>
     <row r="76">
@@ -1755,7 +1755,7 @@
         </is>
       </c>
       <c r="D83" t="n">
-        <v>100</v>
+        <v>106</v>
       </c>
     </row>
     <row r="84">
@@ -1827,7 +1827,7 @@
         </is>
       </c>
       <c r="D87" t="n">
-        <v>130</v>
+        <v>140</v>
       </c>
     </row>
     <row r="88">
@@ -1887,7 +1887,7 @@
       </c>
       <c r="C91" t="inlineStr"/>
       <c r="D91" t="n">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="92">
@@ -1923,7 +1923,7 @@
         </is>
       </c>
       <c r="D93" t="n">
-        <v>68</v>
+        <v>72</v>
       </c>
     </row>
     <row r="94">
@@ -2031,7 +2031,7 @@
         </is>
       </c>
       <c r="D100" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="101">
@@ -2049,7 +2049,7 @@
         </is>
       </c>
       <c r="D101" t="n">
-        <v>24</v>
+        <v>19</v>
       </c>
     </row>
     <row r="102">
@@ -2115,7 +2115,7 @@
         </is>
       </c>
       <c r="D105" t="n">
-        <v>34</v>
+        <v>30</v>
       </c>
     </row>
     <row r="106">
@@ -2147,7 +2147,7 @@
         </is>
       </c>
       <c r="D107" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="108">
@@ -2223,7 +2223,7 @@
       </c>
       <c r="C112" t="inlineStr"/>
       <c r="D112" t="n">
-        <v>189</v>
+        <v>179</v>
       </c>
     </row>
     <row r="113">
@@ -2353,7 +2353,7 @@
         </is>
       </c>
       <c r="D121" t="n">
-        <v>38</v>
+        <v>41</v>
       </c>
     </row>
     <row r="122">
@@ -2371,7 +2371,7 @@
         </is>
       </c>
       <c r="D122" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="123">
@@ -2447,7 +2447,7 @@
         </is>
       </c>
       <c r="D127" t="n">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="128">
@@ -2465,7 +2465,7 @@
         </is>
       </c>
       <c r="D128" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="129">
@@ -2519,7 +2519,7 @@
         </is>
       </c>
       <c r="D131" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="132">
@@ -2537,7 +2537,7 @@
         </is>
       </c>
       <c r="D132" t="n">
-        <v>108</v>
+        <v>81</v>
       </c>
     </row>
     <row r="133">
@@ -2713,7 +2713,7 @@
         </is>
       </c>
       <c r="D143" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="144">
@@ -2771,7 +2771,7 @@
         </is>
       </c>
       <c r="D147" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="148">
@@ -2885,7 +2885,7 @@
         </is>
       </c>
       <c r="D155" t="n">
-        <v>82</v>
+        <v>92</v>
       </c>
     </row>
     <row r="156">
@@ -2967,7 +2967,7 @@
         </is>
       </c>
       <c r="D160" t="n">
-        <v>85</v>
+        <v>94</v>
       </c>
     </row>
     <row r="161">
@@ -3053,7 +3053,7 @@
         </is>
       </c>
       <c r="D165" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="166">
@@ -3145,7 +3145,7 @@
         </is>
       </c>
       <c r="D171" t="n">
-        <v>77</v>
+        <v>79</v>
       </c>
     </row>
     <row r="172">
@@ -3163,7 +3163,7 @@
         </is>
       </c>
       <c r="D172" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="173">
@@ -3271,7 +3271,7 @@
         </is>
       </c>
       <c r="D179" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="180">
@@ -3361,7 +3361,7 @@
         </is>
       </c>
       <c r="D184" t="n">
-        <v>46</v>
+        <v>50</v>
       </c>
     </row>
     <row r="185">
@@ -3439,7 +3439,7 @@
         </is>
       </c>
       <c r="D189" t="n">
-        <v>41</v>
+        <v>38</v>
       </c>
     </row>
     <row r="190">
@@ -3487,7 +3487,7 @@
       </c>
       <c r="C192" t="inlineStr"/>
       <c r="D192" t="n">
-        <v>133</v>
+        <v>127</v>
       </c>
     </row>
     <row r="193">
@@ -3523,7 +3523,7 @@
         </is>
       </c>
       <c r="D194" t="n">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="195">
@@ -3587,7 +3587,7 @@
         </is>
       </c>
       <c r="D198" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
     </row>
     <row r="199">
@@ -3665,7 +3665,7 @@
         </is>
       </c>
       <c r="D203" t="n">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="204">
@@ -3683,7 +3683,7 @@
         </is>
       </c>
       <c r="D204" t="n">
-        <v>79</v>
+        <v>82</v>
       </c>
     </row>
     <row r="205">
@@ -3829,7 +3829,7 @@
         </is>
       </c>
       <c r="D213" t="n">
-        <v>122</v>
+        <v>132</v>
       </c>
     </row>
     <row r="214">
@@ -4025,7 +4025,7 @@
         </is>
       </c>
       <c r="D226" t="n">
-        <v>47</v>
+        <v>43</v>
       </c>
     </row>
     <row r="227">
@@ -4175,7 +4175,7 @@
         </is>
       </c>
       <c r="D235" t="n">
-        <v>83</v>
+        <v>88</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: field/odds refresh 2026-06-08 07:09 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -557,7 +557,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="9">
@@ -716,9 +716,7 @@
         <v>12909</v>
       </c>
       <c r="C18" t="inlineStr"/>
-      <c r="D18" t="n">
-        <v>476</v>
-      </c>
+      <c r="D18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -781,7 +779,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>93</v>
+        <v>95</v>
       </c>
     </row>
     <row r="23">
@@ -839,7 +837,7 @@
       </c>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="n">
-        <v>238</v>
+        <v>241</v>
       </c>
     </row>
     <row r="27">
@@ -969,7 +967,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>202</v>
+        <v>200</v>
       </c>
     </row>
     <row r="35">
@@ -987,7 +985,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>262</v>
+        <v>281</v>
       </c>
     </row>
     <row r="36">
@@ -1089,7 +1087,7 @@
       </c>
       <c r="C42" t="inlineStr"/>
       <c r="D42" t="n">
-        <v>308</v>
+        <v>318</v>
       </c>
     </row>
     <row r="43">
@@ -1135,7 +1133,7 @@
       </c>
       <c r="C45" t="inlineStr"/>
       <c r="D45" t="n">
-        <v>171</v>
+        <v>174</v>
       </c>
     </row>
     <row r="46">
@@ -1197,7 +1195,7 @@
       </c>
       <c r="C49" t="inlineStr"/>
       <c r="D49" t="n">
-        <v>196</v>
+        <v>199</v>
       </c>
     </row>
     <row r="50">
@@ -1215,7 +1213,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>132</v>
+        <v>114</v>
       </c>
     </row>
     <row r="51">
@@ -1319,7 +1317,7 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>407</v>
+        <v>358</v>
       </c>
     </row>
     <row r="57">
@@ -1355,7 +1353,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>185</v>
+        <v>178</v>
       </c>
     </row>
     <row r="59">
@@ -1469,7 +1467,7 @@
       </c>
       <c r="C65" t="inlineStr"/>
       <c r="D65" t="n">
-        <v>217</v>
+        <v>211</v>
       </c>
     </row>
     <row r="66">
@@ -1487,7 +1485,7 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>115</v>
+        <v>122</v>
       </c>
     </row>
     <row r="67">
@@ -1513,7 +1511,7 @@
       </c>
       <c r="C68" t="inlineStr"/>
       <c r="D68" t="n">
-        <v>256</v>
+        <v>273</v>
       </c>
     </row>
     <row r="69">
@@ -1641,7 +1639,7 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="77">
@@ -1673,7 +1671,7 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>160</v>
+        <v>168</v>
       </c>
     </row>
     <row r="79">
@@ -1723,7 +1721,7 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="82">
@@ -1737,7 +1735,7 @@
       </c>
       <c r="C82" t="inlineStr"/>
       <c r="D82" t="n">
-        <v>458</v>
+        <v>467</v>
       </c>
     </row>
     <row r="83">
@@ -1809,7 +1807,7 @@
         </is>
       </c>
       <c r="D86" t="n">
-        <v>123</v>
+        <v>120</v>
       </c>
     </row>
     <row r="87">
@@ -1855,7 +1853,7 @@
       </c>
       <c r="C89" t="inlineStr"/>
       <c r="D89" t="n">
-        <v>151</v>
+        <v>158</v>
       </c>
     </row>
     <row r="90">
@@ -1873,7 +1871,7 @@
         </is>
       </c>
       <c r="D90" t="n">
-        <v>27</v>
+        <v>32</v>
       </c>
     </row>
     <row r="91">
@@ -1905,7 +1903,7 @@
         </is>
       </c>
       <c r="D92" t="n">
-        <v>152</v>
+        <v>136</v>
       </c>
     </row>
     <row r="93">
@@ -1941,7 +1939,7 @@
         </is>
       </c>
       <c r="D94" t="n">
-        <v>84</v>
+        <v>96</v>
       </c>
     </row>
     <row r="95">
@@ -1987,7 +1985,7 @@
       </c>
       <c r="C97" t="inlineStr"/>
       <c r="D97" t="n">
-        <v>145</v>
+        <v>154</v>
       </c>
     </row>
     <row r="98">
@@ -2067,7 +2065,7 @@
         </is>
       </c>
       <c r="D102" t="n">
-        <v>144</v>
+        <v>150</v>
       </c>
     </row>
     <row r="103">
@@ -2085,7 +2083,7 @@
         </is>
       </c>
       <c r="D103" t="n">
-        <v>96</v>
+        <v>103</v>
       </c>
     </row>
     <row r="104">
@@ -2129,7 +2127,7 @@
       </c>
       <c r="C106" t="inlineStr"/>
       <c r="D106" t="n">
-        <v>320</v>
+        <v>333</v>
       </c>
     </row>
     <row r="107">
@@ -2177,7 +2175,7 @@
         </is>
       </c>
       <c r="D109" t="n">
-        <v>111</v>
+        <v>107</v>
       </c>
     </row>
     <row r="110">
@@ -2309,7 +2307,7 @@
         </is>
       </c>
       <c r="D118" t="n">
-        <v>97</v>
+        <v>100</v>
       </c>
     </row>
     <row r="119">
@@ -2335,7 +2333,7 @@
       </c>
       <c r="C120" t="inlineStr"/>
       <c r="D120" t="n">
-        <v>235</v>
+        <v>239</v>
       </c>
     </row>
     <row r="121">
@@ -2483,7 +2481,7 @@
         </is>
       </c>
       <c r="D129" t="n">
-        <v>88</v>
+        <v>97</v>
       </c>
     </row>
     <row r="130">
@@ -2571,7 +2569,7 @@
         </is>
       </c>
       <c r="D134" t="n">
-        <v>95</v>
+        <v>99</v>
       </c>
     </row>
     <row r="135">
@@ -2617,7 +2615,7 @@
         </is>
       </c>
       <c r="D137" t="n">
-        <v>140</v>
+        <v>146</v>
       </c>
     </row>
     <row r="138">
@@ -2635,7 +2633,7 @@
         </is>
       </c>
       <c r="D138" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="139">
@@ -2649,7 +2647,7 @@
       </c>
       <c r="C139" t="inlineStr"/>
       <c r="D139" t="n">
-        <v>136</v>
+        <v>142</v>
       </c>
     </row>
     <row r="140">
@@ -2677,7 +2675,7 @@
       </c>
       <c r="C141" t="inlineStr"/>
       <c r="D141" t="n">
-        <v>78</v>
+        <v>80</v>
       </c>
     </row>
     <row r="142">
@@ -2785,7 +2783,7 @@
       </c>
       <c r="C148" t="inlineStr"/>
       <c r="D148" t="n">
-        <v>121</v>
+        <v>126</v>
       </c>
     </row>
     <row r="149">
@@ -2867,7 +2865,7 @@
         </is>
       </c>
       <c r="D154" t="n">
-        <v>260</v>
+        <v>268</v>
       </c>
     </row>
     <row r="155">
@@ -2949,7 +2947,7 @@
       </c>
       <c r="C159" t="inlineStr"/>
       <c r="D159" t="n">
-        <v>174</v>
+        <v>176</v>
       </c>
     </row>
     <row r="160">
@@ -2985,7 +2983,7 @@
         </is>
       </c>
       <c r="D161" t="n">
-        <v>75</v>
+        <v>77</v>
       </c>
     </row>
     <row r="162">
@@ -2999,7 +2997,7 @@
       </c>
       <c r="C162" t="inlineStr"/>
       <c r="D162" t="n">
-        <v>184</v>
+        <v>185</v>
       </c>
     </row>
     <row r="163">
@@ -3017,7 +3015,7 @@
         </is>
       </c>
       <c r="D163" t="n">
-        <v>81</v>
+        <v>84</v>
       </c>
     </row>
     <row r="164">
@@ -3067,7 +3065,7 @@
       </c>
       <c r="C166" t="inlineStr"/>
       <c r="D166" t="n">
-        <v>163</v>
+        <v>167</v>
       </c>
     </row>
     <row r="167">
@@ -3127,7 +3125,7 @@
         </is>
       </c>
       <c r="D170" t="n">
-        <v>154</v>
+        <v>161</v>
       </c>
     </row>
     <row r="171">
@@ -3191,7 +3189,7 @@
       </c>
       <c r="C174" t="inlineStr"/>
       <c r="D174" t="n">
-        <v>125</v>
+        <v>129</v>
       </c>
     </row>
     <row r="175">
@@ -3227,7 +3225,7 @@
         </is>
       </c>
       <c r="D176" t="n">
-        <v>211</v>
+        <v>220</v>
       </c>
     </row>
     <row r="177">
@@ -3325,7 +3323,7 @@
         </is>
       </c>
       <c r="D182" t="n">
-        <v>65</v>
+        <v>67</v>
       </c>
     </row>
     <row r="183">
@@ -3343,7 +3341,7 @@
         </is>
       </c>
       <c r="D183" t="n">
-        <v>65</v>
+        <v>67</v>
       </c>
     </row>
     <row r="184">
@@ -3389,7 +3387,7 @@
       </c>
       <c r="C186" t="inlineStr"/>
       <c r="D186" t="n">
-        <v>278</v>
+        <v>253</v>
       </c>
     </row>
     <row r="187">
@@ -3537,7 +3535,7 @@
       </c>
       <c r="C195" t="inlineStr"/>
       <c r="D195" t="n">
-        <v>259</v>
+        <v>264</v>
       </c>
     </row>
     <row r="196">
@@ -3633,7 +3631,7 @@
       </c>
       <c r="C201" t="inlineStr"/>
       <c r="D201" t="n">
-        <v>403</v>
+        <v>412</v>
       </c>
     </row>
     <row r="202">
@@ -3647,7 +3645,7 @@
       </c>
       <c r="C202" t="inlineStr"/>
       <c r="D202" t="n">
-        <v>207</v>
+        <v>194</v>
       </c>
     </row>
     <row r="203">
@@ -3719,7 +3717,7 @@
         </is>
       </c>
       <c r="D206" t="n">
-        <v>137</v>
+        <v>135</v>
       </c>
     </row>
     <row r="207">
@@ -3737,7 +3735,7 @@
         </is>
       </c>
       <c r="D207" t="n">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="208">
@@ -3775,7 +3773,7 @@
       </c>
       <c r="C210" t="inlineStr"/>
       <c r="D210" t="n">
-        <v>344</v>
+        <v>366</v>
       </c>
     </row>
     <row r="211">
@@ -3811,7 +3809,7 @@
         </is>
       </c>
       <c r="D212" t="n">
-        <v>175</v>
+        <v>177</v>
       </c>
     </row>
     <row r="213">
@@ -3855,7 +3853,7 @@
       </c>
       <c r="C215" t="inlineStr"/>
       <c r="D215" t="n">
-        <v>276</v>
+        <v>286</v>
       </c>
     </row>
     <row r="216">
@@ -3869,7 +3867,7 @@
       </c>
       <c r="C216" t="inlineStr"/>
       <c r="D216" t="n">
-        <v>276</v>
+        <v>286</v>
       </c>
     </row>
     <row r="217">
@@ -3887,7 +3885,7 @@
         </is>
       </c>
       <c r="D217" t="n">
-        <v>176</v>
+        <v>185</v>
       </c>
     </row>
     <row r="218">
@@ -3901,7 +3899,7 @@
       </c>
       <c r="C218" t="inlineStr"/>
       <c r="D218" t="n">
-        <v>453</v>
+        <v>455</v>
       </c>
     </row>
     <row r="219">
@@ -3915,7 +3913,7 @@
       </c>
       <c r="C219" t="inlineStr"/>
       <c r="D219" t="n">
-        <v>230</v>
+        <v>240</v>
       </c>
     </row>
     <row r="220">
@@ -3933,7 +3931,7 @@
         </is>
       </c>
       <c r="D220" t="n">
-        <v>69</v>
+        <v>74</v>
       </c>
     </row>
     <row r="221">
@@ -3951,7 +3949,7 @@
         </is>
       </c>
       <c r="D221" t="n">
-        <v>298</v>
+        <v>307</v>
       </c>
     </row>
     <row r="222">
@@ -3969,7 +3967,7 @@
         </is>
       </c>
       <c r="D222" t="n">
-        <v>150</v>
+        <v>155</v>
       </c>
     </row>
     <row r="223">
@@ -3995,7 +3993,7 @@
       </c>
       <c r="C224" t="inlineStr"/>
       <c r="D224" t="n">
-        <v>426</v>
+        <v>432</v>
       </c>
     </row>
     <row r="225">
@@ -4039,7 +4037,7 @@
       </c>
       <c r="C227" t="inlineStr"/>
       <c r="D227" t="n">
-        <v>370</v>
+        <v>383</v>
       </c>
     </row>
     <row r="228">
@@ -4121,7 +4119,7 @@
         </is>
       </c>
       <c r="D232" t="n">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="233">

</xml_diff>

<commit_message>
data: field/odds refresh 2026-06-08 11:24 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -557,7 +557,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>93</v>
+        <v>96</v>
       </c>
     </row>
     <row r="9">
@@ -639,7 +639,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
     <row r="14">
@@ -685,7 +685,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>34</v>
+        <v>29</v>
       </c>
     </row>
     <row r="17">
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>118</v>
+        <v>124</v>
       </c>
     </row>
     <row r="18">
@@ -779,7 +779,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="23">
@@ -797,7 +797,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>65</v>
+        <v>68</v>
       </c>
     </row>
     <row r="24">
@@ -837,7 +837,7 @@
       </c>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="n">
-        <v>241</v>
+        <v>249</v>
       </c>
     </row>
     <row r="27">
@@ -855,7 +855,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>45</v>
+        <v>37</v>
       </c>
     </row>
     <row r="28">
@@ -873,7 +873,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>69</v>
+        <v>63</v>
       </c>
     </row>
     <row r="29">
@@ -905,7 +905,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="31">
@@ -967,7 +967,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>200</v>
+        <v>203</v>
       </c>
     </row>
     <row r="35">
@@ -985,7 +985,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>281</v>
+        <v>295</v>
       </c>
     </row>
     <row r="36">
@@ -1087,7 +1087,7 @@
       </c>
       <c r="C42" t="inlineStr"/>
       <c r="D42" t="n">
-        <v>318</v>
+        <v>330</v>
       </c>
     </row>
     <row r="43">
@@ -1133,7 +1133,7 @@
       </c>
       <c r="C45" t="inlineStr"/>
       <c r="D45" t="n">
-        <v>174</v>
+        <v>175</v>
       </c>
     </row>
     <row r="46">
@@ -1181,7 +1181,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="49">
@@ -1195,7 +1195,7 @@
       </c>
       <c r="C49" t="inlineStr"/>
       <c r="D49" t="n">
-        <v>199</v>
+        <v>205</v>
       </c>
     </row>
     <row r="50">
@@ -1213,7 +1213,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>114</v>
+        <v>118</v>
       </c>
     </row>
     <row r="51">
@@ -1249,7 +1249,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="53">
@@ -1299,7 +1299,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="56">
@@ -1317,7 +1317,7 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>358</v>
+        <v>368</v>
       </c>
     </row>
     <row r="57">
@@ -1353,7 +1353,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>178</v>
+        <v>181</v>
       </c>
     </row>
     <row r="59">
@@ -1371,7 +1371,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>104</v>
+        <v>106</v>
       </c>
     </row>
     <row r="60">
@@ -1435,7 +1435,7 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>62</v>
+        <v>67</v>
       </c>
     </row>
     <row r="64">
@@ -1467,7 +1467,7 @@
       </c>
       <c r="C65" t="inlineStr"/>
       <c r="D65" t="n">
-        <v>211</v>
+        <v>214</v>
       </c>
     </row>
     <row r="66">
@@ -1485,7 +1485,7 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="67">
@@ -1511,7 +1511,7 @@
       </c>
       <c r="C68" t="inlineStr"/>
       <c r="D68" t="n">
-        <v>273</v>
+        <v>265</v>
       </c>
     </row>
     <row r="69">
@@ -1529,7 +1529,7 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="70">
@@ -1639,7 +1639,7 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>89</v>
+        <v>92</v>
       </c>
     </row>
     <row r="77">
@@ -1671,7 +1671,7 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>168</v>
+        <v>170</v>
       </c>
     </row>
     <row r="79">
@@ -1703,7 +1703,7 @@
       </c>
       <c r="C80" t="inlineStr"/>
       <c r="D80" t="n">
-        <v>153</v>
+        <v>154</v>
       </c>
     </row>
     <row r="81">
@@ -1721,7 +1721,7 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>85</v>
+        <v>88</v>
       </c>
     </row>
     <row r="82">
@@ -1735,7 +1735,7 @@
       </c>
       <c r="C82" t="inlineStr"/>
       <c r="D82" t="n">
-        <v>467</v>
+        <v>482</v>
       </c>
     </row>
     <row r="83">
@@ -1753,7 +1753,7 @@
         </is>
       </c>
       <c r="D83" t="n">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="84">
@@ -1771,7 +1771,7 @@
         </is>
       </c>
       <c r="D84" t="n">
-        <v>29</v>
+        <v>32</v>
       </c>
     </row>
     <row r="85">
@@ -1807,7 +1807,7 @@
         </is>
       </c>
       <c r="D86" t="n">
-        <v>120</v>
+        <v>117</v>
       </c>
     </row>
     <row r="87">
@@ -1825,7 +1825,7 @@
         </is>
       </c>
       <c r="D87" t="n">
-        <v>140</v>
+        <v>146</v>
       </c>
     </row>
     <row r="88">
@@ -1853,7 +1853,7 @@
       </c>
       <c r="C89" t="inlineStr"/>
       <c r="D89" t="n">
-        <v>158</v>
+        <v>160</v>
       </c>
     </row>
     <row r="90">
@@ -1871,7 +1871,7 @@
         </is>
       </c>
       <c r="D90" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="91">
@@ -1885,7 +1885,7 @@
       </c>
       <c r="C91" t="inlineStr"/>
       <c r="D91" t="n">
-        <v>116</v>
+        <v>119</v>
       </c>
     </row>
     <row r="92">
@@ -1903,7 +1903,7 @@
         </is>
       </c>
       <c r="D92" t="n">
-        <v>136</v>
+        <v>133</v>
       </c>
     </row>
     <row r="93">
@@ -1939,7 +1939,7 @@
         </is>
       </c>
       <c r="D94" t="n">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="95">
@@ -1985,7 +1985,7 @@
       </c>
       <c r="C97" t="inlineStr"/>
       <c r="D97" t="n">
-        <v>154</v>
+        <v>156</v>
       </c>
     </row>
     <row r="98">
@@ -2065,7 +2065,7 @@
         </is>
       </c>
       <c r="D102" t="n">
-        <v>150</v>
+        <v>152</v>
       </c>
     </row>
     <row r="103">
@@ -2083,7 +2083,7 @@
         </is>
       </c>
       <c r="D103" t="n">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="104">
@@ -2127,7 +2127,7 @@
       </c>
       <c r="C106" t="inlineStr"/>
       <c r="D106" t="n">
-        <v>333</v>
+        <v>344</v>
       </c>
     </row>
     <row r="107">
@@ -2175,7 +2175,7 @@
         </is>
       </c>
       <c r="D109" t="n">
-        <v>107</v>
+        <v>109</v>
       </c>
     </row>
     <row r="110">
@@ -2307,7 +2307,7 @@
         </is>
       </c>
       <c r="D118" t="n">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
     <row r="119">
@@ -2333,7 +2333,7 @@
       </c>
       <c r="C120" t="inlineStr"/>
       <c r="D120" t="n">
-        <v>239</v>
+        <v>246</v>
       </c>
     </row>
     <row r="121">
@@ -2351,7 +2351,7 @@
         </is>
       </c>
       <c r="D121" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="122">
@@ -2409,7 +2409,7 @@
       </c>
       <c r="C125" t="inlineStr"/>
       <c r="D125" t="n">
-        <v>454</v>
+        <v>459</v>
       </c>
     </row>
     <row r="126">
@@ -2445,7 +2445,7 @@
         </is>
       </c>
       <c r="D127" t="n">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="128">
@@ -2481,7 +2481,7 @@
         </is>
       </c>
       <c r="D129" t="n">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="130">
@@ -2535,7 +2535,7 @@
         </is>
       </c>
       <c r="D132" t="n">
-        <v>81</v>
+        <v>86</v>
       </c>
     </row>
     <row r="133">
@@ -2569,7 +2569,7 @@
         </is>
       </c>
       <c r="D134" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="135">
@@ -2615,7 +2615,7 @@
         </is>
       </c>
       <c r="D137" t="n">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="138">
@@ -2633,7 +2633,7 @@
         </is>
       </c>
       <c r="D138" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="139">
@@ -2647,7 +2647,7 @@
       </c>
       <c r="C139" t="inlineStr"/>
       <c r="D139" t="n">
-        <v>142</v>
+        <v>138</v>
       </c>
     </row>
     <row r="140">
@@ -2675,7 +2675,7 @@
       </c>
       <c r="C141" t="inlineStr"/>
       <c r="D141" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
     </row>
     <row r="142">
@@ -2711,7 +2711,7 @@
         </is>
       </c>
       <c r="D143" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="144">
@@ -2783,7 +2783,7 @@
       </c>
       <c r="C148" t="inlineStr"/>
       <c r="D148" t="n">
-        <v>126</v>
+        <v>128</v>
       </c>
     </row>
     <row r="149">
@@ -2865,7 +2865,7 @@
         </is>
       </c>
       <c r="D154" t="n">
-        <v>268</v>
+        <v>279</v>
       </c>
     </row>
     <row r="155">
@@ -2883,7 +2883,7 @@
         </is>
       </c>
       <c r="D155" t="n">
-        <v>92</v>
+        <v>94</v>
       </c>
     </row>
     <row r="156">
@@ -2947,7 +2947,7 @@
       </c>
       <c r="C159" t="inlineStr"/>
       <c r="D159" t="n">
-        <v>176</v>
+        <v>178</v>
       </c>
     </row>
     <row r="160">
@@ -2983,7 +2983,7 @@
         </is>
       </c>
       <c r="D161" t="n">
-        <v>77</v>
+        <v>80</v>
       </c>
     </row>
     <row r="162">
@@ -2997,7 +2997,7 @@
       </c>
       <c r="C162" t="inlineStr"/>
       <c r="D162" t="n">
-        <v>185</v>
+        <v>187</v>
       </c>
     </row>
     <row r="163">
@@ -3065,7 +3065,7 @@
       </c>
       <c r="C166" t="inlineStr"/>
       <c r="D166" t="n">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="167">
@@ -3125,7 +3125,7 @@
         </is>
       </c>
       <c r="D170" t="n">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="171">
@@ -3189,7 +3189,7 @@
       </c>
       <c r="C174" t="inlineStr"/>
       <c r="D174" t="n">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="175">
@@ -3225,7 +3225,7 @@
         </is>
       </c>
       <c r="D176" t="n">
-        <v>220</v>
+        <v>226</v>
       </c>
     </row>
     <row r="177">
@@ -3305,7 +3305,7 @@
         </is>
       </c>
       <c r="D181" t="n">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
     <row r="182">
@@ -3323,7 +3323,7 @@
         </is>
       </c>
       <c r="D182" t="n">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="183">
@@ -3341,7 +3341,7 @@
         </is>
       </c>
       <c r="D183" t="n">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="184">
@@ -3535,7 +3535,7 @@
       </c>
       <c r="C195" t="inlineStr"/>
       <c r="D195" t="n">
-        <v>264</v>
+        <v>274</v>
       </c>
     </row>
     <row r="196">
@@ -3617,7 +3617,7 @@
       </c>
       <c r="C200" t="inlineStr"/>
       <c r="D200" t="n">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="201">
@@ -3631,7 +3631,7 @@
       </c>
       <c r="C201" t="inlineStr"/>
       <c r="D201" t="n">
-        <v>412</v>
+        <v>426</v>
       </c>
     </row>
     <row r="202">
@@ -3645,7 +3645,7 @@
       </c>
       <c r="C202" t="inlineStr"/>
       <c r="D202" t="n">
-        <v>194</v>
+        <v>196</v>
       </c>
     </row>
     <row r="203">
@@ -3663,7 +3663,7 @@
         </is>
       </c>
       <c r="D203" t="n">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="204">
@@ -3681,7 +3681,7 @@
         </is>
       </c>
       <c r="D204" t="n">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="205">
@@ -3717,7 +3717,7 @@
         </is>
       </c>
       <c r="D206" t="n">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="207">
@@ -3735,7 +3735,7 @@
         </is>
       </c>
       <c r="D207" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="208">
@@ -3773,7 +3773,7 @@
       </c>
       <c r="C210" t="inlineStr"/>
       <c r="D210" t="n">
-        <v>366</v>
+        <v>377</v>
       </c>
     </row>
     <row r="211">
@@ -3809,7 +3809,7 @@
         </is>
       </c>
       <c r="D212" t="n">
-        <v>177</v>
+        <v>180</v>
       </c>
     </row>
     <row r="213">
@@ -3827,7 +3827,7 @@
         </is>
       </c>
       <c r="D213" t="n">
-        <v>132</v>
+        <v>144</v>
       </c>
     </row>
     <row r="214">
@@ -3853,7 +3853,7 @@
       </c>
       <c r="C215" t="inlineStr"/>
       <c r="D215" t="n">
-        <v>286</v>
+        <v>298</v>
       </c>
     </row>
     <row r="216">
@@ -3867,7 +3867,7 @@
       </c>
       <c r="C216" t="inlineStr"/>
       <c r="D216" t="n">
-        <v>286</v>
+        <v>298</v>
       </c>
     </row>
     <row r="217">
@@ -3885,7 +3885,7 @@
         </is>
       </c>
       <c r="D217" t="n">
-        <v>185</v>
+        <v>188</v>
       </c>
     </row>
     <row r="218">
@@ -3899,7 +3899,7 @@
       </c>
       <c r="C218" t="inlineStr"/>
       <c r="D218" t="n">
-        <v>455</v>
+        <v>461</v>
       </c>
     </row>
     <row r="219">
@@ -3913,7 +3913,7 @@
       </c>
       <c r="C219" t="inlineStr"/>
       <c r="D219" t="n">
-        <v>240</v>
+        <v>244</v>
       </c>
     </row>
     <row r="220">
@@ -3931,7 +3931,7 @@
         </is>
       </c>
       <c r="D220" t="n">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="221">
@@ -3949,7 +3949,7 @@
         </is>
       </c>
       <c r="D221" t="n">
-        <v>307</v>
+        <v>311</v>
       </c>
     </row>
     <row r="222">
@@ -3967,7 +3967,7 @@
         </is>
       </c>
       <c r="D222" t="n">
-        <v>155</v>
+        <v>159</v>
       </c>
     </row>
     <row r="223">
@@ -3993,7 +3993,7 @@
       </c>
       <c r="C224" t="inlineStr"/>
       <c r="D224" t="n">
-        <v>432</v>
+        <v>369</v>
       </c>
     </row>
     <row r="225">
@@ -4037,7 +4037,7 @@
       </c>
       <c r="C227" t="inlineStr"/>
       <c r="D227" t="n">
-        <v>383</v>
+        <v>395</v>
       </c>
     </row>
     <row r="228">
@@ -4069,7 +4069,7 @@
         </is>
       </c>
       <c r="D229" t="n">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="230">
@@ -4119,7 +4119,7 @@
         </is>
       </c>
       <c r="D232" t="n">
-        <v>121</v>
+        <v>127</v>
       </c>
     </row>
     <row r="233">
@@ -4173,7 +4173,7 @@
         </is>
       </c>
       <c r="D235" t="n">
-        <v>88</v>
+        <v>73</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: field/odds refresh 2026-06-08 12:00 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -557,7 +557,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>91</v>
+        <v>96</v>
       </c>
     </row>
     <row r="9">
@@ -639,7 +639,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
     <row r="14">
@@ -685,7 +685,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>34</v>
+        <v>29</v>
       </c>
     </row>
     <row r="17">
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>118</v>
+        <v>124</v>
       </c>
     </row>
     <row r="18">
@@ -716,9 +716,7 @@
         <v>12909</v>
       </c>
       <c r="C18" t="inlineStr"/>
-      <c r="D18" t="n">
-        <v>476</v>
-      </c>
+      <c r="D18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -781,7 +779,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>93</v>
+        <v>97</v>
       </c>
     </row>
     <row r="23">
@@ -799,7 +797,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>65</v>
+        <v>68</v>
       </c>
     </row>
     <row r="24">
@@ -839,7 +837,7 @@
       </c>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="n">
-        <v>238</v>
+        <v>249</v>
       </c>
     </row>
     <row r="27">
@@ -857,7 +855,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>45</v>
+        <v>37</v>
       </c>
     </row>
     <row r="28">
@@ -875,7 +873,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>69</v>
+        <v>63</v>
       </c>
     </row>
     <row r="29">
@@ -907,7 +905,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="31">
@@ -969,7 +967,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>202</v>
+        <v>203</v>
       </c>
     </row>
     <row r="35">
@@ -987,7 +985,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>262</v>
+        <v>295</v>
       </c>
     </row>
     <row r="36">
@@ -1089,7 +1087,7 @@
       </c>
       <c r="C42" t="inlineStr"/>
       <c r="D42" t="n">
-        <v>308</v>
+        <v>330</v>
       </c>
     </row>
     <row r="43">
@@ -1135,7 +1133,7 @@
       </c>
       <c r="C45" t="inlineStr"/>
       <c r="D45" t="n">
-        <v>171</v>
+        <v>175</v>
       </c>
     </row>
     <row r="46">
@@ -1183,7 +1181,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="49">
@@ -1197,7 +1195,7 @@
       </c>
       <c r="C49" t="inlineStr"/>
       <c r="D49" t="n">
-        <v>196</v>
+        <v>205</v>
       </c>
     </row>
     <row r="50">
@@ -1215,7 +1213,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>132</v>
+        <v>118</v>
       </c>
     </row>
     <row r="51">
@@ -1251,7 +1249,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="53">
@@ -1301,7 +1299,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="56">
@@ -1319,7 +1317,7 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>407</v>
+        <v>368</v>
       </c>
     </row>
     <row r="57">
@@ -1355,7 +1353,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>185</v>
+        <v>181</v>
       </c>
     </row>
     <row r="59">
@@ -1373,7 +1371,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>104</v>
+        <v>106</v>
       </c>
     </row>
     <row r="60">
@@ -1437,7 +1435,7 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>62</v>
+        <v>67</v>
       </c>
     </row>
     <row r="64">
@@ -1469,7 +1467,7 @@
       </c>
       <c r="C65" t="inlineStr"/>
       <c r="D65" t="n">
-        <v>217</v>
+        <v>214</v>
       </c>
     </row>
     <row r="66">
@@ -1487,7 +1485,7 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>115</v>
+        <v>120</v>
       </c>
     </row>
     <row r="67">
@@ -1513,7 +1511,7 @@
       </c>
       <c r="C68" t="inlineStr"/>
       <c r="D68" t="n">
-        <v>256</v>
+        <v>265</v>
       </c>
     </row>
     <row r="69">
@@ -1531,7 +1529,7 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="70">
@@ -1641,7 +1639,7 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="77">
@@ -1673,7 +1671,7 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>160</v>
+        <v>170</v>
       </c>
     </row>
     <row r="79">
@@ -1705,7 +1703,7 @@
       </c>
       <c r="C80" t="inlineStr"/>
       <c r="D80" t="n">
-        <v>153</v>
+        <v>154</v>
       </c>
     </row>
     <row r="81">
@@ -1723,7 +1721,7 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>83</v>
+        <v>88</v>
       </c>
     </row>
     <row r="82">
@@ -1737,7 +1735,7 @@
       </c>
       <c r="C82" t="inlineStr"/>
       <c r="D82" t="n">
-        <v>458</v>
+        <v>482</v>
       </c>
     </row>
     <row r="83">
@@ -1755,7 +1753,7 @@
         </is>
       </c>
       <c r="D83" t="n">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="84">
@@ -1773,7 +1771,7 @@
         </is>
       </c>
       <c r="D84" t="n">
-        <v>29</v>
+        <v>32</v>
       </c>
     </row>
     <row r="85">
@@ -1809,7 +1807,7 @@
         </is>
       </c>
       <c r="D86" t="n">
-        <v>123</v>
+        <v>117</v>
       </c>
     </row>
     <row r="87">
@@ -1827,7 +1825,7 @@
         </is>
       </c>
       <c r="D87" t="n">
-        <v>140</v>
+        <v>146</v>
       </c>
     </row>
     <row r="88">
@@ -1855,7 +1853,7 @@
       </c>
       <c r="C89" t="inlineStr"/>
       <c r="D89" t="n">
-        <v>151</v>
+        <v>160</v>
       </c>
     </row>
     <row r="90">
@@ -1873,7 +1871,7 @@
         </is>
       </c>
       <c r="D90" t="n">
-        <v>27</v>
+        <v>33</v>
       </c>
     </row>
     <row r="91">
@@ -1887,7 +1885,7 @@
       </c>
       <c r="C91" t="inlineStr"/>
       <c r="D91" t="n">
-        <v>116</v>
+        <v>119</v>
       </c>
     </row>
     <row r="92">
@@ -1905,7 +1903,7 @@
         </is>
       </c>
       <c r="D92" t="n">
-        <v>152</v>
+        <v>133</v>
       </c>
     </row>
     <row r="93">
@@ -1941,7 +1939,7 @@
         </is>
       </c>
       <c r="D94" t="n">
-        <v>84</v>
+        <v>95</v>
       </c>
     </row>
     <row r="95">
@@ -1987,7 +1985,7 @@
       </c>
       <c r="C97" t="inlineStr"/>
       <c r="D97" t="n">
-        <v>145</v>
+        <v>156</v>
       </c>
     </row>
     <row r="98">
@@ -2067,7 +2065,7 @@
         </is>
       </c>
       <c r="D102" t="n">
-        <v>144</v>
+        <v>152</v>
       </c>
     </row>
     <row r="103">
@@ -2085,7 +2083,7 @@
         </is>
       </c>
       <c r="D103" t="n">
-        <v>96</v>
+        <v>104</v>
       </c>
     </row>
     <row r="104">
@@ -2129,7 +2127,7 @@
       </c>
       <c r="C106" t="inlineStr"/>
       <c r="D106" t="n">
-        <v>320</v>
+        <v>344</v>
       </c>
     </row>
     <row r="107">
@@ -2177,7 +2175,7 @@
         </is>
       </c>
       <c r="D109" t="n">
-        <v>111</v>
+        <v>109</v>
       </c>
     </row>
     <row r="110">
@@ -2309,7 +2307,7 @@
         </is>
       </c>
       <c r="D118" t="n">
-        <v>97</v>
+        <v>102</v>
       </c>
     </row>
     <row r="119">
@@ -2335,7 +2333,7 @@
       </c>
       <c r="C120" t="inlineStr"/>
       <c r="D120" t="n">
-        <v>235</v>
+        <v>246</v>
       </c>
     </row>
     <row r="121">
@@ -2353,7 +2351,7 @@
         </is>
       </c>
       <c r="D121" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="122">
@@ -2411,7 +2409,7 @@
       </c>
       <c r="C125" t="inlineStr"/>
       <c r="D125" t="n">
-        <v>454</v>
+        <v>459</v>
       </c>
     </row>
     <row r="126">
@@ -2447,7 +2445,7 @@
         </is>
       </c>
       <c r="D127" t="n">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="128">
@@ -2483,7 +2481,7 @@
         </is>
       </c>
       <c r="D129" t="n">
-        <v>88</v>
+        <v>98</v>
       </c>
     </row>
     <row r="130">
@@ -2537,7 +2535,7 @@
         </is>
       </c>
       <c r="D132" t="n">
-        <v>81</v>
+        <v>86</v>
       </c>
     </row>
     <row r="133">
@@ -2571,7 +2569,7 @@
         </is>
       </c>
       <c r="D134" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="135">
@@ -2617,7 +2615,7 @@
         </is>
       </c>
       <c r="D137" t="n">
-        <v>140</v>
+        <v>145</v>
       </c>
     </row>
     <row r="138">
@@ -2635,7 +2633,7 @@
         </is>
       </c>
       <c r="D138" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="139">
@@ -2649,7 +2647,7 @@
       </c>
       <c r="C139" t="inlineStr"/>
       <c r="D139" t="n">
-        <v>136</v>
+        <v>138</v>
       </c>
     </row>
     <row r="140">
@@ -2677,7 +2675,7 @@
       </c>
       <c r="C141" t="inlineStr"/>
       <c r="D141" t="n">
-        <v>78</v>
+        <v>82</v>
       </c>
     </row>
     <row r="142">
@@ -2713,7 +2711,7 @@
         </is>
       </c>
       <c r="D143" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="144">
@@ -2785,7 +2783,7 @@
       </c>
       <c r="C148" t="inlineStr"/>
       <c r="D148" t="n">
-        <v>121</v>
+        <v>128</v>
       </c>
     </row>
     <row r="149">
@@ -2867,7 +2865,7 @@
         </is>
       </c>
       <c r="D154" t="n">
-        <v>260</v>
+        <v>279</v>
       </c>
     </row>
     <row r="155">
@@ -2885,7 +2883,7 @@
         </is>
       </c>
       <c r="D155" t="n">
-        <v>92</v>
+        <v>94</v>
       </c>
     </row>
     <row r="156">
@@ -2949,7 +2947,7 @@
       </c>
       <c r="C159" t="inlineStr"/>
       <c r="D159" t="n">
-        <v>174</v>
+        <v>178</v>
       </c>
     </row>
     <row r="160">
@@ -2985,7 +2983,7 @@
         </is>
       </c>
       <c r="D161" t="n">
-        <v>75</v>
+        <v>80</v>
       </c>
     </row>
     <row r="162">
@@ -2999,7 +2997,7 @@
       </c>
       <c r="C162" t="inlineStr"/>
       <c r="D162" t="n">
-        <v>184</v>
+        <v>187</v>
       </c>
     </row>
     <row r="163">
@@ -3017,7 +3015,7 @@
         </is>
       </c>
       <c r="D163" t="n">
-        <v>81</v>
+        <v>84</v>
       </c>
     </row>
     <row r="164">
@@ -3067,7 +3065,7 @@
       </c>
       <c r="C166" t="inlineStr"/>
       <c r="D166" t="n">
-        <v>163</v>
+        <v>168</v>
       </c>
     </row>
     <row r="167">
@@ -3127,7 +3125,7 @@
         </is>
       </c>
       <c r="D170" t="n">
-        <v>154</v>
+        <v>162</v>
       </c>
     </row>
     <row r="171">
@@ -3191,7 +3189,7 @@
       </c>
       <c r="C174" t="inlineStr"/>
       <c r="D174" t="n">
-        <v>125</v>
+        <v>131</v>
       </c>
     </row>
     <row r="175">
@@ -3227,7 +3225,7 @@
         </is>
       </c>
       <c r="D176" t="n">
-        <v>211</v>
+        <v>226</v>
       </c>
     </row>
     <row r="177">
@@ -3307,7 +3305,7 @@
         </is>
       </c>
       <c r="D181" t="n">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
     <row r="182">
@@ -3325,7 +3323,7 @@
         </is>
       </c>
       <c r="D182" t="n">
-        <v>65</v>
+        <v>70</v>
       </c>
     </row>
     <row r="183">
@@ -3343,7 +3341,7 @@
         </is>
       </c>
       <c r="D183" t="n">
-        <v>65</v>
+        <v>70</v>
       </c>
     </row>
     <row r="184">
@@ -3537,7 +3535,7 @@
       </c>
       <c r="C195" t="inlineStr"/>
       <c r="D195" t="n">
-        <v>259</v>
+        <v>274</v>
       </c>
     </row>
     <row r="196">
@@ -3619,7 +3617,7 @@
       </c>
       <c r="C200" t="inlineStr"/>
       <c r="D200" t="n">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="201">
@@ -3633,7 +3631,7 @@
       </c>
       <c r="C201" t="inlineStr"/>
       <c r="D201" t="n">
-        <v>403</v>
+        <v>426</v>
       </c>
     </row>
     <row r="202">
@@ -3647,7 +3645,7 @@
       </c>
       <c r="C202" t="inlineStr"/>
       <c r="D202" t="n">
-        <v>207</v>
+        <v>196</v>
       </c>
     </row>
     <row r="203">
@@ -3665,7 +3663,7 @@
         </is>
       </c>
       <c r="D203" t="n">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="204">
@@ -3683,7 +3681,7 @@
         </is>
       </c>
       <c r="D204" t="n">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="205">
@@ -3719,7 +3717,7 @@
         </is>
       </c>
       <c r="D206" t="n">
-        <v>137</v>
+        <v>134</v>
       </c>
     </row>
     <row r="207">
@@ -3737,7 +3735,7 @@
         </is>
       </c>
       <c r="D207" t="n">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="208">
@@ -3775,7 +3773,7 @@
       </c>
       <c r="C210" t="inlineStr"/>
       <c r="D210" t="n">
-        <v>344</v>
+        <v>377</v>
       </c>
     </row>
     <row r="211">
@@ -3811,7 +3809,7 @@
         </is>
       </c>
       <c r="D212" t="n">
-        <v>175</v>
+        <v>180</v>
       </c>
     </row>
     <row r="213">
@@ -3829,7 +3827,7 @@
         </is>
       </c>
       <c r="D213" t="n">
-        <v>132</v>
+        <v>144</v>
       </c>
     </row>
     <row r="214">
@@ -3855,7 +3853,7 @@
       </c>
       <c r="C215" t="inlineStr"/>
       <c r="D215" t="n">
-        <v>276</v>
+        <v>298</v>
       </c>
     </row>
     <row r="216">
@@ -3869,7 +3867,7 @@
       </c>
       <c r="C216" t="inlineStr"/>
       <c r="D216" t="n">
-        <v>276</v>
+        <v>298</v>
       </c>
     </row>
     <row r="217">
@@ -3887,7 +3885,7 @@
         </is>
       </c>
       <c r="D217" t="n">
-        <v>176</v>
+        <v>188</v>
       </c>
     </row>
     <row r="218">
@@ -3901,7 +3899,7 @@
       </c>
       <c r="C218" t="inlineStr"/>
       <c r="D218" t="n">
-        <v>453</v>
+        <v>461</v>
       </c>
     </row>
     <row r="219">
@@ -3915,7 +3913,7 @@
       </c>
       <c r="C219" t="inlineStr"/>
       <c r="D219" t="n">
-        <v>230</v>
+        <v>244</v>
       </c>
     </row>
     <row r="220">
@@ -3933,7 +3931,7 @@
         </is>
       </c>
       <c r="D220" t="n">
-        <v>69</v>
+        <v>76</v>
       </c>
     </row>
     <row r="221">
@@ -3951,7 +3949,7 @@
         </is>
       </c>
       <c r="D221" t="n">
-        <v>298</v>
+        <v>311</v>
       </c>
     </row>
     <row r="222">
@@ -3969,7 +3967,7 @@
         </is>
       </c>
       <c r="D222" t="n">
-        <v>150</v>
+        <v>159</v>
       </c>
     </row>
     <row r="223">
@@ -3995,7 +3993,7 @@
       </c>
       <c r="C224" t="inlineStr"/>
       <c r="D224" t="n">
-        <v>426</v>
+        <v>369</v>
       </c>
     </row>
     <row r="225">
@@ -4039,7 +4037,7 @@
       </c>
       <c r="C227" t="inlineStr"/>
       <c r="D227" t="n">
-        <v>370</v>
+        <v>395</v>
       </c>
     </row>
     <row r="228">
@@ -4071,7 +4069,7 @@
         </is>
       </c>
       <c r="D229" t="n">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="230">
@@ -4121,7 +4119,7 @@
         </is>
       </c>
       <c r="D232" t="n">
-        <v>122</v>
+        <v>127</v>
       </c>
     </row>
     <row r="233">
@@ -4175,7 +4173,7 @@
         </is>
       </c>
       <c r="D235" t="n">
-        <v>88</v>
+        <v>73</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: field/odds refresh 2026-06-08 14:17 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -2933,7 +2933,7 @@
       </c>
       <c r="C158" t="inlineStr"/>
       <c r="D158" t="n">
-        <v>226</v>
+        <v>240</v>
       </c>
     </row>
     <row r="159">
@@ -3387,7 +3387,7 @@
       </c>
       <c r="C186" t="inlineStr"/>
       <c r="D186" t="n">
-        <v>253</v>
+        <v>263</v>
       </c>
     </row>
     <row r="187">
@@ -3419,7 +3419,7 @@
       </c>
       <c r="C188" t="inlineStr"/>
       <c r="D188" t="n">
-        <v>268</v>
+        <v>283</v>
       </c>
     </row>
     <row r="189">

</xml_diff>

<commit_message>
data: field/odds refresh 2026-06-08 14:18 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -2933,7 +2933,7 @@
       </c>
       <c r="C158" t="inlineStr"/>
       <c r="D158" t="n">
-        <v>226</v>
+        <v>240</v>
       </c>
     </row>
     <row r="159">
@@ -3387,7 +3387,7 @@
       </c>
       <c r="C186" t="inlineStr"/>
       <c r="D186" t="n">
-        <v>278</v>
+        <v>263</v>
       </c>
     </row>
     <row r="187">
@@ -3419,7 +3419,7 @@
       </c>
       <c r="C188" t="inlineStr"/>
       <c r="D188" t="n">
-        <v>268</v>
+        <v>283</v>
       </c>
     </row>
     <row r="189">

</xml_diff>

<commit_message>
data: field/odds refresh 2026-06-11 16:29 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -2189,7 +2189,7 @@
       </c>
       <c r="C110" t="inlineStr"/>
       <c r="D110" t="n">
-        <v>292</v>
+        <v>191</v>
       </c>
     </row>
     <row r="111">
@@ -2847,7 +2847,7 @@
       </c>
       <c r="C153" t="inlineStr"/>
       <c r="D153" t="n">
-        <v>332</v>
+        <v>297</v>
       </c>
     </row>
     <row r="154">

</xml_diff>

<commit_message>
data: field/odds refresh 2026-06-11 18:00 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -2189,7 +2189,7 @@
       </c>
       <c r="C110" t="inlineStr"/>
       <c r="D110" t="n">
-        <v>292</v>
+        <v>191</v>
       </c>
     </row>
     <row r="111">
@@ -2847,7 +2847,7 @@
       </c>
       <c r="C153" t="inlineStr"/>
       <c r="D153" t="n">
-        <v>332</v>
+        <v>297</v>
       </c>
     </row>
     <row r="154">

</xml_diff>

<commit_message>
data: field/odds refresh 2026-06-15 06:00 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -465,7 +465,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3">
@@ -539,7 +539,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>42</v>
+        <v>46</v>
       </c>
     </row>
     <row r="8">
@@ -575,7 +575,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="10">
@@ -589,7 +589,7 @@
       </c>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="n">
-        <v>199</v>
+        <v>206</v>
       </c>
     </row>
     <row r="11">
@@ -607,7 +607,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="12">
@@ -729,7 +729,7 @@
       </c>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="n">
-        <v>74</v>
+        <v>148</v>
       </c>
     </row>
     <row r="20">
@@ -747,7 +747,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="21">
@@ -923,7 +923,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="32">
@@ -1003,7 +1003,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="37">
@@ -1021,7 +1021,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="38">
@@ -1105,7 +1105,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="44">
@@ -1119,7 +1119,7 @@
       </c>
       <c r="C44" t="inlineStr"/>
       <c r="D44" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="45">
@@ -1163,7 +1163,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="48">
@@ -1281,7 +1281,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="55">
@@ -1335,7 +1335,7 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>36</v>
+        <v>23</v>
       </c>
     </row>
     <row r="58">
@@ -1453,7 +1453,7 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="65">
@@ -1559,7 +1559,7 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="72">
@@ -1603,7 +1603,7 @@
         </is>
       </c>
       <c r="D74" t="n">
-        <v>26</v>
+        <v>21</v>
       </c>
     </row>
     <row r="75">
@@ -1653,7 +1653,7 @@
       </c>
       <c r="C77" t="inlineStr"/>
       <c r="D77" t="n">
-        <v>329</v>
+        <v>356</v>
       </c>
     </row>
     <row r="78">
@@ -1689,7 +1689,7 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>59</v>
+        <v>61</v>
       </c>
     </row>
     <row r="80">
@@ -1957,7 +1957,7 @@
         </is>
       </c>
       <c r="D95" t="n">
-        <v>471</v>
+        <v>242</v>
       </c>
     </row>
     <row r="96">
@@ -2029,7 +2029,7 @@
         </is>
       </c>
       <c r="D100" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="101">
@@ -2047,7 +2047,7 @@
         </is>
       </c>
       <c r="D101" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="102">
@@ -2113,7 +2113,7 @@
         </is>
       </c>
       <c r="D105" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="106">
@@ -2145,7 +2145,7 @@
         </is>
       </c>
       <c r="D107" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="108">
@@ -2207,7 +2207,7 @@
         </is>
       </c>
       <c r="D111" t="n">
-        <v>191</v>
+        <v>254</v>
       </c>
     </row>
     <row r="112">
@@ -2289,7 +2289,7 @@
         </is>
       </c>
       <c r="D117" t="n">
-        <v>31</v>
+        <v>36</v>
       </c>
     </row>
     <row r="118">
@@ -2427,7 +2427,7 @@
         </is>
       </c>
       <c r="D126" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
     </row>
     <row r="127">
@@ -2463,7 +2463,7 @@
         </is>
       </c>
       <c r="D128" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="129">
@@ -2597,7 +2597,7 @@
       </c>
       <c r="C136" t="inlineStr"/>
       <c r="D136" t="n">
-        <v>195</v>
+        <v>219</v>
       </c>
     </row>
     <row r="137">
@@ -2693,7 +2693,7 @@
         </is>
       </c>
       <c r="D142" t="n">
-        <v>167</v>
+        <v>79</v>
       </c>
     </row>
     <row r="143">
@@ -2725,7 +2725,7 @@
       </c>
       <c r="C144" t="inlineStr"/>
       <c r="D144" t="n">
-        <v>177</v>
+        <v>270</v>
       </c>
     </row>
     <row r="145">
@@ -2769,7 +2769,7 @@
         </is>
       </c>
       <c r="D147" t="n">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="148">
@@ -2965,7 +2965,7 @@
         </is>
       </c>
       <c r="D160" t="n">
-        <v>94</v>
+        <v>39</v>
       </c>
     </row>
     <row r="161">
@@ -3033,7 +3033,7 @@
         </is>
       </c>
       <c r="D164" t="n">
-        <v>20</v>
+        <v>8</v>
       </c>
     </row>
     <row r="165">
@@ -3095,7 +3095,7 @@
         </is>
       </c>
       <c r="D168" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="169">
@@ -3143,7 +3143,7 @@
         </is>
       </c>
       <c r="D171" t="n">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="172">
@@ -3269,7 +3269,7 @@
         </is>
       </c>
       <c r="D179" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="180">
@@ -3437,7 +3437,7 @@
         </is>
       </c>
       <c r="D189" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="190">
@@ -3455,7 +3455,7 @@
         </is>
       </c>
       <c r="D190" t="n">
-        <v>239</v>
+        <v>132</v>
       </c>
     </row>
     <row r="191">
@@ -3521,7 +3521,7 @@
         </is>
       </c>
       <c r="D194" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="195">
@@ -3553,7 +3553,7 @@
         </is>
       </c>
       <c r="D196" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="197">
@@ -3567,7 +3567,7 @@
       </c>
       <c r="C197" t="inlineStr"/>
       <c r="D197" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="198">
@@ -3585,7 +3585,7 @@
         </is>
       </c>
       <c r="D198" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="199">
@@ -4023,7 +4023,7 @@
         </is>
       </c>
       <c r="D226" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="227">

</xml_diff>

<commit_message>
data: field/odds refresh 2026-06-15 08:31 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -465,7 +465,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3">
@@ -539,7 +539,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>42</v>
+        <v>46</v>
       </c>
     </row>
     <row r="8">
@@ -575,7 +575,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="10">
@@ -589,7 +589,7 @@
       </c>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="n">
-        <v>199</v>
+        <v>206</v>
       </c>
     </row>
     <row r="11">
@@ -607,7 +607,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="12">
@@ -729,7 +729,7 @@
       </c>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="n">
-        <v>74</v>
+        <v>148</v>
       </c>
     </row>
     <row r="20">
@@ -747,7 +747,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="21">
@@ -923,7 +923,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="32">
@@ -1003,7 +1003,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="37">
@@ -1021,7 +1021,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="38">
@@ -1105,7 +1105,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="44">
@@ -1119,7 +1119,7 @@
       </c>
       <c r="C44" t="inlineStr"/>
       <c r="D44" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="45">
@@ -1163,7 +1163,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="48">
@@ -1281,7 +1281,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="55">
@@ -1335,7 +1335,7 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>36</v>
+        <v>23</v>
       </c>
     </row>
     <row r="58">
@@ -1453,7 +1453,7 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="65">
@@ -1559,7 +1559,7 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="72">
@@ -1603,7 +1603,7 @@
         </is>
       </c>
       <c r="D74" t="n">
-        <v>26</v>
+        <v>21</v>
       </c>
     </row>
     <row r="75">
@@ -1653,7 +1653,7 @@
       </c>
       <c r="C77" t="inlineStr"/>
       <c r="D77" t="n">
-        <v>329</v>
+        <v>356</v>
       </c>
     </row>
     <row r="78">
@@ -1689,7 +1689,7 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>59</v>
+        <v>61</v>
       </c>
     </row>
     <row r="80">
@@ -1957,7 +1957,7 @@
         </is>
       </c>
       <c r="D95" t="n">
-        <v>471</v>
+        <v>242</v>
       </c>
     </row>
     <row r="96">
@@ -2029,7 +2029,7 @@
         </is>
       </c>
       <c r="D100" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="101">
@@ -2047,7 +2047,7 @@
         </is>
       </c>
       <c r="D101" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="102">
@@ -2113,7 +2113,7 @@
         </is>
       </c>
       <c r="D105" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="106">
@@ -2145,7 +2145,7 @@
         </is>
       </c>
       <c r="D107" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="108">
@@ -2207,7 +2207,7 @@
         </is>
       </c>
       <c r="D111" t="n">
-        <v>191</v>
+        <v>254</v>
       </c>
     </row>
     <row r="112">
@@ -2289,7 +2289,7 @@
         </is>
       </c>
       <c r="D117" t="n">
-        <v>31</v>
+        <v>36</v>
       </c>
     </row>
     <row r="118">
@@ -2427,7 +2427,7 @@
         </is>
       </c>
       <c r="D126" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
     </row>
     <row r="127">
@@ -2463,7 +2463,7 @@
         </is>
       </c>
       <c r="D128" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="129">
@@ -2597,7 +2597,7 @@
       </c>
       <c r="C136" t="inlineStr"/>
       <c r="D136" t="n">
-        <v>195</v>
+        <v>219</v>
       </c>
     </row>
     <row r="137">
@@ -2693,7 +2693,7 @@
         </is>
       </c>
       <c r="D142" t="n">
-        <v>167</v>
+        <v>79</v>
       </c>
     </row>
     <row r="143">
@@ -2725,7 +2725,7 @@
       </c>
       <c r="C144" t="inlineStr"/>
       <c r="D144" t="n">
-        <v>177</v>
+        <v>270</v>
       </c>
     </row>
     <row r="145">
@@ -2769,7 +2769,7 @@
         </is>
       </c>
       <c r="D147" t="n">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="148">
@@ -2965,7 +2965,7 @@
         </is>
       </c>
       <c r="D160" t="n">
-        <v>94</v>
+        <v>39</v>
       </c>
     </row>
     <row r="161">
@@ -3033,7 +3033,7 @@
         </is>
       </c>
       <c r="D164" t="n">
-        <v>20</v>
+        <v>8</v>
       </c>
     </row>
     <row r="165">
@@ -3095,7 +3095,7 @@
         </is>
       </c>
       <c r="D168" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="169">
@@ -3143,7 +3143,7 @@
         </is>
       </c>
       <c r="D171" t="n">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="172">
@@ -3269,7 +3269,7 @@
         </is>
       </c>
       <c r="D179" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="180">
@@ -3437,7 +3437,7 @@
         </is>
       </c>
       <c r="D189" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="190">
@@ -3455,7 +3455,7 @@
         </is>
       </c>
       <c r="D190" t="n">
-        <v>239</v>
+        <v>132</v>
       </c>
     </row>
     <row r="191">
@@ -3521,7 +3521,7 @@
         </is>
       </c>
       <c r="D194" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="195">
@@ -3553,7 +3553,7 @@
         </is>
       </c>
       <c r="D196" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="197">
@@ -3567,7 +3567,7 @@
       </c>
       <c r="C197" t="inlineStr"/>
       <c r="D197" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="198">
@@ -3585,7 +3585,7 @@
         </is>
       </c>
       <c r="D198" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="199">
@@ -4023,7 +4023,7 @@
         </is>
       </c>
       <c r="D226" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="227">

</xml_diff>

<commit_message>
data: field/odds refresh 2026-06-15 17:13 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -465,7 +465,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3">
@@ -575,7 +575,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="10">
@@ -589,7 +589,7 @@
       </c>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="n">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="11">
@@ -607,7 +607,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="12">
@@ -639,7 +639,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="14">
@@ -685,7 +685,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="17">
@@ -729,7 +729,7 @@
       </c>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="n">
-        <v>148</v>
+        <v>151</v>
       </c>
     </row>
     <row r="20">
@@ -747,7 +747,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="21">
@@ -797,7 +797,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>68</v>
+        <v>40</v>
       </c>
     </row>
     <row r="24">
@@ -855,7 +855,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="28">
@@ -905,7 +905,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="31">
@@ -923,7 +923,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="32">
@@ -1003,7 +1003,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="37">
@@ -1021,7 +1021,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="38">
@@ -1105,7 +1105,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>49</v>
+        <v>52</v>
       </c>
     </row>
     <row r="44">
@@ -1119,7 +1119,7 @@
       </c>
       <c r="C44" t="inlineStr"/>
       <c r="D44" t="n">
-        <v>49</v>
+        <v>52</v>
       </c>
     </row>
     <row r="45">
@@ -1249,7 +1249,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="53">
@@ -1299,7 +1299,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>60</v>
+        <v>55</v>
       </c>
     </row>
     <row r="56">
@@ -1435,7 +1435,7 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="64">
@@ -1485,7 +1485,7 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>120</v>
+        <v>116</v>
       </c>
     </row>
     <row r="67">
@@ -1689,7 +1689,7 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="80">
@@ -1771,7 +1771,7 @@
         </is>
       </c>
       <c r="D84" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="85">
@@ -1825,7 +1825,7 @@
         </is>
       </c>
       <c r="D87" t="n">
-        <v>146</v>
+        <v>135</v>
       </c>
     </row>
     <row r="88">
@@ -1871,7 +1871,7 @@
         </is>
       </c>
       <c r="D90" t="n">
-        <v>33</v>
+        <v>28</v>
       </c>
     </row>
     <row r="91">
@@ -1921,7 +1921,7 @@
         </is>
       </c>
       <c r="D93" t="n">
-        <v>72</v>
+        <v>74</v>
       </c>
     </row>
     <row r="94">
@@ -1957,7 +1957,7 @@
         </is>
       </c>
       <c r="D95" t="n">
-        <v>242</v>
+        <v>245</v>
       </c>
     </row>
     <row r="96">
@@ -2029,7 +2029,7 @@
         </is>
       </c>
       <c r="D100" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="101">
@@ -2065,7 +2065,7 @@
         </is>
       </c>
       <c r="D102" t="n">
-        <v>152</v>
+        <v>141</v>
       </c>
     </row>
     <row r="103">
@@ -2083,7 +2083,7 @@
         </is>
       </c>
       <c r="D103" t="n">
-        <v>104</v>
+        <v>106</v>
       </c>
     </row>
     <row r="104">
@@ -2145,7 +2145,7 @@
         </is>
       </c>
       <c r="D107" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="108">
@@ -2175,7 +2175,7 @@
         </is>
       </c>
       <c r="D109" t="n">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="110">
@@ -2189,7 +2189,7 @@
       </c>
       <c r="C110" t="inlineStr"/>
       <c r="D110" t="n">
-        <v>191</v>
+        <v>184</v>
       </c>
     </row>
     <row r="111">
@@ -2207,7 +2207,7 @@
         </is>
       </c>
       <c r="D111" t="n">
-        <v>254</v>
+        <v>260</v>
       </c>
     </row>
     <row r="112">
@@ -2289,7 +2289,7 @@
         </is>
       </c>
       <c r="D117" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="118">
@@ -2351,7 +2351,7 @@
         </is>
       </c>
       <c r="D121" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="122">
@@ -2427,7 +2427,7 @@
         </is>
       </c>
       <c r="D126" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="127">
@@ -2463,7 +2463,7 @@
         </is>
       </c>
       <c r="D128" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="129">
@@ -2481,7 +2481,7 @@
         </is>
       </c>
       <c r="D129" t="n">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="130">
@@ -2517,7 +2517,7 @@
         </is>
       </c>
       <c r="D131" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="132">
@@ -2597,7 +2597,7 @@
       </c>
       <c r="C136" t="inlineStr"/>
       <c r="D136" t="n">
-        <v>219</v>
+        <v>227</v>
       </c>
     </row>
     <row r="137">
@@ -2647,7 +2647,7 @@
       </c>
       <c r="C139" t="inlineStr"/>
       <c r="D139" t="n">
-        <v>138</v>
+        <v>131</v>
       </c>
     </row>
     <row r="140">
@@ -2693,7 +2693,7 @@
         </is>
       </c>
       <c r="D142" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="143">
@@ -2725,7 +2725,7 @@
       </c>
       <c r="C144" t="inlineStr"/>
       <c r="D144" t="n">
-        <v>270</v>
+        <v>275</v>
       </c>
     </row>
     <row r="145">
@@ -2769,7 +2769,7 @@
         </is>
       </c>
       <c r="D147" t="n">
-        <v>58</v>
+        <v>61</v>
       </c>
     </row>
     <row r="148">
@@ -2947,7 +2947,7 @@
       </c>
       <c r="C159" t="inlineStr"/>
       <c r="D159" t="n">
-        <v>178</v>
+        <v>172</v>
       </c>
     </row>
     <row r="160">
@@ -2965,7 +2965,7 @@
         </is>
       </c>
       <c r="D160" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="161">
@@ -3015,7 +3015,7 @@
         </is>
       </c>
       <c r="D163" t="n">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="164">
@@ -3051,7 +3051,7 @@
         </is>
       </c>
       <c r="D165" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="166">
@@ -3095,7 +3095,7 @@
         </is>
       </c>
       <c r="D168" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="169">
@@ -3161,7 +3161,7 @@
         </is>
       </c>
       <c r="D172" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="173">
@@ -3189,7 +3189,7 @@
       </c>
       <c r="C174" t="inlineStr"/>
       <c r="D174" t="n">
-        <v>131</v>
+        <v>133</v>
       </c>
     </row>
     <row r="175">
@@ -3323,7 +3323,7 @@
         </is>
       </c>
       <c r="D182" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="183">
@@ -3341,7 +3341,7 @@
         </is>
       </c>
       <c r="D183" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="184">
@@ -3359,7 +3359,7 @@
         </is>
       </c>
       <c r="D184" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="185">
@@ -3387,7 +3387,7 @@
       </c>
       <c r="C186" t="inlineStr"/>
       <c r="D186" t="n">
-        <v>263</v>
+        <v>262</v>
       </c>
     </row>
     <row r="187">
@@ -3437,7 +3437,7 @@
         </is>
       </c>
       <c r="D189" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="190">
@@ -3455,7 +3455,7 @@
         </is>
       </c>
       <c r="D190" t="n">
-        <v>132</v>
+        <v>136</v>
       </c>
     </row>
     <row r="191">
@@ -3553,7 +3553,7 @@
         </is>
       </c>
       <c r="D196" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="197">
@@ -3567,7 +3567,7 @@
       </c>
       <c r="C197" t="inlineStr"/>
       <c r="D197" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="198">
@@ -3617,7 +3617,7 @@
       </c>
       <c r="C200" t="inlineStr"/>
       <c r="D200" t="n">
-        <v>167</v>
+        <v>128</v>
       </c>
     </row>
     <row r="201">
@@ -3663,7 +3663,7 @@
         </is>
       </c>
       <c r="D203" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="204">
@@ -3717,7 +3717,7 @@
         </is>
       </c>
       <c r="D206" t="n">
-        <v>134</v>
+        <v>138</v>
       </c>
     </row>
     <row r="207">
@@ -3773,7 +3773,7 @@
       </c>
       <c r="C210" t="inlineStr"/>
       <c r="D210" t="n">
-        <v>377</v>
+        <v>364</v>
       </c>
     </row>
     <row r="211">
@@ -4023,7 +4023,7 @@
         </is>
       </c>
       <c r="D226" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="227">
@@ -4037,7 +4037,7 @@
       </c>
       <c r="C227" t="inlineStr"/>
       <c r="D227" t="n">
-        <v>395</v>
+        <v>386</v>
       </c>
     </row>
     <row r="228">
@@ -4069,7 +4069,7 @@
         </is>
       </c>
       <c r="D229" t="n">
-        <v>110</v>
+        <v>96</v>
       </c>
     </row>
     <row r="230">
@@ -4173,7 +4173,7 @@
         </is>
       </c>
       <c r="D235" t="n">
-        <v>73</v>
+        <v>69</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: field/odds refresh 2026-06-16 06:00 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -465,7 +465,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3">
@@ -575,7 +575,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="10">
@@ -589,7 +589,7 @@
       </c>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="n">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="11">
@@ -607,7 +607,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="12">
@@ -639,7 +639,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="14">
@@ -685,7 +685,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="17">
@@ -729,7 +729,7 @@
       </c>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="n">
-        <v>148</v>
+        <v>151</v>
       </c>
     </row>
     <row r="20">
@@ -747,7 +747,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="21">
@@ -797,7 +797,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>68</v>
+        <v>40</v>
       </c>
     </row>
     <row r="24">
@@ -855,7 +855,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="28">
@@ -905,7 +905,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="31">
@@ -923,7 +923,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="32">
@@ -1003,7 +1003,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="37">
@@ -1021,7 +1021,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="38">
@@ -1105,7 +1105,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>49</v>
+        <v>52</v>
       </c>
     </row>
     <row r="44">
@@ -1119,7 +1119,7 @@
       </c>
       <c r="C44" t="inlineStr"/>
       <c r="D44" t="n">
-        <v>49</v>
+        <v>52</v>
       </c>
     </row>
     <row r="45">
@@ -1249,7 +1249,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="53">
@@ -1299,7 +1299,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>60</v>
+        <v>55</v>
       </c>
     </row>
     <row r="56">
@@ -1435,7 +1435,7 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="64">
@@ -1485,7 +1485,7 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>120</v>
+        <v>116</v>
       </c>
     </row>
     <row r="67">
@@ -1689,7 +1689,7 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="80">
@@ -1771,7 +1771,7 @@
         </is>
       </c>
       <c r="D84" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="85">
@@ -1825,7 +1825,7 @@
         </is>
       </c>
       <c r="D87" t="n">
-        <v>146</v>
+        <v>135</v>
       </c>
     </row>
     <row r="88">
@@ -1871,7 +1871,7 @@
         </is>
       </c>
       <c r="D90" t="n">
-        <v>33</v>
+        <v>28</v>
       </c>
     </row>
     <row r="91">
@@ -1921,7 +1921,7 @@
         </is>
       </c>
       <c r="D93" t="n">
-        <v>72</v>
+        <v>74</v>
       </c>
     </row>
     <row r="94">
@@ -1957,7 +1957,7 @@
         </is>
       </c>
       <c r="D95" t="n">
-        <v>242</v>
+        <v>245</v>
       </c>
     </row>
     <row r="96">
@@ -2029,7 +2029,7 @@
         </is>
       </c>
       <c r="D100" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="101">
@@ -2065,7 +2065,7 @@
         </is>
       </c>
       <c r="D102" t="n">
-        <v>152</v>
+        <v>141</v>
       </c>
     </row>
     <row r="103">
@@ -2083,7 +2083,7 @@
         </is>
       </c>
       <c r="D103" t="n">
-        <v>104</v>
+        <v>106</v>
       </c>
     </row>
     <row r="104">
@@ -2145,7 +2145,7 @@
         </is>
       </c>
       <c r="D107" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="108">
@@ -2175,7 +2175,7 @@
         </is>
       </c>
       <c r="D109" t="n">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="110">
@@ -2189,7 +2189,7 @@
       </c>
       <c r="C110" t="inlineStr"/>
       <c r="D110" t="n">
-        <v>191</v>
+        <v>184</v>
       </c>
     </row>
     <row r="111">
@@ -2207,7 +2207,7 @@
         </is>
       </c>
       <c r="D111" t="n">
-        <v>254</v>
+        <v>260</v>
       </c>
     </row>
     <row r="112">
@@ -2289,7 +2289,7 @@
         </is>
       </c>
       <c r="D117" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="118">
@@ -2351,7 +2351,7 @@
         </is>
       </c>
       <c r="D121" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="122">
@@ -2427,7 +2427,7 @@
         </is>
       </c>
       <c r="D126" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="127">
@@ -2463,7 +2463,7 @@
         </is>
       </c>
       <c r="D128" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="129">
@@ -2481,7 +2481,7 @@
         </is>
       </c>
       <c r="D129" t="n">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="130">
@@ -2517,7 +2517,7 @@
         </is>
       </c>
       <c r="D131" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="132">
@@ -2597,7 +2597,7 @@
       </c>
       <c r="C136" t="inlineStr"/>
       <c r="D136" t="n">
-        <v>219</v>
+        <v>227</v>
       </c>
     </row>
     <row r="137">
@@ -2647,7 +2647,7 @@
       </c>
       <c r="C139" t="inlineStr"/>
       <c r="D139" t="n">
-        <v>138</v>
+        <v>131</v>
       </c>
     </row>
     <row r="140">
@@ -2693,7 +2693,7 @@
         </is>
       </c>
       <c r="D142" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="143">
@@ -2725,7 +2725,7 @@
       </c>
       <c r="C144" t="inlineStr"/>
       <c r="D144" t="n">
-        <v>270</v>
+        <v>275</v>
       </c>
     </row>
     <row r="145">
@@ -2769,7 +2769,7 @@
         </is>
       </c>
       <c r="D147" t="n">
-        <v>58</v>
+        <v>61</v>
       </c>
     </row>
     <row r="148">
@@ -2947,7 +2947,7 @@
       </c>
       <c r="C159" t="inlineStr"/>
       <c r="D159" t="n">
-        <v>178</v>
+        <v>172</v>
       </c>
     </row>
     <row r="160">
@@ -2965,7 +2965,7 @@
         </is>
       </c>
       <c r="D160" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="161">
@@ -3015,7 +3015,7 @@
         </is>
       </c>
       <c r="D163" t="n">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="164">
@@ -3051,7 +3051,7 @@
         </is>
       </c>
       <c r="D165" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="166">
@@ -3095,7 +3095,7 @@
         </is>
       </c>
       <c r="D168" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="169">
@@ -3161,7 +3161,7 @@
         </is>
       </c>
       <c r="D172" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="173">
@@ -3189,7 +3189,7 @@
       </c>
       <c r="C174" t="inlineStr"/>
       <c r="D174" t="n">
-        <v>131</v>
+        <v>133</v>
       </c>
     </row>
     <row r="175">
@@ -3323,7 +3323,7 @@
         </is>
       </c>
       <c r="D182" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="183">
@@ -3341,7 +3341,7 @@
         </is>
       </c>
       <c r="D183" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="184">
@@ -3359,7 +3359,7 @@
         </is>
       </c>
       <c r="D184" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="185">
@@ -3387,7 +3387,7 @@
       </c>
       <c r="C186" t="inlineStr"/>
       <c r="D186" t="n">
-        <v>263</v>
+        <v>262</v>
       </c>
     </row>
     <row r="187">
@@ -3437,7 +3437,7 @@
         </is>
       </c>
       <c r="D189" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="190">
@@ -3455,7 +3455,7 @@
         </is>
       </c>
       <c r="D190" t="n">
-        <v>132</v>
+        <v>136</v>
       </c>
     </row>
     <row r="191">
@@ -3553,7 +3553,7 @@
         </is>
       </c>
       <c r="D196" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="197">
@@ -3567,7 +3567,7 @@
       </c>
       <c r="C197" t="inlineStr"/>
       <c r="D197" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="198">
@@ -3617,7 +3617,7 @@
       </c>
       <c r="C200" t="inlineStr"/>
       <c r="D200" t="n">
-        <v>167</v>
+        <v>128</v>
       </c>
     </row>
     <row r="201">
@@ -3663,7 +3663,7 @@
         </is>
       </c>
       <c r="D203" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="204">
@@ -3717,7 +3717,7 @@
         </is>
       </c>
       <c r="D206" t="n">
-        <v>134</v>
+        <v>138</v>
       </c>
     </row>
     <row r="207">
@@ -3773,7 +3773,7 @@
       </c>
       <c r="C210" t="inlineStr"/>
       <c r="D210" t="n">
-        <v>377</v>
+        <v>364</v>
       </c>
     </row>
     <row r="211">
@@ -4023,7 +4023,7 @@
         </is>
       </c>
       <c r="D226" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="227">
@@ -4037,7 +4037,7 @@
       </c>
       <c r="C227" t="inlineStr"/>
       <c r="D227" t="n">
-        <v>395</v>
+        <v>386</v>
       </c>
     </row>
     <row r="228">
@@ -4069,7 +4069,7 @@
         </is>
       </c>
       <c r="D229" t="n">
-        <v>110</v>
+        <v>96</v>
       </c>
     </row>
     <row r="230">
@@ -4173,7 +4173,7 @@
         </is>
       </c>
       <c r="D235" t="n">
-        <v>73</v>
+        <v>69</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: field/odds refresh 2026-06-22 08:17 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>124</v>
+        <v>126</v>
       </c>
     </row>
     <row r="18">
@@ -873,7 +873,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="29">
@@ -1181,7 +1181,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>111</v>
+        <v>109</v>
       </c>
     </row>
     <row r="49">
@@ -1371,7 +1371,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="60">
@@ -1753,7 +1753,7 @@
         </is>
       </c>
       <c r="D83" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="84">
@@ -1885,7 +1885,7 @@
       </c>
       <c r="C91" t="inlineStr"/>
       <c r="D91" t="n">
-        <v>119</v>
+        <v>121</v>
       </c>
     </row>
     <row r="92">
@@ -2535,7 +2535,7 @@
         </is>
       </c>
       <c r="D132" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="133">
@@ -2883,7 +2883,7 @@
         </is>
       </c>
       <c r="D155" t="n">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="156">
@@ -3485,7 +3485,7 @@
       </c>
       <c r="C192" t="inlineStr"/>
       <c r="D192" t="n">
-        <v>127</v>
+        <v>123</v>
       </c>
     </row>
     <row r="193">
@@ -3827,7 +3827,7 @@
         </is>
       </c>
       <c r="D213" t="n">
-        <v>144</v>
+        <v>150</v>
       </c>
     </row>
     <row r="214">

</xml_diff>

<commit_message>
data: field/odds refresh 2026-06-22 12:00 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>124</v>
+        <v>126</v>
       </c>
     </row>
     <row r="18">
@@ -873,7 +873,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="29">
@@ -1181,7 +1181,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>111</v>
+        <v>109</v>
       </c>
     </row>
     <row r="49">
@@ -1371,7 +1371,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="60">
@@ -1753,7 +1753,7 @@
         </is>
       </c>
       <c r="D83" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="84">
@@ -1885,7 +1885,7 @@
       </c>
       <c r="C91" t="inlineStr"/>
       <c r="D91" t="n">
-        <v>119</v>
+        <v>121</v>
       </c>
     </row>
     <row r="92">
@@ -2535,7 +2535,7 @@
         </is>
       </c>
       <c r="D132" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="133">
@@ -2883,7 +2883,7 @@
         </is>
       </c>
       <c r="D155" t="n">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="156">
@@ -3485,7 +3485,7 @@
       </c>
       <c r="C192" t="inlineStr"/>
       <c r="D192" t="n">
-        <v>127</v>
+        <v>123</v>
       </c>
     </row>
     <row r="193">
@@ -3827,7 +3827,7 @@
         </is>
       </c>
       <c r="D213" t="n">
-        <v>144</v>
+        <v>150</v>
       </c>
     </row>
     <row r="214">

</xml_diff>

<commit_message>
data: field/odds refresh 2026-06-22 12:25 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -465,7 +465,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3">
@@ -539,7 +539,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>46</v>
+        <v>50</v>
       </c>
     </row>
     <row r="8">
@@ -575,7 +575,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="10">
@@ -607,7 +607,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="12">
@@ -685,7 +685,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
     </row>
     <row r="17">
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="18">
@@ -747,7 +747,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="21">
@@ -855,7 +855,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>34</v>
+        <v>8</v>
       </c>
     </row>
     <row r="28">
@@ -873,7 +873,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="29">
@@ -905,7 +905,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="31">
@@ -1105,7 +1105,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="44">
@@ -1119,7 +1119,7 @@
       </c>
       <c r="C44" t="inlineStr"/>
       <c r="D44" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="45">
@@ -1163,7 +1163,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="48">
@@ -1181,7 +1181,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="49">
@@ -1249,7 +1249,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="53">
@@ -1281,7 +1281,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="55">
@@ -1299,7 +1299,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="56">
@@ -1335,7 +1335,7 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="58">
@@ -1371,7 +1371,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>107</v>
+        <v>109</v>
       </c>
     </row>
     <row r="60">
@@ -1417,7 +1417,7 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="63">
@@ -1453,7 +1453,7 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
     </row>
     <row r="65">
@@ -1529,7 +1529,7 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>66</v>
+        <v>70</v>
       </c>
     </row>
     <row r="70">
@@ -1559,7 +1559,7 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="72">
@@ -1753,7 +1753,7 @@
         </is>
       </c>
       <c r="D83" t="n">
-        <v>108</v>
+        <v>112</v>
       </c>
     </row>
     <row r="84">
@@ -1771,7 +1771,7 @@
         </is>
       </c>
       <c r="D84" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="85">
@@ -1871,7 +1871,7 @@
         </is>
       </c>
       <c r="D90" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="91">
@@ -1885,7 +1885,7 @@
       </c>
       <c r="C91" t="inlineStr"/>
       <c r="D91" t="n">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="92">
@@ -1921,7 +1921,7 @@
         </is>
       </c>
       <c r="D93" t="n">
-        <v>74</v>
+        <v>79</v>
       </c>
     </row>
     <row r="94">
@@ -2029,7 +2029,7 @@
         </is>
       </c>
       <c r="D100" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="101">
@@ -2047,7 +2047,7 @@
         </is>
       </c>
       <c r="D101" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="102">
@@ -2113,7 +2113,7 @@
         </is>
       </c>
       <c r="D105" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="106">
@@ -2145,7 +2145,7 @@
         </is>
       </c>
       <c r="D107" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="108">
@@ -2289,7 +2289,7 @@
         </is>
       </c>
       <c r="D117" t="n">
-        <v>35</v>
+        <v>39</v>
       </c>
     </row>
     <row r="118">
@@ -2351,7 +2351,7 @@
         </is>
       </c>
       <c r="D121" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="122">
@@ -2369,7 +2369,7 @@
         </is>
       </c>
       <c r="D122" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="123">
@@ -2427,7 +2427,7 @@
         </is>
       </c>
       <c r="D126" t="n">
-        <v>24</v>
+        <v>28</v>
       </c>
     </row>
     <row r="127">
@@ -2463,7 +2463,7 @@
         </is>
       </c>
       <c r="D128" t="n">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="129">
@@ -2517,7 +2517,7 @@
         </is>
       </c>
       <c r="D131" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="132">
@@ -2535,7 +2535,7 @@
         </is>
       </c>
       <c r="D132" t="n">
-        <v>87</v>
+        <v>90</v>
       </c>
     </row>
     <row r="133">
@@ -2569,7 +2569,7 @@
         </is>
       </c>
       <c r="D134" t="n">
-        <v>100</v>
+        <v>68</v>
       </c>
     </row>
     <row r="135">
@@ -2633,7 +2633,7 @@
         </is>
       </c>
       <c r="D138" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="139">
@@ -2711,7 +2711,7 @@
         </is>
       </c>
       <c r="D143" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
     </row>
     <row r="144">
@@ -2769,7 +2769,7 @@
         </is>
       </c>
       <c r="D147" t="n">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="148">
@@ -2883,7 +2883,7 @@
         </is>
       </c>
       <c r="D155" t="n">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="156">
@@ -2965,7 +2965,7 @@
         </is>
       </c>
       <c r="D160" t="n">
-        <v>38</v>
+        <v>32</v>
       </c>
     </row>
     <row r="161">
@@ -3051,7 +3051,7 @@
         </is>
       </c>
       <c r="D165" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="166">
@@ -3161,7 +3161,7 @@
         </is>
       </c>
       <c r="D172" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="173">
@@ -3269,7 +3269,7 @@
         </is>
       </c>
       <c r="D179" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="180">
@@ -3359,7 +3359,7 @@
         </is>
       </c>
       <c r="D184" t="n">
-        <v>49</v>
+        <v>52</v>
       </c>
     </row>
     <row r="185">
@@ -3437,7 +3437,7 @@
         </is>
       </c>
       <c r="D189" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="190">
@@ -3485,7 +3485,7 @@
       </c>
       <c r="C192" t="inlineStr"/>
       <c r="D192" t="n">
-        <v>123</v>
+        <v>121</v>
       </c>
     </row>
     <row r="193">
@@ -3503,7 +3503,7 @@
         </is>
       </c>
       <c r="D193" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="194">
@@ -3521,7 +3521,7 @@
         </is>
       </c>
       <c r="D194" t="n">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="195">
@@ -3553,7 +3553,7 @@
         </is>
       </c>
       <c r="D196" t="n">
-        <v>54</v>
+        <v>46</v>
       </c>
     </row>
     <row r="197">
@@ -3567,7 +3567,7 @@
       </c>
       <c r="C197" t="inlineStr"/>
       <c r="D197" t="n">
-        <v>54</v>
+        <v>46</v>
       </c>
     </row>
     <row r="198">
@@ -3585,7 +3585,7 @@
         </is>
       </c>
       <c r="D198" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
     </row>
     <row r="199">
@@ -3617,7 +3617,7 @@
       </c>
       <c r="C200" t="inlineStr"/>
       <c r="D200" t="n">
-        <v>128</v>
+        <v>130</v>
       </c>
     </row>
     <row r="201">
@@ -3663,7 +3663,7 @@
         </is>
       </c>
       <c r="D203" t="n">
-        <v>63</v>
+        <v>65</v>
       </c>
     </row>
     <row r="204">
@@ -3681,7 +3681,7 @@
         </is>
       </c>
       <c r="D204" t="n">
-        <v>83</v>
+        <v>73</v>
       </c>
     </row>
     <row r="205">
@@ -3699,7 +3699,7 @@
         </is>
       </c>
       <c r="D205" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="206">
@@ -3827,7 +3827,7 @@
         </is>
       </c>
       <c r="D213" t="n">
-        <v>150</v>
+        <v>154</v>
       </c>
     </row>
     <row r="214">
@@ -4023,7 +4023,7 @@
         </is>
       </c>
       <c r="D226" t="n">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="227">
@@ -4173,7 +4173,7 @@
         </is>
       </c>
       <c r="D235" t="n">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: field/odds refresh 2026-06-22 18:00 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -465,7 +465,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3">
@@ -539,7 +539,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>46</v>
+        <v>50</v>
       </c>
     </row>
     <row r="8">
@@ -575,7 +575,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="10">
@@ -607,7 +607,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="12">
@@ -685,7 +685,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
     </row>
     <row r="17">
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="18">
@@ -747,7 +747,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="21">
@@ -855,7 +855,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>34</v>
+        <v>8</v>
       </c>
     </row>
     <row r="28">
@@ -873,7 +873,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="29">
@@ -905,7 +905,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="31">
@@ -1105,7 +1105,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="44">
@@ -1119,7 +1119,7 @@
       </c>
       <c r="C44" t="inlineStr"/>
       <c r="D44" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="45">
@@ -1163,7 +1163,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="48">
@@ -1181,7 +1181,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="49">
@@ -1249,7 +1249,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="53">
@@ -1281,7 +1281,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="55">
@@ -1299,7 +1299,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="56">
@@ -1335,7 +1335,7 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="58">
@@ -1371,7 +1371,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>107</v>
+        <v>109</v>
       </c>
     </row>
     <row r="60">
@@ -1417,7 +1417,7 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="63">
@@ -1453,7 +1453,7 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
     </row>
     <row r="65">
@@ -1529,7 +1529,7 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>66</v>
+        <v>70</v>
       </c>
     </row>
     <row r="70">
@@ -1559,7 +1559,7 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="72">
@@ -1753,7 +1753,7 @@
         </is>
       </c>
       <c r="D83" t="n">
-        <v>108</v>
+        <v>112</v>
       </c>
     </row>
     <row r="84">
@@ -1771,7 +1771,7 @@
         </is>
       </c>
       <c r="D84" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="85">
@@ -1871,7 +1871,7 @@
         </is>
       </c>
       <c r="D90" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="91">
@@ -1885,7 +1885,7 @@
       </c>
       <c r="C91" t="inlineStr"/>
       <c r="D91" t="n">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="92">
@@ -1921,7 +1921,7 @@
         </is>
       </c>
       <c r="D93" t="n">
-        <v>74</v>
+        <v>79</v>
       </c>
     </row>
     <row r="94">
@@ -2029,7 +2029,7 @@
         </is>
       </c>
       <c r="D100" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="101">
@@ -2047,7 +2047,7 @@
         </is>
       </c>
       <c r="D101" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="102">
@@ -2113,7 +2113,7 @@
         </is>
       </c>
       <c r="D105" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="106">
@@ -2145,7 +2145,7 @@
         </is>
       </c>
       <c r="D107" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="108">
@@ -2289,7 +2289,7 @@
         </is>
       </c>
       <c r="D117" t="n">
-        <v>35</v>
+        <v>39</v>
       </c>
     </row>
     <row r="118">
@@ -2351,7 +2351,7 @@
         </is>
       </c>
       <c r="D121" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="122">
@@ -2369,7 +2369,7 @@
         </is>
       </c>
       <c r="D122" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="123">
@@ -2427,7 +2427,7 @@
         </is>
       </c>
       <c r="D126" t="n">
-        <v>24</v>
+        <v>28</v>
       </c>
     </row>
     <row r="127">
@@ -2463,7 +2463,7 @@
         </is>
       </c>
       <c r="D128" t="n">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="129">
@@ -2517,7 +2517,7 @@
         </is>
       </c>
       <c r="D131" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="132">
@@ -2535,7 +2535,7 @@
         </is>
       </c>
       <c r="D132" t="n">
-        <v>87</v>
+        <v>90</v>
       </c>
     </row>
     <row r="133">
@@ -2569,7 +2569,7 @@
         </is>
       </c>
       <c r="D134" t="n">
-        <v>100</v>
+        <v>68</v>
       </c>
     </row>
     <row r="135">
@@ -2633,7 +2633,7 @@
         </is>
       </c>
       <c r="D138" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="139">
@@ -2711,7 +2711,7 @@
         </is>
       </c>
       <c r="D143" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
     </row>
     <row r="144">
@@ -2769,7 +2769,7 @@
         </is>
       </c>
       <c r="D147" t="n">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="148">
@@ -2883,7 +2883,7 @@
         </is>
       </c>
       <c r="D155" t="n">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="156">
@@ -2965,7 +2965,7 @@
         </is>
       </c>
       <c r="D160" t="n">
-        <v>38</v>
+        <v>32</v>
       </c>
     </row>
     <row r="161">
@@ -3051,7 +3051,7 @@
         </is>
       </c>
       <c r="D165" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="166">
@@ -3161,7 +3161,7 @@
         </is>
       </c>
       <c r="D172" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="173">
@@ -3269,7 +3269,7 @@
         </is>
       </c>
       <c r="D179" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="180">
@@ -3359,7 +3359,7 @@
         </is>
       </c>
       <c r="D184" t="n">
-        <v>49</v>
+        <v>52</v>
       </c>
     </row>
     <row r="185">
@@ -3437,7 +3437,7 @@
         </is>
       </c>
       <c r="D189" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="190">
@@ -3485,7 +3485,7 @@
       </c>
       <c r="C192" t="inlineStr"/>
       <c r="D192" t="n">
-        <v>123</v>
+        <v>121</v>
       </c>
     </row>
     <row r="193">
@@ -3503,7 +3503,7 @@
         </is>
       </c>
       <c r="D193" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="194">
@@ -3521,7 +3521,7 @@
         </is>
       </c>
       <c r="D194" t="n">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="195">
@@ -3553,7 +3553,7 @@
         </is>
       </c>
       <c r="D196" t="n">
-        <v>54</v>
+        <v>46</v>
       </c>
     </row>
     <row r="197">
@@ -3567,7 +3567,7 @@
       </c>
       <c r="C197" t="inlineStr"/>
       <c r="D197" t="n">
-        <v>54</v>
+        <v>46</v>
       </c>
     </row>
     <row r="198">
@@ -3585,7 +3585,7 @@
         </is>
       </c>
       <c r="D198" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
     </row>
     <row r="199">
@@ -3617,7 +3617,7 @@
       </c>
       <c r="C200" t="inlineStr"/>
       <c r="D200" t="n">
-        <v>128</v>
+        <v>130</v>
       </c>
     </row>
     <row r="201">
@@ -3663,7 +3663,7 @@
         </is>
       </c>
       <c r="D203" t="n">
-        <v>63</v>
+        <v>65</v>
       </c>
     </row>
     <row r="204">
@@ -3681,7 +3681,7 @@
         </is>
       </c>
       <c r="D204" t="n">
-        <v>83</v>
+        <v>73</v>
       </c>
     </row>
     <row r="205">
@@ -3699,7 +3699,7 @@
         </is>
       </c>
       <c r="D205" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="206">
@@ -3827,7 +3827,7 @@
         </is>
       </c>
       <c r="D213" t="n">
-        <v>150</v>
+        <v>154</v>
       </c>
     </row>
     <row r="214">
@@ -4023,7 +4023,7 @@
         </is>
       </c>
       <c r="D226" t="n">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="227">
@@ -4173,7 +4173,7 @@
         </is>
       </c>
       <c r="D235" t="n">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: field/odds refresh 2026-06-29 11:26 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -557,7 +557,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
     <row r="9">
@@ -589,7 +589,7 @@
       </c>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="n">
-        <v>204</v>
+        <v>187</v>
       </c>
     </row>
     <row r="11">
@@ -837,7 +837,7 @@
       </c>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="n">
-        <v>249</v>
+        <v>257</v>
       </c>
     </row>
     <row r="27">
@@ -923,7 +923,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="32">
@@ -967,7 +967,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>203</v>
+        <v>209</v>
       </c>
     </row>
     <row r="35">
@@ -1087,7 +1087,7 @@
       </c>
       <c r="C42" t="inlineStr"/>
       <c r="D42" t="n">
-        <v>330</v>
+        <v>356</v>
       </c>
     </row>
     <row r="43">
@@ -1133,7 +1133,7 @@
       </c>
       <c r="C45" t="inlineStr"/>
       <c r="D45" t="n">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="46">
@@ -1195,7 +1195,7 @@
       </c>
       <c r="C49" t="inlineStr"/>
       <c r="D49" t="n">
-        <v>205</v>
+        <v>202</v>
       </c>
     </row>
     <row r="50">
@@ -1213,7 +1213,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>118</v>
+        <v>120</v>
       </c>
     </row>
     <row r="51">
@@ -1317,7 +1317,7 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>368</v>
+        <v>241</v>
       </c>
     </row>
     <row r="57">
@@ -1353,7 +1353,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>181</v>
+        <v>177</v>
       </c>
     </row>
     <row r="59">
@@ -1385,7 +1385,7 @@
       </c>
       <c r="C60" t="inlineStr"/>
       <c r="D60" t="n">
-        <v>325</v>
+        <v>354</v>
       </c>
     </row>
     <row r="61">
@@ -1435,7 +1435,7 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>68</v>
+        <v>71</v>
       </c>
     </row>
     <row r="64">
@@ -1467,7 +1467,7 @@
       </c>
       <c r="C65" t="inlineStr"/>
       <c r="D65" t="n">
-        <v>214</v>
+        <v>223</v>
       </c>
     </row>
     <row r="66">
@@ -1485,7 +1485,7 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>116</v>
+        <v>107</v>
       </c>
     </row>
     <row r="67">
@@ -1511,7 +1511,7 @@
       </c>
       <c r="C68" t="inlineStr"/>
       <c r="D68" t="n">
-        <v>265</v>
+        <v>250</v>
       </c>
     </row>
     <row r="69">
@@ -1639,7 +1639,7 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>92</v>
+        <v>102</v>
       </c>
     </row>
     <row r="77">
@@ -1653,7 +1653,7 @@
       </c>
       <c r="C77" t="inlineStr"/>
       <c r="D77" t="n">
-        <v>356</v>
+        <v>320</v>
       </c>
     </row>
     <row r="78">
@@ -1671,7 +1671,7 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>170</v>
+        <v>174</v>
       </c>
     </row>
     <row r="79">
@@ -1703,7 +1703,7 @@
       </c>
       <c r="C80" t="inlineStr"/>
       <c r="D80" t="n">
-        <v>154</v>
+        <v>157</v>
       </c>
     </row>
     <row r="81">
@@ -1721,7 +1721,7 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>88</v>
+        <v>92</v>
       </c>
     </row>
     <row r="82">
@@ -1807,7 +1807,7 @@
         </is>
       </c>
       <c r="D86" t="n">
-        <v>117</v>
+        <v>111</v>
       </c>
     </row>
     <row r="87">
@@ -1853,7 +1853,7 @@
       </c>
       <c r="C89" t="inlineStr"/>
       <c r="D89" t="n">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="90">
@@ -1903,7 +1903,7 @@
         </is>
       </c>
       <c r="D92" t="n">
-        <v>133</v>
+        <v>139</v>
       </c>
     </row>
     <row r="93">
@@ -1939,7 +1939,7 @@
         </is>
       </c>
       <c r="D94" t="n">
-        <v>95</v>
+        <v>99</v>
       </c>
     </row>
     <row r="95">
@@ -1971,7 +1971,7 @@
       </c>
       <c r="C96" t="inlineStr"/>
       <c r="D96" t="n">
-        <v>321</v>
+        <v>416</v>
       </c>
     </row>
     <row r="97">
@@ -1985,7 +1985,7 @@
       </c>
       <c r="C97" t="inlineStr"/>
       <c r="D97" t="n">
-        <v>156</v>
+        <v>152</v>
       </c>
     </row>
     <row r="98">
@@ -2011,7 +2011,7 @@
       </c>
       <c r="C99" t="inlineStr"/>
       <c r="D99" t="n">
-        <v>291</v>
+        <v>253</v>
       </c>
     </row>
     <row r="100">
@@ -2065,7 +2065,7 @@
         </is>
       </c>
       <c r="D102" t="n">
-        <v>141</v>
+        <v>64</v>
       </c>
     </row>
     <row r="103">
@@ -2127,7 +2127,7 @@
       </c>
       <c r="C106" t="inlineStr"/>
       <c r="D106" t="n">
-        <v>344</v>
+        <v>375</v>
       </c>
     </row>
     <row r="107">
@@ -2189,7 +2189,7 @@
       </c>
       <c r="C110" t="inlineStr"/>
       <c r="D110" t="n">
-        <v>184</v>
+        <v>168</v>
       </c>
     </row>
     <row r="111">
@@ -2207,7 +2207,7 @@
         </is>
       </c>
       <c r="D111" t="n">
-        <v>260</v>
+        <v>217</v>
       </c>
     </row>
     <row r="112">
@@ -2307,7 +2307,7 @@
         </is>
       </c>
       <c r="D118" t="n">
-        <v>102</v>
+        <v>106</v>
       </c>
     </row>
     <row r="119">
@@ -2333,7 +2333,7 @@
       </c>
       <c r="C120" t="inlineStr"/>
       <c r="D120" t="n">
-        <v>246</v>
+        <v>263</v>
       </c>
     </row>
     <row r="121">
@@ -2409,7 +2409,7 @@
       </c>
       <c r="C125" t="inlineStr"/>
       <c r="D125" t="n">
-        <v>459</v>
+        <v>479</v>
       </c>
     </row>
     <row r="126">
@@ -2481,7 +2481,7 @@
         </is>
       </c>
       <c r="D129" t="n">
-        <v>99</v>
+        <v>94</v>
       </c>
     </row>
     <row r="130">
@@ -2615,7 +2615,7 @@
         </is>
       </c>
       <c r="D137" t="n">
-        <v>145</v>
+        <v>140</v>
       </c>
     </row>
     <row r="138">
@@ -2647,7 +2647,7 @@
       </c>
       <c r="C139" t="inlineStr"/>
       <c r="D139" t="n">
-        <v>131</v>
+        <v>129</v>
       </c>
     </row>
     <row r="140">
@@ -2783,7 +2783,7 @@
       </c>
       <c r="C148" t="inlineStr"/>
       <c r="D148" t="n">
-        <v>128</v>
+        <v>133</v>
       </c>
     </row>
     <row r="149">
@@ -2847,7 +2847,7 @@
       </c>
       <c r="C153" t="inlineStr"/>
       <c r="D153" t="n">
-        <v>297</v>
+        <v>301</v>
       </c>
     </row>
     <row r="154">
@@ -2865,7 +2865,7 @@
         </is>
       </c>
       <c r="D154" t="n">
-        <v>279</v>
+        <v>264</v>
       </c>
     </row>
     <row r="155">
@@ -2933,7 +2933,7 @@
       </c>
       <c r="C158" t="inlineStr"/>
       <c r="D158" t="n">
-        <v>240</v>
+        <v>247</v>
       </c>
     </row>
     <row r="159">
@@ -2983,7 +2983,7 @@
         </is>
       </c>
       <c r="D161" t="n">
-        <v>80</v>
+        <v>74</v>
       </c>
     </row>
     <row r="162">
@@ -2997,7 +2997,7 @@
       </c>
       <c r="C162" t="inlineStr"/>
       <c r="D162" t="n">
-        <v>187</v>
+        <v>195</v>
       </c>
     </row>
     <row r="163">
@@ -3015,7 +3015,7 @@
         </is>
       </c>
       <c r="D163" t="n">
-        <v>85</v>
+        <v>88</v>
       </c>
     </row>
     <row r="164">
@@ -3065,7 +3065,7 @@
       </c>
       <c r="C166" t="inlineStr"/>
       <c r="D166" t="n">
-        <v>168</v>
+        <v>170</v>
       </c>
     </row>
     <row r="167">
@@ -3125,7 +3125,7 @@
         </is>
       </c>
       <c r="D170" t="n">
-        <v>162</v>
+        <v>167</v>
       </c>
     </row>
     <row r="171">
@@ -3143,7 +3143,7 @@
         </is>
       </c>
       <c r="D171" t="n">
-        <v>81</v>
+        <v>84</v>
       </c>
     </row>
     <row r="172">
@@ -3189,7 +3189,7 @@
       </c>
       <c r="C174" t="inlineStr"/>
       <c r="D174" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="175">
@@ -3305,7 +3305,7 @@
         </is>
       </c>
       <c r="D181" t="n">
-        <v>165</v>
+        <v>169</v>
       </c>
     </row>
     <row r="182">
@@ -3387,7 +3387,7 @@
       </c>
       <c r="C186" t="inlineStr"/>
       <c r="D186" t="n">
-        <v>262</v>
+        <v>273</v>
       </c>
     </row>
     <row r="187">
@@ -3405,7 +3405,7 @@
         </is>
       </c>
       <c r="D187" t="n">
-        <v>441</v>
+        <v>463</v>
       </c>
     </row>
     <row r="188">
@@ -3419,7 +3419,7 @@
       </c>
       <c r="C188" t="inlineStr"/>
       <c r="D188" t="n">
-        <v>283</v>
+        <v>271</v>
       </c>
     </row>
     <row r="189">
@@ -3535,7 +3535,7 @@
       </c>
       <c r="C195" t="inlineStr"/>
       <c r="D195" t="n">
-        <v>274</v>
+        <v>285</v>
       </c>
     </row>
     <row r="196">
@@ -3603,7 +3603,7 @@
         </is>
       </c>
       <c r="D199" t="n">
-        <v>425</v>
+        <v>420</v>
       </c>
     </row>
     <row r="200">
@@ -3631,7 +3631,7 @@
       </c>
       <c r="C201" t="inlineStr"/>
       <c r="D201" t="n">
-        <v>426</v>
+        <v>428</v>
       </c>
     </row>
     <row r="202">
@@ -3717,7 +3717,7 @@
         </is>
       </c>
       <c r="D206" t="n">
-        <v>138</v>
+        <v>148</v>
       </c>
     </row>
     <row r="207">
@@ -3735,7 +3735,7 @@
         </is>
       </c>
       <c r="D207" t="n">
-        <v>74</v>
+        <v>80</v>
       </c>
     </row>
     <row r="208">
@@ -3773,7 +3773,7 @@
       </c>
       <c r="C210" t="inlineStr"/>
       <c r="D210" t="n">
-        <v>364</v>
+        <v>379</v>
       </c>
     </row>
     <row r="211">
@@ -3809,7 +3809,7 @@
         </is>
       </c>
       <c r="D212" t="n">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
     <row r="213">
@@ -3853,7 +3853,7 @@
       </c>
       <c r="C215" t="inlineStr"/>
       <c r="D215" t="n">
-        <v>298</v>
+        <v>304</v>
       </c>
     </row>
     <row r="216">
@@ -3867,7 +3867,7 @@
       </c>
       <c r="C216" t="inlineStr"/>
       <c r="D216" t="n">
-        <v>298</v>
+        <v>304</v>
       </c>
     </row>
     <row r="217">
@@ -3885,7 +3885,7 @@
         </is>
       </c>
       <c r="D217" t="n">
-        <v>188</v>
+        <v>196</v>
       </c>
     </row>
     <row r="218">
@@ -3899,7 +3899,7 @@
       </c>
       <c r="C218" t="inlineStr"/>
       <c r="D218" t="n">
-        <v>461</v>
+        <v>495</v>
       </c>
     </row>
     <row r="219">
@@ -3913,7 +3913,7 @@
       </c>
       <c r="C219" t="inlineStr"/>
       <c r="D219" t="n">
-        <v>244</v>
+        <v>249</v>
       </c>
     </row>
     <row r="220">
@@ -3931,7 +3931,7 @@
         </is>
       </c>
       <c r="D220" t="n">
-        <v>76</v>
+        <v>83</v>
       </c>
     </row>
     <row r="221">
@@ -3967,7 +3967,7 @@
         </is>
       </c>
       <c r="D222" t="n">
-        <v>159</v>
+        <v>162</v>
       </c>
     </row>
     <row r="223">
@@ -4037,7 +4037,7 @@
       </c>
       <c r="C227" t="inlineStr"/>
       <c r="D227" t="n">
-        <v>386</v>
+        <v>379</v>
       </c>
     </row>
     <row r="228">
@@ -4069,7 +4069,7 @@
         </is>
       </c>
       <c r="D229" t="n">
-        <v>96</v>
+        <v>100</v>
       </c>
     </row>
     <row r="230">
@@ -4101,7 +4101,7 @@
       </c>
       <c r="C231" t="inlineStr"/>
       <c r="D231" t="n">
-        <v>169</v>
+        <v>182</v>
       </c>
     </row>
     <row r="232">
@@ -4119,7 +4119,7 @@
         </is>
       </c>
       <c r="D232" t="n">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="233">

</xml_diff>

<commit_message>
data: field/odds refresh 2026-06-29 14:02 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -539,7 +539,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>50</v>
+        <v>47</v>
       </c>
     </row>
     <row r="8">
@@ -557,7 +557,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="9">
@@ -639,7 +639,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="14">
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>127</v>
+        <v>128</v>
       </c>
     </row>
     <row r="18">
@@ -811,7 +811,7 @@
       </c>
       <c r="C24" t="inlineStr"/>
       <c r="D24" t="n">
-        <v>319</v>
+        <v>362</v>
       </c>
     </row>
     <row r="25">
@@ -837,7 +837,7 @@
       </c>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="n">
-        <v>257</v>
+        <v>270</v>
       </c>
     </row>
     <row r="27">
@@ -873,7 +873,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>66</v>
+        <v>69</v>
       </c>
     </row>
     <row r="29">
@@ -923,7 +923,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="32">
@@ -967,7 +967,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>209</v>
+        <v>211</v>
       </c>
     </row>
     <row r="35">
@@ -1087,7 +1087,7 @@
       </c>
       <c r="C42" t="inlineStr"/>
       <c r="D42" t="n">
-        <v>356</v>
+        <v>360</v>
       </c>
     </row>
     <row r="43">
@@ -1133,7 +1133,7 @@
       </c>
       <c r="C45" t="inlineStr"/>
       <c r="D45" t="n">
-        <v>176</v>
+        <v>180</v>
       </c>
     </row>
     <row r="46">
@@ -1181,7 +1181,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>110</v>
+        <v>113</v>
       </c>
     </row>
     <row r="49">
@@ -1195,7 +1195,7 @@
       </c>
       <c r="C49" t="inlineStr"/>
       <c r="D49" t="n">
-        <v>202</v>
+        <v>207</v>
       </c>
     </row>
     <row r="50">
@@ -1213,7 +1213,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>120</v>
+        <v>123</v>
       </c>
     </row>
     <row r="51">
@@ -1317,7 +1317,7 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>241</v>
+        <v>240</v>
       </c>
     </row>
     <row r="57">
@@ -1353,7 +1353,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>177</v>
+        <v>174</v>
       </c>
     </row>
     <row r="59">
@@ -1371,7 +1371,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>109</v>
+        <v>115</v>
       </c>
     </row>
     <row r="60">
@@ -1385,7 +1385,7 @@
       </c>
       <c r="C60" t="inlineStr"/>
       <c r="D60" t="n">
-        <v>354</v>
+        <v>362</v>
       </c>
     </row>
     <row r="61">
@@ -1417,7 +1417,7 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="63">
@@ -1435,7 +1435,7 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="64">
@@ -1453,7 +1453,7 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="65">
@@ -1467,7 +1467,7 @@
       </c>
       <c r="C65" t="inlineStr"/>
       <c r="D65" t="n">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="66">
@@ -1485,7 +1485,7 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>107</v>
+        <v>109</v>
       </c>
     </row>
     <row r="67">
@@ -1511,7 +1511,7 @@
       </c>
       <c r="C68" t="inlineStr"/>
       <c r="D68" t="n">
-        <v>250</v>
+        <v>262</v>
       </c>
     </row>
     <row r="69">
@@ -1639,7 +1639,7 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>102</v>
+        <v>104</v>
       </c>
     </row>
     <row r="77">
@@ -1653,7 +1653,7 @@
       </c>
       <c r="C77" t="inlineStr"/>
       <c r="D77" t="n">
-        <v>320</v>
+        <v>326</v>
       </c>
     </row>
     <row r="78">
@@ -1671,7 +1671,7 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>174</v>
+        <v>179</v>
       </c>
     </row>
     <row r="79">
@@ -1689,7 +1689,7 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="80">
@@ -1703,7 +1703,7 @@
       </c>
       <c r="C80" t="inlineStr"/>
       <c r="D80" t="n">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="81">
@@ -1753,7 +1753,7 @@
         </is>
       </c>
       <c r="D83" t="n">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="84">
@@ -1807,7 +1807,7 @@
         </is>
       </c>
       <c r="D86" t="n">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="87">
@@ -1853,7 +1853,7 @@
       </c>
       <c r="C89" t="inlineStr"/>
       <c r="D89" t="n">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="90">
@@ -1885,7 +1885,7 @@
       </c>
       <c r="C91" t="inlineStr"/>
       <c r="D91" t="n">
-        <v>122</v>
+        <v>127</v>
       </c>
     </row>
     <row r="92">
@@ -1903,7 +1903,7 @@
         </is>
       </c>
       <c r="D92" t="n">
-        <v>139</v>
+        <v>145</v>
       </c>
     </row>
     <row r="93">
@@ -1921,7 +1921,7 @@
         </is>
       </c>
       <c r="D93" t="n">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="94">
@@ -1939,7 +1939,7 @@
         </is>
       </c>
       <c r="D94" t="n">
-        <v>99</v>
+        <v>96</v>
       </c>
     </row>
     <row r="95">
@@ -1971,7 +1971,7 @@
       </c>
       <c r="C96" t="inlineStr"/>
       <c r="D96" t="n">
-        <v>416</v>
+        <v>430</v>
       </c>
     </row>
     <row r="97">
@@ -1985,7 +1985,7 @@
       </c>
       <c r="C97" t="inlineStr"/>
       <c r="D97" t="n">
-        <v>152</v>
+        <v>154</v>
       </c>
     </row>
     <row r="98">
@@ -2011,7 +2011,7 @@
       </c>
       <c r="C99" t="inlineStr"/>
       <c r="D99" t="n">
-        <v>253</v>
+        <v>256</v>
       </c>
     </row>
     <row r="100">
@@ -2029,7 +2029,7 @@
         </is>
       </c>
       <c r="D100" t="n">
-        <v>51</v>
+        <v>48</v>
       </c>
     </row>
     <row r="101">
@@ -2065,7 +2065,7 @@
         </is>
       </c>
       <c r="D102" t="n">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="103">
@@ -2127,7 +2127,7 @@
       </c>
       <c r="C106" t="inlineStr"/>
       <c r="D106" t="n">
-        <v>375</v>
+        <v>384</v>
       </c>
     </row>
     <row r="107">
@@ -2189,7 +2189,7 @@
       </c>
       <c r="C110" t="inlineStr"/>
       <c r="D110" t="n">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="111">
@@ -2207,7 +2207,7 @@
         </is>
       </c>
       <c r="D111" t="n">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="112">
@@ -2221,7 +2221,7 @@
       </c>
       <c r="C112" t="inlineStr"/>
       <c r="D112" t="n">
-        <v>179</v>
+        <v>181</v>
       </c>
     </row>
     <row r="113">
@@ -2307,7 +2307,7 @@
         </is>
       </c>
       <c r="D118" t="n">
-        <v>106</v>
+        <v>108</v>
       </c>
     </row>
     <row r="119">
@@ -2333,7 +2333,7 @@
       </c>
       <c r="C120" t="inlineStr"/>
       <c r="D120" t="n">
-        <v>263</v>
+        <v>265</v>
       </c>
     </row>
     <row r="121">
@@ -2409,7 +2409,7 @@
       </c>
       <c r="C125" t="inlineStr"/>
       <c r="D125" t="n">
-        <v>479</v>
+        <v>490</v>
       </c>
     </row>
     <row r="126">
@@ -2445,7 +2445,7 @@
         </is>
       </c>
       <c r="D127" t="n">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="128">
@@ -2535,7 +2535,7 @@
         </is>
       </c>
       <c r="D132" t="n">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="133">
@@ -2615,7 +2615,7 @@
         </is>
       </c>
       <c r="D137" t="n">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="138">
@@ -2769,7 +2769,7 @@
         </is>
       </c>
       <c r="D147" t="n">
-        <v>63</v>
+        <v>65</v>
       </c>
     </row>
     <row r="148">
@@ -2783,7 +2783,7 @@
       </c>
       <c r="C148" t="inlineStr"/>
       <c r="D148" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="149">
@@ -2847,7 +2847,7 @@
       </c>
       <c r="C153" t="inlineStr"/>
       <c r="D153" t="n">
-        <v>301</v>
+        <v>304</v>
       </c>
     </row>
     <row r="154">
@@ -2865,7 +2865,7 @@
         </is>
       </c>
       <c r="D154" t="n">
-        <v>264</v>
+        <v>269</v>
       </c>
     </row>
     <row r="155">
@@ -2933,7 +2933,7 @@
       </c>
       <c r="C158" t="inlineStr"/>
       <c r="D158" t="n">
-        <v>247</v>
+        <v>252</v>
       </c>
     </row>
     <row r="159">
@@ -2947,7 +2947,7 @@
       </c>
       <c r="C159" t="inlineStr"/>
       <c r="D159" t="n">
-        <v>172</v>
+        <v>173</v>
       </c>
     </row>
     <row r="160">
@@ -2997,7 +2997,7 @@
       </c>
       <c r="C162" t="inlineStr"/>
       <c r="D162" t="n">
-        <v>195</v>
+        <v>198</v>
       </c>
     </row>
     <row r="163">
@@ -3065,7 +3065,7 @@
       </c>
       <c r="C166" t="inlineStr"/>
       <c r="D166" t="n">
-        <v>170</v>
+        <v>172</v>
       </c>
     </row>
     <row r="167">
@@ -3143,7 +3143,7 @@
         </is>
       </c>
       <c r="D171" t="n">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="172">
@@ -3189,7 +3189,7 @@
       </c>
       <c r="C174" t="inlineStr"/>
       <c r="D174" t="n">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="175">
@@ -3305,7 +3305,7 @@
         </is>
       </c>
       <c r="D181" t="n">
-        <v>169</v>
+        <v>171</v>
       </c>
     </row>
     <row r="182">
@@ -3387,7 +3387,7 @@
       </c>
       <c r="C186" t="inlineStr"/>
       <c r="D186" t="n">
-        <v>273</v>
+        <v>276</v>
       </c>
     </row>
     <row r="187">
@@ -3405,7 +3405,7 @@
         </is>
       </c>
       <c r="D187" t="n">
-        <v>463</v>
+        <v>476</v>
       </c>
     </row>
     <row r="188">
@@ -3521,7 +3521,7 @@
         </is>
       </c>
       <c r="D194" t="n">
-        <v>49</v>
+        <v>53</v>
       </c>
     </row>
     <row r="195">
@@ -3535,7 +3535,7 @@
       </c>
       <c r="C195" t="inlineStr"/>
       <c r="D195" t="n">
-        <v>285</v>
+        <v>287</v>
       </c>
     </row>
     <row r="196">
@@ -3603,7 +3603,7 @@
         </is>
       </c>
       <c r="D199" t="n">
-        <v>420</v>
+        <v>437</v>
       </c>
     </row>
     <row r="200">
@@ -3617,7 +3617,7 @@
       </c>
       <c r="C200" t="inlineStr"/>
       <c r="D200" t="n">
-        <v>130</v>
+        <v>126</v>
       </c>
     </row>
     <row r="201">
@@ -3631,7 +3631,7 @@
       </c>
       <c r="C201" t="inlineStr"/>
       <c r="D201" t="n">
-        <v>428</v>
+        <v>438</v>
       </c>
     </row>
     <row r="202">
@@ -3735,7 +3735,7 @@
         </is>
       </c>
       <c r="D207" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
     </row>
     <row r="208">
@@ -3809,7 +3809,7 @@
         </is>
       </c>
       <c r="D212" t="n">
-        <v>181</v>
+        <v>183</v>
       </c>
     </row>
     <row r="213">
@@ -3827,7 +3827,7 @@
         </is>
       </c>
       <c r="D213" t="n">
-        <v>154</v>
+        <v>156</v>
       </c>
     </row>
     <row r="214">
@@ -3853,7 +3853,7 @@
       </c>
       <c r="C215" t="inlineStr"/>
       <c r="D215" t="n">
-        <v>304</v>
+        <v>311</v>
       </c>
     </row>
     <row r="216">
@@ -3867,7 +3867,7 @@
       </c>
       <c r="C216" t="inlineStr"/>
       <c r="D216" t="n">
-        <v>304</v>
+        <v>311</v>
       </c>
     </row>
     <row r="217">
@@ -3913,7 +3913,7 @@
       </c>
       <c r="C219" t="inlineStr"/>
       <c r="D219" t="n">
-        <v>249</v>
+        <v>254</v>
       </c>
     </row>
     <row r="220">
@@ -3931,7 +3931,7 @@
         </is>
       </c>
       <c r="D220" t="n">
-        <v>83</v>
+        <v>70</v>
       </c>
     </row>
     <row r="221">
@@ -3967,7 +3967,7 @@
         </is>
       </c>
       <c r="D222" t="n">
-        <v>162</v>
+        <v>166</v>
       </c>
     </row>
     <row r="223">
@@ -4037,7 +4037,7 @@
       </c>
       <c r="C227" t="inlineStr"/>
       <c r="D227" t="n">
-        <v>379</v>
+        <v>377</v>
       </c>
     </row>
     <row r="228">
@@ -4069,7 +4069,7 @@
         </is>
       </c>
       <c r="D229" t="n">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="230">
@@ -4101,7 +4101,7 @@
       </c>
       <c r="C231" t="inlineStr"/>
       <c r="D231" t="n">
-        <v>182</v>
+        <v>175</v>
       </c>
     </row>
     <row r="232">
@@ -4119,7 +4119,7 @@
         </is>
       </c>
       <c r="D232" t="n">
-        <v>125</v>
+        <v>130</v>
       </c>
     </row>
     <row r="233">

</xml_diff>

<commit_message>
data: field/odds refresh 2026-06-29 18:01 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -539,7 +539,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>50</v>
+        <v>47</v>
       </c>
     </row>
     <row r="8">
@@ -557,7 +557,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>96</v>
+        <v>100</v>
       </c>
     </row>
     <row r="9">
@@ -589,7 +589,7 @@
       </c>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="n">
-        <v>204</v>
+        <v>187</v>
       </c>
     </row>
     <row r="11">
@@ -639,7 +639,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="14">
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>127</v>
+        <v>128</v>
       </c>
     </row>
     <row r="18">
@@ -811,7 +811,7 @@
       </c>
       <c r="C24" t="inlineStr"/>
       <c r="D24" t="n">
-        <v>319</v>
+        <v>362</v>
       </c>
     </row>
     <row r="25">
@@ -837,7 +837,7 @@
       </c>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="n">
-        <v>249</v>
+        <v>270</v>
       </c>
     </row>
     <row r="27">
@@ -873,7 +873,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>66</v>
+        <v>69</v>
       </c>
     </row>
     <row r="29">
@@ -923,7 +923,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="32">
@@ -967,7 +967,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>203</v>
+        <v>211</v>
       </c>
     </row>
     <row r="35">
@@ -1087,7 +1087,7 @@
       </c>
       <c r="C42" t="inlineStr"/>
       <c r="D42" t="n">
-        <v>330</v>
+        <v>360</v>
       </c>
     </row>
     <row r="43">
@@ -1133,7 +1133,7 @@
       </c>
       <c r="C45" t="inlineStr"/>
       <c r="D45" t="n">
-        <v>175</v>
+        <v>180</v>
       </c>
     </row>
     <row r="46">
@@ -1181,7 +1181,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>110</v>
+        <v>113</v>
       </c>
     </row>
     <row r="49">
@@ -1195,7 +1195,7 @@
       </c>
       <c r="C49" t="inlineStr"/>
       <c r="D49" t="n">
-        <v>205</v>
+        <v>207</v>
       </c>
     </row>
     <row r="50">
@@ -1213,7 +1213,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>118</v>
+        <v>123</v>
       </c>
     </row>
     <row r="51">
@@ -1317,7 +1317,7 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>368</v>
+        <v>240</v>
       </c>
     </row>
     <row r="57">
@@ -1353,7 +1353,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>181</v>
+        <v>174</v>
       </c>
     </row>
     <row r="59">
@@ -1371,7 +1371,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>109</v>
+        <v>115</v>
       </c>
     </row>
     <row r="60">
@@ -1385,7 +1385,7 @@
       </c>
       <c r="C60" t="inlineStr"/>
       <c r="D60" t="n">
-        <v>325</v>
+        <v>362</v>
       </c>
     </row>
     <row r="61">
@@ -1417,7 +1417,7 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="63">
@@ -1435,7 +1435,7 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>68</v>
+        <v>73</v>
       </c>
     </row>
     <row r="64">
@@ -1453,7 +1453,7 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="65">
@@ -1467,7 +1467,7 @@
       </c>
       <c r="C65" t="inlineStr"/>
       <c r="D65" t="n">
-        <v>214</v>
+        <v>222</v>
       </c>
     </row>
     <row r="66">
@@ -1485,7 +1485,7 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>116</v>
+        <v>109</v>
       </c>
     </row>
     <row r="67">
@@ -1511,7 +1511,7 @@
       </c>
       <c r="C68" t="inlineStr"/>
       <c r="D68" t="n">
-        <v>265</v>
+        <v>262</v>
       </c>
     </row>
     <row r="69">
@@ -1639,7 +1639,7 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>92</v>
+        <v>104</v>
       </c>
     </row>
     <row r="77">
@@ -1653,7 +1653,7 @@
       </c>
       <c r="C77" t="inlineStr"/>
       <c r="D77" t="n">
-        <v>356</v>
+        <v>326</v>
       </c>
     </row>
     <row r="78">
@@ -1671,7 +1671,7 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>170</v>
+        <v>179</v>
       </c>
     </row>
     <row r="79">
@@ -1689,7 +1689,7 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="80">
@@ -1703,7 +1703,7 @@
       </c>
       <c r="C80" t="inlineStr"/>
       <c r="D80" t="n">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="81">
@@ -1721,7 +1721,7 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>88</v>
+        <v>92</v>
       </c>
     </row>
     <row r="82">
@@ -1753,7 +1753,7 @@
         </is>
       </c>
       <c r="D83" t="n">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="84">
@@ -1807,7 +1807,7 @@
         </is>
       </c>
       <c r="D86" t="n">
-        <v>117</v>
+        <v>112</v>
       </c>
     </row>
     <row r="87">
@@ -1853,7 +1853,7 @@
       </c>
       <c r="C89" t="inlineStr"/>
       <c r="D89" t="n">
-        <v>160</v>
+        <v>158</v>
       </c>
     </row>
     <row r="90">
@@ -1885,7 +1885,7 @@
       </c>
       <c r="C91" t="inlineStr"/>
       <c r="D91" t="n">
-        <v>122</v>
+        <v>127</v>
       </c>
     </row>
     <row r="92">
@@ -1903,7 +1903,7 @@
         </is>
       </c>
       <c r="D92" t="n">
-        <v>133</v>
+        <v>145</v>
       </c>
     </row>
     <row r="93">
@@ -1921,7 +1921,7 @@
         </is>
       </c>
       <c r="D93" t="n">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="94">
@@ -1939,7 +1939,7 @@
         </is>
       </c>
       <c r="D94" t="n">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
     <row r="95">
@@ -1971,7 +1971,7 @@
       </c>
       <c r="C96" t="inlineStr"/>
       <c r="D96" t="n">
-        <v>321</v>
+        <v>430</v>
       </c>
     </row>
     <row r="97">
@@ -1985,7 +1985,7 @@
       </c>
       <c r="C97" t="inlineStr"/>
       <c r="D97" t="n">
-        <v>156</v>
+        <v>154</v>
       </c>
     </row>
     <row r="98">
@@ -2011,7 +2011,7 @@
       </c>
       <c r="C99" t="inlineStr"/>
       <c r="D99" t="n">
-        <v>291</v>
+        <v>256</v>
       </c>
     </row>
     <row r="100">
@@ -2029,7 +2029,7 @@
         </is>
       </c>
       <c r="D100" t="n">
-        <v>51</v>
+        <v>48</v>
       </c>
     </row>
     <row r="101">
@@ -2065,7 +2065,7 @@
         </is>
       </c>
       <c r="D102" t="n">
-        <v>141</v>
+        <v>66</v>
       </c>
     </row>
     <row r="103">
@@ -2127,7 +2127,7 @@
       </c>
       <c r="C106" t="inlineStr"/>
       <c r="D106" t="n">
-        <v>344</v>
+        <v>384</v>
       </c>
     </row>
     <row r="107">
@@ -2189,7 +2189,7 @@
       </c>
       <c r="C110" t="inlineStr"/>
       <c r="D110" t="n">
-        <v>184</v>
+        <v>169</v>
       </c>
     </row>
     <row r="111">
@@ -2207,7 +2207,7 @@
         </is>
       </c>
       <c r="D111" t="n">
-        <v>260</v>
+        <v>218</v>
       </c>
     </row>
     <row r="112">
@@ -2221,7 +2221,7 @@
       </c>
       <c r="C112" t="inlineStr"/>
       <c r="D112" t="n">
-        <v>179</v>
+        <v>181</v>
       </c>
     </row>
     <row r="113">
@@ -2307,7 +2307,7 @@
         </is>
       </c>
       <c r="D118" t="n">
-        <v>102</v>
+        <v>108</v>
       </c>
     </row>
     <row r="119">
@@ -2333,7 +2333,7 @@
       </c>
       <c r="C120" t="inlineStr"/>
       <c r="D120" t="n">
-        <v>246</v>
+        <v>265</v>
       </c>
     </row>
     <row r="121">
@@ -2409,7 +2409,7 @@
       </c>
       <c r="C125" t="inlineStr"/>
       <c r="D125" t="n">
-        <v>459</v>
+        <v>490</v>
       </c>
     </row>
     <row r="126">
@@ -2445,7 +2445,7 @@
         </is>
       </c>
       <c r="D127" t="n">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="128">
@@ -2481,7 +2481,7 @@
         </is>
       </c>
       <c r="D129" t="n">
-        <v>99</v>
+        <v>94</v>
       </c>
     </row>
     <row r="130">
@@ -2535,7 +2535,7 @@
         </is>
       </c>
       <c r="D132" t="n">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="133">
@@ -2615,7 +2615,7 @@
         </is>
       </c>
       <c r="D137" t="n">
-        <v>145</v>
+        <v>138</v>
       </c>
     </row>
     <row r="138">
@@ -2647,7 +2647,7 @@
       </c>
       <c r="C139" t="inlineStr"/>
       <c r="D139" t="n">
-        <v>131</v>
+        <v>129</v>
       </c>
     </row>
     <row r="140">
@@ -2769,7 +2769,7 @@
         </is>
       </c>
       <c r="D147" t="n">
-        <v>63</v>
+        <v>65</v>
       </c>
     </row>
     <row r="148">
@@ -2783,7 +2783,7 @@
       </c>
       <c r="C148" t="inlineStr"/>
       <c r="D148" t="n">
-        <v>128</v>
+        <v>134</v>
       </c>
     </row>
     <row r="149">
@@ -2847,7 +2847,7 @@
       </c>
       <c r="C153" t="inlineStr"/>
       <c r="D153" t="n">
-        <v>297</v>
+        <v>304</v>
       </c>
     </row>
     <row r="154">
@@ -2865,7 +2865,7 @@
         </is>
       </c>
       <c r="D154" t="n">
-        <v>279</v>
+        <v>269</v>
       </c>
     </row>
     <row r="155">
@@ -2933,7 +2933,7 @@
       </c>
       <c r="C158" t="inlineStr"/>
       <c r="D158" t="n">
-        <v>240</v>
+        <v>252</v>
       </c>
     </row>
     <row r="159">
@@ -2947,7 +2947,7 @@
       </c>
       <c r="C159" t="inlineStr"/>
       <c r="D159" t="n">
-        <v>172</v>
+        <v>173</v>
       </c>
     </row>
     <row r="160">
@@ -2983,7 +2983,7 @@
         </is>
       </c>
       <c r="D161" t="n">
-        <v>80</v>
+        <v>74</v>
       </c>
     </row>
     <row r="162">
@@ -2997,7 +2997,7 @@
       </c>
       <c r="C162" t="inlineStr"/>
       <c r="D162" t="n">
-        <v>187</v>
+        <v>198</v>
       </c>
     </row>
     <row r="163">
@@ -3015,7 +3015,7 @@
         </is>
       </c>
       <c r="D163" t="n">
-        <v>85</v>
+        <v>88</v>
       </c>
     </row>
     <row r="164">
@@ -3065,7 +3065,7 @@
       </c>
       <c r="C166" t="inlineStr"/>
       <c r="D166" t="n">
-        <v>168</v>
+        <v>172</v>
       </c>
     </row>
     <row r="167">
@@ -3125,7 +3125,7 @@
         </is>
       </c>
       <c r="D170" t="n">
-        <v>162</v>
+        <v>167</v>
       </c>
     </row>
     <row r="171">
@@ -3143,7 +3143,7 @@
         </is>
       </c>
       <c r="D171" t="n">
-        <v>81</v>
+        <v>85</v>
       </c>
     </row>
     <row r="172">
@@ -3189,7 +3189,7 @@
       </c>
       <c r="C174" t="inlineStr"/>
       <c r="D174" t="n">
-        <v>133</v>
+        <v>135</v>
       </c>
     </row>
     <row r="175">
@@ -3305,7 +3305,7 @@
         </is>
       </c>
       <c r="D181" t="n">
-        <v>165</v>
+        <v>171</v>
       </c>
     </row>
     <row r="182">
@@ -3387,7 +3387,7 @@
       </c>
       <c r="C186" t="inlineStr"/>
       <c r="D186" t="n">
-        <v>262</v>
+        <v>276</v>
       </c>
     </row>
     <row r="187">
@@ -3405,7 +3405,7 @@
         </is>
       </c>
       <c r="D187" t="n">
-        <v>441</v>
+        <v>476</v>
       </c>
     </row>
     <row r="188">
@@ -3419,7 +3419,7 @@
       </c>
       <c r="C188" t="inlineStr"/>
       <c r="D188" t="n">
-        <v>283</v>
+        <v>271</v>
       </c>
     </row>
     <row r="189">
@@ -3521,7 +3521,7 @@
         </is>
       </c>
       <c r="D194" t="n">
-        <v>49</v>
+        <v>53</v>
       </c>
     </row>
     <row r="195">
@@ -3535,7 +3535,7 @@
       </c>
       <c r="C195" t="inlineStr"/>
       <c r="D195" t="n">
-        <v>274</v>
+        <v>287</v>
       </c>
     </row>
     <row r="196">
@@ -3603,7 +3603,7 @@
         </is>
       </c>
       <c r="D199" t="n">
-        <v>425</v>
+        <v>437</v>
       </c>
     </row>
     <row r="200">
@@ -3617,7 +3617,7 @@
       </c>
       <c r="C200" t="inlineStr"/>
       <c r="D200" t="n">
-        <v>130</v>
+        <v>126</v>
       </c>
     </row>
     <row r="201">
@@ -3631,7 +3631,7 @@
       </c>
       <c r="C201" t="inlineStr"/>
       <c r="D201" t="n">
-        <v>426</v>
+        <v>438</v>
       </c>
     </row>
     <row r="202">
@@ -3717,7 +3717,7 @@
         </is>
       </c>
       <c r="D206" t="n">
-        <v>138</v>
+        <v>148</v>
       </c>
     </row>
     <row r="207">
@@ -3735,7 +3735,7 @@
         </is>
       </c>
       <c r="D207" t="n">
-        <v>74</v>
+        <v>82</v>
       </c>
     </row>
     <row r="208">
@@ -3773,7 +3773,7 @@
       </c>
       <c r="C210" t="inlineStr"/>
       <c r="D210" t="n">
-        <v>364</v>
+        <v>379</v>
       </c>
     </row>
     <row r="211">
@@ -3809,7 +3809,7 @@
         </is>
       </c>
       <c r="D212" t="n">
-        <v>180</v>
+        <v>183</v>
       </c>
     </row>
     <row r="213">
@@ -3827,7 +3827,7 @@
         </is>
       </c>
       <c r="D213" t="n">
-        <v>154</v>
+        <v>156</v>
       </c>
     </row>
     <row r="214">
@@ -3853,7 +3853,7 @@
       </c>
       <c r="C215" t="inlineStr"/>
       <c r="D215" t="n">
-        <v>298</v>
+        <v>311</v>
       </c>
     </row>
     <row r="216">
@@ -3867,7 +3867,7 @@
       </c>
       <c r="C216" t="inlineStr"/>
       <c r="D216" t="n">
-        <v>298</v>
+        <v>311</v>
       </c>
     </row>
     <row r="217">
@@ -3885,7 +3885,7 @@
         </is>
       </c>
       <c r="D217" t="n">
-        <v>188</v>
+        <v>196</v>
       </c>
     </row>
     <row r="218">
@@ -3899,7 +3899,7 @@
       </c>
       <c r="C218" t="inlineStr"/>
       <c r="D218" t="n">
-        <v>461</v>
+        <v>495</v>
       </c>
     </row>
     <row r="219">
@@ -3913,7 +3913,7 @@
       </c>
       <c r="C219" t="inlineStr"/>
       <c r="D219" t="n">
-        <v>244</v>
+        <v>254</v>
       </c>
     </row>
     <row r="220">
@@ -3931,7 +3931,7 @@
         </is>
       </c>
       <c r="D220" t="n">
-        <v>76</v>
+        <v>70</v>
       </c>
     </row>
     <row r="221">
@@ -3967,7 +3967,7 @@
         </is>
       </c>
       <c r="D222" t="n">
-        <v>159</v>
+        <v>166</v>
       </c>
     </row>
     <row r="223">
@@ -4037,7 +4037,7 @@
       </c>
       <c r="C227" t="inlineStr"/>
       <c r="D227" t="n">
-        <v>386</v>
+        <v>377</v>
       </c>
     </row>
     <row r="228">
@@ -4069,7 +4069,7 @@
         </is>
       </c>
       <c r="D229" t="n">
-        <v>96</v>
+        <v>99</v>
       </c>
     </row>
     <row r="230">
@@ -4101,7 +4101,7 @@
       </c>
       <c r="C231" t="inlineStr"/>
       <c r="D231" t="n">
-        <v>169</v>
+        <v>175</v>
       </c>
     </row>
     <row r="232">
@@ -4119,7 +4119,7 @@
         </is>
       </c>
       <c r="D232" t="n">
-        <v>127</v>
+        <v>130</v>
       </c>
     </row>
     <row r="233">

</xml_diff>

<commit_message>
data: field/odds refresh 2026-07-06 06:51 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -465,7 +465,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>14</v>
+        <v>19</v>
       </c>
     </row>
     <row r="3">
@@ -729,7 +729,7 @@
       </c>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="n">
-        <v>151</v>
+        <v>144</v>
       </c>
     </row>
     <row r="20">
@@ -747,7 +747,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="21">
@@ -855,7 +855,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="28">
@@ -905,7 +905,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>55</v>
+        <v>50</v>
       </c>
     </row>
     <row r="31">
@@ -985,7 +985,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>295</v>
+        <v>320</v>
       </c>
     </row>
     <row r="36">
@@ -1105,7 +1105,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="44">
@@ -1119,7 +1119,7 @@
       </c>
       <c r="C44" t="inlineStr"/>
       <c r="D44" t="n">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="45">
@@ -1163,7 +1163,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>24</v>
+        <v>29</v>
       </c>
     </row>
     <row r="48">
@@ -1299,7 +1299,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="56">
@@ -1335,7 +1335,7 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="58">
@@ -1529,7 +1529,7 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="70">
@@ -1559,7 +1559,7 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>58</v>
+        <v>61</v>
       </c>
     </row>
     <row r="72">
@@ -1734,9 +1734,7 @@
         <v>5768</v>
       </c>
       <c r="C82" t="inlineStr"/>
-      <c r="D82" t="n">
-        <v>482</v>
-      </c>
+      <c r="D82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -1771,7 +1769,7 @@
         </is>
       </c>
       <c r="D84" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="85">
@@ -1789,7 +1787,7 @@
         </is>
       </c>
       <c r="D85" t="n">
-        <v>70</v>
+        <v>84</v>
       </c>
     </row>
     <row r="86">
@@ -1825,7 +1823,7 @@
         </is>
       </c>
       <c r="D87" t="n">
-        <v>135</v>
+        <v>149</v>
       </c>
     </row>
     <row r="88">
@@ -1839,7 +1837,7 @@
       </c>
       <c r="C88" t="inlineStr"/>
       <c r="D88" t="n">
-        <v>353</v>
+        <v>465</v>
       </c>
     </row>
     <row r="89">
@@ -1871,7 +1869,7 @@
         </is>
       </c>
       <c r="D90" t="n">
-        <v>30</v>
+        <v>12</v>
       </c>
     </row>
     <row r="91">
@@ -2047,7 +2045,7 @@
         </is>
       </c>
       <c r="D101" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="102">
@@ -2083,7 +2081,7 @@
         </is>
       </c>
       <c r="D103" t="n">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="104">
@@ -2175,7 +2173,7 @@
         </is>
       </c>
       <c r="D109" t="n">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
     <row r="110">
@@ -2259,7 +2257,7 @@
       </c>
       <c r="C115" t="inlineStr"/>
       <c r="D115" t="n">
-        <v>80</v>
+        <v>152</v>
       </c>
     </row>
     <row r="116">
@@ -2369,7 +2367,7 @@
         </is>
       </c>
       <c r="D122" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="123">
@@ -2395,7 +2393,7 @@
       </c>
       <c r="C124" t="inlineStr"/>
       <c r="D124" t="n">
-        <v>226</v>
+        <v>330</v>
       </c>
     </row>
     <row r="125">
@@ -2463,7 +2461,7 @@
         </is>
       </c>
       <c r="D128" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="129">
@@ -2583,7 +2581,7 @@
       </c>
       <c r="C135" t="inlineStr"/>
       <c r="D135" t="n">
-        <v>280</v>
+        <v>293</v>
       </c>
     </row>
     <row r="136">
@@ -2675,7 +2673,7 @@
       </c>
       <c r="C141" t="inlineStr"/>
       <c r="D141" t="n">
-        <v>82</v>
+        <v>87</v>
       </c>
     </row>
     <row r="142">
@@ -2711,7 +2709,7 @@
         </is>
       </c>
       <c r="D143" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="144">
@@ -2725,7 +2723,7 @@
       </c>
       <c r="C144" t="inlineStr"/>
       <c r="D144" t="n">
-        <v>275</v>
+        <v>263</v>
       </c>
     </row>
     <row r="145">
@@ -2901,7 +2899,7 @@
         </is>
       </c>
       <c r="D156" t="n">
-        <v>40</v>
+        <v>51</v>
       </c>
     </row>
     <row r="157">
@@ -2919,7 +2917,7 @@
         </is>
       </c>
       <c r="D157" t="n">
-        <v>153</v>
+        <v>212</v>
       </c>
     </row>
     <row r="158">
@@ -3033,7 +3031,7 @@
         </is>
       </c>
       <c r="D164" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
     <row r="165">
@@ -3051,7 +3049,7 @@
         </is>
       </c>
       <c r="D165" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="166">
@@ -3095,7 +3093,7 @@
         </is>
       </c>
       <c r="D168" t="n">
-        <v>27</v>
+        <v>31</v>
       </c>
     </row>
     <row r="169">
@@ -3207,7 +3205,7 @@
         </is>
       </c>
       <c r="D175" t="n">
-        <v>163</v>
+        <v>203</v>
       </c>
     </row>
     <row r="176">
@@ -3269,7 +3267,7 @@
         </is>
       </c>
       <c r="D179" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="180">
@@ -3323,7 +3321,7 @@
         </is>
       </c>
       <c r="D182" t="n">
-        <v>71</v>
+        <v>80</v>
       </c>
     </row>
     <row r="183">
@@ -3341,7 +3339,7 @@
         </is>
       </c>
       <c r="D183" t="n">
-        <v>71</v>
+        <v>80</v>
       </c>
     </row>
     <row r="184">
@@ -3359,7 +3357,7 @@
         </is>
       </c>
       <c r="D184" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
     </row>
     <row r="185">
@@ -3503,7 +3501,7 @@
         </is>
       </c>
       <c r="D193" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="194">
@@ -3585,7 +3583,7 @@
         </is>
       </c>
       <c r="D198" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="199">
@@ -3645,7 +3643,7 @@
       </c>
       <c r="C202" t="inlineStr"/>
       <c r="D202" t="n">
-        <v>196</v>
+        <v>162</v>
       </c>
     </row>
     <row r="203">
@@ -3663,7 +3661,7 @@
         </is>
       </c>
       <c r="D203" t="n">
-        <v>65</v>
+        <v>67</v>
       </c>
     </row>
     <row r="204">
@@ -3681,7 +3679,7 @@
         </is>
       </c>
       <c r="D204" t="n">
-        <v>73</v>
+        <v>76</v>
       </c>
     </row>
     <row r="205">
@@ -3949,7 +3947,7 @@
         </is>
       </c>
       <c r="D221" t="n">
-        <v>311</v>
+        <v>338</v>
       </c>
     </row>
     <row r="222">
@@ -3993,7 +3991,7 @@
       </c>
       <c r="C224" t="inlineStr"/>
       <c r="D224" t="n">
-        <v>369</v>
+        <v>391</v>
       </c>
     </row>
     <row r="225">
@@ -4155,7 +4153,7 @@
         </is>
       </c>
       <c r="D234" t="n">
-        <v>72</v>
+        <v>83</v>
       </c>
     </row>
     <row r="235">
@@ -4173,7 +4171,7 @@
         </is>
       </c>
       <c r="D235" t="n">
-        <v>67</v>
+        <v>62</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: field/odds refresh 2026-07-06 10:54 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>128</v>
+        <v>134</v>
       </c>
     </row>
     <row r="18">
@@ -729,7 +729,7 @@
       </c>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="n">
-        <v>144</v>
+        <v>149</v>
       </c>
     </row>
     <row r="20">
@@ -779,7 +779,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>97</v>
+        <v>99</v>
       </c>
     </row>
     <row r="23">
@@ -797,7 +797,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="24">
@@ -855,7 +855,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="28">
@@ -873,7 +873,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="29">
@@ -905,7 +905,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="31">
@@ -923,7 +923,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="32">
@@ -985,7 +985,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>320</v>
+        <v>336</v>
       </c>
     </row>
     <row r="36">
@@ -1105,7 +1105,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="44">
@@ -1119,7 +1119,7 @@
       </c>
       <c r="C44" t="inlineStr"/>
       <c r="D44" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="45">
@@ -1133,7 +1133,7 @@
       </c>
       <c r="C45" t="inlineStr"/>
       <c r="D45" t="n">
-        <v>180</v>
+        <v>189</v>
       </c>
     </row>
     <row r="46">
@@ -1249,7 +1249,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="53">
@@ -1353,7 +1353,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>174</v>
+        <v>155</v>
       </c>
     </row>
     <row r="59">
@@ -1417,7 +1417,7 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
     </row>
     <row r="63">
@@ -1435,7 +1435,7 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>73</v>
+        <v>75</v>
       </c>
     </row>
     <row r="64">
@@ -1559,7 +1559,7 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="72">
@@ -1671,7 +1671,7 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>179</v>
+        <v>186</v>
       </c>
     </row>
     <row r="79">
@@ -1787,7 +1787,7 @@
         </is>
       </c>
       <c r="D85" t="n">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="86">
@@ -1823,7 +1823,7 @@
         </is>
       </c>
       <c r="D87" t="n">
-        <v>149</v>
+        <v>157</v>
       </c>
     </row>
     <row r="88">
@@ -1837,7 +1837,7 @@
       </c>
       <c r="C88" t="inlineStr"/>
       <c r="D88" t="n">
-        <v>465</v>
+        <v>475</v>
       </c>
     </row>
     <row r="89">
@@ -1869,7 +1869,7 @@
         </is>
       </c>
       <c r="D90" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="91">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="C91" t="inlineStr"/>
       <c r="D91" t="n">
-        <v>127</v>
+        <v>130</v>
       </c>
     </row>
     <row r="92">
@@ -1919,7 +1919,7 @@
         </is>
       </c>
       <c r="D93" t="n">
-        <v>78</v>
+        <v>80</v>
       </c>
     </row>
     <row r="94">
@@ -2027,7 +2027,7 @@
         </is>
       </c>
       <c r="D100" t="n">
-        <v>48</v>
+        <v>51</v>
       </c>
     </row>
     <row r="101">
@@ -2081,7 +2081,7 @@
         </is>
       </c>
       <c r="D103" t="n">
-        <v>107</v>
+        <v>110</v>
       </c>
     </row>
     <row r="104">
@@ -2173,7 +2173,7 @@
         </is>
       </c>
       <c r="D109" t="n">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="110">
@@ -2257,7 +2257,7 @@
       </c>
       <c r="C115" t="inlineStr"/>
       <c r="D115" t="n">
-        <v>152</v>
+        <v>159</v>
       </c>
     </row>
     <row r="116">
@@ -2393,7 +2393,7 @@
       </c>
       <c r="C124" t="inlineStr"/>
       <c r="D124" t="n">
-        <v>330</v>
+        <v>340</v>
       </c>
     </row>
     <row r="125">
@@ -2479,7 +2479,7 @@
         </is>
       </c>
       <c r="D129" t="n">
-        <v>94</v>
+        <v>97</v>
       </c>
     </row>
     <row r="130">
@@ -2533,7 +2533,7 @@
         </is>
       </c>
       <c r="D132" t="n">
-        <v>89</v>
+        <v>84</v>
       </c>
     </row>
     <row r="133">
@@ -2581,7 +2581,7 @@
       </c>
       <c r="C135" t="inlineStr"/>
       <c r="D135" t="n">
-        <v>293</v>
+        <v>298</v>
       </c>
     </row>
     <row r="136">
@@ -2613,7 +2613,7 @@
         </is>
       </c>
       <c r="D137" t="n">
-        <v>138</v>
+        <v>147</v>
       </c>
     </row>
     <row r="138">
@@ -2673,7 +2673,7 @@
       </c>
       <c r="C141" t="inlineStr"/>
       <c r="D141" t="n">
-        <v>87</v>
+        <v>90</v>
       </c>
     </row>
     <row r="142">
@@ -2781,7 +2781,7 @@
       </c>
       <c r="C148" t="inlineStr"/>
       <c r="D148" t="n">
-        <v>134</v>
+        <v>142</v>
       </c>
     </row>
     <row r="149">
@@ -2863,7 +2863,7 @@
         </is>
       </c>
       <c r="D154" t="n">
-        <v>269</v>
+        <v>273</v>
       </c>
     </row>
     <row r="155">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="D156" t="n">
-        <v>51</v>
+        <v>48</v>
       </c>
     </row>
     <row r="157">
@@ -2917,7 +2917,7 @@
         </is>
       </c>
       <c r="D157" t="n">
-        <v>212</v>
+        <v>198</v>
       </c>
     </row>
     <row r="158">
@@ -2945,7 +2945,7 @@
       </c>
       <c r="C159" t="inlineStr"/>
       <c r="D159" t="n">
-        <v>173</v>
+        <v>175</v>
       </c>
     </row>
     <row r="160">
@@ -2981,7 +2981,7 @@
         </is>
       </c>
       <c r="D161" t="n">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="162">
@@ -3013,7 +3013,7 @@
         </is>
       </c>
       <c r="D163" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="164">
@@ -3049,7 +3049,7 @@
         </is>
       </c>
       <c r="D165" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="166">
@@ -3123,7 +3123,7 @@
         </is>
       </c>
       <c r="D170" t="n">
-        <v>167</v>
+        <v>174</v>
       </c>
     </row>
     <row r="171">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="C174" t="inlineStr"/>
       <c r="D174" t="n">
-        <v>135</v>
+        <v>140</v>
       </c>
     </row>
     <row r="175">
@@ -3205,7 +3205,7 @@
         </is>
       </c>
       <c r="D175" t="n">
-        <v>203</v>
+        <v>209</v>
       </c>
     </row>
     <row r="176">
@@ -3267,7 +3267,7 @@
         </is>
       </c>
       <c r="D179" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="180">
@@ -3321,7 +3321,7 @@
         </is>
       </c>
       <c r="D182" t="n">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="183">
@@ -3339,7 +3339,7 @@
         </is>
       </c>
       <c r="D183" t="n">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="184">
@@ -3483,7 +3483,7 @@
       </c>
       <c r="C192" t="inlineStr"/>
       <c r="D192" t="n">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="193">
@@ -3501,7 +3501,7 @@
         </is>
       </c>
       <c r="D193" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="194">
@@ -3643,7 +3643,7 @@
       </c>
       <c r="C202" t="inlineStr"/>
       <c r="D202" t="n">
-        <v>162</v>
+        <v>170</v>
       </c>
     </row>
     <row r="203">
@@ -3661,7 +3661,7 @@
         </is>
       </c>
       <c r="D203" t="n">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="204">
@@ -3697,7 +3697,7 @@
         </is>
       </c>
       <c r="D205" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="206">
@@ -3733,7 +3733,7 @@
         </is>
       </c>
       <c r="D207" t="n">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="208">
@@ -3807,7 +3807,7 @@
         </is>
       </c>
       <c r="D212" t="n">
-        <v>183</v>
+        <v>181</v>
       </c>
     </row>
     <row r="213">
@@ -3929,7 +3929,7 @@
         </is>
       </c>
       <c r="D220" t="n">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="221">
@@ -3947,7 +3947,7 @@
         </is>
       </c>
       <c r="D221" t="n">
-        <v>338</v>
+        <v>342</v>
       </c>
     </row>
     <row r="222">
@@ -3991,7 +3991,7 @@
       </c>
       <c r="C224" t="inlineStr"/>
       <c r="D224" t="n">
-        <v>391</v>
+        <v>396</v>
       </c>
     </row>
     <row r="225">
@@ -4067,7 +4067,7 @@
         </is>
       </c>
       <c r="D229" t="n">
-        <v>99</v>
+        <v>104</v>
       </c>
     </row>
     <row r="230">
@@ -4117,7 +4117,7 @@
         </is>
       </c>
       <c r="D232" t="n">
-        <v>130</v>
+        <v>124</v>
       </c>
     </row>
     <row r="233">
@@ -4153,7 +4153,7 @@
         </is>
       </c>
       <c r="D234" t="n">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="235">

</xml_diff>

<commit_message>
data: field/odds refresh 2026-07-06 18:10 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -465,7 +465,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>14</v>
+        <v>19</v>
       </c>
     </row>
     <row r="3">
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>128</v>
+        <v>134</v>
       </c>
     </row>
     <row r="18">
@@ -729,7 +729,7 @@
       </c>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="n">
-        <v>151</v>
+        <v>149</v>
       </c>
     </row>
     <row r="20">
@@ -747,7 +747,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="21">
@@ -779,7 +779,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>97</v>
+        <v>99</v>
       </c>
     </row>
     <row r="23">
@@ -797,7 +797,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="24">
@@ -873,7 +873,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="29">
@@ -905,7 +905,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>55</v>
+        <v>52</v>
       </c>
     </row>
     <row r="31">
@@ -923,7 +923,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="32">
@@ -985,7 +985,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>295</v>
+        <v>336</v>
       </c>
     </row>
     <row r="36">
@@ -1133,7 +1133,7 @@
       </c>
       <c r="C45" t="inlineStr"/>
       <c r="D45" t="n">
-        <v>180</v>
+        <v>189</v>
       </c>
     </row>
     <row r="46">
@@ -1163,7 +1163,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>24</v>
+        <v>29</v>
       </c>
     </row>
     <row r="48">
@@ -1249,7 +1249,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="53">
@@ -1299,7 +1299,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="56">
@@ -1335,7 +1335,7 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="58">
@@ -1353,7 +1353,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>174</v>
+        <v>155</v>
       </c>
     </row>
     <row r="59">
@@ -1417,7 +1417,7 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
     </row>
     <row r="63">
@@ -1435,7 +1435,7 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>73</v>
+        <v>75</v>
       </c>
     </row>
     <row r="64">
@@ -1529,7 +1529,7 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="70">
@@ -1559,7 +1559,7 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>58</v>
+        <v>63</v>
       </c>
     </row>
     <row r="72">
@@ -1671,7 +1671,7 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>179</v>
+        <v>186</v>
       </c>
     </row>
     <row r="79">
@@ -1734,9 +1734,7 @@
         <v>5768</v>
       </c>
       <c r="C82" t="inlineStr"/>
-      <c r="D82" t="n">
-        <v>482</v>
-      </c>
+      <c r="D82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -1771,7 +1769,7 @@
         </is>
       </c>
       <c r="D84" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="85">
@@ -1789,7 +1787,7 @@
         </is>
       </c>
       <c r="D85" t="n">
-        <v>70</v>
+        <v>86</v>
       </c>
     </row>
     <row r="86">
@@ -1825,7 +1823,7 @@
         </is>
       </c>
       <c r="D87" t="n">
-        <v>135</v>
+        <v>157</v>
       </c>
     </row>
     <row r="88">
@@ -1839,7 +1837,7 @@
       </c>
       <c r="C88" t="inlineStr"/>
       <c r="D88" t="n">
-        <v>353</v>
+        <v>475</v>
       </c>
     </row>
     <row r="89">
@@ -1871,7 +1869,7 @@
         </is>
       </c>
       <c r="D90" t="n">
-        <v>30</v>
+        <v>13</v>
       </c>
     </row>
     <row r="91">
@@ -1885,7 +1883,7 @@
       </c>
       <c r="C91" t="inlineStr"/>
       <c r="D91" t="n">
-        <v>127</v>
+        <v>130</v>
       </c>
     </row>
     <row r="92">
@@ -1921,7 +1919,7 @@
         </is>
       </c>
       <c r="D93" t="n">
-        <v>78</v>
+        <v>80</v>
       </c>
     </row>
     <row r="94">
@@ -2029,7 +2027,7 @@
         </is>
       </c>
       <c r="D100" t="n">
-        <v>48</v>
+        <v>51</v>
       </c>
     </row>
     <row r="101">
@@ -2047,7 +2045,7 @@
         </is>
       </c>
       <c r="D101" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="102">
@@ -2083,7 +2081,7 @@
         </is>
       </c>
       <c r="D103" t="n">
-        <v>106</v>
+        <v>110</v>
       </c>
     </row>
     <row r="104">
@@ -2175,7 +2173,7 @@
         </is>
       </c>
       <c r="D109" t="n">
-        <v>110</v>
+        <v>115</v>
       </c>
     </row>
     <row r="110">
@@ -2259,7 +2257,7 @@
       </c>
       <c r="C115" t="inlineStr"/>
       <c r="D115" t="n">
-        <v>80</v>
+        <v>159</v>
       </c>
     </row>
     <row r="116">
@@ -2369,7 +2367,7 @@
         </is>
       </c>
       <c r="D122" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="123">
@@ -2395,7 +2393,7 @@
       </c>
       <c r="C124" t="inlineStr"/>
       <c r="D124" t="n">
-        <v>226</v>
+        <v>340</v>
       </c>
     </row>
     <row r="125">
@@ -2463,7 +2461,7 @@
         </is>
       </c>
       <c r="D128" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="129">
@@ -2481,7 +2479,7 @@
         </is>
       </c>
       <c r="D129" t="n">
-        <v>94</v>
+        <v>97</v>
       </c>
     </row>
     <row r="130">
@@ -2535,7 +2533,7 @@
         </is>
       </c>
       <c r="D132" t="n">
-        <v>89</v>
+        <v>84</v>
       </c>
     </row>
     <row r="133">
@@ -2583,7 +2581,7 @@
       </c>
       <c r="C135" t="inlineStr"/>
       <c r="D135" t="n">
-        <v>280</v>
+        <v>298</v>
       </c>
     </row>
     <row r="136">
@@ -2615,7 +2613,7 @@
         </is>
       </c>
       <c r="D137" t="n">
-        <v>138</v>
+        <v>147</v>
       </c>
     </row>
     <row r="138">
@@ -2675,7 +2673,7 @@
       </c>
       <c r="C141" t="inlineStr"/>
       <c r="D141" t="n">
-        <v>82</v>
+        <v>90</v>
       </c>
     </row>
     <row r="142">
@@ -2711,7 +2709,7 @@
         </is>
       </c>
       <c r="D143" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="144">
@@ -2725,7 +2723,7 @@
       </c>
       <c r="C144" t="inlineStr"/>
       <c r="D144" t="n">
-        <v>275</v>
+        <v>263</v>
       </c>
     </row>
     <row r="145">
@@ -2783,7 +2781,7 @@
       </c>
       <c r="C148" t="inlineStr"/>
       <c r="D148" t="n">
-        <v>134</v>
+        <v>142</v>
       </c>
     </row>
     <row r="149">
@@ -2865,7 +2863,7 @@
         </is>
       </c>
       <c r="D154" t="n">
-        <v>269</v>
+        <v>273</v>
       </c>
     </row>
     <row r="155">
@@ -2901,7 +2899,7 @@
         </is>
       </c>
       <c r="D156" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
     </row>
     <row r="157">
@@ -2919,7 +2917,7 @@
         </is>
       </c>
       <c r="D157" t="n">
-        <v>153</v>
+        <v>198</v>
       </c>
     </row>
     <row r="158">
@@ -2983,7 +2981,7 @@
         </is>
       </c>
       <c r="D161" t="n">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="162">
@@ -3015,7 +3013,7 @@
         </is>
       </c>
       <c r="D163" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="164">
@@ -3033,7 +3031,7 @@
         </is>
       </c>
       <c r="D164" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
     <row r="165">
@@ -3095,7 +3093,7 @@
         </is>
       </c>
       <c r="D168" t="n">
-        <v>27</v>
+        <v>31</v>
       </c>
     </row>
     <row r="169">
@@ -3125,7 +3123,7 @@
         </is>
       </c>
       <c r="D170" t="n">
-        <v>167</v>
+        <v>174</v>
       </c>
     </row>
     <row r="171">
@@ -3189,7 +3187,7 @@
       </c>
       <c r="C174" t="inlineStr"/>
       <c r="D174" t="n">
-        <v>135</v>
+        <v>140</v>
       </c>
     </row>
     <row r="175">
@@ -3207,7 +3205,7 @@
         </is>
       </c>
       <c r="D175" t="n">
-        <v>163</v>
+        <v>209</v>
       </c>
     </row>
     <row r="176">
@@ -3269,7 +3267,7 @@
         </is>
       </c>
       <c r="D179" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="180">
@@ -3323,7 +3321,7 @@
         </is>
       </c>
       <c r="D182" t="n">
-        <v>71</v>
+        <v>78</v>
       </c>
     </row>
     <row r="183">
@@ -3341,7 +3339,7 @@
         </is>
       </c>
       <c r="D183" t="n">
-        <v>71</v>
+        <v>78</v>
       </c>
     </row>
     <row r="184">
@@ -3359,7 +3357,7 @@
         </is>
       </c>
       <c r="D184" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
     </row>
     <row r="185">
@@ -3485,7 +3483,7 @@
       </c>
       <c r="C192" t="inlineStr"/>
       <c r="D192" t="n">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="193">
@@ -3585,7 +3583,7 @@
         </is>
       </c>
       <c r="D198" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="199">
@@ -3645,7 +3643,7 @@
       </c>
       <c r="C202" t="inlineStr"/>
       <c r="D202" t="n">
-        <v>196</v>
+        <v>170</v>
       </c>
     </row>
     <row r="203">
@@ -3663,7 +3661,7 @@
         </is>
       </c>
       <c r="D203" t="n">
-        <v>65</v>
+        <v>70</v>
       </c>
     </row>
     <row r="204">
@@ -3681,7 +3679,7 @@
         </is>
       </c>
       <c r="D204" t="n">
-        <v>73</v>
+        <v>76</v>
       </c>
     </row>
     <row r="205">
@@ -3699,7 +3697,7 @@
         </is>
       </c>
       <c r="D205" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="206">
@@ -3735,7 +3733,7 @@
         </is>
       </c>
       <c r="D207" t="n">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="208">
@@ -3809,7 +3807,7 @@
         </is>
       </c>
       <c r="D212" t="n">
-        <v>183</v>
+        <v>181</v>
       </c>
     </row>
     <row r="213">
@@ -3885,7 +3883,7 @@
         </is>
       </c>
       <c r="D217" t="n">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="218">
@@ -3931,7 +3929,7 @@
         </is>
       </c>
       <c r="D220" t="n">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="221">
@@ -3949,7 +3947,7 @@
         </is>
       </c>
       <c r="D221" t="n">
-        <v>311</v>
+        <v>342</v>
       </c>
     </row>
     <row r="222">
@@ -3993,7 +3991,7 @@
       </c>
       <c r="C224" t="inlineStr"/>
       <c r="D224" t="n">
-        <v>369</v>
+        <v>396</v>
       </c>
     </row>
     <row r="225">
@@ -4069,7 +4067,7 @@
         </is>
       </c>
       <c r="D229" t="n">
-        <v>99</v>
+        <v>104</v>
       </c>
     </row>
     <row r="230">
@@ -4119,7 +4117,7 @@
         </is>
       </c>
       <c r="D232" t="n">
-        <v>130</v>
+        <v>124</v>
       </c>
     </row>
     <row r="233">
@@ -4155,7 +4153,7 @@
         </is>
       </c>
       <c r="D234" t="n">
-        <v>72</v>
+        <v>85</v>
       </c>
     </row>
     <row r="235">
@@ -4173,7 +4171,7 @@
         </is>
       </c>
       <c r="D235" t="n">
-        <v>67</v>
+        <v>62</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: field/odds refresh 2026-07-13 05:39 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -465,7 +465,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3">
@@ -539,7 +539,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="8">
@@ -575,7 +575,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="10">
@@ -607,7 +607,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>38</v>
+        <v>41</v>
       </c>
     </row>
     <row r="12">
@@ -639,7 +639,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="14">
@@ -685,7 +685,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
     </row>
     <row r="17">
@@ -729,7 +729,7 @@
       </c>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="n">
-        <v>149</v>
+        <v>143</v>
       </c>
     </row>
     <row r="20">
@@ -747,7 +747,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="21">
@@ -797,7 +797,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="24">
@@ -873,7 +873,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>67</v>
+        <v>71</v>
       </c>
     </row>
     <row r="29">
@@ -905,7 +905,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="31">
@@ -923,7 +923,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>58</v>
+        <v>61</v>
       </c>
     </row>
     <row r="32">
@@ -1003,7 +1003,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>47</v>
+        <v>54</v>
       </c>
     </row>
     <row r="37">
@@ -1021,7 +1021,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>32</v>
+        <v>37</v>
       </c>
     </row>
     <row r="38">
@@ -1047,7 +1047,7 @@
       </c>
       <c r="C39" t="inlineStr"/>
       <c r="D39" t="n">
-        <v>61</v>
+        <v>80</v>
       </c>
     </row>
     <row r="40">
@@ -1105,7 +1105,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="44">
@@ -1119,7 +1119,7 @@
       </c>
       <c r="C44" t="inlineStr"/>
       <c r="D44" t="n">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="45">
@@ -1163,7 +1163,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>29</v>
+        <v>32</v>
       </c>
     </row>
     <row r="48">
@@ -1231,7 +1231,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="52">
@@ -1417,7 +1417,7 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="63">
@@ -1435,7 +1435,7 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>75</v>
+        <v>77</v>
       </c>
     </row>
     <row r="64">
@@ -1529,7 +1529,7 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>72</v>
+        <v>76</v>
       </c>
     </row>
     <row r="70">
@@ -1559,7 +1559,7 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="72">
@@ -1603,7 +1603,7 @@
         </is>
       </c>
       <c r="D74" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="75">
@@ -1689,7 +1689,7 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="80">
@@ -1769,7 +1769,7 @@
         </is>
       </c>
       <c r="D84" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="85">
@@ -1787,7 +1787,7 @@
         </is>
       </c>
       <c r="D85" t="n">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="86">
@@ -1805,7 +1805,7 @@
         </is>
       </c>
       <c r="D86" t="n">
-        <v>112</v>
+        <v>74</v>
       </c>
     </row>
     <row r="87">
@@ -1823,7 +1823,7 @@
         </is>
       </c>
       <c r="D87" t="n">
-        <v>157</v>
+        <v>168</v>
       </c>
     </row>
     <row r="88">
@@ -1869,7 +1869,7 @@
         </is>
       </c>
       <c r="D90" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="91">
@@ -1919,7 +1919,7 @@
         </is>
       </c>
       <c r="D93" t="n">
-        <v>80</v>
+        <v>86</v>
       </c>
     </row>
     <row r="94">
@@ -2027,7 +2027,7 @@
         </is>
       </c>
       <c r="D100" t="n">
-        <v>51</v>
+        <v>55</v>
       </c>
     </row>
     <row r="101">
@@ -2045,7 +2045,7 @@
         </is>
       </c>
       <c r="D101" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="102">
@@ -2063,7 +2063,7 @@
         </is>
       </c>
       <c r="D102" t="n">
-        <v>66</v>
+        <v>33</v>
       </c>
     </row>
     <row r="103">
@@ -2111,7 +2111,7 @@
         </is>
       </c>
       <c r="D105" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
     </row>
     <row r="106">
@@ -2143,7 +2143,7 @@
         </is>
       </c>
       <c r="D107" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="108">
@@ -2173,7 +2173,7 @@
         </is>
       </c>
       <c r="D109" t="n">
-        <v>115</v>
+        <v>118</v>
       </c>
     </row>
     <row r="110">
@@ -2287,7 +2287,7 @@
         </is>
       </c>
       <c r="D117" t="n">
-        <v>39</v>
+        <v>24</v>
       </c>
     </row>
     <row r="118">
@@ -2349,7 +2349,7 @@
         </is>
       </c>
       <c r="D121" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="122">
@@ -2367,7 +2367,7 @@
         </is>
       </c>
       <c r="D122" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
     </row>
     <row r="123">
@@ -2425,7 +2425,7 @@
         </is>
       </c>
       <c r="D126" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
     </row>
     <row r="127">
@@ -2461,7 +2461,7 @@
         </is>
       </c>
       <c r="D128" t="n">
-        <v>57</v>
+        <v>63</v>
       </c>
     </row>
     <row r="129">
@@ -2515,7 +2515,7 @@
         </is>
       </c>
       <c r="D131" t="n">
-        <v>36</v>
+        <v>39</v>
       </c>
     </row>
     <row r="132">
@@ -2581,7 +2581,7 @@
       </c>
       <c r="C135" t="inlineStr"/>
       <c r="D135" t="n">
-        <v>298</v>
+        <v>243</v>
       </c>
     </row>
     <row r="136">
@@ -2631,7 +2631,7 @@
         </is>
       </c>
       <c r="D138" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="139">
@@ -2673,7 +2673,7 @@
       </c>
       <c r="C141" t="inlineStr"/>
       <c r="D141" t="n">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="142">
@@ -2691,7 +2691,7 @@
         </is>
       </c>
       <c r="D142" t="n">
-        <v>80</v>
+        <v>48</v>
       </c>
     </row>
     <row r="143">
@@ -2709,7 +2709,7 @@
         </is>
       </c>
       <c r="D143" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="144">
@@ -2767,7 +2767,7 @@
         </is>
       </c>
       <c r="D147" t="n">
-        <v>65</v>
+        <v>69</v>
       </c>
     </row>
     <row r="148">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="D156" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="157">
@@ -2917,7 +2917,7 @@
         </is>
       </c>
       <c r="D157" t="n">
-        <v>198</v>
+        <v>163</v>
       </c>
     </row>
     <row r="158">
@@ -2963,7 +2963,7 @@
         </is>
       </c>
       <c r="D160" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="161">
@@ -3049,7 +3049,7 @@
         </is>
       </c>
       <c r="D165" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="166">
@@ -3093,7 +3093,7 @@
         </is>
       </c>
       <c r="D168" t="n">
-        <v>31</v>
+        <v>26</v>
       </c>
     </row>
     <row r="169">
@@ -3159,7 +3159,7 @@
         </is>
       </c>
       <c r="D172" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="173">
@@ -3205,7 +3205,7 @@
         </is>
       </c>
       <c r="D175" t="n">
-        <v>209</v>
+        <v>216</v>
       </c>
     </row>
     <row r="176">
@@ -3357,7 +3357,7 @@
         </is>
       </c>
       <c r="D184" t="n">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="185">
@@ -3435,7 +3435,7 @@
         </is>
       </c>
       <c r="D189" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="190">
@@ -3453,7 +3453,7 @@
         </is>
       </c>
       <c r="D190" t="n">
-        <v>136</v>
+        <v>140</v>
       </c>
     </row>
     <row r="191">
@@ -3501,7 +3501,7 @@
         </is>
       </c>
       <c r="D193" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="194">
@@ -3519,7 +3519,7 @@
         </is>
       </c>
       <c r="D194" t="n">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
     <row r="195">
@@ -3551,7 +3551,7 @@
         </is>
       </c>
       <c r="D196" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="197">
@@ -3565,7 +3565,7 @@
       </c>
       <c r="C197" t="inlineStr"/>
       <c r="D197" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="198">
@@ -3615,7 +3615,7 @@
       </c>
       <c r="C200" t="inlineStr"/>
       <c r="D200" t="n">
-        <v>126</v>
+        <v>115</v>
       </c>
     </row>
     <row r="201">
@@ -3643,7 +3643,7 @@
       </c>
       <c r="C202" t="inlineStr"/>
       <c r="D202" t="n">
-        <v>170</v>
+        <v>165</v>
       </c>
     </row>
     <row r="203">
@@ -3661,7 +3661,7 @@
         </is>
       </c>
       <c r="D203" t="n">
-        <v>70</v>
+        <v>67</v>
       </c>
     </row>
     <row r="204">
@@ -3679,7 +3679,7 @@
         </is>
       </c>
       <c r="D204" t="n">
-        <v>76</v>
+        <v>81</v>
       </c>
     </row>
     <row r="205">
@@ -3697,7 +3697,7 @@
         </is>
       </c>
       <c r="D205" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="206">
@@ -3733,7 +3733,7 @@
         </is>
       </c>
       <c r="D207" t="n">
-        <v>83</v>
+        <v>70</v>
       </c>
     </row>
     <row r="208">
@@ -3789,7 +3789,7 @@
         </is>
       </c>
       <c r="D211" t="n">
-        <v>60</v>
+        <v>73</v>
       </c>
     </row>
     <row r="212">
@@ -3929,7 +3929,7 @@
         </is>
       </c>
       <c r="D220" t="n">
-        <v>69</v>
+        <v>72</v>
       </c>
     </row>
     <row r="221">
@@ -4021,7 +4021,7 @@
         </is>
       </c>
       <c r="D226" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="227">
@@ -4085,7 +4085,7 @@
         </is>
       </c>
       <c r="D230" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="231">
@@ -4153,7 +4153,7 @@
         </is>
       </c>
       <c r="D234" t="n">
-        <v>85</v>
+        <v>82</v>
       </c>
     </row>
     <row r="235">
@@ -4171,7 +4171,7 @@
         </is>
       </c>
       <c r="D235" t="n">
-        <v>62</v>
+        <v>65</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: field/odds refresh 2026-07-13 13:14 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -465,7 +465,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3">
@@ -539,7 +539,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="8">
@@ -575,7 +575,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="10">
@@ -607,7 +607,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>38</v>
+        <v>41</v>
       </c>
     </row>
     <row r="12">
@@ -639,7 +639,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="14">
@@ -685,7 +685,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
     </row>
     <row r="17">
@@ -729,7 +729,7 @@
       </c>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="n">
-        <v>149</v>
+        <v>143</v>
       </c>
     </row>
     <row r="20">
@@ -747,7 +747,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="21">
@@ -797,7 +797,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="24">
@@ -873,7 +873,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>67</v>
+        <v>71</v>
       </c>
     </row>
     <row r="29">
@@ -905,7 +905,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="31">
@@ -923,7 +923,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>58</v>
+        <v>61</v>
       </c>
     </row>
     <row r="32">
@@ -1003,7 +1003,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>47</v>
+        <v>54</v>
       </c>
     </row>
     <row r="37">
@@ -1021,7 +1021,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>32</v>
+        <v>37</v>
       </c>
     </row>
     <row r="38">
@@ -1047,7 +1047,7 @@
       </c>
       <c r="C39" t="inlineStr"/>
       <c r="D39" t="n">
-        <v>61</v>
+        <v>80</v>
       </c>
     </row>
     <row r="40">
@@ -1105,7 +1105,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="44">
@@ -1119,7 +1119,7 @@
       </c>
       <c r="C44" t="inlineStr"/>
       <c r="D44" t="n">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="45">
@@ -1163,7 +1163,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>29</v>
+        <v>32</v>
       </c>
     </row>
     <row r="48">
@@ -1231,7 +1231,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="52">
@@ -1417,7 +1417,7 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="63">
@@ -1435,7 +1435,7 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>75</v>
+        <v>77</v>
       </c>
     </row>
     <row r="64">
@@ -1529,7 +1529,7 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>72</v>
+        <v>76</v>
       </c>
     </row>
     <row r="70">
@@ -1559,7 +1559,7 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="72">
@@ -1603,7 +1603,7 @@
         </is>
       </c>
       <c r="D74" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="75">
@@ -1689,7 +1689,7 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="80">
@@ -1769,7 +1769,7 @@
         </is>
       </c>
       <c r="D84" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="85">
@@ -1787,7 +1787,7 @@
         </is>
       </c>
       <c r="D85" t="n">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="86">
@@ -1805,7 +1805,7 @@
         </is>
       </c>
       <c r="D86" t="n">
-        <v>112</v>
+        <v>74</v>
       </c>
     </row>
     <row r="87">
@@ -1823,7 +1823,7 @@
         </is>
       </c>
       <c r="D87" t="n">
-        <v>157</v>
+        <v>168</v>
       </c>
     </row>
     <row r="88">
@@ -1869,7 +1869,7 @@
         </is>
       </c>
       <c r="D90" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="91">
@@ -1919,7 +1919,7 @@
         </is>
       </c>
       <c r="D93" t="n">
-        <v>80</v>
+        <v>86</v>
       </c>
     </row>
     <row r="94">
@@ -2027,7 +2027,7 @@
         </is>
       </c>
       <c r="D100" t="n">
-        <v>51</v>
+        <v>55</v>
       </c>
     </row>
     <row r="101">
@@ -2045,7 +2045,7 @@
         </is>
       </c>
       <c r="D101" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="102">
@@ -2063,7 +2063,7 @@
         </is>
       </c>
       <c r="D102" t="n">
-        <v>66</v>
+        <v>33</v>
       </c>
     </row>
     <row r="103">
@@ -2111,7 +2111,7 @@
         </is>
       </c>
       <c r="D105" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
     </row>
     <row r="106">
@@ -2143,7 +2143,7 @@
         </is>
       </c>
       <c r="D107" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="108">
@@ -2173,7 +2173,7 @@
         </is>
       </c>
       <c r="D109" t="n">
-        <v>115</v>
+        <v>118</v>
       </c>
     </row>
     <row r="110">
@@ -2287,7 +2287,7 @@
         </is>
       </c>
       <c r="D117" t="n">
-        <v>39</v>
+        <v>24</v>
       </c>
     </row>
     <row r="118">
@@ -2349,7 +2349,7 @@
         </is>
       </c>
       <c r="D121" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="122">
@@ -2367,7 +2367,7 @@
         </is>
       </c>
       <c r="D122" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
     </row>
     <row r="123">
@@ -2425,7 +2425,7 @@
         </is>
       </c>
       <c r="D126" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
     </row>
     <row r="127">
@@ -2461,7 +2461,7 @@
         </is>
       </c>
       <c r="D128" t="n">
-        <v>57</v>
+        <v>63</v>
       </c>
     </row>
     <row r="129">
@@ -2515,7 +2515,7 @@
         </is>
       </c>
       <c r="D131" t="n">
-        <v>36</v>
+        <v>39</v>
       </c>
     </row>
     <row r="132">
@@ -2581,7 +2581,7 @@
       </c>
       <c r="C135" t="inlineStr"/>
       <c r="D135" t="n">
-        <v>298</v>
+        <v>243</v>
       </c>
     </row>
     <row r="136">
@@ -2631,7 +2631,7 @@
         </is>
       </c>
       <c r="D138" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="139">
@@ -2673,7 +2673,7 @@
       </c>
       <c r="C141" t="inlineStr"/>
       <c r="D141" t="n">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="142">
@@ -2691,7 +2691,7 @@
         </is>
       </c>
       <c r="D142" t="n">
-        <v>80</v>
+        <v>48</v>
       </c>
     </row>
     <row r="143">
@@ -2709,7 +2709,7 @@
         </is>
       </c>
       <c r="D143" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="144">
@@ -2767,7 +2767,7 @@
         </is>
       </c>
       <c r="D147" t="n">
-        <v>65</v>
+        <v>69</v>
       </c>
     </row>
     <row r="148">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="D156" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="157">
@@ -2917,7 +2917,7 @@
         </is>
       </c>
       <c r="D157" t="n">
-        <v>198</v>
+        <v>163</v>
       </c>
     </row>
     <row r="158">
@@ -2963,7 +2963,7 @@
         </is>
       </c>
       <c r="D160" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="161">
@@ -2981,7 +2981,7 @@
         </is>
       </c>
       <c r="D161" t="n">
-        <v>77</v>
+        <v>83</v>
       </c>
     </row>
     <row r="162">
@@ -3049,7 +3049,7 @@
         </is>
       </c>
       <c r="D165" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="166">
@@ -3093,7 +3093,7 @@
         </is>
       </c>
       <c r="D168" t="n">
-        <v>31</v>
+        <v>26</v>
       </c>
     </row>
     <row r="169">
@@ -3159,7 +3159,7 @@
         </is>
       </c>
       <c r="D172" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="173">
@@ -3205,7 +3205,7 @@
         </is>
       </c>
       <c r="D175" t="n">
-        <v>209</v>
+        <v>216</v>
       </c>
     </row>
     <row r="176">
@@ -3357,7 +3357,7 @@
         </is>
       </c>
       <c r="D184" t="n">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="185">
@@ -3435,7 +3435,7 @@
         </is>
       </c>
       <c r="D189" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="190">
@@ -3453,7 +3453,7 @@
         </is>
       </c>
       <c r="D190" t="n">
-        <v>136</v>
+        <v>140</v>
       </c>
     </row>
     <row r="191">
@@ -3501,7 +3501,7 @@
         </is>
       </c>
       <c r="D193" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="194">
@@ -3519,7 +3519,7 @@
         </is>
       </c>
       <c r="D194" t="n">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
     <row r="195">
@@ -3551,7 +3551,7 @@
         </is>
       </c>
       <c r="D196" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="197">
@@ -3565,7 +3565,7 @@
       </c>
       <c r="C197" t="inlineStr"/>
       <c r="D197" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="198">
@@ -3615,7 +3615,7 @@
       </c>
       <c r="C200" t="inlineStr"/>
       <c r="D200" t="n">
-        <v>126</v>
+        <v>115</v>
       </c>
     </row>
     <row r="201">
@@ -3643,7 +3643,7 @@
       </c>
       <c r="C202" t="inlineStr"/>
       <c r="D202" t="n">
-        <v>170</v>
+        <v>165</v>
       </c>
     </row>
     <row r="203">
@@ -3661,7 +3661,7 @@
         </is>
       </c>
       <c r="D203" t="n">
-        <v>70</v>
+        <v>67</v>
       </c>
     </row>
     <row r="204">
@@ -3679,7 +3679,7 @@
         </is>
       </c>
       <c r="D204" t="n">
-        <v>76</v>
+        <v>81</v>
       </c>
     </row>
     <row r="205">
@@ -3697,7 +3697,7 @@
         </is>
       </c>
       <c r="D205" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="206">
@@ -3733,7 +3733,7 @@
         </is>
       </c>
       <c r="D207" t="n">
-        <v>83</v>
+        <v>70</v>
       </c>
     </row>
     <row r="208">
@@ -3789,7 +3789,7 @@
         </is>
       </c>
       <c r="D211" t="n">
-        <v>60</v>
+        <v>73</v>
       </c>
     </row>
     <row r="212">
@@ -3929,7 +3929,7 @@
         </is>
       </c>
       <c r="D220" t="n">
-        <v>69</v>
+        <v>72</v>
       </c>
     </row>
     <row r="221">
@@ -4021,7 +4021,7 @@
         </is>
       </c>
       <c r="D226" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="227">
@@ -4085,7 +4085,7 @@
         </is>
       </c>
       <c r="D230" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="231">
@@ -4153,7 +4153,7 @@
         </is>
       </c>
       <c r="D234" t="n">
-        <v>85</v>
+        <v>82</v>
       </c>
     </row>
     <row r="235">
@@ -4171,7 +4171,7 @@
         </is>
       </c>
       <c r="D235" t="n">
-        <v>62</v>
+        <v>65</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: field/odds refresh 2026-07-19 18:00 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -557,7 +557,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>100</v>
+        <v>96</v>
       </c>
     </row>
     <row r="9">
@@ -589,7 +589,7 @@
       </c>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="n">
-        <v>187</v>
+        <v>157</v>
       </c>
     </row>
     <row r="11">
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>134</v>
+        <v>139</v>
       </c>
     </row>
     <row r="18">
@@ -811,7 +811,7 @@
       </c>
       <c r="C24" t="inlineStr"/>
       <c r="D24" t="n">
-        <v>362</v>
+        <v>367</v>
       </c>
     </row>
     <row r="25">
@@ -837,7 +837,7 @@
       </c>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="n">
-        <v>270</v>
+        <v>286</v>
       </c>
     </row>
     <row r="27">
@@ -967,7 +967,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="35">
@@ -985,7 +985,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>336</v>
+        <v>287</v>
       </c>
     </row>
     <row r="36">
@@ -1087,7 +1087,7 @@
       </c>
       <c r="C42" t="inlineStr"/>
       <c r="D42" t="n">
-        <v>360</v>
+        <v>368</v>
       </c>
     </row>
     <row r="43">
@@ -1133,7 +1133,7 @@
       </c>
       <c r="C45" t="inlineStr"/>
       <c r="D45" t="n">
-        <v>189</v>
+        <v>183</v>
       </c>
     </row>
     <row r="46">
@@ -1181,7 +1181,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>113</v>
+        <v>123</v>
       </c>
     </row>
     <row r="49">
@@ -1195,7 +1195,7 @@
       </c>
       <c r="C49" t="inlineStr"/>
       <c r="D49" t="n">
-        <v>207</v>
+        <v>225</v>
       </c>
     </row>
     <row r="50">
@@ -1213,7 +1213,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>123</v>
+        <v>79</v>
       </c>
     </row>
     <row r="51">
@@ -1317,7 +1317,7 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>240</v>
+        <v>246</v>
       </c>
     </row>
     <row r="57">
@@ -1353,7 +1353,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>155</v>
+        <v>159</v>
       </c>
     </row>
     <row r="59">
@@ -1371,7 +1371,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>115</v>
+        <v>89</v>
       </c>
     </row>
     <row r="60">
@@ -1399,7 +1399,7 @@
       </c>
       <c r="C61" t="inlineStr"/>
       <c r="D61" t="n">
-        <v>457</v>
+        <v>461</v>
       </c>
     </row>
     <row r="62">
@@ -1467,7 +1467,7 @@
       </c>
       <c r="C65" t="inlineStr"/>
       <c r="D65" t="n">
-        <v>222</v>
+        <v>218</v>
       </c>
     </row>
     <row r="66">
@@ -1485,7 +1485,7 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>109</v>
+        <v>113</v>
       </c>
     </row>
     <row r="67">
@@ -1511,7 +1511,7 @@
       </c>
       <c r="C68" t="inlineStr"/>
       <c r="D68" t="n">
-        <v>262</v>
+        <v>274</v>
       </c>
     </row>
     <row r="69">
@@ -1639,7 +1639,7 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>104</v>
+        <v>107</v>
       </c>
     </row>
     <row r="77">
@@ -1671,7 +1671,7 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>186</v>
+        <v>193</v>
       </c>
     </row>
     <row r="79">
@@ -1703,7 +1703,7 @@
       </c>
       <c r="C80" t="inlineStr"/>
       <c r="D80" t="n">
-        <v>155</v>
+        <v>119</v>
       </c>
     </row>
     <row r="81">
@@ -1721,7 +1721,7 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>92</v>
+        <v>101</v>
       </c>
     </row>
     <row r="82">
@@ -1751,7 +1751,7 @@
         </is>
       </c>
       <c r="D83" t="n">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="84">
@@ -1851,7 +1851,7 @@
       </c>
       <c r="C89" t="inlineStr"/>
       <c r="D89" t="n">
-        <v>158</v>
+        <v>161</v>
       </c>
     </row>
     <row r="90">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="C91" t="inlineStr"/>
       <c r="D91" t="n">
-        <v>130</v>
+        <v>133</v>
       </c>
     </row>
     <row r="92">
@@ -1901,7 +1901,7 @@
         </is>
       </c>
       <c r="D92" t="n">
-        <v>145</v>
+        <v>141</v>
       </c>
     </row>
     <row r="93">
@@ -1937,7 +1937,7 @@
         </is>
       </c>
       <c r="D94" t="n">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
     <row r="95">
@@ -1983,7 +1983,7 @@
       </c>
       <c r="C97" t="inlineStr"/>
       <c r="D97" t="n">
-        <v>154</v>
+        <v>156</v>
       </c>
     </row>
     <row r="98">
@@ -2081,7 +2081,7 @@
         </is>
       </c>
       <c r="D103" t="n">
-        <v>110</v>
+        <v>116</v>
       </c>
     </row>
     <row r="104">
@@ -2125,7 +2125,7 @@
       </c>
       <c r="C106" t="inlineStr"/>
       <c r="D106" t="n">
-        <v>384</v>
+        <v>400</v>
       </c>
     </row>
     <row r="107">
@@ -2187,7 +2187,7 @@
       </c>
       <c r="C110" t="inlineStr"/>
       <c r="D110" t="n">
-        <v>169</v>
+        <v>125</v>
       </c>
     </row>
     <row r="111">
@@ -2205,7 +2205,7 @@
         </is>
       </c>
       <c r="D111" t="n">
-        <v>218</v>
+        <v>203</v>
       </c>
     </row>
     <row r="112">
@@ -2219,7 +2219,7 @@
       </c>
       <c r="C112" t="inlineStr"/>
       <c r="D112" t="n">
-        <v>181</v>
+        <v>179</v>
       </c>
     </row>
     <row r="113">
@@ -2305,7 +2305,7 @@
         </is>
       </c>
       <c r="D118" t="n">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="119">
@@ -2331,7 +2331,7 @@
       </c>
       <c r="C120" t="inlineStr"/>
       <c r="D120" t="n">
-        <v>265</v>
+        <v>276</v>
       </c>
     </row>
     <row r="121">
@@ -2407,7 +2407,7 @@
       </c>
       <c r="C125" t="inlineStr"/>
       <c r="D125" t="n">
-        <v>490</v>
+        <v>481</v>
       </c>
     </row>
     <row r="126">
@@ -2443,7 +2443,7 @@
         </is>
       </c>
       <c r="D127" t="n">
-        <v>102</v>
+        <v>108</v>
       </c>
     </row>
     <row r="128">
@@ -2479,7 +2479,7 @@
         </is>
       </c>
       <c r="D129" t="n">
-        <v>97</v>
+        <v>102</v>
       </c>
     </row>
     <row r="130">
@@ -2613,7 +2613,7 @@
         </is>
       </c>
       <c r="D137" t="n">
-        <v>147</v>
+        <v>151</v>
       </c>
     </row>
     <row r="138">
@@ -2645,7 +2645,7 @@
       </c>
       <c r="C139" t="inlineStr"/>
       <c r="D139" t="n">
-        <v>129</v>
+        <v>126</v>
       </c>
     </row>
     <row r="140">
@@ -2737,7 +2737,7 @@
       </c>
       <c r="C145" t="inlineStr"/>
       <c r="D145" t="n">
-        <v>367</v>
+        <v>446</v>
       </c>
     </row>
     <row r="146">
@@ -2781,7 +2781,7 @@
       </c>
       <c r="C148" t="inlineStr"/>
       <c r="D148" t="n">
-        <v>142</v>
+        <v>146</v>
       </c>
     </row>
     <row r="149">
@@ -2845,7 +2845,7 @@
       </c>
       <c r="C153" t="inlineStr"/>
       <c r="D153" t="n">
-        <v>304</v>
+        <v>315</v>
       </c>
     </row>
     <row r="154">
@@ -2863,7 +2863,7 @@
         </is>
       </c>
       <c r="D154" t="n">
-        <v>273</v>
+        <v>278</v>
       </c>
     </row>
     <row r="155">
@@ -2881,7 +2881,7 @@
         </is>
       </c>
       <c r="D155" t="n">
-        <v>93</v>
+        <v>87</v>
       </c>
     </row>
     <row r="156">
@@ -2931,7 +2931,7 @@
       </c>
       <c r="C158" t="inlineStr"/>
       <c r="D158" t="n">
-        <v>252</v>
+        <v>261</v>
       </c>
     </row>
     <row r="159">
@@ -2945,7 +2945,7 @@
       </c>
       <c r="C159" t="inlineStr"/>
       <c r="D159" t="n">
-        <v>173</v>
+        <v>167</v>
       </c>
     </row>
     <row r="160">
@@ -2995,7 +2995,7 @@
       </c>
       <c r="C162" t="inlineStr"/>
       <c r="D162" t="n">
-        <v>198</v>
+        <v>213</v>
       </c>
     </row>
     <row r="163">
@@ -3013,7 +3013,7 @@
         </is>
       </c>
       <c r="D163" t="n">
-        <v>89</v>
+        <v>93</v>
       </c>
     </row>
     <row r="164">
@@ -3063,7 +3063,7 @@
       </c>
       <c r="C166" t="inlineStr"/>
       <c r="D166" t="n">
-        <v>172</v>
+        <v>182</v>
       </c>
     </row>
     <row r="167">
@@ -3123,7 +3123,7 @@
         </is>
       </c>
       <c r="D170" t="n">
-        <v>174</v>
+        <v>176</v>
       </c>
     </row>
     <row r="171">
@@ -3141,7 +3141,7 @@
         </is>
       </c>
       <c r="D171" t="n">
-        <v>85</v>
+        <v>92</v>
       </c>
     </row>
     <row r="172">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="C174" t="inlineStr"/>
       <c r="D174" t="n">
-        <v>140</v>
+        <v>117</v>
       </c>
     </row>
     <row r="175">
@@ -3303,7 +3303,7 @@
         </is>
       </c>
       <c r="D181" t="n">
-        <v>171</v>
+        <v>184</v>
       </c>
     </row>
     <row r="182">
@@ -3321,7 +3321,7 @@
         </is>
       </c>
       <c r="D182" t="n">
-        <v>78</v>
+        <v>75</v>
       </c>
     </row>
     <row r="183">
@@ -3339,7 +3339,7 @@
         </is>
       </c>
       <c r="D183" t="n">
-        <v>78</v>
+        <v>75</v>
       </c>
     </row>
     <row r="184">
@@ -3385,7 +3385,7 @@
       </c>
       <c r="C186" t="inlineStr"/>
       <c r="D186" t="n">
-        <v>276</v>
+        <v>214</v>
       </c>
     </row>
     <row r="187">
@@ -3417,7 +3417,7 @@
       </c>
       <c r="C188" t="inlineStr"/>
       <c r="D188" t="n">
-        <v>271</v>
+        <v>266</v>
       </c>
     </row>
     <row r="189">
@@ -3483,7 +3483,7 @@
       </c>
       <c r="C192" t="inlineStr"/>
       <c r="D192" t="n">
-        <v>119</v>
+        <v>124</v>
       </c>
     </row>
     <row r="193">
@@ -3533,7 +3533,7 @@
       </c>
       <c r="C195" t="inlineStr"/>
       <c r="D195" t="n">
-        <v>287</v>
+        <v>298</v>
       </c>
     </row>
     <row r="196">
@@ -3601,7 +3601,7 @@
         </is>
       </c>
       <c r="D199" t="n">
-        <v>437</v>
+        <v>439</v>
       </c>
     </row>
     <row r="200">
@@ -3629,7 +3629,7 @@
       </c>
       <c r="C201" t="inlineStr"/>
       <c r="D201" t="n">
-        <v>438</v>
+        <v>459</v>
       </c>
     </row>
     <row r="202">
@@ -3715,7 +3715,7 @@
         </is>
       </c>
       <c r="D206" t="n">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="207">
@@ -3771,7 +3771,7 @@
       </c>
       <c r="C210" t="inlineStr"/>
       <c r="D210" t="n">
-        <v>379</v>
+        <v>383</v>
       </c>
     </row>
     <row r="211">
@@ -3807,7 +3807,7 @@
         </is>
       </c>
       <c r="D212" t="n">
-        <v>181</v>
+        <v>185</v>
       </c>
     </row>
     <row r="213">
@@ -3851,7 +3851,7 @@
       </c>
       <c r="C215" t="inlineStr"/>
       <c r="D215" t="n">
-        <v>311</v>
+        <v>270</v>
       </c>
     </row>
     <row r="216">
@@ -3865,7 +3865,7 @@
       </c>
       <c r="C216" t="inlineStr"/>
       <c r="D216" t="n">
-        <v>311</v>
+        <v>270</v>
       </c>
     </row>
     <row r="217">
@@ -3883,7 +3883,7 @@
         </is>
       </c>
       <c r="D217" t="n">
-        <v>197</v>
+        <v>191</v>
       </c>
     </row>
     <row r="218">
@@ -3897,7 +3897,7 @@
       </c>
       <c r="C218" t="inlineStr"/>
       <c r="D218" t="n">
-        <v>495</v>
+        <v>489</v>
       </c>
     </row>
     <row r="219">
@@ -3911,7 +3911,7 @@
       </c>
       <c r="C219" t="inlineStr"/>
       <c r="D219" t="n">
-        <v>254</v>
+        <v>264</v>
       </c>
     </row>
     <row r="220">
@@ -3965,7 +3965,7 @@
         </is>
       </c>
       <c r="D222" t="n">
-        <v>166</v>
+        <v>180</v>
       </c>
     </row>
     <row r="223">
@@ -4035,7 +4035,7 @@
       </c>
       <c r="C227" t="inlineStr"/>
       <c r="D227" t="n">
-        <v>377</v>
+        <v>375</v>
       </c>
     </row>
     <row r="228">
@@ -4067,7 +4067,7 @@
         </is>
       </c>
       <c r="D229" t="n">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="230">
@@ -4117,7 +4117,7 @@
         </is>
       </c>
       <c r="D232" t="n">
-        <v>124</v>
+        <v>131</v>
       </c>
     </row>
     <row r="233">

</xml_diff>

<commit_message>
data: field/odds refresh 2026-07-20 05:26 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -557,7 +557,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>100</v>
+        <v>96</v>
       </c>
     </row>
     <row r="9">
@@ -589,7 +589,7 @@
       </c>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="n">
-        <v>187</v>
+        <v>157</v>
       </c>
     </row>
     <row r="11">
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>134</v>
+        <v>139</v>
       </c>
     </row>
     <row r="18">
@@ -811,7 +811,7 @@
       </c>
       <c r="C24" t="inlineStr"/>
       <c r="D24" t="n">
-        <v>362</v>
+        <v>367</v>
       </c>
     </row>
     <row r="25">
@@ -837,7 +837,7 @@
       </c>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="n">
-        <v>270</v>
+        <v>286</v>
       </c>
     </row>
     <row r="27">
@@ -967,7 +967,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="35">
@@ -985,7 +985,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>336</v>
+        <v>287</v>
       </c>
     </row>
     <row r="36">
@@ -1087,7 +1087,7 @@
       </c>
       <c r="C42" t="inlineStr"/>
       <c r="D42" t="n">
-        <v>360</v>
+        <v>368</v>
       </c>
     </row>
     <row r="43">
@@ -1133,7 +1133,7 @@
       </c>
       <c r="C45" t="inlineStr"/>
       <c r="D45" t="n">
-        <v>189</v>
+        <v>183</v>
       </c>
     </row>
     <row r="46">
@@ -1181,7 +1181,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>113</v>
+        <v>123</v>
       </c>
     </row>
     <row r="49">
@@ -1195,7 +1195,7 @@
       </c>
       <c r="C49" t="inlineStr"/>
       <c r="D49" t="n">
-        <v>207</v>
+        <v>225</v>
       </c>
     </row>
     <row r="50">
@@ -1213,7 +1213,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>123</v>
+        <v>79</v>
       </c>
     </row>
     <row r="51">
@@ -1317,7 +1317,7 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>240</v>
+        <v>246</v>
       </c>
     </row>
     <row r="57">
@@ -1353,7 +1353,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>155</v>
+        <v>159</v>
       </c>
     </row>
     <row r="59">
@@ -1371,7 +1371,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>115</v>
+        <v>89</v>
       </c>
     </row>
     <row r="60">
@@ -1399,7 +1399,7 @@
       </c>
       <c r="C61" t="inlineStr"/>
       <c r="D61" t="n">
-        <v>457</v>
+        <v>461</v>
       </c>
     </row>
     <row r="62">
@@ -1467,7 +1467,7 @@
       </c>
       <c r="C65" t="inlineStr"/>
       <c r="D65" t="n">
-        <v>222</v>
+        <v>218</v>
       </c>
     </row>
     <row r="66">
@@ -1485,7 +1485,7 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>109</v>
+        <v>113</v>
       </c>
     </row>
     <row r="67">
@@ -1511,7 +1511,7 @@
       </c>
       <c r="C68" t="inlineStr"/>
       <c r="D68" t="n">
-        <v>262</v>
+        <v>274</v>
       </c>
     </row>
     <row r="69">
@@ -1639,7 +1639,7 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>104</v>
+        <v>107</v>
       </c>
     </row>
     <row r="77">
@@ -1653,7 +1653,7 @@
       </c>
       <c r="C77" t="inlineStr"/>
       <c r="D77" t="n">
-        <v>326</v>
+        <v>320</v>
       </c>
     </row>
     <row r="78">
@@ -1671,7 +1671,7 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>186</v>
+        <v>193</v>
       </c>
     </row>
     <row r="79">
@@ -1703,7 +1703,7 @@
       </c>
       <c r="C80" t="inlineStr"/>
       <c r="D80" t="n">
-        <v>155</v>
+        <v>119</v>
       </c>
     </row>
     <row r="81">
@@ -1721,7 +1721,7 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>92</v>
+        <v>101</v>
       </c>
     </row>
     <row r="82">
@@ -1751,7 +1751,7 @@
         </is>
       </c>
       <c r="D83" t="n">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="84">
@@ -1851,7 +1851,7 @@
       </c>
       <c r="C89" t="inlineStr"/>
       <c r="D89" t="n">
-        <v>158</v>
+        <v>161</v>
       </c>
     </row>
     <row r="90">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="C91" t="inlineStr"/>
       <c r="D91" t="n">
-        <v>130</v>
+        <v>133</v>
       </c>
     </row>
     <row r="92">
@@ -1901,7 +1901,7 @@
         </is>
       </c>
       <c r="D92" t="n">
-        <v>145</v>
+        <v>141</v>
       </c>
     </row>
     <row r="93">
@@ -1937,7 +1937,7 @@
         </is>
       </c>
       <c r="D94" t="n">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
     <row r="95">
@@ -1983,7 +1983,7 @@
       </c>
       <c r="C97" t="inlineStr"/>
       <c r="D97" t="n">
-        <v>154</v>
+        <v>156</v>
       </c>
     </row>
     <row r="98">
@@ -2081,7 +2081,7 @@
         </is>
       </c>
       <c r="D103" t="n">
-        <v>110</v>
+        <v>116</v>
       </c>
     </row>
     <row r="104">
@@ -2125,7 +2125,7 @@
       </c>
       <c r="C106" t="inlineStr"/>
       <c r="D106" t="n">
-        <v>384</v>
+        <v>400</v>
       </c>
     </row>
     <row r="107">
@@ -2187,7 +2187,7 @@
       </c>
       <c r="C110" t="inlineStr"/>
       <c r="D110" t="n">
-        <v>169</v>
+        <v>125</v>
       </c>
     </row>
     <row r="111">
@@ -2205,7 +2205,7 @@
         </is>
       </c>
       <c r="D111" t="n">
-        <v>218</v>
+        <v>203</v>
       </c>
     </row>
     <row r="112">
@@ -2219,7 +2219,7 @@
       </c>
       <c r="C112" t="inlineStr"/>
       <c r="D112" t="n">
-        <v>181</v>
+        <v>179</v>
       </c>
     </row>
     <row r="113">
@@ -2305,7 +2305,7 @@
         </is>
       </c>
       <c r="D118" t="n">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="119">
@@ -2331,7 +2331,7 @@
       </c>
       <c r="C120" t="inlineStr"/>
       <c r="D120" t="n">
-        <v>265</v>
+        <v>276</v>
       </c>
     </row>
     <row r="121">
@@ -2407,7 +2407,7 @@
       </c>
       <c r="C125" t="inlineStr"/>
       <c r="D125" t="n">
-        <v>490</v>
+        <v>481</v>
       </c>
     </row>
     <row r="126">
@@ -2443,7 +2443,7 @@
         </is>
       </c>
       <c r="D127" t="n">
-        <v>102</v>
+        <v>108</v>
       </c>
     </row>
     <row r="128">
@@ -2479,7 +2479,7 @@
         </is>
       </c>
       <c r="D129" t="n">
-        <v>97</v>
+        <v>102</v>
       </c>
     </row>
     <row r="130">
@@ -2613,7 +2613,7 @@
         </is>
       </c>
       <c r="D137" t="n">
-        <v>147</v>
+        <v>151</v>
       </c>
     </row>
     <row r="138">
@@ -2645,7 +2645,7 @@
       </c>
       <c r="C139" t="inlineStr"/>
       <c r="D139" t="n">
-        <v>129</v>
+        <v>126</v>
       </c>
     </row>
     <row r="140">
@@ -2781,7 +2781,7 @@
       </c>
       <c r="C148" t="inlineStr"/>
       <c r="D148" t="n">
-        <v>142</v>
+        <v>146</v>
       </c>
     </row>
     <row r="149">
@@ -2845,7 +2845,7 @@
       </c>
       <c r="C153" t="inlineStr"/>
       <c r="D153" t="n">
-        <v>304</v>
+        <v>315</v>
       </c>
     </row>
     <row r="154">
@@ -2863,7 +2863,7 @@
         </is>
       </c>
       <c r="D154" t="n">
-        <v>273</v>
+        <v>278</v>
       </c>
     </row>
     <row r="155">
@@ -2881,7 +2881,7 @@
         </is>
       </c>
       <c r="D155" t="n">
-        <v>93</v>
+        <v>87</v>
       </c>
     </row>
     <row r="156">
@@ -2931,7 +2931,7 @@
       </c>
       <c r="C158" t="inlineStr"/>
       <c r="D158" t="n">
-        <v>252</v>
+        <v>261</v>
       </c>
     </row>
     <row r="159">
@@ -2945,7 +2945,7 @@
       </c>
       <c r="C159" t="inlineStr"/>
       <c r="D159" t="n">
-        <v>175</v>
+        <v>167</v>
       </c>
     </row>
     <row r="160">
@@ -2995,7 +2995,7 @@
       </c>
       <c r="C162" t="inlineStr"/>
       <c r="D162" t="n">
-        <v>198</v>
+        <v>213</v>
       </c>
     </row>
     <row r="163">
@@ -3013,7 +3013,7 @@
         </is>
       </c>
       <c r="D163" t="n">
-        <v>89</v>
+        <v>93</v>
       </c>
     </row>
     <row r="164">
@@ -3063,7 +3063,7 @@
       </c>
       <c r="C166" t="inlineStr"/>
       <c r="D166" t="n">
-        <v>180</v>
+        <v>182</v>
       </c>
     </row>
     <row r="167">
@@ -3123,7 +3123,7 @@
         </is>
       </c>
       <c r="D170" t="n">
-        <v>174</v>
+        <v>176</v>
       </c>
     </row>
     <row r="171">
@@ -3141,7 +3141,7 @@
         </is>
       </c>
       <c r="D171" t="n">
-        <v>85</v>
+        <v>92</v>
       </c>
     </row>
     <row r="172">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="C174" t="inlineStr"/>
       <c r="D174" t="n">
-        <v>140</v>
+        <v>117</v>
       </c>
     </row>
     <row r="175">
@@ -3303,7 +3303,7 @@
         </is>
       </c>
       <c r="D181" t="n">
-        <v>171</v>
+        <v>184</v>
       </c>
     </row>
     <row r="182">
@@ -3321,7 +3321,7 @@
         </is>
       </c>
       <c r="D182" t="n">
-        <v>78</v>
+        <v>75</v>
       </c>
     </row>
     <row r="183">
@@ -3339,7 +3339,7 @@
         </is>
       </c>
       <c r="D183" t="n">
-        <v>78</v>
+        <v>75</v>
       </c>
     </row>
     <row r="184">
@@ -3385,7 +3385,7 @@
       </c>
       <c r="C186" t="inlineStr"/>
       <c r="D186" t="n">
-        <v>276</v>
+        <v>214</v>
       </c>
     </row>
     <row r="187">
@@ -3417,7 +3417,7 @@
       </c>
       <c r="C188" t="inlineStr"/>
       <c r="D188" t="n">
-        <v>271</v>
+        <v>266</v>
       </c>
     </row>
     <row r="189">
@@ -3483,7 +3483,7 @@
       </c>
       <c r="C192" t="inlineStr"/>
       <c r="D192" t="n">
-        <v>119</v>
+        <v>124</v>
       </c>
     </row>
     <row r="193">
@@ -3533,7 +3533,7 @@
       </c>
       <c r="C195" t="inlineStr"/>
       <c r="D195" t="n">
-        <v>287</v>
+        <v>298</v>
       </c>
     </row>
     <row r="196">
@@ -3601,7 +3601,7 @@
         </is>
       </c>
       <c r="D199" t="n">
-        <v>437</v>
+        <v>439</v>
       </c>
     </row>
     <row r="200">
@@ -3629,7 +3629,7 @@
       </c>
       <c r="C201" t="inlineStr"/>
       <c r="D201" t="n">
-        <v>438</v>
+        <v>459</v>
       </c>
     </row>
     <row r="202">
@@ -3715,7 +3715,7 @@
         </is>
       </c>
       <c r="D206" t="n">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="207">
@@ -3771,7 +3771,7 @@
       </c>
       <c r="C210" t="inlineStr"/>
       <c r="D210" t="n">
-        <v>379</v>
+        <v>383</v>
       </c>
     </row>
     <row r="211">
@@ -3807,7 +3807,7 @@
         </is>
       </c>
       <c r="D212" t="n">
-        <v>181</v>
+        <v>185</v>
       </c>
     </row>
     <row r="213">
@@ -3851,7 +3851,7 @@
       </c>
       <c r="C215" t="inlineStr"/>
       <c r="D215" t="n">
-        <v>311</v>
+        <v>270</v>
       </c>
     </row>
     <row r="216">
@@ -3865,7 +3865,7 @@
       </c>
       <c r="C216" t="inlineStr"/>
       <c r="D216" t="n">
-        <v>311</v>
+        <v>270</v>
       </c>
     </row>
     <row r="217">
@@ -3883,7 +3883,7 @@
         </is>
       </c>
       <c r="D217" t="n">
-        <v>197</v>
+        <v>191</v>
       </c>
     </row>
     <row r="218">
@@ -3897,7 +3897,7 @@
       </c>
       <c r="C218" t="inlineStr"/>
       <c r="D218" t="n">
-        <v>495</v>
+        <v>489</v>
       </c>
     </row>
     <row r="219">
@@ -3911,7 +3911,7 @@
       </c>
       <c r="C219" t="inlineStr"/>
       <c r="D219" t="n">
-        <v>254</v>
+        <v>264</v>
       </c>
     </row>
     <row r="220">
@@ -3965,7 +3965,7 @@
         </is>
       </c>
       <c r="D222" t="n">
-        <v>166</v>
+        <v>180</v>
       </c>
     </row>
     <row r="223">
@@ -4035,7 +4035,7 @@
       </c>
       <c r="C227" t="inlineStr"/>
       <c r="D227" t="n">
-        <v>377</v>
+        <v>375</v>
       </c>
     </row>
     <row r="228">
@@ -4067,7 +4067,7 @@
         </is>
       </c>
       <c r="D229" t="n">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="230">
@@ -4117,7 +4117,7 @@
         </is>
       </c>
       <c r="D232" t="n">
-        <v>124</v>
+        <v>131</v>
       </c>
     </row>
     <row r="233">

</xml_diff>

<commit_message>
data: field/odds refresh 2026-07-20 09:45 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -557,7 +557,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
     <row r="9">
@@ -589,7 +589,7 @@
       </c>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="n">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="11">
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>139</v>
+        <v>140</v>
       </c>
     </row>
     <row r="18">
@@ -811,7 +811,7 @@
       </c>
       <c r="C24" t="inlineStr"/>
       <c r="D24" t="n">
-        <v>367</v>
+        <v>373</v>
       </c>
     </row>
     <row r="25">
@@ -837,7 +837,7 @@
       </c>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="n">
-        <v>286</v>
+        <v>296</v>
       </c>
     </row>
     <row r="27">
@@ -905,7 +905,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>53</v>
+        <v>48</v>
       </c>
     </row>
     <row r="31">
@@ -923,7 +923,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>61</v>
+        <v>58</v>
       </c>
     </row>
     <row r="32">
@@ -967,7 +967,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="35">
@@ -985,7 +985,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>287</v>
+        <v>297</v>
       </c>
     </row>
     <row r="36">
@@ -1003,7 +1003,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="37">
@@ -1087,7 +1087,7 @@
       </c>
       <c r="C42" t="inlineStr"/>
       <c r="D42" t="n">
-        <v>368</v>
+        <v>362</v>
       </c>
     </row>
     <row r="43">
@@ -1133,7 +1133,7 @@
       </c>
       <c r="C45" t="inlineStr"/>
       <c r="D45" t="n">
-        <v>183</v>
+        <v>187</v>
       </c>
     </row>
     <row r="46">
@@ -1181,7 +1181,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="49">
@@ -1195,7 +1195,7 @@
       </c>
       <c r="C49" t="inlineStr"/>
       <c r="D49" t="n">
-        <v>225</v>
+        <v>230</v>
       </c>
     </row>
     <row r="50">
@@ -1213,7 +1213,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>79</v>
+        <v>84</v>
       </c>
     </row>
     <row r="51">
@@ -1317,7 +1317,7 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>246</v>
+        <v>253</v>
       </c>
     </row>
     <row r="57">
@@ -1353,7 +1353,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>159</v>
+        <v>162</v>
       </c>
     </row>
     <row r="59">
@@ -1371,7 +1371,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="60">
@@ -1399,7 +1399,7 @@
       </c>
       <c r="C61" t="inlineStr"/>
       <c r="D61" t="n">
-        <v>461</v>
+        <v>360</v>
       </c>
     </row>
     <row r="62">
@@ -1435,7 +1435,7 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>77</v>
+        <v>85</v>
       </c>
     </row>
     <row r="64">
@@ -1467,7 +1467,7 @@
       </c>
       <c r="C65" t="inlineStr"/>
       <c r="D65" t="n">
-        <v>218</v>
+        <v>226</v>
       </c>
     </row>
     <row r="66">
@@ -1511,7 +1511,7 @@
       </c>
       <c r="C68" t="inlineStr"/>
       <c r="D68" t="n">
-        <v>274</v>
+        <v>281</v>
       </c>
     </row>
     <row r="69">
@@ -1559,7 +1559,7 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="72">
@@ -1639,7 +1639,7 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>107</v>
+        <v>105</v>
       </c>
     </row>
     <row r="77">
@@ -1653,7 +1653,7 @@
       </c>
       <c r="C77" t="inlineStr"/>
       <c r="D77" t="n">
-        <v>320</v>
+        <v>322</v>
       </c>
     </row>
     <row r="78">
@@ -1671,7 +1671,7 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>193</v>
+        <v>185</v>
       </c>
     </row>
     <row r="79">
@@ -1703,7 +1703,7 @@
       </c>
       <c r="C80" t="inlineStr"/>
       <c r="D80" t="n">
-        <v>119</v>
+        <v>125</v>
       </c>
     </row>
     <row r="81">
@@ -1721,7 +1721,7 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>101</v>
+        <v>110</v>
       </c>
     </row>
     <row r="82">
@@ -1751,7 +1751,7 @@
         </is>
       </c>
       <c r="D83" t="n">
-        <v>112</v>
+        <v>114</v>
       </c>
     </row>
     <row r="84">
@@ -1787,7 +1787,7 @@
         </is>
       </c>
       <c r="D85" t="n">
-        <v>88</v>
+        <v>91</v>
       </c>
     </row>
     <row r="86">
@@ -1805,7 +1805,7 @@
         </is>
       </c>
       <c r="D86" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="87">
@@ -1823,7 +1823,7 @@
         </is>
       </c>
       <c r="D87" t="n">
-        <v>168</v>
+        <v>176</v>
       </c>
     </row>
     <row r="88">
@@ -1851,7 +1851,7 @@
       </c>
       <c r="C89" t="inlineStr"/>
       <c r="D89" t="n">
-        <v>161</v>
+        <v>164</v>
       </c>
     </row>
     <row r="90">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="C91" t="inlineStr"/>
       <c r="D91" t="n">
-        <v>133</v>
+        <v>136</v>
       </c>
     </row>
     <row r="92">
@@ -1919,7 +1919,7 @@
         </is>
       </c>
       <c r="D93" t="n">
-        <v>86</v>
+        <v>77</v>
       </c>
     </row>
     <row r="94">
@@ -1937,7 +1937,7 @@
         </is>
       </c>
       <c r="D94" t="n">
-        <v>98</v>
+        <v>101</v>
       </c>
     </row>
     <row r="95">
@@ -1983,7 +1983,7 @@
       </c>
       <c r="C97" t="inlineStr"/>
       <c r="D97" t="n">
-        <v>156</v>
+        <v>161</v>
       </c>
     </row>
     <row r="98">
@@ -2027,7 +2027,7 @@
         </is>
       </c>
       <c r="D100" t="n">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="101">
@@ -2063,7 +2063,7 @@
         </is>
       </c>
       <c r="D102" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="103">
@@ -2081,7 +2081,7 @@
         </is>
       </c>
       <c r="D103" t="n">
-        <v>116</v>
+        <v>118</v>
       </c>
     </row>
     <row r="104">
@@ -2111,7 +2111,7 @@
         </is>
       </c>
       <c r="D105" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="106">
@@ -2125,7 +2125,7 @@
       </c>
       <c r="C106" t="inlineStr"/>
       <c r="D106" t="n">
-        <v>400</v>
+        <v>407</v>
       </c>
     </row>
     <row r="107">
@@ -2143,7 +2143,7 @@
         </is>
       </c>
       <c r="D107" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="108">
@@ -2187,7 +2187,7 @@
       </c>
       <c r="C110" t="inlineStr"/>
       <c r="D110" t="n">
-        <v>125</v>
+        <v>128</v>
       </c>
     </row>
     <row r="111">
@@ -2205,7 +2205,7 @@
         </is>
       </c>
       <c r="D111" t="n">
-        <v>203</v>
+        <v>206</v>
       </c>
     </row>
     <row r="112">
@@ -2219,7 +2219,7 @@
       </c>
       <c r="C112" t="inlineStr"/>
       <c r="D112" t="n">
-        <v>179</v>
+        <v>180</v>
       </c>
     </row>
     <row r="113">
@@ -2305,7 +2305,7 @@
         </is>
       </c>
       <c r="D118" t="n">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="119">
@@ -2318,7 +2318,9 @@
         <v>7960</v>
       </c>
       <c r="C119" t="inlineStr"/>
-      <c r="D119" t="inlineStr"/>
+      <c r="D119" t="n">
+        <v>492</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -2331,7 +2333,7 @@
       </c>
       <c r="C120" t="inlineStr"/>
       <c r="D120" t="n">
-        <v>276</v>
+        <v>286</v>
       </c>
     </row>
     <row r="121">
@@ -2407,7 +2409,7 @@
       </c>
       <c r="C125" t="inlineStr"/>
       <c r="D125" t="n">
-        <v>481</v>
+        <v>488</v>
       </c>
     </row>
     <row r="126">
@@ -2425,7 +2427,7 @@
         </is>
       </c>
       <c r="D126" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="127">
@@ -2443,7 +2445,7 @@
         </is>
       </c>
       <c r="D127" t="n">
-        <v>108</v>
+        <v>103</v>
       </c>
     </row>
     <row r="128">
@@ -2479,7 +2481,7 @@
         </is>
       </c>
       <c r="D129" t="n">
-        <v>102</v>
+        <v>100</v>
       </c>
     </row>
     <row r="130">
@@ -2515,7 +2517,7 @@
         </is>
       </c>
       <c r="D131" t="n">
-        <v>39</v>
+        <v>42</v>
       </c>
     </row>
     <row r="132">
@@ -2533,7 +2535,7 @@
         </is>
       </c>
       <c r="D132" t="n">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="133">
@@ -2567,7 +2569,7 @@
         </is>
       </c>
       <c r="D134" t="n">
-        <v>68</v>
+        <v>73</v>
       </c>
     </row>
     <row r="135">
@@ -2613,7 +2615,7 @@
         </is>
       </c>
       <c r="D137" t="n">
-        <v>151</v>
+        <v>149</v>
       </c>
     </row>
     <row r="138">
@@ -2645,7 +2647,7 @@
       </c>
       <c r="C139" t="inlineStr"/>
       <c r="D139" t="n">
-        <v>126</v>
+        <v>129</v>
       </c>
     </row>
     <row r="140">
@@ -2673,7 +2675,7 @@
       </c>
       <c r="C141" t="inlineStr"/>
       <c r="D141" t="n">
-        <v>91</v>
+        <v>79</v>
       </c>
     </row>
     <row r="142">
@@ -2781,7 +2783,7 @@
       </c>
       <c r="C148" t="inlineStr"/>
       <c r="D148" t="n">
-        <v>146</v>
+        <v>150</v>
       </c>
     </row>
     <row r="149">
@@ -2845,7 +2847,7 @@
       </c>
       <c r="C153" t="inlineStr"/>
       <c r="D153" t="n">
-        <v>315</v>
+        <v>319</v>
       </c>
     </row>
     <row r="154">
@@ -2863,7 +2865,7 @@
         </is>
       </c>
       <c r="D154" t="n">
-        <v>278</v>
+        <v>283</v>
       </c>
     </row>
     <row r="155">
@@ -2881,7 +2883,7 @@
         </is>
       </c>
       <c r="D155" t="n">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
     <row r="156">
@@ -2931,7 +2933,7 @@
       </c>
       <c r="C158" t="inlineStr"/>
       <c r="D158" t="n">
-        <v>261</v>
+        <v>258</v>
       </c>
     </row>
     <row r="159">
@@ -2945,7 +2947,7 @@
       </c>
       <c r="C159" t="inlineStr"/>
       <c r="D159" t="n">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="160">
@@ -2981,7 +2983,7 @@
         </is>
       </c>
       <c r="D161" t="n">
-        <v>83</v>
+        <v>87</v>
       </c>
     </row>
     <row r="162">
@@ -2995,7 +2997,7 @@
       </c>
       <c r="C162" t="inlineStr"/>
       <c r="D162" t="n">
-        <v>213</v>
+        <v>203</v>
       </c>
     </row>
     <row r="163">
@@ -3013,7 +3015,7 @@
         </is>
       </c>
       <c r="D163" t="n">
-        <v>93</v>
+        <v>96</v>
       </c>
     </row>
     <row r="164">
@@ -3123,7 +3125,7 @@
         </is>
       </c>
       <c r="D170" t="n">
-        <v>176</v>
+        <v>177</v>
       </c>
     </row>
     <row r="171">
@@ -3141,7 +3143,7 @@
         </is>
       </c>
       <c r="D171" t="n">
-        <v>92</v>
+        <v>95</v>
       </c>
     </row>
     <row r="172">
@@ -3187,7 +3189,7 @@
       </c>
       <c r="C174" t="inlineStr"/>
       <c r="D174" t="n">
-        <v>117</v>
+        <v>120</v>
       </c>
     </row>
     <row r="175">
@@ -3250,7 +3252,9 @@
         <v>30814</v>
       </c>
       <c r="C178" t="inlineStr"/>
-      <c r="D178" t="inlineStr"/>
+      <c r="D178" t="n">
+        <v>343</v>
+      </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -3321,7 +3325,7 @@
         </is>
       </c>
       <c r="D182" t="n">
-        <v>75</v>
+        <v>81</v>
       </c>
     </row>
     <row r="183">
@@ -3339,7 +3343,7 @@
         </is>
       </c>
       <c r="D183" t="n">
-        <v>75</v>
+        <v>81</v>
       </c>
     </row>
     <row r="184">
@@ -3385,7 +3389,7 @@
       </c>
       <c r="C186" t="inlineStr"/>
       <c r="D186" t="n">
-        <v>214</v>
+        <v>219</v>
       </c>
     </row>
     <row r="187">
@@ -3417,7 +3421,7 @@
       </c>
       <c r="C188" t="inlineStr"/>
       <c r="D188" t="n">
-        <v>266</v>
+        <v>268</v>
       </c>
     </row>
     <row r="189">
@@ -3483,7 +3487,7 @@
       </c>
       <c r="C192" t="inlineStr"/>
       <c r="D192" t="n">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="193">
@@ -3533,7 +3537,7 @@
       </c>
       <c r="C195" t="inlineStr"/>
       <c r="D195" t="n">
-        <v>298</v>
+        <v>291</v>
       </c>
     </row>
     <row r="196">
@@ -3551,7 +3555,7 @@
         </is>
       </c>
       <c r="D196" t="n">
-        <v>47</v>
+        <v>52</v>
       </c>
     </row>
     <row r="197">
@@ -3565,7 +3569,7 @@
       </c>
       <c r="C197" t="inlineStr"/>
       <c r="D197" t="n">
-        <v>47</v>
+        <v>52</v>
       </c>
     </row>
     <row r="198">
@@ -3601,7 +3605,7 @@
         </is>
       </c>
       <c r="D199" t="n">
-        <v>439</v>
+        <v>448</v>
       </c>
     </row>
     <row r="200">
@@ -3615,7 +3619,7 @@
       </c>
       <c r="C200" t="inlineStr"/>
       <c r="D200" t="n">
-        <v>115</v>
+        <v>104</v>
       </c>
     </row>
     <row r="201">
@@ -3629,7 +3633,7 @@
       </c>
       <c r="C201" t="inlineStr"/>
       <c r="D201" t="n">
-        <v>459</v>
+        <v>467</v>
       </c>
     </row>
     <row r="202">
@@ -3643,7 +3647,7 @@
       </c>
       <c r="C202" t="inlineStr"/>
       <c r="D202" t="n">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="203">
@@ -3715,7 +3719,7 @@
         </is>
       </c>
       <c r="D206" t="n">
-        <v>150</v>
+        <v>148</v>
       </c>
     </row>
     <row r="207">
@@ -3771,7 +3775,7 @@
       </c>
       <c r="C210" t="inlineStr"/>
       <c r="D210" t="n">
-        <v>383</v>
+        <v>388</v>
       </c>
     </row>
     <row r="211">
@@ -3807,7 +3811,7 @@
         </is>
       </c>
       <c r="D212" t="n">
-        <v>185</v>
+        <v>190</v>
       </c>
     </row>
     <row r="213">
@@ -3851,7 +3855,7 @@
       </c>
       <c r="C215" t="inlineStr"/>
       <c r="D215" t="n">
-        <v>270</v>
+        <v>260</v>
       </c>
     </row>
     <row r="216">
@@ -3865,7 +3869,7 @@
       </c>
       <c r="C216" t="inlineStr"/>
       <c r="D216" t="n">
-        <v>270</v>
+        <v>260</v>
       </c>
     </row>
     <row r="217">
@@ -3897,7 +3901,7 @@
       </c>
       <c r="C218" t="inlineStr"/>
       <c r="D218" t="n">
-        <v>489</v>
+        <v>479</v>
       </c>
     </row>
     <row r="219">
@@ -3911,7 +3915,7 @@
       </c>
       <c r="C219" t="inlineStr"/>
       <c r="D219" t="n">
-        <v>264</v>
+        <v>270</v>
       </c>
     </row>
     <row r="220">
@@ -3965,7 +3969,7 @@
         </is>
       </c>
       <c r="D222" t="n">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
     <row r="223">
@@ -4004,7 +4008,9 @@
         <v>22051</v>
       </c>
       <c r="C225" t="inlineStr"/>
-      <c r="D225" t="inlineStr"/>
+      <c r="D225" t="n">
+        <v>464</v>
+      </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
@@ -4021,7 +4027,7 @@
         </is>
       </c>
       <c r="D226" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="227">
@@ -4035,7 +4041,7 @@
       </c>
       <c r="C227" t="inlineStr"/>
       <c r="D227" t="n">
-        <v>375</v>
+        <v>385</v>
       </c>
     </row>
     <row r="228">
@@ -4067,7 +4073,7 @@
         </is>
       </c>
       <c r="D229" t="n">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="230">
@@ -4117,7 +4123,7 @@
         </is>
       </c>
       <c r="D232" t="n">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="233">
@@ -4153,7 +4159,7 @@
         </is>
       </c>
       <c r="D234" t="n">
-        <v>82</v>
+        <v>63</v>
       </c>
     </row>
     <row r="235">

</xml_diff>

<commit_message>
data: field/odds refresh 2026-07-20 13:38 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -557,7 +557,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
     <row r="9">
@@ -589,7 +589,7 @@
       </c>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="n">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="11">
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>139</v>
+        <v>140</v>
       </c>
     </row>
     <row r="18">
@@ -811,7 +811,7 @@
       </c>
       <c r="C24" t="inlineStr"/>
       <c r="D24" t="n">
-        <v>367</v>
+        <v>373</v>
       </c>
     </row>
     <row r="25">
@@ -837,7 +837,7 @@
       </c>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="n">
-        <v>286</v>
+        <v>296</v>
       </c>
     </row>
     <row r="27">
@@ -905,7 +905,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>53</v>
+        <v>48</v>
       </c>
     </row>
     <row r="31">
@@ -923,7 +923,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>61</v>
+        <v>58</v>
       </c>
     </row>
     <row r="32">
@@ -967,7 +967,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="35">
@@ -985,7 +985,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>287</v>
+        <v>297</v>
       </c>
     </row>
     <row r="36">
@@ -1003,7 +1003,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="37">
@@ -1087,7 +1087,7 @@
       </c>
       <c r="C42" t="inlineStr"/>
       <c r="D42" t="n">
-        <v>368</v>
+        <v>362</v>
       </c>
     </row>
     <row r="43">
@@ -1133,7 +1133,7 @@
       </c>
       <c r="C45" t="inlineStr"/>
       <c r="D45" t="n">
-        <v>183</v>
+        <v>187</v>
       </c>
     </row>
     <row r="46">
@@ -1181,7 +1181,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="49">
@@ -1195,7 +1195,7 @@
       </c>
       <c r="C49" t="inlineStr"/>
       <c r="D49" t="n">
-        <v>225</v>
+        <v>230</v>
       </c>
     </row>
     <row r="50">
@@ -1213,7 +1213,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>79</v>
+        <v>84</v>
       </c>
     </row>
     <row r="51">
@@ -1317,7 +1317,7 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>246</v>
+        <v>253</v>
       </c>
     </row>
     <row r="57">
@@ -1353,7 +1353,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>159</v>
+        <v>162</v>
       </c>
     </row>
     <row r="59">
@@ -1371,7 +1371,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="60">
@@ -1399,7 +1399,7 @@
       </c>
       <c r="C61" t="inlineStr"/>
       <c r="D61" t="n">
-        <v>461</v>
+        <v>360</v>
       </c>
     </row>
     <row r="62">
@@ -1435,7 +1435,7 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>77</v>
+        <v>85</v>
       </c>
     </row>
     <row r="64">
@@ -1467,7 +1467,7 @@
       </c>
       <c r="C65" t="inlineStr"/>
       <c r="D65" t="n">
-        <v>218</v>
+        <v>226</v>
       </c>
     </row>
     <row r="66">
@@ -1511,7 +1511,7 @@
       </c>
       <c r="C68" t="inlineStr"/>
       <c r="D68" t="n">
-        <v>274</v>
+        <v>281</v>
       </c>
     </row>
     <row r="69">
@@ -1559,7 +1559,7 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="72">
@@ -1639,7 +1639,7 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>107</v>
+        <v>105</v>
       </c>
     </row>
     <row r="77">
@@ -1653,7 +1653,7 @@
       </c>
       <c r="C77" t="inlineStr"/>
       <c r="D77" t="n">
-        <v>320</v>
+        <v>322</v>
       </c>
     </row>
     <row r="78">
@@ -1671,7 +1671,7 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>193</v>
+        <v>185</v>
       </c>
     </row>
     <row r="79">
@@ -1703,7 +1703,7 @@
       </c>
       <c r="C80" t="inlineStr"/>
       <c r="D80" t="n">
-        <v>119</v>
+        <v>125</v>
       </c>
     </row>
     <row r="81">
@@ -1721,7 +1721,7 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>101</v>
+        <v>110</v>
       </c>
     </row>
     <row r="82">
@@ -1751,7 +1751,7 @@
         </is>
       </c>
       <c r="D83" t="n">
-        <v>112</v>
+        <v>114</v>
       </c>
     </row>
     <row r="84">
@@ -1787,7 +1787,7 @@
         </is>
       </c>
       <c r="D85" t="n">
-        <v>88</v>
+        <v>91</v>
       </c>
     </row>
     <row r="86">
@@ -1805,7 +1805,7 @@
         </is>
       </c>
       <c r="D86" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="87">
@@ -1823,7 +1823,7 @@
         </is>
       </c>
       <c r="D87" t="n">
-        <v>168</v>
+        <v>176</v>
       </c>
     </row>
     <row r="88">
@@ -1851,7 +1851,7 @@
       </c>
       <c r="C89" t="inlineStr"/>
       <c r="D89" t="n">
-        <v>161</v>
+        <v>164</v>
       </c>
     </row>
     <row r="90">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="C91" t="inlineStr"/>
       <c r="D91" t="n">
-        <v>133</v>
+        <v>136</v>
       </c>
     </row>
     <row r="92">
@@ -1919,7 +1919,7 @@
         </is>
       </c>
       <c r="D93" t="n">
-        <v>86</v>
+        <v>77</v>
       </c>
     </row>
     <row r="94">
@@ -1937,7 +1937,7 @@
         </is>
       </c>
       <c r="D94" t="n">
-        <v>98</v>
+        <v>101</v>
       </c>
     </row>
     <row r="95">
@@ -1983,7 +1983,7 @@
       </c>
       <c r="C97" t="inlineStr"/>
       <c r="D97" t="n">
-        <v>156</v>
+        <v>161</v>
       </c>
     </row>
     <row r="98">
@@ -2027,7 +2027,7 @@
         </is>
       </c>
       <c r="D100" t="n">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="101">
@@ -2063,7 +2063,7 @@
         </is>
       </c>
       <c r="D102" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="103">
@@ -2081,7 +2081,7 @@
         </is>
       </c>
       <c r="D103" t="n">
-        <v>116</v>
+        <v>118</v>
       </c>
     </row>
     <row r="104">
@@ -2111,7 +2111,7 @@
         </is>
       </c>
       <c r="D105" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="106">
@@ -2125,7 +2125,7 @@
       </c>
       <c r="C106" t="inlineStr"/>
       <c r="D106" t="n">
-        <v>400</v>
+        <v>407</v>
       </c>
     </row>
     <row r="107">
@@ -2143,7 +2143,7 @@
         </is>
       </c>
       <c r="D107" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="108">
@@ -2187,7 +2187,7 @@
       </c>
       <c r="C110" t="inlineStr"/>
       <c r="D110" t="n">
-        <v>125</v>
+        <v>128</v>
       </c>
     </row>
     <row r="111">
@@ -2205,7 +2205,7 @@
         </is>
       </c>
       <c r="D111" t="n">
-        <v>203</v>
+        <v>206</v>
       </c>
     </row>
     <row r="112">
@@ -2219,7 +2219,7 @@
       </c>
       <c r="C112" t="inlineStr"/>
       <c r="D112" t="n">
-        <v>179</v>
+        <v>180</v>
       </c>
     </row>
     <row r="113">
@@ -2305,7 +2305,7 @@
         </is>
       </c>
       <c r="D118" t="n">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="119">
@@ -2318,7 +2318,9 @@
         <v>7960</v>
       </c>
       <c r="C119" t="inlineStr"/>
-      <c r="D119" t="inlineStr"/>
+      <c r="D119" t="n">
+        <v>492</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -2331,7 +2333,7 @@
       </c>
       <c r="C120" t="inlineStr"/>
       <c r="D120" t="n">
-        <v>276</v>
+        <v>286</v>
       </c>
     </row>
     <row r="121">
@@ -2407,7 +2409,7 @@
       </c>
       <c r="C125" t="inlineStr"/>
       <c r="D125" t="n">
-        <v>481</v>
+        <v>488</v>
       </c>
     </row>
     <row r="126">
@@ -2425,7 +2427,7 @@
         </is>
       </c>
       <c r="D126" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="127">
@@ -2443,7 +2445,7 @@
         </is>
       </c>
       <c r="D127" t="n">
-        <v>108</v>
+        <v>103</v>
       </c>
     </row>
     <row r="128">
@@ -2479,7 +2481,7 @@
         </is>
       </c>
       <c r="D129" t="n">
-        <v>102</v>
+        <v>100</v>
       </c>
     </row>
     <row r="130">
@@ -2515,7 +2517,7 @@
         </is>
       </c>
       <c r="D131" t="n">
-        <v>39</v>
+        <v>42</v>
       </c>
     </row>
     <row r="132">
@@ -2533,7 +2535,7 @@
         </is>
       </c>
       <c r="D132" t="n">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="133">
@@ -2567,7 +2569,7 @@
         </is>
       </c>
       <c r="D134" t="n">
-        <v>68</v>
+        <v>73</v>
       </c>
     </row>
     <row r="135">
@@ -2613,7 +2615,7 @@
         </is>
       </c>
       <c r="D137" t="n">
-        <v>151</v>
+        <v>149</v>
       </c>
     </row>
     <row r="138">
@@ -2645,7 +2647,7 @@
       </c>
       <c r="C139" t="inlineStr"/>
       <c r="D139" t="n">
-        <v>126</v>
+        <v>129</v>
       </c>
     </row>
     <row r="140">
@@ -2673,7 +2675,7 @@
       </c>
       <c r="C141" t="inlineStr"/>
       <c r="D141" t="n">
-        <v>91</v>
+        <v>79</v>
       </c>
     </row>
     <row r="142">
@@ -2781,7 +2783,7 @@
       </c>
       <c r="C148" t="inlineStr"/>
       <c r="D148" t="n">
-        <v>146</v>
+        <v>150</v>
       </c>
     </row>
     <row r="149">
@@ -2845,7 +2847,7 @@
       </c>
       <c r="C153" t="inlineStr"/>
       <c r="D153" t="n">
-        <v>315</v>
+        <v>319</v>
       </c>
     </row>
     <row r="154">
@@ -2863,7 +2865,7 @@
         </is>
       </c>
       <c r="D154" t="n">
-        <v>278</v>
+        <v>283</v>
       </c>
     </row>
     <row r="155">
@@ -2881,7 +2883,7 @@
         </is>
       </c>
       <c r="D155" t="n">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
     <row r="156">
@@ -2931,7 +2933,7 @@
       </c>
       <c r="C158" t="inlineStr"/>
       <c r="D158" t="n">
-        <v>261</v>
+        <v>258</v>
       </c>
     </row>
     <row r="159">
@@ -2945,7 +2947,7 @@
       </c>
       <c r="C159" t="inlineStr"/>
       <c r="D159" t="n">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="160">
@@ -2981,7 +2983,7 @@
         </is>
       </c>
       <c r="D161" t="n">
-        <v>83</v>
+        <v>87</v>
       </c>
     </row>
     <row r="162">
@@ -2995,7 +2997,7 @@
       </c>
       <c r="C162" t="inlineStr"/>
       <c r="D162" t="n">
-        <v>213</v>
+        <v>203</v>
       </c>
     </row>
     <row r="163">
@@ -3013,7 +3015,7 @@
         </is>
       </c>
       <c r="D163" t="n">
-        <v>93</v>
+        <v>96</v>
       </c>
     </row>
     <row r="164">
@@ -3123,7 +3125,7 @@
         </is>
       </c>
       <c r="D170" t="n">
-        <v>176</v>
+        <v>177</v>
       </c>
     </row>
     <row r="171">
@@ -3141,7 +3143,7 @@
         </is>
       </c>
       <c r="D171" t="n">
-        <v>92</v>
+        <v>95</v>
       </c>
     </row>
     <row r="172">
@@ -3187,7 +3189,7 @@
       </c>
       <c r="C174" t="inlineStr"/>
       <c r="D174" t="n">
-        <v>117</v>
+        <v>120</v>
       </c>
     </row>
     <row r="175">
@@ -3250,7 +3252,9 @@
         <v>30814</v>
       </c>
       <c r="C178" t="inlineStr"/>
-      <c r="D178" t="inlineStr"/>
+      <c r="D178" t="n">
+        <v>343</v>
+      </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -3321,7 +3325,7 @@
         </is>
       </c>
       <c r="D182" t="n">
-        <v>75</v>
+        <v>81</v>
       </c>
     </row>
     <row r="183">
@@ -3339,7 +3343,7 @@
         </is>
       </c>
       <c r="D183" t="n">
-        <v>75</v>
+        <v>81</v>
       </c>
     </row>
     <row r="184">
@@ -3385,7 +3389,7 @@
       </c>
       <c r="C186" t="inlineStr"/>
       <c r="D186" t="n">
-        <v>214</v>
+        <v>219</v>
       </c>
     </row>
     <row r="187">
@@ -3417,7 +3421,7 @@
       </c>
       <c r="C188" t="inlineStr"/>
       <c r="D188" t="n">
-        <v>266</v>
+        <v>268</v>
       </c>
     </row>
     <row r="189">
@@ -3483,7 +3487,7 @@
       </c>
       <c r="C192" t="inlineStr"/>
       <c r="D192" t="n">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="193">
@@ -3533,7 +3537,7 @@
       </c>
       <c r="C195" t="inlineStr"/>
       <c r="D195" t="n">
-        <v>298</v>
+        <v>291</v>
       </c>
     </row>
     <row r="196">
@@ -3551,7 +3555,7 @@
         </is>
       </c>
       <c r="D196" t="n">
-        <v>47</v>
+        <v>52</v>
       </c>
     </row>
     <row r="197">
@@ -3565,7 +3569,7 @@
       </c>
       <c r="C197" t="inlineStr"/>
       <c r="D197" t="n">
-        <v>47</v>
+        <v>52</v>
       </c>
     </row>
     <row r="198">
@@ -3601,7 +3605,7 @@
         </is>
       </c>
       <c r="D199" t="n">
-        <v>439</v>
+        <v>448</v>
       </c>
     </row>
     <row r="200">
@@ -3615,7 +3619,7 @@
       </c>
       <c r="C200" t="inlineStr"/>
       <c r="D200" t="n">
-        <v>115</v>
+        <v>104</v>
       </c>
     </row>
     <row r="201">
@@ -3629,7 +3633,7 @@
       </c>
       <c r="C201" t="inlineStr"/>
       <c r="D201" t="n">
-        <v>459</v>
+        <v>467</v>
       </c>
     </row>
     <row r="202">
@@ -3643,7 +3647,7 @@
       </c>
       <c r="C202" t="inlineStr"/>
       <c r="D202" t="n">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="203">
@@ -3715,7 +3719,7 @@
         </is>
       </c>
       <c r="D206" t="n">
-        <v>150</v>
+        <v>148</v>
       </c>
     </row>
     <row r="207">
@@ -3771,7 +3775,7 @@
       </c>
       <c r="C210" t="inlineStr"/>
       <c r="D210" t="n">
-        <v>383</v>
+        <v>388</v>
       </c>
     </row>
     <row r="211">
@@ -3807,7 +3811,7 @@
         </is>
       </c>
       <c r="D212" t="n">
-        <v>185</v>
+        <v>190</v>
       </c>
     </row>
     <row r="213">
@@ -3851,7 +3855,7 @@
       </c>
       <c r="C215" t="inlineStr"/>
       <c r="D215" t="n">
-        <v>270</v>
+        <v>260</v>
       </c>
     </row>
     <row r="216">
@@ -3865,7 +3869,7 @@
       </c>
       <c r="C216" t="inlineStr"/>
       <c r="D216" t="n">
-        <v>270</v>
+        <v>260</v>
       </c>
     </row>
     <row r="217">
@@ -3897,7 +3901,7 @@
       </c>
       <c r="C218" t="inlineStr"/>
       <c r="D218" t="n">
-        <v>489</v>
+        <v>479</v>
       </c>
     </row>
     <row r="219">
@@ -3911,7 +3915,7 @@
       </c>
       <c r="C219" t="inlineStr"/>
       <c r="D219" t="n">
-        <v>264</v>
+        <v>270</v>
       </c>
     </row>
     <row r="220">
@@ -3965,7 +3969,7 @@
         </is>
       </c>
       <c r="D222" t="n">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
     <row r="223">
@@ -4004,7 +4008,9 @@
         <v>22051</v>
       </c>
       <c r="C225" t="inlineStr"/>
-      <c r="D225" t="inlineStr"/>
+      <c r="D225" t="n">
+        <v>464</v>
+      </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
@@ -4021,7 +4027,7 @@
         </is>
       </c>
       <c r="D226" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="227">
@@ -4035,7 +4041,7 @@
       </c>
       <c r="C227" t="inlineStr"/>
       <c r="D227" t="n">
-        <v>375</v>
+        <v>385</v>
       </c>
     </row>
     <row r="228">
@@ -4067,7 +4073,7 @@
         </is>
       </c>
       <c r="D229" t="n">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="230">
@@ -4117,7 +4123,7 @@
         </is>
       </c>
       <c r="D232" t="n">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="233">
@@ -4153,7 +4159,7 @@
         </is>
       </c>
       <c r="D234" t="n">
-        <v>82</v>
+        <v>63</v>
       </c>
     </row>
     <row r="235">

</xml_diff>

<commit_message>
data: field/odds refresh 2026-07-27 06:02 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -575,7 +575,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>29</v>
+        <v>32</v>
       </c>
     </row>
     <row r="10">
@@ -607,7 +607,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="12">
@@ -639,7 +639,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="14">
@@ -747,7 +747,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="21">
@@ -855,7 +855,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="28">
@@ -1105,7 +1105,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="44">
@@ -1119,7 +1119,7 @@
       </c>
       <c r="C44" t="inlineStr"/>
       <c r="D44" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="45">
@@ -1163,7 +1163,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="48">
@@ -1281,7 +1281,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="55">
@@ -1335,7 +1335,7 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>28</v>
+        <v>24</v>
       </c>
     </row>
     <row r="58">
@@ -1417,7 +1417,7 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="63">
@@ -1453,7 +1453,7 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
     </row>
     <row r="65">
@@ -1529,7 +1529,7 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>76</v>
+        <v>83</v>
       </c>
     </row>
     <row r="70">
@@ -1769,7 +1769,7 @@
         </is>
       </c>
       <c r="D84" t="n">
-        <v>35</v>
+        <v>38</v>
       </c>
     </row>
     <row r="85">
@@ -2045,7 +2045,7 @@
         </is>
       </c>
       <c r="D101" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
     </row>
     <row r="102">
@@ -2173,7 +2173,7 @@
         </is>
       </c>
       <c r="D109" t="n">
-        <v>118</v>
+        <v>111</v>
       </c>
     </row>
     <row r="110">
@@ -2463,7 +2463,7 @@
         </is>
       </c>
       <c r="D128" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="129">
@@ -2769,7 +2769,7 @@
         </is>
       </c>
       <c r="D147" t="n">
-        <v>69</v>
+        <v>74</v>
       </c>
     </row>
     <row r="148">
@@ -3271,7 +3271,7 @@
         </is>
       </c>
       <c r="D179" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="180">
@@ -3406,9 +3406,7 @@
           <t>https://pga-tour-res.cloudinary.com/image/upload/c_fill,g_face:center,q_auto,f_auto,dpr_2.0,h_220,w_200,d_stub:default_avatar_light.webp/headshots_29221</t>
         </is>
       </c>
-      <c r="D187" t="n">
-        <v>476</v>
-      </c>
+      <c r="D187" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -3505,7 +3503,7 @@
         </is>
       </c>
       <c r="D193" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="194">
@@ -3523,7 +3521,7 @@
         </is>
       </c>
       <c r="D194" t="n">
-        <v>51</v>
+        <v>55</v>
       </c>
     </row>
     <row r="195">
@@ -3665,7 +3663,7 @@
         </is>
       </c>
       <c r="D203" t="n">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="204">
@@ -3737,7 +3735,7 @@
         </is>
       </c>
       <c r="D207" t="n">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="208">
@@ -4091,7 +4089,7 @@
         </is>
       </c>
       <c r="D230" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="231">

</xml_diff>

<commit_message>
data: field/odds refresh 2026-07-27 10:08 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -557,7 +557,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="9">
@@ -607,7 +607,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="12">
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>140</v>
+        <v>148</v>
       </c>
     </row>
     <row r="18">
@@ -779,7 +779,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="23">
@@ -837,7 +837,7 @@
       </c>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="n">
-        <v>296</v>
+        <v>305</v>
       </c>
     </row>
     <row r="27">
@@ -873,7 +873,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="29">
@@ -905,7 +905,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="31">
@@ -923,7 +923,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>58</v>
+        <v>62</v>
       </c>
     </row>
     <row r="32">
@@ -967,7 +967,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>209</v>
+        <v>206</v>
       </c>
     </row>
     <row r="35">
@@ -985,7 +985,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>297</v>
+        <v>307</v>
       </c>
     </row>
     <row r="36">
@@ -1003,7 +1003,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>56</v>
+        <v>59</v>
       </c>
     </row>
     <row r="37">
@@ -1087,7 +1087,7 @@
       </c>
       <c r="C42" t="inlineStr"/>
       <c r="D42" t="n">
-        <v>362</v>
+        <v>368</v>
       </c>
     </row>
     <row r="43">
@@ -1105,7 +1105,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="44">
@@ -1119,7 +1119,7 @@
       </c>
       <c r="C44" t="inlineStr"/>
       <c r="D44" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="45">
@@ -1163,7 +1163,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="48">
@@ -1181,7 +1181,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>122</v>
+        <v>130</v>
       </c>
     </row>
     <row r="49">
@@ -1195,7 +1195,7 @@
       </c>
       <c r="C49" t="inlineStr"/>
       <c r="D49" t="n">
-        <v>230</v>
+        <v>210</v>
       </c>
     </row>
     <row r="50">
@@ -1213,7 +1213,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="51">
@@ -1317,7 +1317,7 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>253</v>
+        <v>260</v>
       </c>
     </row>
     <row r="57">
@@ -1353,7 +1353,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>162</v>
+        <v>169</v>
       </c>
     </row>
     <row r="59">
@@ -1371,7 +1371,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>90</v>
+        <v>93</v>
       </c>
     </row>
     <row r="60">
@@ -1435,7 +1435,7 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="64">
@@ -1485,7 +1485,7 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>113</v>
+        <v>101</v>
       </c>
     </row>
     <row r="67">
@@ -1529,7 +1529,7 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>83</v>
+        <v>86</v>
       </c>
     </row>
     <row r="70">
@@ -1639,7 +1639,7 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="77">
@@ -1671,7 +1671,7 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>185</v>
+        <v>193</v>
       </c>
     </row>
     <row r="79">
@@ -1689,7 +1689,7 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>62</v>
+        <v>65</v>
       </c>
     </row>
     <row r="80">
@@ -1703,7 +1703,7 @@
       </c>
       <c r="C80" t="inlineStr"/>
       <c r="D80" t="n">
-        <v>125</v>
+        <v>122</v>
       </c>
     </row>
     <row r="81">
@@ -1721,7 +1721,7 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="82">
@@ -1751,7 +1751,7 @@
         </is>
       </c>
       <c r="D83" t="n">
-        <v>114</v>
+        <v>118</v>
       </c>
     </row>
     <row r="84">
@@ -1787,7 +1787,7 @@
         </is>
       </c>
       <c r="D85" t="n">
-        <v>91</v>
+        <v>95</v>
       </c>
     </row>
     <row r="86">
@@ -1823,7 +1823,7 @@
         </is>
       </c>
       <c r="D87" t="n">
-        <v>176</v>
+        <v>164</v>
       </c>
     </row>
     <row r="88">
@@ -1851,7 +1851,7 @@
       </c>
       <c r="C89" t="inlineStr"/>
       <c r="D89" t="n">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="90">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="C91" t="inlineStr"/>
       <c r="D91" t="n">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="92">
@@ -1901,7 +1901,7 @@
         </is>
       </c>
       <c r="D92" t="n">
-        <v>141</v>
+        <v>146</v>
       </c>
     </row>
     <row r="93">
@@ -1919,7 +1919,7 @@
         </is>
       </c>
       <c r="D93" t="n">
-        <v>77</v>
+        <v>79</v>
       </c>
     </row>
     <row r="94">
@@ -1937,7 +1937,7 @@
         </is>
       </c>
       <c r="D94" t="n">
-        <v>101</v>
+        <v>106</v>
       </c>
     </row>
     <row r="95">
@@ -1983,7 +1983,7 @@
       </c>
       <c r="C97" t="inlineStr"/>
       <c r="D97" t="n">
-        <v>161</v>
+        <v>166</v>
       </c>
     </row>
     <row r="98">
@@ -2027,7 +2027,7 @@
         </is>
       </c>
       <c r="D100" t="n">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="101">
@@ -2081,7 +2081,7 @@
         </is>
       </c>
       <c r="D103" t="n">
-        <v>118</v>
+        <v>120</v>
       </c>
     </row>
     <row r="104">
@@ -2125,7 +2125,7 @@
       </c>
       <c r="C106" t="inlineStr"/>
       <c r="D106" t="n">
-        <v>407</v>
+        <v>428</v>
       </c>
     </row>
     <row r="107">
@@ -2143,7 +2143,7 @@
         </is>
       </c>
       <c r="D107" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="108">
@@ -2173,7 +2173,7 @@
         </is>
       </c>
       <c r="D109" t="n">
-        <v>111</v>
+        <v>113</v>
       </c>
     </row>
     <row r="110">
@@ -2187,7 +2187,7 @@
       </c>
       <c r="C110" t="inlineStr"/>
       <c r="D110" t="n">
-        <v>128</v>
+        <v>114</v>
       </c>
     </row>
     <row r="111">
@@ -2205,7 +2205,7 @@
         </is>
       </c>
       <c r="D111" t="n">
-        <v>206</v>
+        <v>73</v>
       </c>
     </row>
     <row r="112">
@@ -2219,7 +2219,7 @@
       </c>
       <c r="C112" t="inlineStr"/>
       <c r="D112" t="n">
-        <v>180</v>
+        <v>185</v>
       </c>
     </row>
     <row r="113">
@@ -2305,7 +2305,7 @@
         </is>
       </c>
       <c r="D118" t="n">
-        <v>112</v>
+        <v>115</v>
       </c>
     </row>
     <row r="119">
@@ -2427,7 +2427,7 @@
         </is>
       </c>
       <c r="D126" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
     </row>
     <row r="127">
@@ -2445,7 +2445,7 @@
         </is>
       </c>
       <c r="D127" t="n">
-        <v>103</v>
+        <v>90</v>
       </c>
     </row>
     <row r="128">
@@ -2463,7 +2463,7 @@
         </is>
       </c>
       <c r="D128" t="n">
-        <v>64</v>
+        <v>67</v>
       </c>
     </row>
     <row r="129">
@@ -2481,7 +2481,7 @@
         </is>
       </c>
       <c r="D129" t="n">
-        <v>100</v>
+        <v>107</v>
       </c>
     </row>
     <row r="130">
@@ -2535,7 +2535,7 @@
         </is>
       </c>
       <c r="D132" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="133">
@@ -2615,7 +2615,7 @@
         </is>
       </c>
       <c r="D137" t="n">
-        <v>149</v>
+        <v>153</v>
       </c>
     </row>
     <row r="138">
@@ -2647,7 +2647,7 @@
       </c>
       <c r="C139" t="inlineStr"/>
       <c r="D139" t="n">
-        <v>129</v>
+        <v>133</v>
       </c>
     </row>
     <row r="140">
@@ -2675,7 +2675,7 @@
       </c>
       <c r="C141" t="inlineStr"/>
       <c r="D141" t="n">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="142">
@@ -2769,7 +2769,7 @@
         </is>
       </c>
       <c r="D147" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="148">
@@ -2783,7 +2783,7 @@
       </c>
       <c r="C148" t="inlineStr"/>
       <c r="D148" t="n">
-        <v>150</v>
+        <v>158</v>
       </c>
     </row>
     <row r="149">
@@ -2865,7 +2865,7 @@
         </is>
       </c>
       <c r="D154" t="n">
-        <v>283</v>
+        <v>290</v>
       </c>
     </row>
     <row r="155">
@@ -2883,7 +2883,7 @@
         </is>
       </c>
       <c r="D155" t="n">
-        <v>89</v>
+        <v>92</v>
       </c>
     </row>
     <row r="156">
@@ -2901,7 +2901,7 @@
         </is>
       </c>
       <c r="D156" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="157">
@@ -2947,7 +2947,7 @@
       </c>
       <c r="C159" t="inlineStr"/>
       <c r="D159" t="n">
-        <v>168</v>
+        <v>132</v>
       </c>
     </row>
     <row r="160">
@@ -2983,7 +2983,7 @@
         </is>
       </c>
       <c r="D161" t="n">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="162">
@@ -2997,7 +2997,7 @@
       </c>
       <c r="C162" t="inlineStr"/>
       <c r="D162" t="n">
-        <v>203</v>
+        <v>184</v>
       </c>
     </row>
     <row r="163">
@@ -3065,7 +3065,7 @@
       </c>
       <c r="C166" t="inlineStr"/>
       <c r="D166" t="n">
-        <v>182</v>
+        <v>186</v>
       </c>
     </row>
     <row r="167">
@@ -3125,7 +3125,7 @@
         </is>
       </c>
       <c r="D170" t="n">
-        <v>177</v>
+        <v>180</v>
       </c>
     </row>
     <row r="171">
@@ -3143,7 +3143,7 @@
         </is>
       </c>
       <c r="D171" t="n">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="172">
@@ -3189,7 +3189,7 @@
       </c>
       <c r="C174" t="inlineStr"/>
       <c r="D174" t="n">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="175">
@@ -3253,7 +3253,7 @@
       </c>
       <c r="C178" t="inlineStr"/>
       <c r="D178" t="n">
-        <v>343</v>
+        <v>345</v>
       </c>
     </row>
     <row r="179">
@@ -3307,7 +3307,7 @@
         </is>
       </c>
       <c r="D181" t="n">
-        <v>184</v>
+        <v>190</v>
       </c>
     </row>
     <row r="182">
@@ -3325,7 +3325,7 @@
         </is>
       </c>
       <c r="D182" t="n">
-        <v>81</v>
+        <v>84</v>
       </c>
     </row>
     <row r="183">
@@ -3343,7 +3343,7 @@
         </is>
       </c>
       <c r="D183" t="n">
-        <v>81</v>
+        <v>84</v>
       </c>
     </row>
     <row r="184">
@@ -3485,7 +3485,7 @@
       </c>
       <c r="C192" t="inlineStr"/>
       <c r="D192" t="n">
-        <v>123</v>
+        <v>129</v>
       </c>
     </row>
     <row r="193">
@@ -3521,7 +3521,7 @@
         </is>
       </c>
       <c r="D194" t="n">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="195">
@@ -3553,7 +3553,7 @@
         </is>
       </c>
       <c r="D196" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="197">
@@ -3567,7 +3567,7 @@
       </c>
       <c r="C197" t="inlineStr"/>
       <c r="D197" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="198">
@@ -3603,7 +3603,7 @@
         </is>
       </c>
       <c r="D199" t="n">
-        <v>448</v>
+        <v>397</v>
       </c>
     </row>
     <row r="200">
@@ -3617,7 +3617,7 @@
       </c>
       <c r="C200" t="inlineStr"/>
       <c r="D200" t="n">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="201">
@@ -3631,7 +3631,7 @@
       </c>
       <c r="C201" t="inlineStr"/>
       <c r="D201" t="n">
-        <v>467</v>
+        <v>476</v>
       </c>
     </row>
     <row r="202">
@@ -3645,7 +3645,7 @@
       </c>
       <c r="C202" t="inlineStr"/>
       <c r="D202" t="n">
-        <v>166</v>
+        <v>168</v>
       </c>
     </row>
     <row r="203">
@@ -3663,7 +3663,7 @@
         </is>
       </c>
       <c r="D203" t="n">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="204">
@@ -3717,7 +3717,7 @@
         </is>
       </c>
       <c r="D206" t="n">
-        <v>148</v>
+        <v>136</v>
       </c>
     </row>
     <row r="207">
@@ -3773,7 +3773,7 @@
       </c>
       <c r="C210" t="inlineStr"/>
       <c r="D210" t="n">
-        <v>388</v>
+        <v>396</v>
       </c>
     </row>
     <row r="211">
@@ -3809,7 +3809,7 @@
         </is>
       </c>
       <c r="D212" t="n">
-        <v>190</v>
+        <v>195</v>
       </c>
     </row>
     <row r="213">
@@ -3853,7 +3853,7 @@
       </c>
       <c r="C215" t="inlineStr"/>
       <c r="D215" t="n">
-        <v>260</v>
+        <v>262</v>
       </c>
     </row>
     <row r="216">
@@ -3867,7 +3867,7 @@
       </c>
       <c r="C216" t="inlineStr"/>
       <c r="D216" t="n">
-        <v>260</v>
+        <v>262</v>
       </c>
     </row>
     <row r="217">
@@ -3885,7 +3885,7 @@
         </is>
       </c>
       <c r="D217" t="n">
-        <v>191</v>
+        <v>196</v>
       </c>
     </row>
     <row r="218">
@@ -3913,7 +3913,7 @@
       </c>
       <c r="C219" t="inlineStr"/>
       <c r="D219" t="n">
-        <v>270</v>
+        <v>277</v>
       </c>
     </row>
     <row r="220">
@@ -3931,7 +3931,7 @@
         </is>
       </c>
       <c r="D220" t="n">
-        <v>72</v>
+        <v>74</v>
       </c>
     </row>
     <row r="221">
@@ -4007,7 +4007,7 @@
       </c>
       <c r="C225" t="inlineStr"/>
       <c r="D225" t="n">
-        <v>464</v>
+        <v>466</v>
       </c>
     </row>
     <row r="226">
@@ -4039,7 +4039,7 @@
       </c>
       <c r="C227" t="inlineStr"/>
       <c r="D227" t="n">
-        <v>385</v>
+        <v>388</v>
       </c>
     </row>
     <row r="228">
@@ -4071,7 +4071,7 @@
         </is>
       </c>
       <c r="D229" t="n">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="230">
@@ -4121,7 +4121,7 @@
         </is>
       </c>
       <c r="D232" t="n">
-        <v>132</v>
+        <v>127</v>
       </c>
     </row>
     <row r="233">

</xml_diff>

<commit_message>
data: field/odds refresh 2026-07-27 12:00 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -557,7 +557,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="9">
@@ -575,7 +575,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>29</v>
+        <v>32</v>
       </c>
     </row>
     <row r="10">
@@ -607,7 +607,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>41</v>
+        <v>44</v>
       </c>
     </row>
     <row r="12">
@@ -639,7 +639,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="14">
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>140</v>
+        <v>148</v>
       </c>
     </row>
     <row r="18">
@@ -747,7 +747,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="21">
@@ -779,7 +779,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="23">
@@ -837,7 +837,7 @@
       </c>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="n">
-        <v>296</v>
+        <v>305</v>
       </c>
     </row>
     <row r="27">
@@ -855,7 +855,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="28">
@@ -873,7 +873,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="29">
@@ -905,7 +905,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="31">
@@ -923,7 +923,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>58</v>
+        <v>62</v>
       </c>
     </row>
     <row r="32">
@@ -967,7 +967,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>209</v>
+        <v>206</v>
       </c>
     </row>
     <row r="35">
@@ -985,7 +985,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>297</v>
+        <v>307</v>
       </c>
     </row>
     <row r="36">
@@ -1003,7 +1003,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>56</v>
+        <v>59</v>
       </c>
     </row>
     <row r="37">
@@ -1087,7 +1087,7 @@
       </c>
       <c r="C42" t="inlineStr"/>
       <c r="D42" t="n">
-        <v>362</v>
+        <v>368</v>
       </c>
     </row>
     <row r="43">
@@ -1105,7 +1105,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>52</v>
+        <v>56</v>
       </c>
     </row>
     <row r="44">
@@ -1119,7 +1119,7 @@
       </c>
       <c r="C44" t="inlineStr"/>
       <c r="D44" t="n">
-        <v>52</v>
+        <v>56</v>
       </c>
     </row>
     <row r="45">
@@ -1163,7 +1163,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="48">
@@ -1181,7 +1181,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>122</v>
+        <v>130</v>
       </c>
     </row>
     <row r="49">
@@ -1195,7 +1195,7 @@
       </c>
       <c r="C49" t="inlineStr"/>
       <c r="D49" t="n">
-        <v>230</v>
+        <v>210</v>
       </c>
     </row>
     <row r="50">
@@ -1213,7 +1213,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="51">
@@ -1281,7 +1281,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="55">
@@ -1317,7 +1317,7 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>253</v>
+        <v>260</v>
       </c>
     </row>
     <row r="57">
@@ -1335,7 +1335,7 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>28</v>
+        <v>24</v>
       </c>
     </row>
     <row r="58">
@@ -1353,7 +1353,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>162</v>
+        <v>169</v>
       </c>
     </row>
     <row r="59">
@@ -1371,7 +1371,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>90</v>
+        <v>93</v>
       </c>
     </row>
     <row r="60">
@@ -1417,7 +1417,7 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="63">
@@ -1435,7 +1435,7 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="64">
@@ -1453,7 +1453,7 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
     </row>
     <row r="65">
@@ -1485,7 +1485,7 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>113</v>
+        <v>101</v>
       </c>
     </row>
     <row r="67">
@@ -1529,7 +1529,7 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>76</v>
+        <v>86</v>
       </c>
     </row>
     <row r="70">
@@ -1639,7 +1639,7 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="77">
@@ -1671,7 +1671,7 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>185</v>
+        <v>193</v>
       </c>
     </row>
     <row r="79">
@@ -1689,7 +1689,7 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>62</v>
+        <v>65</v>
       </c>
     </row>
     <row r="80">
@@ -1703,7 +1703,7 @@
       </c>
       <c r="C80" t="inlineStr"/>
       <c r="D80" t="n">
-        <v>125</v>
+        <v>122</v>
       </c>
     </row>
     <row r="81">
@@ -1721,7 +1721,7 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="82">
@@ -1751,7 +1751,7 @@
         </is>
       </c>
       <c r="D83" t="n">
-        <v>114</v>
+        <v>118</v>
       </c>
     </row>
     <row r="84">
@@ -1769,7 +1769,7 @@
         </is>
       </c>
       <c r="D84" t="n">
-        <v>35</v>
+        <v>38</v>
       </c>
     </row>
     <row r="85">
@@ -1787,7 +1787,7 @@
         </is>
       </c>
       <c r="D85" t="n">
-        <v>91</v>
+        <v>95</v>
       </c>
     </row>
     <row r="86">
@@ -1823,7 +1823,7 @@
         </is>
       </c>
       <c r="D87" t="n">
-        <v>176</v>
+        <v>164</v>
       </c>
     </row>
     <row r="88">
@@ -1851,7 +1851,7 @@
       </c>
       <c r="C89" t="inlineStr"/>
       <c r="D89" t="n">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="90">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="C91" t="inlineStr"/>
       <c r="D91" t="n">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="92">
@@ -1901,7 +1901,7 @@
         </is>
       </c>
       <c r="D92" t="n">
-        <v>141</v>
+        <v>146</v>
       </c>
     </row>
     <row r="93">
@@ -1919,7 +1919,7 @@
         </is>
       </c>
       <c r="D93" t="n">
-        <v>77</v>
+        <v>79</v>
       </c>
     </row>
     <row r="94">
@@ -1937,7 +1937,7 @@
         </is>
       </c>
       <c r="D94" t="n">
-        <v>101</v>
+        <v>106</v>
       </c>
     </row>
     <row r="95">
@@ -1983,7 +1983,7 @@
       </c>
       <c r="C97" t="inlineStr"/>
       <c r="D97" t="n">
-        <v>161</v>
+        <v>166</v>
       </c>
     </row>
     <row r="98">
@@ -2027,7 +2027,7 @@
         </is>
       </c>
       <c r="D100" t="n">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="101">
@@ -2045,7 +2045,7 @@
         </is>
       </c>
       <c r="D101" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
     </row>
     <row r="102">
@@ -2081,7 +2081,7 @@
         </is>
       </c>
       <c r="D103" t="n">
-        <v>118</v>
+        <v>120</v>
       </c>
     </row>
     <row r="104">
@@ -2125,7 +2125,7 @@
       </c>
       <c r="C106" t="inlineStr"/>
       <c r="D106" t="n">
-        <v>407</v>
+        <v>428</v>
       </c>
     </row>
     <row r="107">
@@ -2143,7 +2143,7 @@
         </is>
       </c>
       <c r="D107" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="108">
@@ -2173,7 +2173,7 @@
         </is>
       </c>
       <c r="D109" t="n">
-        <v>118</v>
+        <v>113</v>
       </c>
     </row>
     <row r="110">
@@ -2187,7 +2187,7 @@
       </c>
       <c r="C110" t="inlineStr"/>
       <c r="D110" t="n">
-        <v>128</v>
+        <v>114</v>
       </c>
     </row>
     <row r="111">
@@ -2205,7 +2205,7 @@
         </is>
       </c>
       <c r="D111" t="n">
-        <v>206</v>
+        <v>73</v>
       </c>
     </row>
     <row r="112">
@@ -2219,7 +2219,7 @@
       </c>
       <c r="C112" t="inlineStr"/>
       <c r="D112" t="n">
-        <v>180</v>
+        <v>185</v>
       </c>
     </row>
     <row r="113">
@@ -2305,7 +2305,7 @@
         </is>
       </c>
       <c r="D118" t="n">
-        <v>112</v>
+        <v>115</v>
       </c>
     </row>
     <row r="119">
@@ -2427,7 +2427,7 @@
         </is>
       </c>
       <c r="D126" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
     </row>
     <row r="127">
@@ -2445,7 +2445,7 @@
         </is>
       </c>
       <c r="D127" t="n">
-        <v>103</v>
+        <v>90</v>
       </c>
     </row>
     <row r="128">
@@ -2463,7 +2463,7 @@
         </is>
       </c>
       <c r="D128" t="n">
-        <v>63</v>
+        <v>67</v>
       </c>
     </row>
     <row r="129">
@@ -2481,7 +2481,7 @@
         </is>
       </c>
       <c r="D129" t="n">
-        <v>100</v>
+        <v>107</v>
       </c>
     </row>
     <row r="130">
@@ -2535,7 +2535,7 @@
         </is>
       </c>
       <c r="D132" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="133">
@@ -2615,7 +2615,7 @@
         </is>
       </c>
       <c r="D137" t="n">
-        <v>149</v>
+        <v>153</v>
       </c>
     </row>
     <row r="138">
@@ -2647,7 +2647,7 @@
       </c>
       <c r="C139" t="inlineStr"/>
       <c r="D139" t="n">
-        <v>129</v>
+        <v>133</v>
       </c>
     </row>
     <row r="140">
@@ -2675,7 +2675,7 @@
       </c>
       <c r="C141" t="inlineStr"/>
       <c r="D141" t="n">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="142">
@@ -2769,7 +2769,7 @@
         </is>
       </c>
       <c r="D147" t="n">
-        <v>69</v>
+        <v>75</v>
       </c>
     </row>
     <row r="148">
@@ -2783,7 +2783,7 @@
       </c>
       <c r="C148" t="inlineStr"/>
       <c r="D148" t="n">
-        <v>150</v>
+        <v>158</v>
       </c>
     </row>
     <row r="149">
@@ -2865,7 +2865,7 @@
         </is>
       </c>
       <c r="D154" t="n">
-        <v>283</v>
+        <v>290</v>
       </c>
     </row>
     <row r="155">
@@ -2883,7 +2883,7 @@
         </is>
       </c>
       <c r="D155" t="n">
-        <v>89</v>
+        <v>92</v>
       </c>
     </row>
     <row r="156">
@@ -2901,7 +2901,7 @@
         </is>
       </c>
       <c r="D156" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="157">
@@ -2947,7 +2947,7 @@
       </c>
       <c r="C159" t="inlineStr"/>
       <c r="D159" t="n">
-        <v>168</v>
+        <v>132</v>
       </c>
     </row>
     <row r="160">
@@ -2983,7 +2983,7 @@
         </is>
       </c>
       <c r="D161" t="n">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="162">
@@ -2997,7 +2997,7 @@
       </c>
       <c r="C162" t="inlineStr"/>
       <c r="D162" t="n">
-        <v>203</v>
+        <v>184</v>
       </c>
     </row>
     <row r="163">
@@ -3065,7 +3065,7 @@
       </c>
       <c r="C166" t="inlineStr"/>
       <c r="D166" t="n">
-        <v>182</v>
+        <v>186</v>
       </c>
     </row>
     <row r="167">
@@ -3125,7 +3125,7 @@
         </is>
       </c>
       <c r="D170" t="n">
-        <v>177</v>
+        <v>180</v>
       </c>
     </row>
     <row r="171">
@@ -3143,7 +3143,7 @@
         </is>
       </c>
       <c r="D171" t="n">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="172">
@@ -3189,7 +3189,7 @@
       </c>
       <c r="C174" t="inlineStr"/>
       <c r="D174" t="n">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="175">
@@ -3253,7 +3253,7 @@
       </c>
       <c r="C178" t="inlineStr"/>
       <c r="D178" t="n">
-        <v>343</v>
+        <v>345</v>
       </c>
     </row>
     <row r="179">
@@ -3271,7 +3271,7 @@
         </is>
       </c>
       <c r="D179" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="180">
@@ -3307,7 +3307,7 @@
         </is>
       </c>
       <c r="D181" t="n">
-        <v>184</v>
+        <v>190</v>
       </c>
     </row>
     <row r="182">
@@ -3325,7 +3325,7 @@
         </is>
       </c>
       <c r="D182" t="n">
-        <v>81</v>
+        <v>84</v>
       </c>
     </row>
     <row r="183">
@@ -3343,7 +3343,7 @@
         </is>
       </c>
       <c r="D183" t="n">
-        <v>81</v>
+        <v>84</v>
       </c>
     </row>
     <row r="184">
@@ -3406,9 +3406,7 @@
           <t>https://pga-tour-res.cloudinary.com/image/upload/c_fill,g_face:center,q_auto,f_auto,dpr_2.0,h_220,w_200,d_stub:default_avatar_light.webp/headshots_29221</t>
         </is>
       </c>
-      <c r="D187" t="n">
-        <v>476</v>
-      </c>
+      <c r="D187" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -3487,7 +3485,7 @@
       </c>
       <c r="C192" t="inlineStr"/>
       <c r="D192" t="n">
-        <v>123</v>
+        <v>129</v>
       </c>
     </row>
     <row r="193">
@@ -3505,7 +3503,7 @@
         </is>
       </c>
       <c r="D193" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="194">
@@ -3523,7 +3521,7 @@
         </is>
       </c>
       <c r="D194" t="n">
-        <v>51</v>
+        <v>57</v>
       </c>
     </row>
     <row r="195">
@@ -3555,7 +3553,7 @@
         </is>
       </c>
       <c r="D196" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="197">
@@ -3569,7 +3567,7 @@
       </c>
       <c r="C197" t="inlineStr"/>
       <c r="D197" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="198">
@@ -3605,7 +3603,7 @@
         </is>
       </c>
       <c r="D199" t="n">
-        <v>448</v>
+        <v>397</v>
       </c>
     </row>
     <row r="200">
@@ -3619,7 +3617,7 @@
       </c>
       <c r="C200" t="inlineStr"/>
       <c r="D200" t="n">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="201">
@@ -3633,7 +3631,7 @@
       </c>
       <c r="C201" t="inlineStr"/>
       <c r="D201" t="n">
-        <v>467</v>
+        <v>476</v>
       </c>
     </row>
     <row r="202">
@@ -3647,7 +3645,7 @@
       </c>
       <c r="C202" t="inlineStr"/>
       <c r="D202" t="n">
-        <v>166</v>
+        <v>168</v>
       </c>
     </row>
     <row r="203">
@@ -3665,7 +3663,7 @@
         </is>
       </c>
       <c r="D203" t="n">
-        <v>67</v>
+        <v>72</v>
       </c>
     </row>
     <row r="204">
@@ -3719,7 +3717,7 @@
         </is>
       </c>
       <c r="D206" t="n">
-        <v>148</v>
+        <v>136</v>
       </c>
     </row>
     <row r="207">
@@ -3737,7 +3735,7 @@
         </is>
       </c>
       <c r="D207" t="n">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="208">
@@ -3775,7 +3773,7 @@
       </c>
       <c r="C210" t="inlineStr"/>
       <c r="D210" t="n">
-        <v>388</v>
+        <v>396</v>
       </c>
     </row>
     <row r="211">
@@ -3811,7 +3809,7 @@
         </is>
       </c>
       <c r="D212" t="n">
-        <v>190</v>
+        <v>195</v>
       </c>
     </row>
     <row r="213">
@@ -3855,7 +3853,7 @@
       </c>
       <c r="C215" t="inlineStr"/>
       <c r="D215" t="n">
-        <v>260</v>
+        <v>262</v>
       </c>
     </row>
     <row r="216">
@@ -3869,7 +3867,7 @@
       </c>
       <c r="C216" t="inlineStr"/>
       <c r="D216" t="n">
-        <v>260</v>
+        <v>262</v>
       </c>
     </row>
     <row r="217">
@@ -3887,7 +3885,7 @@
         </is>
       </c>
       <c r="D217" t="n">
-        <v>191</v>
+        <v>196</v>
       </c>
     </row>
     <row r="218">
@@ -3915,7 +3913,7 @@
       </c>
       <c r="C219" t="inlineStr"/>
       <c r="D219" t="n">
-        <v>270</v>
+        <v>277</v>
       </c>
     </row>
     <row r="220">
@@ -3933,7 +3931,7 @@
         </is>
       </c>
       <c r="D220" t="n">
-        <v>72</v>
+        <v>74</v>
       </c>
     </row>
     <row r="221">
@@ -4009,7 +4007,7 @@
       </c>
       <c r="C225" t="inlineStr"/>
       <c r="D225" t="n">
-        <v>464</v>
+        <v>466</v>
       </c>
     </row>
     <row r="226">
@@ -4041,7 +4039,7 @@
       </c>
       <c r="C227" t="inlineStr"/>
       <c r="D227" t="n">
-        <v>385</v>
+        <v>388</v>
       </c>
     </row>
     <row r="228">
@@ -4073,7 +4071,7 @@
         </is>
       </c>
       <c r="D229" t="n">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="230">
@@ -4091,7 +4089,7 @@
         </is>
       </c>
       <c r="D230" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="231">
@@ -4123,7 +4121,7 @@
         </is>
       </c>
       <c r="D232" t="n">
-        <v>132</v>
+        <v>127</v>
       </c>
     </row>
     <row r="233">

</xml_diff>

<commit_message>
data: field/odds refresh 2026-07-27 15:44 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -589,7 +589,7 @@
       </c>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="n">
-        <v>155</v>
+        <v>142</v>
       </c>
     </row>
     <row r="11">
@@ -3535,7 +3535,7 @@
       </c>
       <c r="C195" t="inlineStr"/>
       <c r="D195" t="n">
-        <v>291</v>
+        <v>298</v>
       </c>
     </row>
     <row r="196">

</xml_diff>

<commit_message>
data: field/odds refresh 2026-07-28 12:01 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -589,7 +589,7 @@
       </c>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="n">
-        <v>155</v>
+        <v>142</v>
       </c>
     </row>
     <row r="11">
@@ -3535,7 +3535,7 @@
       </c>
       <c r="C195" t="inlineStr"/>
       <c r="D195" t="n">
-        <v>291</v>
+        <v>298</v>
       </c>
     </row>
     <row r="196">

</xml_diff>

<commit_message>
data: field/odds refresh 2026-08-03 05:57 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -539,7 +539,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>49</v>
+        <v>54</v>
       </c>
     </row>
     <row r="8">
@@ -1559,7 +1559,7 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>66</v>
+        <v>58</v>
       </c>
     </row>
     <row r="72">
@@ -2063,7 +2063,7 @@
         </is>
       </c>
       <c r="D102" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="103">
@@ -2569,7 +2569,7 @@
         </is>
       </c>
       <c r="D134" t="n">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
     <row r="135">
@@ -2711,7 +2711,7 @@
         </is>
       </c>
       <c r="D143" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="144">
@@ -2965,7 +2965,7 @@
         </is>
       </c>
       <c r="D160" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="161">
@@ -3051,7 +3051,7 @@
         </is>
       </c>
       <c r="D165" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
     </row>
     <row r="166">
@@ -3437,7 +3437,7 @@
         </is>
       </c>
       <c r="D189" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="190">
@@ -3585,7 +3585,7 @@
         </is>
       </c>
       <c r="D198" t="n">
-        <v>23</v>
+        <v>26</v>
       </c>
     </row>
     <row r="199">
@@ -3699,7 +3699,7 @@
         </is>
       </c>
       <c r="D205" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
     </row>
     <row r="206">
@@ -4175,7 +4175,7 @@
         </is>
       </c>
       <c r="D235" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: field/odds refresh 2026-08-03 06:00 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -539,7 +539,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>49</v>
+        <v>54</v>
       </c>
     </row>
     <row r="8">
@@ -1559,7 +1559,7 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>66</v>
+        <v>58</v>
       </c>
     </row>
     <row r="72">
@@ -2063,7 +2063,7 @@
         </is>
       </c>
       <c r="D102" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="103">
@@ -2569,7 +2569,7 @@
         </is>
       </c>
       <c r="D134" t="n">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
     <row r="135">
@@ -2711,7 +2711,7 @@
         </is>
       </c>
       <c r="D143" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="144">
@@ -2965,7 +2965,7 @@
         </is>
       </c>
       <c r="D160" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="161">
@@ -3051,7 +3051,7 @@
         </is>
       </c>
       <c r="D165" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
     </row>
     <row r="166">
@@ -3437,7 +3437,7 @@
         </is>
       </c>
       <c r="D189" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="190">
@@ -3585,7 +3585,7 @@
         </is>
       </c>
       <c r="D198" t="n">
-        <v>23</v>
+        <v>26</v>
       </c>
     </row>
     <row r="199">
@@ -3699,7 +3699,7 @@
         </is>
       </c>
       <c r="D205" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
     </row>
     <row r="206">
@@ -4175,7 +4175,7 @@
         </is>
       </c>
       <c r="D235" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: field/odds refresh 2026-08-03 10:12 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -539,7 +539,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="8">
@@ -557,7 +557,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="9">
@@ -589,7 +589,7 @@
       </c>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="n">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="11">
@@ -607,7 +607,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="12">
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="18">
@@ -779,7 +779,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>102</v>
+        <v>96</v>
       </c>
     </row>
     <row r="23">
@@ -797,7 +797,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="24">
@@ -837,7 +837,7 @@
       </c>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="n">
-        <v>305</v>
+        <v>269</v>
       </c>
     </row>
     <row r="27">
@@ -873,7 +873,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>70</v>
+        <v>74</v>
       </c>
     </row>
     <row r="29">
@@ -923,7 +923,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="32">
@@ -967,7 +967,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>206</v>
+        <v>211</v>
       </c>
     </row>
     <row r="35">
@@ -985,7 +985,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>307</v>
+        <v>317</v>
       </c>
     </row>
     <row r="36">
@@ -1003,7 +1003,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>59</v>
+        <v>61</v>
       </c>
     </row>
     <row r="37">
@@ -1087,7 +1087,7 @@
       </c>
       <c r="C42" t="inlineStr"/>
       <c r="D42" t="n">
-        <v>368</v>
+        <v>386</v>
       </c>
     </row>
     <row r="43">
@@ -1105,7 +1105,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>56</v>
+        <v>59</v>
       </c>
     </row>
     <row r="44">
@@ -1119,7 +1119,7 @@
       </c>
       <c r="C44" t="inlineStr"/>
       <c r="D44" t="n">
-        <v>56</v>
+        <v>59</v>
       </c>
     </row>
     <row r="45">
@@ -1163,7 +1163,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="48">
@@ -1181,7 +1181,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>130</v>
+        <v>134</v>
       </c>
     </row>
     <row r="49">
@@ -1195,7 +1195,7 @@
       </c>
       <c r="C49" t="inlineStr"/>
       <c r="D49" t="n">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="50">
@@ -1213,7 +1213,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="51">
@@ -1317,7 +1317,7 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>260</v>
+        <v>265</v>
       </c>
     </row>
     <row r="57">
@@ -1335,7 +1335,7 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="58">
@@ -1353,7 +1353,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>169</v>
+        <v>155</v>
       </c>
     </row>
     <row r="59">
@@ -1371,7 +1371,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>93</v>
+        <v>100</v>
       </c>
     </row>
     <row r="60">
@@ -1435,7 +1435,7 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="64">
@@ -1453,7 +1453,7 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="65">
@@ -1467,7 +1467,7 @@
       </c>
       <c r="C65" t="inlineStr"/>
       <c r="D65" t="n">
-        <v>226</v>
+        <v>233</v>
       </c>
     </row>
     <row r="66">
@@ -1485,7 +1485,7 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>101</v>
+        <v>99</v>
       </c>
     </row>
     <row r="67">
@@ -1529,7 +1529,7 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="70">
@@ -1559,7 +1559,7 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="72">
@@ -1639,7 +1639,7 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>110</v>
+        <v>117</v>
       </c>
     </row>
     <row r="77">
@@ -1671,7 +1671,7 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>193</v>
+        <v>194</v>
       </c>
     </row>
     <row r="79">
@@ -1689,7 +1689,7 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="80">
@@ -1703,7 +1703,7 @@
       </c>
       <c r="C80" t="inlineStr"/>
       <c r="D80" t="n">
-        <v>122</v>
+        <v>130</v>
       </c>
     </row>
     <row r="81">
@@ -1721,7 +1721,7 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>112</v>
+        <v>103</v>
       </c>
     </row>
     <row r="82">
@@ -1751,7 +1751,7 @@
         </is>
       </c>
       <c r="D83" t="n">
-        <v>118</v>
+        <v>124</v>
       </c>
     </row>
     <row r="84">
@@ -1787,7 +1787,7 @@
         </is>
       </c>
       <c r="D85" t="n">
-        <v>95</v>
+        <v>77</v>
       </c>
     </row>
     <row r="86">
@@ -1823,7 +1823,7 @@
         </is>
       </c>
       <c r="D87" t="n">
-        <v>164</v>
+        <v>176</v>
       </c>
     </row>
     <row r="88">
@@ -1851,7 +1851,7 @@
       </c>
       <c r="C89" t="inlineStr"/>
       <c r="D89" t="n">
-        <v>163</v>
+        <v>165</v>
       </c>
     </row>
     <row r="90">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="C91" t="inlineStr"/>
       <c r="D91" t="n">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="92">
@@ -1901,7 +1901,7 @@
         </is>
       </c>
       <c r="D92" t="n">
-        <v>146</v>
+        <v>150</v>
       </c>
     </row>
     <row r="93">
@@ -1919,7 +1919,7 @@
         </is>
       </c>
       <c r="D93" t="n">
-        <v>79</v>
+        <v>75</v>
       </c>
     </row>
     <row r="94">
@@ -1937,7 +1937,7 @@
         </is>
       </c>
       <c r="D94" t="n">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="95">
@@ -1983,7 +1983,7 @@
       </c>
       <c r="C97" t="inlineStr"/>
       <c r="D97" t="n">
-        <v>166</v>
+        <v>171</v>
       </c>
     </row>
     <row r="98">
@@ -2027,7 +2027,7 @@
         </is>
       </c>
       <c r="D100" t="n">
-        <v>55</v>
+        <v>51</v>
       </c>
     </row>
     <row r="101">
@@ -2063,7 +2063,7 @@
         </is>
       </c>
       <c r="D102" t="n">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="103">
@@ -2081,7 +2081,7 @@
         </is>
       </c>
       <c r="D103" t="n">
-        <v>120</v>
+        <v>105</v>
       </c>
     </row>
     <row r="104">
@@ -2125,7 +2125,7 @@
       </c>
       <c r="C106" t="inlineStr"/>
       <c r="D106" t="n">
-        <v>428</v>
+        <v>447</v>
       </c>
     </row>
     <row r="107">
@@ -2173,7 +2173,7 @@
         </is>
       </c>
       <c r="D109" t="n">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="110">
@@ -2187,7 +2187,7 @@
       </c>
       <c r="C110" t="inlineStr"/>
       <c r="D110" t="n">
-        <v>114</v>
+        <v>108</v>
       </c>
     </row>
     <row r="111">
@@ -2205,7 +2205,7 @@
         </is>
       </c>
       <c r="D111" t="n">
-        <v>73</v>
+        <v>70</v>
       </c>
     </row>
     <row r="112">
@@ -2219,7 +2219,7 @@
       </c>
       <c r="C112" t="inlineStr"/>
       <c r="D112" t="n">
-        <v>185</v>
+        <v>182</v>
       </c>
     </row>
     <row r="113">
@@ -2333,7 +2333,7 @@
       </c>
       <c r="C120" t="inlineStr"/>
       <c r="D120" t="n">
-        <v>294</v>
+        <v>285</v>
       </c>
     </row>
     <row r="121">
@@ -2427,7 +2427,7 @@
         </is>
       </c>
       <c r="D126" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="127">
@@ -2445,7 +2445,7 @@
         </is>
       </c>
       <c r="D127" t="n">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="128">
@@ -2463,7 +2463,7 @@
         </is>
       </c>
       <c r="D128" t="n">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="129">
@@ -2481,7 +2481,7 @@
         </is>
       </c>
       <c r="D129" t="n">
-        <v>107</v>
+        <v>111</v>
       </c>
     </row>
     <row r="130">
@@ -2517,7 +2517,7 @@
         </is>
       </c>
       <c r="D131" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="132">
@@ -2535,7 +2535,7 @@
         </is>
       </c>
       <c r="D132" t="n">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="133">
@@ -2569,7 +2569,7 @@
         </is>
       </c>
       <c r="D134" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="135">
@@ -2615,7 +2615,7 @@
         </is>
       </c>
       <c r="D137" t="n">
-        <v>153</v>
+        <v>158</v>
       </c>
     </row>
     <row r="138">
@@ -2647,7 +2647,7 @@
       </c>
       <c r="C139" t="inlineStr"/>
       <c r="D139" t="n">
-        <v>133</v>
+        <v>136</v>
       </c>
     </row>
     <row r="140">
@@ -2675,7 +2675,7 @@
       </c>
       <c r="C141" t="inlineStr"/>
       <c r="D141" t="n">
-        <v>77</v>
+        <v>80</v>
       </c>
     </row>
     <row r="142">
@@ -2769,7 +2769,7 @@
         </is>
       </c>
       <c r="D147" t="n">
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="148">
@@ -2783,7 +2783,7 @@
       </c>
       <c r="C148" t="inlineStr"/>
       <c r="D148" t="n">
-        <v>158</v>
+        <v>152</v>
       </c>
     </row>
     <row r="149">
@@ -2865,7 +2865,7 @@
         </is>
       </c>
       <c r="D154" t="n">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="155">
@@ -2883,7 +2883,7 @@
         </is>
       </c>
       <c r="D155" t="n">
-        <v>92</v>
+        <v>95</v>
       </c>
     </row>
     <row r="156">
@@ -2901,7 +2901,7 @@
         </is>
       </c>
       <c r="D156" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="157">
@@ -2947,7 +2947,7 @@
       </c>
       <c r="C159" t="inlineStr"/>
       <c r="D159" t="n">
-        <v>132</v>
+        <v>135</v>
       </c>
     </row>
     <row r="160">
@@ -2965,7 +2965,7 @@
         </is>
       </c>
       <c r="D160" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="161">
@@ -2983,7 +2983,7 @@
         </is>
       </c>
       <c r="D161" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="162">
@@ -2997,7 +2997,7 @@
       </c>
       <c r="C162" t="inlineStr"/>
       <c r="D162" t="n">
-        <v>184</v>
+        <v>190</v>
       </c>
     </row>
     <row r="163">
@@ -3015,7 +3015,7 @@
         </is>
       </c>
       <c r="D163" t="n">
-        <v>96</v>
+        <v>101</v>
       </c>
     </row>
     <row r="164">
@@ -3051,7 +3051,7 @@
         </is>
       </c>
       <c r="D165" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="166">
@@ -3065,7 +3065,7 @@
       </c>
       <c r="C166" t="inlineStr"/>
       <c r="D166" t="n">
-        <v>186</v>
+        <v>191</v>
       </c>
     </row>
     <row r="167">
@@ -3125,7 +3125,7 @@
         </is>
       </c>
       <c r="D170" t="n">
-        <v>180</v>
+        <v>116</v>
       </c>
     </row>
     <row r="171">
@@ -3143,7 +3143,7 @@
         </is>
       </c>
       <c r="D171" t="n">
-        <v>97</v>
+        <v>102</v>
       </c>
     </row>
     <row r="172">
@@ -3189,7 +3189,7 @@
       </c>
       <c r="C174" t="inlineStr"/>
       <c r="D174" t="n">
-        <v>121</v>
+        <v>118</v>
       </c>
     </row>
     <row r="175">
@@ -3253,7 +3253,7 @@
       </c>
       <c r="C178" t="inlineStr"/>
       <c r="D178" t="n">
-        <v>345</v>
+        <v>326</v>
       </c>
     </row>
     <row r="179">
@@ -3307,7 +3307,7 @@
         </is>
       </c>
       <c r="D181" t="n">
-        <v>190</v>
+        <v>187</v>
       </c>
     </row>
     <row r="182">
@@ -3325,7 +3325,7 @@
         </is>
       </c>
       <c r="D182" t="n">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="183">
@@ -3343,7 +3343,7 @@
         </is>
       </c>
       <c r="D183" t="n">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="184">
@@ -3437,7 +3437,7 @@
         </is>
       </c>
       <c r="D189" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="190">
@@ -3485,7 +3485,7 @@
       </c>
       <c r="C192" t="inlineStr"/>
       <c r="D192" t="n">
-        <v>129</v>
+        <v>127</v>
       </c>
     </row>
     <row r="193">
@@ -3553,7 +3553,7 @@
         </is>
       </c>
       <c r="D196" t="n">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="197">
@@ -3567,7 +3567,7 @@
       </c>
       <c r="C197" t="inlineStr"/>
       <c r="D197" t="n">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="198">
@@ -3603,7 +3603,7 @@
         </is>
       </c>
       <c r="D199" t="n">
-        <v>397</v>
+        <v>407</v>
       </c>
     </row>
     <row r="200">
@@ -3617,7 +3617,7 @@
       </c>
       <c r="C200" t="inlineStr"/>
       <c r="D200" t="n">
-        <v>105</v>
+        <v>109</v>
       </c>
     </row>
     <row r="201">
@@ -3631,7 +3631,7 @@
       </c>
       <c r="C201" t="inlineStr"/>
       <c r="D201" t="n">
-        <v>476</v>
+        <v>475</v>
       </c>
     </row>
     <row r="202">
@@ -3645,7 +3645,7 @@
       </c>
       <c r="C202" t="inlineStr"/>
       <c r="D202" t="n">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="203">
@@ -3663,7 +3663,7 @@
         </is>
       </c>
       <c r="D203" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="204">
@@ -3681,7 +3681,7 @@
         </is>
       </c>
       <c r="D204" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="205">
@@ -3717,7 +3717,7 @@
         </is>
       </c>
       <c r="D206" t="n">
-        <v>136</v>
+        <v>123</v>
       </c>
     </row>
     <row r="207">
@@ -3773,7 +3773,7 @@
       </c>
       <c r="C210" t="inlineStr"/>
       <c r="D210" t="n">
-        <v>396</v>
+        <v>410</v>
       </c>
     </row>
     <row r="211">
@@ -3809,7 +3809,7 @@
         </is>
       </c>
       <c r="D212" t="n">
-        <v>195</v>
+        <v>198</v>
       </c>
     </row>
     <row r="213">
@@ -3853,7 +3853,7 @@
       </c>
       <c r="C215" t="inlineStr"/>
       <c r="D215" t="n">
-        <v>262</v>
+        <v>192</v>
       </c>
     </row>
     <row r="216">
@@ -3867,7 +3867,7 @@
       </c>
       <c r="C216" t="inlineStr"/>
       <c r="D216" t="n">
-        <v>262</v>
+        <v>192</v>
       </c>
     </row>
     <row r="217">
@@ -3885,7 +3885,7 @@
         </is>
       </c>
       <c r="D217" t="n">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="218">
@@ -3913,7 +3913,7 @@
       </c>
       <c r="C219" t="inlineStr"/>
       <c r="D219" t="n">
-        <v>277</v>
+        <v>284</v>
       </c>
     </row>
     <row r="220">
@@ -3931,7 +3931,7 @@
         </is>
       </c>
       <c r="D220" t="n">
-        <v>74</v>
+        <v>62</v>
       </c>
     </row>
     <row r="221">
@@ -3967,7 +3967,7 @@
         </is>
       </c>
       <c r="D222" t="n">
-        <v>181</v>
+        <v>184</v>
       </c>
     </row>
     <row r="223">
@@ -4007,7 +4007,7 @@
       </c>
       <c r="C225" t="inlineStr"/>
       <c r="D225" t="n">
-        <v>466</v>
+        <v>460</v>
       </c>
     </row>
     <row r="226">
@@ -4039,7 +4039,7 @@
       </c>
       <c r="C227" t="inlineStr"/>
       <c r="D227" t="n">
-        <v>388</v>
+        <v>389</v>
       </c>
     </row>
     <row r="228">
@@ -4121,7 +4121,7 @@
         </is>
       </c>
       <c r="D232" t="n">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="233">
@@ -4175,7 +4175,7 @@
         </is>
       </c>
       <c r="D235" t="n">
-        <v>66</v>
+        <v>68</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: field/odds refresh 2026-08-03 13:44 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -539,7 +539,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="8">
@@ -557,7 +557,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="9">
@@ -589,7 +589,7 @@
       </c>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="n">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="11">
@@ -607,7 +607,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="12">
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="18">
@@ -779,7 +779,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>102</v>
+        <v>96</v>
       </c>
     </row>
     <row r="23">
@@ -797,7 +797,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="24">
@@ -837,7 +837,7 @@
       </c>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="n">
-        <v>305</v>
+        <v>269</v>
       </c>
     </row>
     <row r="27">
@@ -873,7 +873,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>70</v>
+        <v>74</v>
       </c>
     </row>
     <row r="29">
@@ -923,7 +923,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="32">
@@ -967,7 +967,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>206</v>
+        <v>211</v>
       </c>
     </row>
     <row r="35">
@@ -985,7 +985,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>307</v>
+        <v>317</v>
       </c>
     </row>
     <row r="36">
@@ -1003,7 +1003,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>59</v>
+        <v>61</v>
       </c>
     </row>
     <row r="37">
@@ -1087,7 +1087,7 @@
       </c>
       <c r="C42" t="inlineStr"/>
       <c r="D42" t="n">
-        <v>368</v>
+        <v>386</v>
       </c>
     </row>
     <row r="43">
@@ -1105,7 +1105,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>56</v>
+        <v>59</v>
       </c>
     </row>
     <row r="44">
@@ -1119,7 +1119,7 @@
       </c>
       <c r="C44" t="inlineStr"/>
       <c r="D44" t="n">
-        <v>56</v>
+        <v>59</v>
       </c>
     </row>
     <row r="45">
@@ -1163,7 +1163,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="48">
@@ -1181,7 +1181,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>130</v>
+        <v>134</v>
       </c>
     </row>
     <row r="49">
@@ -1195,7 +1195,7 @@
       </c>
       <c r="C49" t="inlineStr"/>
       <c r="D49" t="n">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="50">
@@ -1213,7 +1213,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="51">
@@ -1317,7 +1317,7 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>260</v>
+        <v>265</v>
       </c>
     </row>
     <row r="57">
@@ -1335,7 +1335,7 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="58">
@@ -1353,7 +1353,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>169</v>
+        <v>155</v>
       </c>
     </row>
     <row r="59">
@@ -1371,7 +1371,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>93</v>
+        <v>100</v>
       </c>
     </row>
     <row r="60">
@@ -1435,7 +1435,7 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="64">
@@ -1453,7 +1453,7 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="65">
@@ -1467,7 +1467,7 @@
       </c>
       <c r="C65" t="inlineStr"/>
       <c r="D65" t="n">
-        <v>226</v>
+        <v>233</v>
       </c>
     </row>
     <row r="66">
@@ -1485,7 +1485,7 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>101</v>
+        <v>99</v>
       </c>
     </row>
     <row r="67">
@@ -1529,7 +1529,7 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="70">
@@ -1559,7 +1559,7 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="72">
@@ -1639,7 +1639,7 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>110</v>
+        <v>117</v>
       </c>
     </row>
     <row r="77">
@@ -1671,7 +1671,7 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>193</v>
+        <v>194</v>
       </c>
     </row>
     <row r="79">
@@ -1689,7 +1689,7 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="80">
@@ -1703,7 +1703,7 @@
       </c>
       <c r="C80" t="inlineStr"/>
       <c r="D80" t="n">
-        <v>122</v>
+        <v>130</v>
       </c>
     </row>
     <row r="81">
@@ -1721,7 +1721,7 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>112</v>
+        <v>103</v>
       </c>
     </row>
     <row r="82">
@@ -1751,7 +1751,7 @@
         </is>
       </c>
       <c r="D83" t="n">
-        <v>118</v>
+        <v>124</v>
       </c>
     </row>
     <row r="84">
@@ -1787,7 +1787,7 @@
         </is>
       </c>
       <c r="D85" t="n">
-        <v>95</v>
+        <v>77</v>
       </c>
     </row>
     <row r="86">
@@ -1823,7 +1823,7 @@
         </is>
       </c>
       <c r="D87" t="n">
-        <v>164</v>
+        <v>176</v>
       </c>
     </row>
     <row r="88">
@@ -1851,7 +1851,7 @@
       </c>
       <c r="C89" t="inlineStr"/>
       <c r="D89" t="n">
-        <v>163</v>
+        <v>165</v>
       </c>
     </row>
     <row r="90">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="C91" t="inlineStr"/>
       <c r="D91" t="n">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="92">
@@ -1901,7 +1901,7 @@
         </is>
       </c>
       <c r="D92" t="n">
-        <v>146</v>
+        <v>150</v>
       </c>
     </row>
     <row r="93">
@@ -1919,7 +1919,7 @@
         </is>
       </c>
       <c r="D93" t="n">
-        <v>79</v>
+        <v>75</v>
       </c>
     </row>
     <row r="94">
@@ -1937,7 +1937,7 @@
         </is>
       </c>
       <c r="D94" t="n">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="95">
@@ -1983,7 +1983,7 @@
       </c>
       <c r="C97" t="inlineStr"/>
       <c r="D97" t="n">
-        <v>166</v>
+        <v>171</v>
       </c>
     </row>
     <row r="98">
@@ -2027,7 +2027,7 @@
         </is>
       </c>
       <c r="D100" t="n">
-        <v>55</v>
+        <v>51</v>
       </c>
     </row>
     <row r="101">
@@ -2063,7 +2063,7 @@
         </is>
       </c>
       <c r="D102" t="n">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="103">
@@ -2081,7 +2081,7 @@
         </is>
       </c>
       <c r="D103" t="n">
-        <v>120</v>
+        <v>105</v>
       </c>
     </row>
     <row r="104">
@@ -2125,7 +2125,7 @@
       </c>
       <c r="C106" t="inlineStr"/>
       <c r="D106" t="n">
-        <v>428</v>
+        <v>447</v>
       </c>
     </row>
     <row r="107">
@@ -2173,7 +2173,7 @@
         </is>
       </c>
       <c r="D109" t="n">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="110">
@@ -2187,7 +2187,7 @@
       </c>
       <c r="C110" t="inlineStr"/>
       <c r="D110" t="n">
-        <v>114</v>
+        <v>108</v>
       </c>
     </row>
     <row r="111">
@@ -2205,7 +2205,7 @@
         </is>
       </c>
       <c r="D111" t="n">
-        <v>73</v>
+        <v>70</v>
       </c>
     </row>
     <row r="112">
@@ -2219,7 +2219,7 @@
       </c>
       <c r="C112" t="inlineStr"/>
       <c r="D112" t="n">
-        <v>185</v>
+        <v>182</v>
       </c>
     </row>
     <row r="113">
@@ -2333,7 +2333,7 @@
       </c>
       <c r="C120" t="inlineStr"/>
       <c r="D120" t="n">
-        <v>294</v>
+        <v>285</v>
       </c>
     </row>
     <row r="121">
@@ -2427,7 +2427,7 @@
         </is>
       </c>
       <c r="D126" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="127">
@@ -2445,7 +2445,7 @@
         </is>
       </c>
       <c r="D127" t="n">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="128">
@@ -2463,7 +2463,7 @@
         </is>
       </c>
       <c r="D128" t="n">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="129">
@@ -2481,7 +2481,7 @@
         </is>
       </c>
       <c r="D129" t="n">
-        <v>107</v>
+        <v>111</v>
       </c>
     </row>
     <row r="130">
@@ -2517,7 +2517,7 @@
         </is>
       </c>
       <c r="D131" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="132">
@@ -2535,7 +2535,7 @@
         </is>
       </c>
       <c r="D132" t="n">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="133">
@@ -2569,7 +2569,7 @@
         </is>
       </c>
       <c r="D134" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="135">
@@ -2615,7 +2615,7 @@
         </is>
       </c>
       <c r="D137" t="n">
-        <v>153</v>
+        <v>158</v>
       </c>
     </row>
     <row r="138">
@@ -2647,7 +2647,7 @@
       </c>
       <c r="C139" t="inlineStr"/>
       <c r="D139" t="n">
-        <v>133</v>
+        <v>136</v>
       </c>
     </row>
     <row r="140">
@@ -2675,7 +2675,7 @@
       </c>
       <c r="C141" t="inlineStr"/>
       <c r="D141" t="n">
-        <v>77</v>
+        <v>80</v>
       </c>
     </row>
     <row r="142">
@@ -2769,7 +2769,7 @@
         </is>
       </c>
       <c r="D147" t="n">
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="148">
@@ -2783,7 +2783,7 @@
       </c>
       <c r="C148" t="inlineStr"/>
       <c r="D148" t="n">
-        <v>158</v>
+        <v>152</v>
       </c>
     </row>
     <row r="149">
@@ -2865,7 +2865,7 @@
         </is>
       </c>
       <c r="D154" t="n">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="155">
@@ -2883,7 +2883,7 @@
         </is>
       </c>
       <c r="D155" t="n">
-        <v>92</v>
+        <v>95</v>
       </c>
     </row>
     <row r="156">
@@ -2901,7 +2901,7 @@
         </is>
       </c>
       <c r="D156" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="157">
@@ -2947,7 +2947,7 @@
       </c>
       <c r="C159" t="inlineStr"/>
       <c r="D159" t="n">
-        <v>132</v>
+        <v>135</v>
       </c>
     </row>
     <row r="160">
@@ -2965,7 +2965,7 @@
         </is>
       </c>
       <c r="D160" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="161">
@@ -2983,7 +2983,7 @@
         </is>
       </c>
       <c r="D161" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="162">
@@ -2997,7 +2997,7 @@
       </c>
       <c r="C162" t="inlineStr"/>
       <c r="D162" t="n">
-        <v>184</v>
+        <v>190</v>
       </c>
     </row>
     <row r="163">
@@ -3015,7 +3015,7 @@
         </is>
       </c>
       <c r="D163" t="n">
-        <v>96</v>
+        <v>101</v>
       </c>
     </row>
     <row r="164">
@@ -3051,7 +3051,7 @@
         </is>
       </c>
       <c r="D165" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="166">
@@ -3065,7 +3065,7 @@
       </c>
       <c r="C166" t="inlineStr"/>
       <c r="D166" t="n">
-        <v>186</v>
+        <v>191</v>
       </c>
     </row>
     <row r="167">
@@ -3125,7 +3125,7 @@
         </is>
       </c>
       <c r="D170" t="n">
-        <v>180</v>
+        <v>116</v>
       </c>
     </row>
     <row r="171">
@@ -3143,7 +3143,7 @@
         </is>
       </c>
       <c r="D171" t="n">
-        <v>97</v>
+        <v>102</v>
       </c>
     </row>
     <row r="172">
@@ -3189,7 +3189,7 @@
       </c>
       <c r="C174" t="inlineStr"/>
       <c r="D174" t="n">
-        <v>121</v>
+        <v>118</v>
       </c>
     </row>
     <row r="175">
@@ -3253,7 +3253,7 @@
       </c>
       <c r="C178" t="inlineStr"/>
       <c r="D178" t="n">
-        <v>345</v>
+        <v>326</v>
       </c>
     </row>
     <row r="179">
@@ -3307,7 +3307,7 @@
         </is>
       </c>
       <c r="D181" t="n">
-        <v>190</v>
+        <v>187</v>
       </c>
     </row>
     <row r="182">
@@ -3325,7 +3325,7 @@
         </is>
       </c>
       <c r="D182" t="n">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="183">
@@ -3343,7 +3343,7 @@
         </is>
       </c>
       <c r="D183" t="n">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="184">
@@ -3437,7 +3437,7 @@
         </is>
       </c>
       <c r="D189" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="190">
@@ -3485,7 +3485,7 @@
       </c>
       <c r="C192" t="inlineStr"/>
       <c r="D192" t="n">
-        <v>129</v>
+        <v>127</v>
       </c>
     </row>
     <row r="193">
@@ -3535,7 +3535,7 @@
       </c>
       <c r="C195" t="inlineStr"/>
       <c r="D195" t="n">
-        <v>298</v>
+        <v>309</v>
       </c>
     </row>
     <row r="196">
@@ -3553,7 +3553,7 @@
         </is>
       </c>
       <c r="D196" t="n">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="197">
@@ -3567,7 +3567,7 @@
       </c>
       <c r="C197" t="inlineStr"/>
       <c r="D197" t="n">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="198">
@@ -3603,7 +3603,7 @@
         </is>
       </c>
       <c r="D199" t="n">
-        <v>397</v>
+        <v>407</v>
       </c>
     </row>
     <row r="200">
@@ -3617,7 +3617,7 @@
       </c>
       <c r="C200" t="inlineStr"/>
       <c r="D200" t="n">
-        <v>105</v>
+        <v>109</v>
       </c>
     </row>
     <row r="201">
@@ -3631,7 +3631,7 @@
       </c>
       <c r="C201" t="inlineStr"/>
       <c r="D201" t="n">
-        <v>476</v>
+        <v>475</v>
       </c>
     </row>
     <row r="202">
@@ -3645,7 +3645,7 @@
       </c>
       <c r="C202" t="inlineStr"/>
       <c r="D202" t="n">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="203">
@@ -3663,7 +3663,7 @@
         </is>
       </c>
       <c r="D203" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="204">
@@ -3681,7 +3681,7 @@
         </is>
       </c>
       <c r="D204" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="205">
@@ -3717,7 +3717,7 @@
         </is>
       </c>
       <c r="D206" t="n">
-        <v>136</v>
+        <v>123</v>
       </c>
     </row>
     <row r="207">
@@ -3773,7 +3773,7 @@
       </c>
       <c r="C210" t="inlineStr"/>
       <c r="D210" t="n">
-        <v>396</v>
+        <v>410</v>
       </c>
     </row>
     <row r="211">
@@ -3809,7 +3809,7 @@
         </is>
       </c>
       <c r="D212" t="n">
-        <v>195</v>
+        <v>198</v>
       </c>
     </row>
     <row r="213">
@@ -3853,7 +3853,7 @@
       </c>
       <c r="C215" t="inlineStr"/>
       <c r="D215" t="n">
-        <v>262</v>
+        <v>192</v>
       </c>
     </row>
     <row r="216">
@@ -3867,7 +3867,7 @@
       </c>
       <c r="C216" t="inlineStr"/>
       <c r="D216" t="n">
-        <v>262</v>
+        <v>192</v>
       </c>
     </row>
     <row r="217">
@@ -3885,7 +3885,7 @@
         </is>
       </c>
       <c r="D217" t="n">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="218">
@@ -3899,7 +3899,7 @@
       </c>
       <c r="C218" t="inlineStr"/>
       <c r="D218" t="n">
-        <v>479</v>
+        <v>473</v>
       </c>
     </row>
     <row r="219">
@@ -3913,7 +3913,7 @@
       </c>
       <c r="C219" t="inlineStr"/>
       <c r="D219" t="n">
-        <v>277</v>
+        <v>284</v>
       </c>
     </row>
     <row r="220">
@@ -3931,7 +3931,7 @@
         </is>
       </c>
       <c r="D220" t="n">
-        <v>74</v>
+        <v>62</v>
       </c>
     </row>
     <row r="221">
@@ -3967,7 +3967,7 @@
         </is>
       </c>
       <c r="D222" t="n">
-        <v>181</v>
+        <v>184</v>
       </c>
     </row>
     <row r="223">
@@ -4007,7 +4007,7 @@
       </c>
       <c r="C225" t="inlineStr"/>
       <c r="D225" t="n">
-        <v>466</v>
+        <v>460</v>
       </c>
     </row>
     <row r="226">
@@ -4039,7 +4039,7 @@
       </c>
       <c r="C227" t="inlineStr"/>
       <c r="D227" t="n">
-        <v>388</v>
+        <v>389</v>
       </c>
     </row>
     <row r="228">
@@ -4121,7 +4121,7 @@
         </is>
       </c>
       <c r="D232" t="n">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="233">
@@ -4175,7 +4175,7 @@
         </is>
       </c>
       <c r="D235" t="n">
-        <v>66</v>
+        <v>68</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: field/odds refresh 2026-08-03 13:45 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -3535,7 +3535,7 @@
       </c>
       <c r="C195" t="inlineStr"/>
       <c r="D195" t="n">
-        <v>298</v>
+        <v>309</v>
       </c>
     </row>
     <row r="196">
@@ -3899,7 +3899,7 @@
       </c>
       <c r="C218" t="inlineStr"/>
       <c r="D218" t="n">
-        <v>479</v>
+        <v>473</v>
       </c>
     </row>
     <row r="219">

</xml_diff>

<commit_message>
data: field/odds refresh 2026-08-03 16:53 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -2318,9 +2318,7 @@
         <v>7960</v>
       </c>
       <c r="C119" t="inlineStr"/>
-      <c r="D119" t="n">
-        <v>492</v>
-      </c>
+      <c r="D119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">

</xml_diff>

<commit_message>
data: field/odds refresh 2026-08-04 12:00 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -2318,9 +2318,7 @@
         <v>7960</v>
       </c>
       <c r="C119" t="inlineStr"/>
-      <c r="D119" t="n">
-        <v>492</v>
-      </c>
+      <c r="D119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -3389,7 +3387,7 @@
       </c>
       <c r="C186" t="inlineStr"/>
       <c r="D186" t="n">
-        <v>221</v>
+        <v>228</v>
       </c>
     </row>
     <row r="187">

</xml_diff>

<commit_message>
data: field/odds refresh 2026-08-10 03:52 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -465,7 +465,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
     </row>
     <row r="3">
@@ -639,7 +639,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="14">
@@ -685,7 +685,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>18</v>
+        <v>11</v>
       </c>
     </row>
     <row r="17">
@@ -855,7 +855,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="28">
@@ -1231,7 +1231,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="52">
@@ -1249,7 +1249,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="53">
@@ -1299,7 +1299,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>56</v>
+        <v>23</v>
       </c>
     </row>
     <row r="56">
@@ -1805,7 +1805,7 @@
         </is>
       </c>
       <c r="D86" t="n">
-        <v>75</v>
+        <v>79</v>
       </c>
     </row>
     <row r="87">
@@ -1869,7 +1869,7 @@
         </is>
       </c>
       <c r="D90" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="91">
@@ -2143,7 +2143,7 @@
         </is>
       </c>
       <c r="D107" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="108">
@@ -2287,7 +2287,7 @@
         </is>
       </c>
       <c r="D117" t="n">
-        <v>24</v>
+        <v>28</v>
       </c>
     </row>
     <row r="118">
@@ -2349,7 +2349,7 @@
         </is>
       </c>
       <c r="D121" t="n">
-        <v>46</v>
+        <v>49</v>
       </c>
     </row>
     <row r="122">
@@ -2367,7 +2367,7 @@
         </is>
       </c>
       <c r="D122" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="123">
@@ -2631,7 +2631,7 @@
         </is>
       </c>
       <c r="D138" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="139">
@@ -3159,7 +3159,7 @@
         </is>
       </c>
       <c r="D172" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="173">
@@ -3269,7 +3269,7 @@
         </is>
       </c>
       <c r="D179" t="n">
-        <v>15</v>
+        <v>9</v>
       </c>
     </row>
     <row r="180">
@@ -3359,7 +3359,7 @@
         </is>
       </c>
       <c r="D184" t="n">
-        <v>57</v>
+        <v>53</v>
       </c>
     </row>
     <row r="185">
@@ -3501,7 +3501,7 @@
         </is>
       </c>
       <c r="D193" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="194">
@@ -3733,7 +3733,7 @@
         </is>
       </c>
       <c r="D207" t="n">
-        <v>68</v>
+        <v>40</v>
       </c>
     </row>
     <row r="208">
@@ -4023,7 +4023,7 @@
         </is>
       </c>
       <c r="D226" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="227">
@@ -4069,7 +4069,7 @@
         </is>
       </c>
       <c r="D229" t="n">
-        <v>103</v>
+        <v>106</v>
       </c>
     </row>
     <row r="230">

</xml_diff>

<commit_message>
data: field/odds refresh 2026-08-10 08:41 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -575,7 +575,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="10">
@@ -639,7 +639,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="14">
@@ -747,7 +747,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="21">
@@ -797,7 +797,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="24">
@@ -855,7 +855,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="28">
@@ -873,7 +873,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="29">
@@ -905,7 +905,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="31">
@@ -1105,7 +1105,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
     <row r="44">
@@ -1119,7 +1119,7 @@
       </c>
       <c r="C44" t="inlineStr"/>
       <c r="D44" t="n">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
     <row r="45">
@@ -1163,7 +1163,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="48">
@@ -1281,7 +1281,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>41</v>
+        <v>44</v>
       </c>
     </row>
     <row r="55">
@@ -1299,7 +1299,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="56">
@@ -1529,7 +1529,7 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>88</v>
+        <v>77</v>
       </c>
     </row>
     <row r="70">
@@ -1559,7 +1559,7 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="72">
@@ -1769,7 +1769,7 @@
         </is>
       </c>
       <c r="D84" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="85">
@@ -1805,7 +1805,7 @@
         </is>
       </c>
       <c r="D86" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="87">
@@ -1919,7 +1919,7 @@
         </is>
       </c>
       <c r="D93" t="n">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="94">
@@ -2027,7 +2027,7 @@
         </is>
       </c>
       <c r="D100" t="n">
-        <v>51</v>
+        <v>59</v>
       </c>
     </row>
     <row r="101">
@@ -2063,7 +2063,7 @@
         </is>
       </c>
       <c r="D102" t="n">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="103">
@@ -2143,7 +2143,7 @@
         </is>
       </c>
       <c r="D107" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="108">
@@ -2205,7 +2205,7 @@
         </is>
       </c>
       <c r="D111" t="n">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="112">
@@ -2287,7 +2287,7 @@
         </is>
       </c>
       <c r="D117" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="118">
@@ -2349,7 +2349,7 @@
         </is>
       </c>
       <c r="D121" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="122">
@@ -2461,7 +2461,7 @@
         </is>
       </c>
       <c r="D128" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="129">
@@ -2515,7 +2515,7 @@
         </is>
       </c>
       <c r="D131" t="n">
-        <v>44</v>
+        <v>47</v>
       </c>
     </row>
     <row r="132">
@@ -2567,7 +2567,7 @@
         </is>
       </c>
       <c r="D134" t="n">
-        <v>72</v>
+        <v>74</v>
       </c>
     </row>
     <row r="135">
@@ -2631,7 +2631,7 @@
         </is>
       </c>
       <c r="D138" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="139">
@@ -2709,7 +2709,7 @@
         </is>
       </c>
       <c r="D143" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="144">
@@ -2963,7 +2963,7 @@
         </is>
       </c>
       <c r="D160" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="161">
@@ -3141,7 +3141,7 @@
         </is>
       </c>
       <c r="D171" t="n">
-        <v>102</v>
+        <v>105</v>
       </c>
     </row>
     <row r="172">
@@ -3359,7 +3359,7 @@
         </is>
       </c>
       <c r="D184" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="185">
@@ -3551,7 +3551,7 @@
         </is>
       </c>
       <c r="D196" t="n">
-        <v>55</v>
+        <v>58</v>
       </c>
     </row>
     <row r="197">
@@ -3565,7 +3565,7 @@
       </c>
       <c r="C197" t="inlineStr"/>
       <c r="D197" t="n">
-        <v>55</v>
+        <v>58</v>
       </c>
     </row>
     <row r="198">
@@ -3583,7 +3583,7 @@
         </is>
       </c>
       <c r="D198" t="n">
-        <v>26</v>
+        <v>29</v>
       </c>
     </row>
     <row r="199">
@@ -3661,7 +3661,7 @@
         </is>
       </c>
       <c r="D203" t="n">
-        <v>73</v>
+        <v>78</v>
       </c>
     </row>
     <row r="204">
@@ -3679,7 +3679,7 @@
         </is>
       </c>
       <c r="D204" t="n">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="205">
@@ -3697,7 +3697,7 @@
         </is>
       </c>
       <c r="D205" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="206">
@@ -3733,7 +3733,7 @@
         </is>
       </c>
       <c r="D207" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="208">
@@ -4023,7 +4023,7 @@
         </is>
       </c>
       <c r="D226" t="n">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="227">
@@ -4069,7 +4069,7 @@
         </is>
       </c>
       <c r="D229" t="n">
-        <v>106</v>
+        <v>108</v>
       </c>
     </row>
     <row r="230">

</xml_diff>

<commit_message>
data: field/odds refresh 2026-08-17 08:54 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -465,7 +465,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="3">
@@ -685,7 +685,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
     </row>
     <row r="17">
@@ -747,7 +747,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>41</v>
+        <v>38</v>
       </c>
     </row>
     <row r="21">
@@ -797,7 +797,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="24">
@@ -1249,7 +1249,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="53">
@@ -1299,7 +1299,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="56">
@@ -1335,7 +1335,7 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="58">
@@ -1417,7 +1417,7 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="63">
@@ -1453,7 +1453,7 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="65">
@@ -1621,7 +1621,7 @@
         </is>
       </c>
       <c r="D75" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="76">
@@ -1689,7 +1689,7 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>66</v>
+        <v>69</v>
       </c>
     </row>
     <row r="80">
@@ -1919,7 +1919,7 @@
         </is>
       </c>
       <c r="D93" t="n">
-        <v>73</v>
+        <v>62</v>
       </c>
     </row>
     <row r="94">
@@ -2045,7 +2045,7 @@
         </is>
       </c>
       <c r="D101" t="n">
-        <v>18</v>
+        <v>13</v>
       </c>
     </row>
     <row r="102">
@@ -2063,7 +2063,7 @@
         </is>
       </c>
       <c r="D102" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="103">
@@ -2143,7 +2143,7 @@
         </is>
       </c>
       <c r="D107" t="n">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="108">
@@ -2367,7 +2367,7 @@
         </is>
       </c>
       <c r="D122" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="123">
@@ -2425,7 +2425,7 @@
         </is>
       </c>
       <c r="D126" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="127">
@@ -2461,7 +2461,7 @@
         </is>
       </c>
       <c r="D128" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="129">
@@ -2515,7 +2515,7 @@
         </is>
       </c>
       <c r="D131" t="n">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="132">
@@ -2631,7 +2631,7 @@
         </is>
       </c>
       <c r="D138" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="139">
@@ -2709,7 +2709,7 @@
         </is>
       </c>
       <c r="D143" t="n">
-        <v>26</v>
+        <v>18</v>
       </c>
     </row>
     <row r="144">
@@ -2963,7 +2963,7 @@
         </is>
       </c>
       <c r="D160" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="161">
@@ -3049,7 +3049,7 @@
         </is>
       </c>
       <c r="D165" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="166">
@@ -3269,7 +3269,7 @@
         </is>
       </c>
       <c r="D179" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="180">
@@ -3359,7 +3359,7 @@
         </is>
       </c>
       <c r="D184" t="n">
-        <v>54</v>
+        <v>51</v>
       </c>
     </row>
     <row r="185">
@@ -3435,7 +3435,7 @@
         </is>
       </c>
       <c r="D189" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="190">
@@ -3501,7 +3501,7 @@
         </is>
       </c>
       <c r="D193" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="194">
@@ -3583,7 +3583,7 @@
         </is>
       </c>
       <c r="D198" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="199">
@@ -3679,7 +3679,7 @@
         </is>
       </c>
       <c r="D204" t="n">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="205">
@@ -3733,7 +3733,7 @@
         </is>
       </c>
       <c r="D207" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="208">
@@ -4023,7 +4023,7 @@
         </is>
       </c>
       <c r="D226" t="n">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="227">
@@ -4173,7 +4173,7 @@
         </is>
       </c>
       <c r="D235" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: field/odds refresh 2026-08-24 14:49 ET
</commit_message>
<xml_diff>
--- a/Data/in Use/All_players.xlsx
+++ b/Data/in Use/All_players.xlsx
@@ -639,7 +639,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>31</v>
+        <v>28</v>
       </c>
     </row>
     <row r="14">
@@ -685,7 +685,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="17">
@@ -747,7 +747,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>38</v>
+        <v>26</v>
       </c>
     </row>
     <row r="21">
@@ -855,7 +855,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="28">
@@ -1249,7 +1249,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="53">
@@ -1299,7 +1299,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="56">
@@ -1335,7 +1335,7 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="58">
@@ -1417,7 +1417,7 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="63">
@@ -1869,7 +1869,7 @@
         </is>
       </c>
       <c r="D90" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="91">
@@ -2063,7 +2063,7 @@
         </is>
       </c>
       <c r="D102" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="103">
@@ -2287,7 +2287,7 @@
         </is>
       </c>
       <c r="D117" t="n">
-        <v>27</v>
+        <v>31</v>
       </c>
     </row>
     <row r="118">
@@ -2367,7 +2367,7 @@
         </is>
       </c>
       <c r="D122" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="123">
@@ -2425,7 +2425,7 @@
         </is>
       </c>
       <c r="D126" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="127">
@@ -2631,7 +2631,7 @@
         </is>
       </c>
       <c r="D138" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="139">
@@ -3159,7 +3159,7 @@
         </is>
       </c>
       <c r="D172" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="173">
@@ -3269,7 +3269,7 @@
         </is>
       </c>
       <c r="D179" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="180">
@@ -3435,7 +3435,7 @@
         </is>
       </c>
       <c r="D189" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="190">
@@ -4023,7 +4023,7 @@
         </is>
       </c>
       <c r="D226" t="n">
-        <v>47</v>
+        <v>42</v>
       </c>
     </row>
     <row r="227">
@@ -4173,7 +4173,7 @@
         </is>
       </c>
       <c r="D235" t="n">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
   </sheetData>

</xml_diff>